<commit_message>
Log August 18 chest workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R75764a6ada614460"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rfa1f3eefedd54b80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rd1c1ce0774924baf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R05fc8eeffae94058"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rcfb190a300ba4b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R6ff6ec66dada4d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R40fa810806dc4b45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Raf9d0dcee54f4c3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R53b1efe2afd041f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rca1d23cdee7c4d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R915f5342e1054fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2e459d9c55d246b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra9230cdbd06c4046"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R3ad06fea062247bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rfc7f664136ea48b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R4cfe7d32addd4d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R82670c6b5c0e4732"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R925469b572994334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R15b6f11f423541bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R19774d1b30ed49c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc0fab02e29af4e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rb82c135a065249a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8e5692fc95574915"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb64eba7362274ee2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N271" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N289" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1803,7 +1803,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D42" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2494,7 +2494,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R846ba9219395484b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f461e00cc1e42fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3897,7 +3897,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4397180e14a94a52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd20978317e43470e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3975,7 +3975,7 @@
       </x:c>
       <x:c r="L3" s="140" t="n">
         <x:f>SUMIF('Session Summary'!$B$5:$B$200,K3,'Session Summary'!$C$5:$C$200)</x:f>
-        <x:v>12</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -4026,7 +4026,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4422,7 +4422,7 @@
       <x:c r="K18" s="59" t="n"/>
       <x:c r="L18" s="59" t="n"/>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="92" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Sunday</x:t>
@@ -4439,26 +4439,26 @@
           <x:t xml:space="preserve">Chest</x:t>
         </x:is>
       </x:c>
-      <x:c r="E19" s="59" t="str">
+      <x:c r="E19" s="222" t="str">
         <x:v>Flat Bench Press</x:v>
       </x:c>
-      <x:c r="F19" s="59" t="str">
+      <x:c r="F19" s="222" t="str">
         <x:v>22.5 kg/side x 7 @ RIR 1</x:v>
       </x:c>
-      <x:c r="G19" s="59" t="str">
+      <x:c r="G19" s="222" t="str">
         <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
       </x:c>
-      <x:c r="H19" s="59" t="str">
+      <x:c r="H19" s="222" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I19" s="59" t="str">
-        <x:v>Bar excluded</x:v>
+      <x:c r="I19" s="222" t="str">
+        <x:v>Bar excluded; improve reserve</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
       <x:c r="L19" s="59" t="n"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="59" t="n"/>
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
@@ -4467,20 +4467,20 @@
           <x:t xml:space="preserve">Chest</x:t>
         </x:is>
       </x:c>
-      <x:c r="E20" s="59" t="str">
+      <x:c r="E20" s="222" t="str">
         <x:v>Incline Barbell Bench</x:v>
       </x:c>
-      <x:c r="F20" s="59" t="str">
-        <x:v>15 kg/side x 8 nearly assisted</x:v>
-      </x:c>
-      <x:c r="G20" s="59" t="str">
-        <x:v>15 kg/side x 8 clean @ RIR 2</x:v>
-      </x:c>
-      <x:c r="H20" s="59" t="str">
-        <x:v>Verify clean rep</x:v>
-      </x:c>
-      <x:c r="I20" s="59" t="str">
-        <x:v>Separate from incline DB</x:v>
+      <x:c r="F20" s="222" t="str">
+        <x:v>15 kg/side x 9 @ RIR 1 clean</x:v>
+      </x:c>
+      <x:c r="G20" s="222" t="str">
+        <x:v>15 kg/side x 9 @ RIR 2</x:v>
+      </x:c>
+      <x:c r="H20" s="222" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I20" s="222" t="str">
+        <x:v>No assistance; do not add load</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4621,7 +4621,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c040a6728294c52"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ebd4c6a1f724bcc"/>
 </x:worksheet>
 </file>
 
@@ -15626,292 +15626,760 @@
       </x:c>
     </x:row>
     <x:row r="272">
-      <x:c r="A272" s="220"/>
-      <x:c r="B272" s="170"/>
-      <x:c r="C272" s="170"/>
-      <x:c r="D272" s="170"/>
-      <x:c r="E272" s="170"/>
-      <x:c r="F272" s="170"/>
-      <x:c r="G272" s="170"/>
-      <x:c r="H272" s="170"/>
-      <x:c r="I272" s="170"/>
-      <x:c r="J272" s="170"/>
-      <x:c r="K272" s="170"/>
+      <x:c r="A272" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B272" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C272" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D272" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E272" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F272" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G272" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H272" s="170" t="str">
+        <x:v>No assistance; prescribed preparation-set completion To verify</x:v>
+      </x:c>
+      <x:c r="I272" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J272" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K272" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L272" s="170"/>
-      <x:c r="M272" s="170"/>
-      <x:c r="N272" s="170"/>
+      <x:c r="M272" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N272" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="273">
-      <x:c r="A273" s="220"/>
-      <x:c r="B273" s="170"/>
-      <x:c r="C273" s="170"/>
-      <x:c r="D273" s="170"/>
-      <x:c r="E273" s="170"/>
-      <x:c r="F273" s="170"/>
-      <x:c r="G273" s="170"/>
-      <x:c r="H273" s="170"/>
-      <x:c r="I273" s="170"/>
-      <x:c r="J273" s="170"/>
-      <x:c r="K273" s="170"/>
+      <x:c r="A273" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B273" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C273" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D273" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E273" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F273" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G273" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H273" s="170" t="str">
+        <x:v>No assistance; rep target met but harder than planned</x:v>
+      </x:c>
+      <x:c r="I273" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J273" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K273" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L273" s="170"/>
-      <x:c r="M273" s="170"/>
-      <x:c r="N273" s="170"/>
+      <x:c r="M273" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N273" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="274">
-      <x:c r="A274" s="220"/>
-      <x:c r="B274" s="170"/>
-      <x:c r="C274" s="170"/>
-      <x:c r="D274" s="170"/>
-      <x:c r="E274" s="170"/>
-      <x:c r="F274" s="170"/>
-      <x:c r="G274" s="170"/>
-      <x:c r="H274" s="170"/>
-      <x:c r="I274" s="170"/>
-      <x:c r="J274" s="170"/>
-      <x:c r="K274" s="170"/>
+      <x:c r="A274" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B274" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C274" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D274" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E274" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F274" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G274" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H274" s="170" t="str">
+        <x:v>No assistance; matched prior result</x:v>
+      </x:c>
+      <x:c r="I274" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J274" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K274" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L274" s="170"/>
-      <x:c r="M274" s="170"/>
-      <x:c r="N274" s="170"/>
+      <x:c r="M274" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N274" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="275">
-      <x:c r="A275" s="220"/>
-      <x:c r="B275" s="170"/>
-      <x:c r="C275" s="170"/>
-      <x:c r="D275" s="170"/>
-      <x:c r="E275" s="170"/>
-      <x:c r="F275" s="170"/>
-      <x:c r="G275" s="170"/>
-      <x:c r="H275" s="170"/>
-      <x:c r="I275" s="170"/>
-      <x:c r="J275" s="170"/>
-      <x:c r="K275" s="170"/>
+      <x:c r="A275" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B275" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C275" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D275" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E275" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F275" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G275" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H275" s="170" t="str">
+        <x:v>No assistance; performed before plate chest press</x:v>
+      </x:c>
+      <x:c r="I275" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J275" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K275" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L275" s="170"/>
-      <x:c r="M275" s="170"/>
-      <x:c r="N275" s="170"/>
+      <x:c r="M275" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N275" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="276">
-      <x:c r="A276" s="220"/>
-      <x:c r="B276" s="170"/>
-      <x:c r="C276" s="170"/>
-      <x:c r="D276" s="170"/>
-      <x:c r="E276" s="170"/>
-      <x:c r="F276" s="170"/>
-      <x:c r="G276" s="170"/>
-      <x:c r="H276" s="170"/>
-      <x:c r="I276" s="170"/>
-      <x:c r="J276" s="170"/>
-      <x:c r="K276" s="170"/>
+      <x:c r="A276" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B276" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C276" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D276" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E276" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F276" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G276" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H276" s="170" t="str">
+        <x:v>No assistance; performed before plate chest press</x:v>
+      </x:c>
+      <x:c r="I276" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J276" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K276" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L276" s="170"/>
-      <x:c r="M276" s="170"/>
-      <x:c r="N276" s="170"/>
+      <x:c r="M276" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N276" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="277">
-      <x:c r="A277" s="220"/>
-      <x:c r="B277" s="170"/>
-      <x:c r="C277" s="170"/>
-      <x:c r="D277" s="170"/>
-      <x:c r="E277" s="170"/>
-      <x:c r="F277" s="170"/>
-      <x:c r="G277" s="170"/>
-      <x:c r="H277" s="170"/>
-      <x:c r="I277" s="170"/>
-      <x:c r="J277" s="170"/>
-      <x:c r="K277" s="170"/>
+      <x:c r="A277" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B277" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C277" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D277" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E277" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F277" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G277" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H277" s="170" t="str">
+        <x:v>No assistance; progressed from 8 nearly assisted reps to 9 clean reps</x:v>
+      </x:c>
+      <x:c r="I277" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J277" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K277" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L277" s="170"/>
-      <x:c r="M277" s="170"/>
-      <x:c r="N277" s="170"/>
+      <x:c r="M277" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N277" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="278">
-      <x:c r="A278" s="220"/>
-      <x:c r="B278" s="170"/>
-      <x:c r="C278" s="170"/>
-      <x:c r="D278" s="170"/>
-      <x:c r="E278" s="170"/>
-      <x:c r="F278" s="170"/>
-      <x:c r="G278" s="170"/>
-      <x:c r="H278" s="170"/>
-      <x:c r="I278" s="170"/>
-      <x:c r="J278" s="170"/>
-      <x:c r="K278" s="170"/>
+      <x:c r="A278" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B278" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C278" s="170" t="str">
+        <x:v>Plate Chest Press</x:v>
+      </x:c>
+      <x:c r="D278" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E278" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F278" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G278" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H278" s="170" t="str">
+        <x:v>Clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I278" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J278" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K278" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L278" s="170"/>
-      <x:c r="M278" s="170"/>
-      <x:c r="N278" s="170"/>
+      <x:c r="M278" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N278" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="279">
-      <x:c r="A279" s="220"/>
-      <x:c r="B279" s="170"/>
-      <x:c r="C279" s="170"/>
-      <x:c r="D279" s="170"/>
-      <x:c r="E279" s="170"/>
-      <x:c r="F279" s="170"/>
-      <x:c r="G279" s="170"/>
-      <x:c r="H279" s="170"/>
-      <x:c r="I279" s="170"/>
-      <x:c r="J279" s="170"/>
-      <x:c r="K279" s="170"/>
+      <x:c r="A279" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B279" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C279" s="170" t="str">
+        <x:v>Plate Chest Press</x:v>
+      </x:c>
+      <x:c r="D279" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E279" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F279" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G279" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H279" s="170" t="str">
+        <x:v>Clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I279" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J279" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K279" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L279" s="170"/>
-      <x:c r="M279" s="170"/>
-      <x:c r="N279" s="170"/>
+      <x:c r="M279" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N279" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="280">
-      <x:c r="A280" s="220"/>
-      <x:c r="B280" s="170"/>
-      <x:c r="C280" s="170"/>
-      <x:c r="D280" s="170"/>
-      <x:c r="E280" s="170"/>
-      <x:c r="F280" s="170"/>
-      <x:c r="G280" s="170"/>
-      <x:c r="H280" s="170"/>
-      <x:c r="I280" s="170"/>
-      <x:c r="J280" s="170"/>
-      <x:c r="K280" s="170"/>
+      <x:c r="A280" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B280" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C280" s="170" t="str">
+        <x:v>Plate Chest Press</x:v>
+      </x:c>
+      <x:c r="D280" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E280" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F280" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G280" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H280" s="170" t="str">
+        <x:v>New baseline; explicitly confirmed clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I280" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J280" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K280" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L280" s="170"/>
-      <x:c r="M280" s="170"/>
-      <x:c r="N280" s="170"/>
+      <x:c r="M280" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N280" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="281">
-      <x:c r="A281" s="220"/>
-      <x:c r="B281" s="170"/>
-      <x:c r="C281" s="170"/>
-      <x:c r="D281" s="170"/>
-      <x:c r="E281" s="170"/>
-      <x:c r="F281" s="170"/>
-      <x:c r="G281" s="170"/>
-      <x:c r="H281" s="170"/>
-      <x:c r="I281" s="170"/>
-      <x:c r="J281" s="170"/>
-      <x:c r="K281" s="170"/>
+      <x:c r="A281" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B281" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C281" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D281" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E281" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F281" s="170" t="str">
+        <x:v>kg total machine stack</x:v>
+      </x:c>
+      <x:c r="G281" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H281" s="170" t="str">
+        <x:v>No assistance reported</x:v>
+      </x:c>
+      <x:c r="I281" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J281" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K281" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L281" s="170"/>
-      <x:c r="M281" s="170"/>
-      <x:c r="N281" s="170"/>
+      <x:c r="M281" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N281" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="282">
-      <x:c r="A282" s="220"/>
-      <x:c r="B282" s="170"/>
-      <x:c r="C282" s="170"/>
-      <x:c r="D282" s="170"/>
-      <x:c r="E282" s="170"/>
-      <x:c r="F282" s="170"/>
-      <x:c r="G282" s="170"/>
-      <x:c r="H282" s="170"/>
-      <x:c r="I282" s="170"/>
-      <x:c r="J282" s="170"/>
-      <x:c r="K282" s="170"/>
+      <x:c r="A282" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B282" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C282" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D282" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E282" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F282" s="170" t="str">
+        <x:v>kg total machine stack</x:v>
+      </x:c>
+      <x:c r="G282" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H282" s="170" t="str">
+        <x:v>No assistance reported</x:v>
+      </x:c>
+      <x:c r="I282" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J282" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K282" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L282" s="170"/>
-      <x:c r="M282" s="170"/>
-      <x:c r="N282" s="170"/>
+      <x:c r="M282" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N282" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="283">
-      <x:c r="A283" s="220"/>
-      <x:c r="B283" s="170"/>
-      <x:c r="C283" s="170"/>
-      <x:c r="D283" s="170"/>
-      <x:c r="E283" s="170"/>
-      <x:c r="F283" s="170"/>
-      <x:c r="G283" s="170"/>
-      <x:c r="H283" s="170"/>
-      <x:c r="I283" s="170"/>
-      <x:c r="J283" s="170"/>
-      <x:c r="K283" s="170"/>
+      <x:c r="A283" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B283" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C283" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D283" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E283" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F283" s="170" t="str">
+        <x:v>kg total machine stack</x:v>
+      </x:c>
+      <x:c r="G283" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H283" s="170" t="str">
+        <x:v>Progressed from 11 to 12 reps; no assistance</x:v>
+      </x:c>
+      <x:c r="I283" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J283" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K283" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L283" s="170"/>
-      <x:c r="M283" s="170"/>
-      <x:c r="N283" s="170"/>
+      <x:c r="M283" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N283" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="284">
-      <x:c r="A284" s="220"/>
-      <x:c r="B284" s="170"/>
-      <x:c r="C284" s="170"/>
-      <x:c r="D284" s="170"/>
-      <x:c r="E284" s="170"/>
-      <x:c r="F284" s="170"/>
-      <x:c r="G284" s="170"/>
-      <x:c r="H284" s="170"/>
-      <x:c r="I284" s="170"/>
-      <x:c r="J284" s="170"/>
-      <x:c r="K284" s="170"/>
+      <x:c r="A284" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B284" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C284" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="D284" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E284" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F284" s="170" t="str">
+        <x:v>kg each side; conventional horizontal path</x:v>
+      </x:c>
+      <x:c r="G284" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H284" s="170" t="str">
+        <x:v>No assistance; load now too light for efficient working use</x:v>
+      </x:c>
+      <x:c r="I284" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J284" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K284" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L284" s="170"/>
-      <x:c r="M284" s="170"/>
-      <x:c r="N284" s="170"/>
+      <x:c r="M284" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N284" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="285">
-      <x:c r="A285" s="220"/>
-      <x:c r="B285" s="170"/>
-      <x:c r="C285" s="170"/>
-      <x:c r="D285" s="170"/>
-      <x:c r="E285" s="170"/>
-      <x:c r="F285" s="170"/>
-      <x:c r="G285" s="170"/>
-      <x:c r="H285" s="170"/>
-      <x:c r="I285" s="170"/>
-      <x:c r="J285" s="170"/>
-      <x:c r="K285" s="170"/>
+      <x:c r="A285" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B285" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C285" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="D285" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E285" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F285" s="170" t="str">
+        <x:v>kg each side; conventional horizontal path</x:v>
+      </x:c>
+      <x:c r="G285" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H285" s="170" t="str">
+        <x:v>No assistance; controlled-form detail To verify</x:v>
+      </x:c>
+      <x:c r="I285" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J285" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K285" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L285" s="170"/>
-      <x:c r="M285" s="170"/>
-      <x:c r="N285" s="170"/>
+      <x:c r="M285" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N285" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="286">
-      <x:c r="A286" s="220"/>
-      <x:c r="B286" s="170"/>
-      <x:c r="C286" s="170"/>
-      <x:c r="D286" s="170"/>
-      <x:c r="E286" s="170"/>
-      <x:c r="F286" s="170"/>
-      <x:c r="G286" s="170"/>
-      <x:c r="H286" s="170"/>
-      <x:c r="I286" s="170"/>
-      <x:c r="J286" s="170"/>
-      <x:c r="K286" s="170"/>
+      <x:c r="A286" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B286" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C286" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="D286" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E286" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F286" s="170" t="str">
+        <x:v>kg each side; conventional horizontal path</x:v>
+      </x:c>
+      <x:c r="G286" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H286" s="170" t="str">
+        <x:v>No assistance; progressed from 10 to 12 reps</x:v>
+      </x:c>
+      <x:c r="I286" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J286" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K286" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L286" s="170"/>
-      <x:c r="M286" s="170"/>
-      <x:c r="N286" s="170"/>
+      <x:c r="M286" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N286" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="287">
-      <x:c r="A287" s="220"/>
-      <x:c r="B287" s="170"/>
-      <x:c r="C287" s="170"/>
-      <x:c r="D287" s="170"/>
-      <x:c r="E287" s="170"/>
-      <x:c r="F287" s="170"/>
-      <x:c r="G287" s="170"/>
-      <x:c r="H287" s="170"/>
-      <x:c r="I287" s="170"/>
-      <x:c r="J287" s="170"/>
-      <x:c r="K287" s="170"/>
+      <x:c r="A287" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B287" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C287" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="D287" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E287" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="F287" s="170" t="str">
+        <x:v>seconds</x:v>
+      </x:c>
+      <x:c r="G287" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H287" s="170" t="str">
+        <x:v>Strict completion; no hip sag or lower-back discomfort</x:v>
+      </x:c>
+      <x:c r="I287" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J287" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K287" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L287" s="170"/>
-      <x:c r="M287" s="170"/>
-      <x:c r="N287" s="170"/>
+      <x:c r="M287" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="N287" s="170" t="str">
+        <x:v>To verify</x:v>
+      </x:c>
     </x:row>
     <x:row r="288">
-      <x:c r="A288" s="220"/>
-      <x:c r="B288" s="170"/>
-      <x:c r="C288" s="170"/>
-      <x:c r="D288" s="170"/>
-      <x:c r="E288" s="170"/>
-      <x:c r="F288" s="170"/>
-      <x:c r="G288" s="170"/>
-      <x:c r="H288" s="170"/>
-      <x:c r="I288" s="170"/>
-      <x:c r="J288" s="170"/>
-      <x:c r="K288" s="170"/>
+      <x:c r="A288" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B288" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C288" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="D288" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E288" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="F288" s="170" t="str">
+        <x:v>seconds</x:v>
+      </x:c>
+      <x:c r="G288" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H288" s="170" t="str">
+        <x:v>Strict completion; no hip sag or lower-back discomfort</x:v>
+      </x:c>
+      <x:c r="I288" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J288" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K288" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L288" s="170"/>
-      <x:c r="M288" s="170"/>
-      <x:c r="N288" s="170"/>
+      <x:c r="M288" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="N288" s="170" t="str">
+        <x:v>To verify</x:v>
+      </x:c>
     </x:row>
     <x:row r="289">
-      <x:c r="A289" s="220"/>
-      <x:c r="B289" s="170"/>
-      <x:c r="C289" s="170"/>
-      <x:c r="D289" s="170"/>
-      <x:c r="E289" s="170"/>
-      <x:c r="F289" s="170"/>
-      <x:c r="G289" s="170"/>
-      <x:c r="H289" s="170"/>
-      <x:c r="I289" s="170"/>
-      <x:c r="J289" s="170"/>
-      <x:c r="K289" s="170"/>
+      <x:c r="A289" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B289" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C289" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="D289" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E289" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="F289" s="170" t="str">
+        <x:v>seconds</x:v>
+      </x:c>
+      <x:c r="G289" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H289" s="170" t="str">
+        <x:v>Strict completion; no hip sag or lower-back discomfort</x:v>
+      </x:c>
+      <x:c r="I289" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable-fly set; exact side and resolution To verify</x:v>
+      </x:c>
+      <x:c r="J289" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="K289" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L289" s="170"/>
-      <x:c r="M289" s="170"/>
-      <x:c r="N289" s="170"/>
+      <x:c r="M289" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="N289" s="170" t="str">
+        <x:v>To verify</x:v>
+      </x:c>
     </x:row>
     <x:row r="290">
       <x:c r="A290" s="220"/>
@@ -16088,6 +16556,326 @@
       <x:c r="L300" s="170"/>
       <x:c r="M300" s="170"/>
       <x:c r="N300" s="170"/>
+    </x:row>
+    <x:row r="301">
+      <x:c r="A301" s="220"/>
+      <x:c r="B301" s="170"/>
+      <x:c r="C301" s="170"/>
+      <x:c r="D301" s="170"/>
+      <x:c r="E301" s="170"/>
+      <x:c r="F301" s="170"/>
+      <x:c r="G301" s="170"/>
+      <x:c r="H301" s="170"/>
+      <x:c r="I301" s="170"/>
+      <x:c r="J301" s="170"/>
+      <x:c r="K301" s="170"/>
+      <x:c r="L301" s="170"/>
+      <x:c r="M301" s="170"/>
+      <x:c r="N301" s="170"/>
+    </x:row>
+    <x:row r="302">
+      <x:c r="A302" s="220"/>
+      <x:c r="B302" s="170"/>
+      <x:c r="C302" s="170"/>
+      <x:c r="D302" s="170"/>
+      <x:c r="E302" s="170"/>
+      <x:c r="F302" s="170"/>
+      <x:c r="G302" s="170"/>
+      <x:c r="H302" s="170"/>
+      <x:c r="I302" s="170"/>
+      <x:c r="J302" s="170"/>
+      <x:c r="K302" s="170"/>
+      <x:c r="L302" s="170"/>
+      <x:c r="M302" s="170"/>
+      <x:c r="N302" s="170"/>
+    </x:row>
+    <x:row r="303">
+      <x:c r="A303" s="220"/>
+      <x:c r="B303" s="170"/>
+      <x:c r="C303" s="170"/>
+      <x:c r="D303" s="170"/>
+      <x:c r="E303" s="170"/>
+      <x:c r="F303" s="170"/>
+      <x:c r="G303" s="170"/>
+      <x:c r="H303" s="170"/>
+      <x:c r="I303" s="170"/>
+      <x:c r="J303" s="170"/>
+      <x:c r="K303" s="170"/>
+      <x:c r="L303" s="170"/>
+      <x:c r="M303" s="170"/>
+      <x:c r="N303" s="170"/>
+    </x:row>
+    <x:row r="304">
+      <x:c r="A304" s="220"/>
+      <x:c r="B304" s="170"/>
+      <x:c r="C304" s="170"/>
+      <x:c r="D304" s="170"/>
+      <x:c r="E304" s="170"/>
+      <x:c r="F304" s="170"/>
+      <x:c r="G304" s="170"/>
+      <x:c r="H304" s="170"/>
+      <x:c r="I304" s="170"/>
+      <x:c r="J304" s="170"/>
+      <x:c r="K304" s="170"/>
+      <x:c r="L304" s="170"/>
+      <x:c r="M304" s="170"/>
+      <x:c r="N304" s="170"/>
+    </x:row>
+    <x:row r="305">
+      <x:c r="A305" s="220"/>
+      <x:c r="B305" s="170"/>
+      <x:c r="C305" s="170"/>
+      <x:c r="D305" s="170"/>
+      <x:c r="E305" s="170"/>
+      <x:c r="F305" s="170"/>
+      <x:c r="G305" s="170"/>
+      <x:c r="H305" s="170"/>
+      <x:c r="I305" s="170"/>
+      <x:c r="J305" s="170"/>
+      <x:c r="K305" s="170"/>
+      <x:c r="L305" s="170"/>
+      <x:c r="M305" s="170"/>
+      <x:c r="N305" s="170"/>
+    </x:row>
+    <x:row r="306">
+      <x:c r="A306" s="220"/>
+      <x:c r="B306" s="170"/>
+      <x:c r="C306" s="170"/>
+      <x:c r="D306" s="170"/>
+      <x:c r="E306" s="170"/>
+      <x:c r="F306" s="170"/>
+      <x:c r="G306" s="170"/>
+      <x:c r="H306" s="170"/>
+      <x:c r="I306" s="170"/>
+      <x:c r="J306" s="170"/>
+      <x:c r="K306" s="170"/>
+      <x:c r="L306" s="170"/>
+      <x:c r="M306" s="170"/>
+      <x:c r="N306" s="170"/>
+    </x:row>
+    <x:row r="307">
+      <x:c r="A307" s="220"/>
+      <x:c r="B307" s="170"/>
+      <x:c r="C307" s="170"/>
+      <x:c r="D307" s="170"/>
+      <x:c r="E307" s="170"/>
+      <x:c r="F307" s="170"/>
+      <x:c r="G307" s="170"/>
+      <x:c r="H307" s="170"/>
+      <x:c r="I307" s="170"/>
+      <x:c r="J307" s="170"/>
+      <x:c r="K307" s="170"/>
+      <x:c r="L307" s="170"/>
+      <x:c r="M307" s="170"/>
+      <x:c r="N307" s="170"/>
+    </x:row>
+    <x:row r="308">
+      <x:c r="A308" s="220"/>
+      <x:c r="B308" s="170"/>
+      <x:c r="C308" s="170"/>
+      <x:c r="D308" s="170"/>
+      <x:c r="E308" s="170"/>
+      <x:c r="F308" s="170"/>
+      <x:c r="G308" s="170"/>
+      <x:c r="H308" s="170"/>
+      <x:c r="I308" s="170"/>
+      <x:c r="J308" s="170"/>
+      <x:c r="K308" s="170"/>
+      <x:c r="L308" s="170"/>
+      <x:c r="M308" s="170"/>
+      <x:c r="N308" s="170"/>
+    </x:row>
+    <x:row r="309">
+      <x:c r="A309" s="220"/>
+      <x:c r="B309" s="170"/>
+      <x:c r="C309" s="170"/>
+      <x:c r="D309" s="170"/>
+      <x:c r="E309" s="170"/>
+      <x:c r="F309" s="170"/>
+      <x:c r="G309" s="170"/>
+      <x:c r="H309" s="170"/>
+      <x:c r="I309" s="170"/>
+      <x:c r="J309" s="170"/>
+      <x:c r="K309" s="170"/>
+      <x:c r="L309" s="170"/>
+      <x:c r="M309" s="170"/>
+      <x:c r="N309" s="170"/>
+    </x:row>
+    <x:row r="310">
+      <x:c r="A310" s="220"/>
+      <x:c r="B310" s="170"/>
+      <x:c r="C310" s="170"/>
+      <x:c r="D310" s="170"/>
+      <x:c r="E310" s="170"/>
+      <x:c r="F310" s="170"/>
+      <x:c r="G310" s="170"/>
+      <x:c r="H310" s="170"/>
+      <x:c r="I310" s="170"/>
+      <x:c r="J310" s="170"/>
+      <x:c r="K310" s="170"/>
+      <x:c r="L310" s="170"/>
+      <x:c r="M310" s="170"/>
+      <x:c r="N310" s="170"/>
+    </x:row>
+    <x:row r="311">
+      <x:c r="A311" s="220"/>
+      <x:c r="B311" s="170"/>
+      <x:c r="C311" s="170"/>
+      <x:c r="D311" s="170"/>
+      <x:c r="E311" s="170"/>
+      <x:c r="F311" s="170"/>
+      <x:c r="G311" s="170"/>
+      <x:c r="H311" s="170"/>
+      <x:c r="I311" s="170"/>
+      <x:c r="J311" s="170"/>
+      <x:c r="K311" s="170"/>
+      <x:c r="L311" s="170"/>
+      <x:c r="M311" s="170"/>
+      <x:c r="N311" s="170"/>
+    </x:row>
+    <x:row r="312">
+      <x:c r="A312" s="220"/>
+      <x:c r="B312" s="170"/>
+      <x:c r="C312" s="170"/>
+      <x:c r="D312" s="170"/>
+      <x:c r="E312" s="170"/>
+      <x:c r="F312" s="170"/>
+      <x:c r="G312" s="170"/>
+      <x:c r="H312" s="170"/>
+      <x:c r="I312" s="170"/>
+      <x:c r="J312" s="170"/>
+      <x:c r="K312" s="170"/>
+      <x:c r="L312" s="170"/>
+      <x:c r="M312" s="170"/>
+      <x:c r="N312" s="170"/>
+    </x:row>
+    <x:row r="313">
+      <x:c r="A313" s="220"/>
+      <x:c r="B313" s="170"/>
+      <x:c r="C313" s="170"/>
+      <x:c r="D313" s="170"/>
+      <x:c r="E313" s="170"/>
+      <x:c r="F313" s="170"/>
+      <x:c r="G313" s="170"/>
+      <x:c r="H313" s="170"/>
+      <x:c r="I313" s="170"/>
+      <x:c r="J313" s="170"/>
+      <x:c r="K313" s="170"/>
+      <x:c r="L313" s="170"/>
+      <x:c r="M313" s="170"/>
+      <x:c r="N313" s="170"/>
+    </x:row>
+    <x:row r="314">
+      <x:c r="A314" s="220"/>
+      <x:c r="B314" s="170"/>
+      <x:c r="C314" s="170"/>
+      <x:c r="D314" s="170"/>
+      <x:c r="E314" s="170"/>
+      <x:c r="F314" s="170"/>
+      <x:c r="G314" s="170"/>
+      <x:c r="H314" s="170"/>
+      <x:c r="I314" s="170"/>
+      <x:c r="J314" s="170"/>
+      <x:c r="K314" s="170"/>
+      <x:c r="L314" s="170"/>
+      <x:c r="M314" s="170"/>
+      <x:c r="N314" s="170"/>
+    </x:row>
+    <x:row r="315">
+      <x:c r="A315" s="220"/>
+      <x:c r="B315" s="170"/>
+      <x:c r="C315" s="170"/>
+      <x:c r="D315" s="170"/>
+      <x:c r="E315" s="170"/>
+      <x:c r="F315" s="170"/>
+      <x:c r="G315" s="170"/>
+      <x:c r="H315" s="170"/>
+      <x:c r="I315" s="170"/>
+      <x:c r="J315" s="170"/>
+      <x:c r="K315" s="170"/>
+      <x:c r="L315" s="170"/>
+      <x:c r="M315" s="170"/>
+      <x:c r="N315" s="170"/>
+    </x:row>
+    <x:row r="316">
+      <x:c r="A316" s="220"/>
+      <x:c r="B316" s="170"/>
+      <x:c r="C316" s="170"/>
+      <x:c r="D316" s="170"/>
+      <x:c r="E316" s="170"/>
+      <x:c r="F316" s="170"/>
+      <x:c r="G316" s="170"/>
+      <x:c r="H316" s="170"/>
+      <x:c r="I316" s="170"/>
+      <x:c r="J316" s="170"/>
+      <x:c r="K316" s="170"/>
+      <x:c r="L316" s="170"/>
+      <x:c r="M316" s="170"/>
+      <x:c r="N316" s="170"/>
+    </x:row>
+    <x:row r="317">
+      <x:c r="A317" s="220"/>
+      <x:c r="B317" s="170"/>
+      <x:c r="C317" s="170"/>
+      <x:c r="D317" s="170"/>
+      <x:c r="E317" s="170"/>
+      <x:c r="F317" s="170"/>
+      <x:c r="G317" s="170"/>
+      <x:c r="H317" s="170"/>
+      <x:c r="I317" s="170"/>
+      <x:c r="J317" s="170"/>
+      <x:c r="K317" s="170"/>
+      <x:c r="L317" s="170"/>
+      <x:c r="M317" s="170"/>
+      <x:c r="N317" s="170"/>
+    </x:row>
+    <x:row r="318">
+      <x:c r="A318" s="220"/>
+      <x:c r="B318" s="170"/>
+      <x:c r="C318" s="170"/>
+      <x:c r="D318" s="170"/>
+      <x:c r="E318" s="170"/>
+      <x:c r="F318" s="170"/>
+      <x:c r="G318" s="170"/>
+      <x:c r="H318" s="170"/>
+      <x:c r="I318" s="170"/>
+      <x:c r="J318" s="170"/>
+      <x:c r="K318" s="170"/>
+      <x:c r="L318" s="170"/>
+      <x:c r="M318" s="170"/>
+      <x:c r="N318" s="170"/>
+    </x:row>
+    <x:row r="319">
+      <x:c r="A319" s="220"/>
+      <x:c r="B319" s="170"/>
+      <x:c r="C319" s="170"/>
+      <x:c r="D319" s="170"/>
+      <x:c r="E319" s="170"/>
+      <x:c r="F319" s="170"/>
+      <x:c r="G319" s="170"/>
+      <x:c r="H319" s="170"/>
+      <x:c r="I319" s="170"/>
+      <x:c r="J319" s="170"/>
+      <x:c r="K319" s="170"/>
+      <x:c r="L319" s="170"/>
+      <x:c r="M319" s="170"/>
+      <x:c r="N319" s="170"/>
+    </x:row>
+    <x:row r="320">
+      <x:c r="A320" s="220"/>
+      <x:c r="B320" s="170"/>
+      <x:c r="C320" s="170"/>
+      <x:c r="D320" s="170"/>
+      <x:c r="E320" s="170"/>
+      <x:c r="F320" s="170"/>
+      <x:c r="G320" s="170"/>
+      <x:c r="H320" s="170"/>
+      <x:c r="I320" s="170"/>
+      <x:c r="J320" s="170"/>
+      <x:c r="K320" s="170"/>
+      <x:c r="L320" s="170"/>
+      <x:c r="M320" s="170"/>
+      <x:c r="N320" s="170"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -16121,7 +16909,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d9b2c83e1d34293"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbac0593a15924b20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16341,7 +17129,7 @@
         <x:v>Do not use 55 kg yet</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" ht="40" hidden="0" customHeight="1">
       <x:c r="A9" s="222" t="str">
         <x:v>Chest</x:v>
       </x:c>
@@ -16352,13 +17140,13 @@
         <x:v>22.5 kg/side x 7 @ RIR 1</x:v>
       </x:c>
       <x:c r="D9" s="222" t="str">
-        <x:v>20-22.5 kg/side</x:v>
+        <x:v>17.5-22.5 kg/side</x:v>
       </x:c>
       <x:c r="E9" s="222" t="str">
         <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
       </x:c>
       <x:c r="F9" s="222" t="str">
-        <x:v>Add reps before load</x:v>
+        <x:v>Improve reserve; add rep before load</x:v>
       </x:c>
       <x:c r="G9" s="222" t="str">
         <x:v>Shoulder blades set</x:v>
@@ -16367,10 +17155,10 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I9" s="222" t="str">
-        <x:v>Bar excluded</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+        <x:v>20 kg/side x 10 reached only RIR 1; bar excluded</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="40" hidden="0" customHeight="1">
       <x:c r="A10" s="222" t="str">
         <x:v>Chest</x:v>
       </x:c>
@@ -16399,7 +17187,7 @@
         <x:v>Each dumbbell</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+    <x:row r="11" ht="40" hidden="0" customHeight="1">
       <x:c r="A11" s="222" t="str">
         <x:v>Chest</x:v>
       </x:c>
@@ -16407,16 +17195,16 @@
         <x:v>Plate Chest Press</x:v>
       </x:c>
       <x:c r="C11" s="222" t="str">
-        <x:v>40 kg/side x 10 @ RIR 1</x:v>
+        <x:v>45 kg/side x 8 @ RIR 1 clean</x:v>
       </x:c>
       <x:c r="D11" s="222" t="str">
-        <x:v>30-40 kg/side</x:v>
+        <x:v>30-45 kg/side</x:v>
       </x:c>
       <x:c r="E11" s="222" t="str">
-        <x:v>40 kg/side x 10-11 @ RIR 2</x:v>
+        <x:v>45 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F11" s="222" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Add clean rep with reserve</x:v>
       </x:c>
       <x:c r="G11" s="222" t="str">
         <x:v>Controlled eccentric</x:v>
@@ -16425,10 +17213,10 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I11" s="222" t="str">
-        <x:v>Use as one of maximum 3 presses</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>New 45 kg/side baseline; clean and unassisted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="40" hidden="0" customHeight="1">
       <x:c r="A12" s="222" t="str">
         <x:v>Chest</x:v>
       </x:c>
@@ -16436,28 +17224,28 @@
         <x:v>Cable Fly</x:v>
       </x:c>
       <x:c r="C12" s="222" t="str">
-        <x:v>25 kg/side x 10 @ RIR 2</x:v>
+        <x:v>25 kg/side x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D12" s="222" t="str">
-        <x:v>15-25 kg/side</x:v>
+        <x:v>20-25 kg/side</x:v>
       </x:c>
       <x:c r="E12" s="222" t="str">
-        <x:v>25 kg/side x 11-12 @ RIR 2</x:v>
+        <x:v>25 kg/side x 12 for 2 sets @ RIR 2</x:v>
       </x:c>
       <x:c r="F12" s="222" t="str">
-        <x:v>Add clean reps</x:v>
+        <x:v>Remove 15 kg working set; build second top set</x:v>
       </x:c>
       <x:c r="G12" s="222" t="str">
-        <x:v>Hugging arc</x:v>
+        <x:v>Soft elbow bend; hugging arc</x:v>
       </x:c>
       <x:c r="H12" s="222" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I12" s="222" t="str">
-        <x:v>Clean form confirmed on 2026-08-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+        <x:v>20 kg x 15-18 @ RIR 3, then two 25 kg sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="40" hidden="0" customHeight="1">
       <x:c r="A13" s="222" t="str">
         <x:v>Chest</x:v>
       </x:c>
@@ -16465,25 +17253,25 @@
         <x:v>Pec Deck Fly</x:v>
       </x:c>
       <x:c r="C13" s="222" t="str">
-        <x:v>55 kg x 11 @ RIR 1</x:v>
+        <x:v>55 kg x 12 @ RIR 1</x:v>
       </x:c>
       <x:c r="D13" s="222" t="str">
         <x:v>45-55 kg</x:v>
       </x:c>
       <x:c r="E13" s="222" t="str">
-        <x:v>55 kg x 11 @ RIR 2</x:v>
+        <x:v>55 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F13" s="222" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Improve reserve; no load increase</x:v>
       </x:c>
       <x:c r="G13" s="222" t="str">
-        <x:v>Slow stretch</x:v>
+        <x:v>Slow stretch; shoulders controlled</x:v>
       </x:c>
       <x:c r="H13" s="222" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I13" s="222" t="str">
-        <x:v>No load increase</x:v>
+        <x:v>Build reserve before load</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -17241,7 +18029,7 @@
         <x:v>+20 kg required pause and caused lower-back pump</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="34" customHeight="1">
+    <x:row r="41" ht="40" customHeight="1">
       <x:c r="A41" s="170" t="str">
         <x:v>Chest</x:v>
       </x:c>
@@ -17249,25 +18037,25 @@
         <x:v>Incline Barbell Bench Press</x:v>
       </x:c>
       <x:c r="C41" s="170" t="str">
-        <x:v>15 kg/side x 8 @ RIR 1; nearly assisted</x:v>
+        <x:v>15 kg/side x 9 @ RIR 1; unassisted</x:v>
       </x:c>
       <x:c r="D41" s="170" t="str">
         <x:v>10-15 kg/side</x:v>
       </x:c>
       <x:c r="E41" s="170" t="str">
-        <x:v>15 kg/side x 8 clean @ RIR 2</x:v>
+        <x:v>15 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F41" s="170" t="str">
-        <x:v>Repeat clean before progression</x:v>
+        <x:v>Improve reserve before load</x:v>
       </x:c>
       <x:c r="G41" s="170" t="str">
         <x:v>Controlled bar path</x:v>
       </x:c>
       <x:c r="H41" s="170" t="str">
-        <x:v>Verify clean rep</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I41" s="170" t="str">
-        <x:v>Bar excluded; separate from incline dumbbells</x:v>
+        <x:v>Bar excluded; 12.5 kg/side target remains 12 reps</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -17384,6 +18172,35 @@
       </x:c>
       <x:c r="I45" s="170" t="str">
         <x:v>Grip and exact effective stack To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="36" customHeight="1">
+      <x:c r="A46" s="170" t="str">
+        <x:v>Core</x:v>
+      </x:c>
+      <x:c r="B46" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="C46" s="170" t="str">
+        <x:v>3 x 60 sec strict</x:v>
+      </x:c>
+      <x:c r="D46" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="E46" s="170" t="str">
+        <x:v>3 x 60 sec strict</x:v>
+      </x:c>
+      <x:c r="F46" s="170" t="str">
+        <x:v>Add time only after perfect sets</x:v>
+      </x:c>
+      <x:c r="G46" s="170" t="str">
+        <x:v>Glutes tight; ribs down; no hip sag</x:v>
+      </x:c>
+      <x:c r="H46" s="170" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I46" s="170" t="str">
+        <x:v>No lower-back discomfort reported</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17411,7 +18228,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf08a17980afc45af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fce9c7079fd4d07"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18032,16 +18849,28 @@
       <x:c r="Q17" s="59" t="n"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="220"/>
+      <x:c r="A18" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
       <x:c r="B18" s="170"/>
       <x:c r="C18" s="170"/>
-      <x:c r="D18" s="170"/>
-      <x:c r="E18" s="170"/>
-      <x:c r="F18" s="170"/>
+      <x:c r="D18" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E18" s="170" t="str">
+        <x:v>Medium to low final</x:v>
+      </x:c>
+      <x:c r="F18" s="170" t="str">
+        <x:v>No pain; little lower-biceps pump after final cable fly</x:v>
+      </x:c>
       <x:c r="G18" s="170"/>
       <x:c r="H18" s="170"/>
-      <x:c r="I18" s="170"/>
-      <x:c r="J18" s="170"/>
+      <x:c r="I18" s="170" t="str">
+        <x:v>Chest workout - 90 min; medium chest pump; 3 x 60-sec strict plank</x:v>
+      </x:c>
+      <x:c r="J18" s="170" t="str">
+        <x:v>Full EAA+ scoop; no black coffee; no assisted reps; lower-biceps pump side and resolution To verify</x:v>
+      </x:c>
       <x:c r="K18" s="59" t="n"/>
       <x:c r="L18" s="59" t="n"/>
       <x:c r="M18" s="59" t="n"/>
@@ -21564,7 +22393,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56763b828aab4199"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cd96f6502da4a20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22229,13 +23058,27 @@
         <x:v>Keep product labels and serving weights To verify; do not count unquantified lentils, sabji, fruit or salad yet</x:v>
       </x:c>
     </x:row>
+    <x:row r="43" ht="46" customHeight="1">
+      <x:c r="A43" s="170" t="str">
+        <x:v>Chest volume cap applied</x:v>
+      </x:c>
+      <x:c r="B43" s="170" t="str">
+        <x:v>The 2026-08-18 Chest session used exactly 15 direct sets plus three 60-second plank sets with no assistance</x:v>
+      </x:c>
+      <x:c r="C43" s="170" t="str">
+        <x:v>Multiple exercises progressed while final energy still fell to Medium-Low</x:v>
+      </x:c>
+      <x:c r="D43" s="170" t="str">
+        <x:v>Retain the 15-set chest cap, improve RIR before load, and keep core work separate</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5e7774955c24736"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R021c79b3fe284834"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22697,14 +23540,30 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="220"/>
-      <x:c r="B18" s="170"/>
-      <x:c r="C18" s="170"/>
-      <x:c r="D18" s="170"/>
-      <x:c r="E18" s="170"/>
-      <x:c r="F18" s="170"/>
-      <x:c r="G18" s="170"/>
-      <x:c r="H18" s="170"/>
+      <x:c r="A18" s="220" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="B18" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C18" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D18" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E18" s="170" t="str">
+        <x:v>Green</x:v>
+      </x:c>
+      <x:c r="F18" s="170" t="str">
+        <x:v>Good sleep; Medium start and Medium-Low final energy; no pain; little lower-biceps pump after final cable fly; medium chest pump; 90 min; no assistance; full EAA+; no coffee; three strict 60-sec planks</x:v>
+      </x:c>
+      <x:c r="G18" s="170" t="str">
+        <x:v>Exactly 15 direct chest sets plus 3 core sets. Incline press, plate press, pec deck and cable fly progressed; flat-bench top set remained unchanged and several early sets were harder than planned.</x:v>
+      </x:c>
+      <x:c r="H18" s="170" t="str">
+        <x:v>Retain 15 direct sets; improve reserve before load; remove 15 kg cable-fly working set; keep 3 x 60-sec strict planks</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="220"/>
@@ -22788,7 +23647,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fd07f3864364cf3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6e29a6a9e26496c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22965,13 +23824,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>No joint pain reported through 2026-08-17. Lower-back muscular pump occurred after an unprescribed +20 kg hyperextension set at RIR 0; no pain.</x:v>
+        <x:v>No joint pain reported through 2026-08-18. A little lower-biceps pump followed the final cable-fly set; exact side and resolution remain To verify.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Continue pre-workout checks; avoid +20 kg hyperextensions next session</x:v>
+        <x:v>Check that the lower-biceps pump resolved before Biceps training</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -23153,13 +24012,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Completed Back on 2026-08-17 in the retained one-body-part split. Next session follows the same split unless Vipin activates the researched Push-Pull-Legs hybrid.</x:v>
+        <x:v>Completed Chest on 2026-08-18 in the retained one-body-part split. Biceps is next, subject to fresh readiness and confirmation that the lower-biceps pump resolved.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Confirm readiness before the next scheduled muscle group</x:v>
+        <x:v>Collect fresh readiness before Biceps</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -23359,7 +24218,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a6764b7c84d4fb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8cfdcf5bf5645ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24462,10 +25321,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37edcd4733a54fb8"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R117f4939ea7c4a3b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a2518aa547a4463"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc122579941814979"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R682b7c492aa34733"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2ff5ff7e7924666"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dc8801c9e59463d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R010627ed54b64ea0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 19 biceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2e459d9c55d246b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra9230cdbd06c4046"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R3ad06fea062247bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rfc7f664136ea48b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R4cfe7d32addd4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R82670c6b5c0e4732"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R925469b572994334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R15b6f11f423541bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R19774d1b30ed49c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc0fab02e29af4e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rb82c135a065249a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra92fbd93b1654c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R3b0a901b44974167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rc74109d616184261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rd4a1850083ed4aab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rf614fde1278e47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Reb512a2733a2429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rd5487c6d211f48c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R06cfe3edd064486f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R74ab6b3ad2ec4fb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R0886202db97e489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rb4aa6ceadcc24db4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1703,13 +1703,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>42</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb64eba7362274ee2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf91945eabb754020"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N289" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N307" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1767,7 +1767,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="PhotoMeasurementTable" displayName="PhotoMeasurementTable" ref="A4:K6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="PhotoMeasurementTable" displayName="PhotoMeasurementTable" ref="A4:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1803,7 +1803,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2479,6 +2479,35 @@
         <x:v>To verify</x:v>
       </x:c>
     </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="220" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B7" s="223" t="n">
+        <x:v>88.3</x:v>
+      </x:c>
+      <x:c r="C7" s="223" t="n">
+        <x:v>96.5</x:v>
+      </x:c>
+      <x:c r="D7" s="223"/>
+      <x:c r="E7" s="223"/>
+      <x:c r="F7" s="223"/>
+      <x:c r="G7" s="170" t="str">
+        <x:v>To link</x:v>
+      </x:c>
+      <x:c r="H7" s="170" t="str">
+        <x:v>To link</x:v>
+      </x:c>
+      <x:c r="I7" s="170" t="str">
+        <x:v>To link</x:v>
+      </x:c>
+      <x:c r="J7" s="170" t="str">
+        <x:v>Verified standardized Sunday measurement: after bathroom, before food/drink, abdomen relaxed, tape at navel level. Weight changed -0.5 kg and waist -2.6 cm versus 2026-08-09. Progress photos were not supplied for this check-in.</x:v>
+      </x:c>
+      <x:c r="K7" s="170" t="str">
+        <x:v>Missing photos</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K2"/>
@@ -2494,7 +2523,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f461e00cc1e42fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1e8f822aed143b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3897,7 +3926,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd20978317e43470e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6336d8963d3a4b8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4009,8 +4038,7 @@
         <x:v>Biceps</x:v>
       </x:c>
       <x:c r="L4" s="140" t="n">
-        <x:f>SUMIF('Session Summary'!$B$5:$B$200,K4,'Session Summary'!$C$5:$C$200)</x:f>
-        <x:v>12</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4026,11 +4054,11 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
-        <x:v>52</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="inlineStr">
@@ -4055,7 +4083,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="59" t="str">
-        <x:v>88.8 kg (2026-08-09)</x:v>
+        <x:v>88.3 kg (2026-08-16)</x:v>
       </x:c>
       <x:c r="C6" s="59" t="n"/>
       <x:c r="D6" s="53" t="n"/>
@@ -4490,25 +4518,23 @@
       <x:c r="A21" s="59" t="n"/>
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
-      <x:c r="D21" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Biceps</x:t>
-        </x:is>
+      <x:c r="D21" s="59" t="str">
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
         <x:v>Straight Bar Curl</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>15 kg/side x 7 @ RIR 1</x:v>
+        <x:v>15 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>15 kg/side x 8 @ RIR 2</x:v>
+        <x:v>15 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>No body swing</x:v>
+        <x:v>Bar excluded; exactly 3 working sets</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4518,25 +4544,23 @@
       <x:c r="A22" s="59" t="n"/>
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
-      <x:c r="D22" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Biceps</x:t>
-        </x:is>
+      <x:c r="D22" s="59" t="str">
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
         <x:v>Hammer Curl</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>17.5 kg x 11 @ RIR 1</x:v>
+        <x:v>17.5 kg each x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>17.5 kg x 12 @ RIR 2</x:v>
+        <x:v>17.5 kg each x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Each dumbbell</x:v>
+        <x:v>No body swing</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4546,25 +4570,23 @@
       <x:c r="A23" s="50" t="n"/>
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
-      <x:c r="D23" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Legs</x:t>
-        </x:is>
+      <x:c r="D23" s="50" t="str">
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Hack Squat</x:v>
+        <x:v>Concentration Curl</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>60 kg/side x 10 @ RIR 1</x:v>
+        <x:v>12.5 kg each x 10 @ RIR 1</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>60 kg/side x 10 @ RIR 2</x:v>
+        <x:v>12.5 kg each x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Keep depth/control</x:v>
+        <x:v>No assistance or body swing</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4574,25 +4596,23 @@
       <x:c r="A24" s="50" t="n"/>
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
-      <x:c r="D24" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Legs</x:t>
-        </x:is>
+      <x:c r="D24" s="50" t="str">
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Leg Press</x:v>
+        <x:v>Reverse EZ Curl</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>150 kg: 4 clean + 4 assisted</x:v>
+        <x:v>10 kg/side x 11 @ RIR 1</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>130 kg x 11-12 @ RIR 2</x:v>
+        <x:v>10 kg/side x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>No hand assistance</x:v>
+        <x:v>Bar excluded; preserve the 18-set cap</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4621,7 +4641,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ebd4c6a1f724bcc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R469c0637645e445d"/>
 </x:worksheet>
 </file>
 
@@ -16382,292 +16402,776 @@
       </x:c>
     </x:row>
     <x:row r="290">
-      <x:c r="A290" s="220"/>
-      <x:c r="B290" s="170"/>
-      <x:c r="C290" s="170"/>
-      <x:c r="D290" s="170"/>
-      <x:c r="E290" s="170"/>
-      <x:c r="F290" s="170"/>
-      <x:c r="G290" s="170"/>
-      <x:c r="H290" s="170"/>
-      <x:c r="I290" s="170"/>
-      <x:c r="J290" s="170"/>
-      <x:c r="K290" s="170"/>
+      <x:c r="A290" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B290" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C290" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D290" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E290" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F290" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G290" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H290" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I290" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J290" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K290" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L290" s="170"/>
-      <x:c r="M290" s="170"/>
-      <x:c r="N290" s="170"/>
+      <x:c r="M290" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N290" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="291">
-      <x:c r="A291" s="220"/>
-      <x:c r="B291" s="170"/>
-      <x:c r="C291" s="170"/>
-      <x:c r="D291" s="170"/>
-      <x:c r="E291" s="170"/>
-      <x:c r="F291" s="170"/>
-      <x:c r="G291" s="170"/>
-      <x:c r="H291" s="170"/>
-      <x:c r="I291" s="170"/>
-      <x:c r="J291" s="170"/>
-      <x:c r="K291" s="170"/>
+      <x:c r="A291" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B291" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C291" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D291" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E291" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F291" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G291" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H291" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I291" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J291" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K291" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L291" s="170"/>
-      <x:c r="M291" s="170"/>
-      <x:c r="N291" s="170"/>
+      <x:c r="M291" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N291" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="292">
-      <x:c r="A292" s="220"/>
-      <x:c r="B292" s="170"/>
-      <x:c r="C292" s="170"/>
-      <x:c r="D292" s="170"/>
-      <x:c r="E292" s="170"/>
-      <x:c r="F292" s="170"/>
-      <x:c r="G292" s="170"/>
-      <x:c r="H292" s="170"/>
-      <x:c r="I292" s="170"/>
-      <x:c r="J292" s="170"/>
-      <x:c r="K292" s="170"/>
+      <x:c r="A292" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B292" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C292" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D292" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E292" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F292" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G292" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H292" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I292" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J292" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K292" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L292" s="170"/>
-      <x:c r="M292" s="170"/>
-      <x:c r="N292" s="170"/>
+      <x:c r="M292" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N292" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="293">
-      <x:c r="A293" s="220"/>
-      <x:c r="B293" s="170"/>
-      <x:c r="C293" s="170"/>
-      <x:c r="D293" s="170"/>
-      <x:c r="E293" s="170"/>
-      <x:c r="F293" s="170"/>
-      <x:c r="G293" s="170"/>
-      <x:c r="H293" s="170"/>
-      <x:c r="I293" s="170"/>
-      <x:c r="J293" s="170"/>
-      <x:c r="K293" s="170"/>
-      <x:c r="L293" s="170"/>
-      <x:c r="M293" s="170"/>
-      <x:c r="N293" s="170"/>
+      <x:c r="A293" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B293" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C293" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D293" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E293" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F293" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G293" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H293" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I293" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J293" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K293" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L293" s="170" t="str">
+        <x:v>Progressed from 7 reps at RIR 1 to 8 reps at RIR 2</x:v>
+      </x:c>
+      <x:c r="M293" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N293" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="294">
-      <x:c r="A294" s="220"/>
-      <x:c r="B294" s="170"/>
-      <x:c r="C294" s="170"/>
-      <x:c r="D294" s="170"/>
-      <x:c r="E294" s="170"/>
-      <x:c r="F294" s="170"/>
-      <x:c r="G294" s="170"/>
-      <x:c r="H294" s="170"/>
-      <x:c r="I294" s="170"/>
-      <x:c r="J294" s="170"/>
-      <x:c r="K294" s="170"/>
+      <x:c r="A294" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B294" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C294" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D294" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E294" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F294" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G294" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H294" s="170" t="str">
+        <x:v>Clean and controlled; no shoulder pain</x:v>
+      </x:c>
+      <x:c r="I294" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J294" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K294" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L294" s="170"/>
-      <x:c r="M294" s="170"/>
-      <x:c r="N294" s="170"/>
+      <x:c r="M294" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N294" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="295">
-      <x:c r="A295" s="220"/>
-      <x:c r="B295" s="170"/>
-      <x:c r="C295" s="170"/>
-      <x:c r="D295" s="170"/>
-      <x:c r="E295" s="170"/>
-      <x:c r="F295" s="170"/>
-      <x:c r="G295" s="170"/>
-      <x:c r="H295" s="170"/>
-      <x:c r="I295" s="170"/>
-      <x:c r="J295" s="170"/>
-      <x:c r="K295" s="170"/>
+      <x:c r="A295" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B295" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C295" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D295" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E295" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F295" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G295" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H295" s="170" t="str">
+        <x:v>Clean and controlled; no shoulder pain</x:v>
+      </x:c>
+      <x:c r="I295" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J295" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K295" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L295" s="170"/>
-      <x:c r="M295" s="170"/>
-      <x:c r="N295" s="170"/>
+      <x:c r="M295" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N295" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="296">
-      <x:c r="A296" s="220"/>
-      <x:c r="B296" s="170"/>
-      <x:c r="C296" s="170"/>
-      <x:c r="D296" s="170"/>
-      <x:c r="E296" s="170"/>
-      <x:c r="F296" s="170"/>
-      <x:c r="G296" s="170"/>
-      <x:c r="H296" s="170"/>
-      <x:c r="I296" s="170"/>
-      <x:c r="J296" s="170"/>
-      <x:c r="K296" s="170"/>
-      <x:c r="L296" s="170"/>
-      <x:c r="M296" s="170"/>
-      <x:c r="N296" s="170"/>
+      <x:c r="A296" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B296" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C296" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D296" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E296" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F296" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G296" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H296" s="170" t="str">
+        <x:v>Clean and controlled; no shoulder pain</x:v>
+      </x:c>
+      <x:c r="I296" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J296" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K296" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L296" s="170" t="str">
+        <x:v>New tracked baseline; replaced Cable Curl in active sequence</x:v>
+      </x:c>
+      <x:c r="M296" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N296" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="297">
-      <x:c r="A297" s="220"/>
-      <x:c r="B297" s="170"/>
-      <x:c r="C297" s="170"/>
-      <x:c r="D297" s="170"/>
-      <x:c r="E297" s="170"/>
-      <x:c r="F297" s="170"/>
-      <x:c r="G297" s="170"/>
-      <x:c r="H297" s="170"/>
-      <x:c r="I297" s="170"/>
-      <x:c r="J297" s="170"/>
-      <x:c r="K297" s="170"/>
+      <x:c r="A297" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B297" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C297" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D297" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E297" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F297" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G297" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H297" s="170" t="str">
+        <x:v>Clean and controlled</x:v>
+      </x:c>
+      <x:c r="I297" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J297" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K297" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L297" s="170"/>
-      <x:c r="M297" s="170"/>
-      <x:c r="N297" s="170"/>
+      <x:c r="M297" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N297" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="298">
-      <x:c r="A298" s="220"/>
-      <x:c r="B298" s="170"/>
-      <x:c r="C298" s="170"/>
-      <x:c r="D298" s="170"/>
-      <x:c r="E298" s="170"/>
-      <x:c r="F298" s="170"/>
-      <x:c r="G298" s="170"/>
-      <x:c r="H298" s="170"/>
-      <x:c r="I298" s="170"/>
-      <x:c r="J298" s="170"/>
-      <x:c r="K298" s="170"/>
+      <x:c r="A298" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B298" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C298" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D298" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E298" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F298" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G298" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H298" s="170" t="str">
+        <x:v>Clean and controlled</x:v>
+      </x:c>
+      <x:c r="I298" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J298" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K298" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L298" s="170"/>
-      <x:c r="M298" s="170"/>
-      <x:c r="N298" s="170"/>
+      <x:c r="M298" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N298" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="299">
-      <x:c r="A299" s="220"/>
-      <x:c r="B299" s="170"/>
-      <x:c r="C299" s="170"/>
-      <x:c r="D299" s="170"/>
-      <x:c r="E299" s="170"/>
-      <x:c r="F299" s="170"/>
-      <x:c r="G299" s="170"/>
-      <x:c r="H299" s="170"/>
-      <x:c r="I299" s="170"/>
-      <x:c r="J299" s="170"/>
-      <x:c r="K299" s="170"/>
-      <x:c r="L299" s="170"/>
-      <x:c r="M299" s="170"/>
-      <x:c r="N299" s="170"/>
+      <x:c r="A299" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B299" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C299" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D299" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E299" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F299" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G299" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H299" s="170" t="str">
+        <x:v>Clean and controlled</x:v>
+      </x:c>
+      <x:c r="I299" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J299" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K299" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L299" s="170" t="str">
+        <x:v>Progressed from 9 reps at RIR 1 to 10 reps at RIR 2</x:v>
+      </x:c>
+      <x:c r="M299" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N299" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="300">
-      <x:c r="A300" s="220"/>
-      <x:c r="B300" s="170"/>
-      <x:c r="C300" s="170"/>
-      <x:c r="D300" s="170"/>
-      <x:c r="E300" s="170"/>
-      <x:c r="F300" s="170"/>
-      <x:c r="G300" s="170"/>
-      <x:c r="H300" s="170"/>
-      <x:c r="I300" s="170"/>
-      <x:c r="J300" s="170"/>
-      <x:c r="K300" s="170"/>
-      <x:c r="L300" s="170"/>
-      <x:c r="M300" s="170"/>
-      <x:c r="N300" s="170"/>
+      <x:c r="A300" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B300" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C300" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D300" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E300" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F300" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G300" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H300" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I300" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J300" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K300" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L300" s="170" t="str">
+        <x:v>Progressed from 15 to 17 reps</x:v>
+      </x:c>
+      <x:c r="M300" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N300" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="301">
-      <x:c r="A301" s="220"/>
-      <x:c r="B301" s="170"/>
-      <x:c r="C301" s="170"/>
-      <x:c r="D301" s="170"/>
-      <x:c r="E301" s="170"/>
-      <x:c r="F301" s="170"/>
-      <x:c r="G301" s="170"/>
-      <x:c r="H301" s="170"/>
-      <x:c r="I301" s="170"/>
-      <x:c r="J301" s="170"/>
-      <x:c r="K301" s="170"/>
+      <x:c r="A301" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B301" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C301" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D301" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E301" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F301" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G301" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H301" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I301" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J301" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K301" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L301" s="170"/>
-      <x:c r="M301" s="170"/>
-      <x:c r="N301" s="170"/>
+      <x:c r="M301" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N301" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="302">
-      <x:c r="A302" s="220"/>
-      <x:c r="B302" s="170"/>
-      <x:c r="C302" s="170"/>
-      <x:c r="D302" s="170"/>
-      <x:c r="E302" s="170"/>
-      <x:c r="F302" s="170"/>
-      <x:c r="G302" s="170"/>
-      <x:c r="H302" s="170"/>
-      <x:c r="I302" s="170"/>
-      <x:c r="J302" s="170"/>
-      <x:c r="K302" s="170"/>
-      <x:c r="L302" s="170"/>
-      <x:c r="M302" s="170"/>
-      <x:c r="N302" s="170"/>
+      <x:c r="A302" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B302" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C302" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D302" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E302" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F302" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G302" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H302" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I302" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J302" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K302" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L302" s="170" t="str">
+        <x:v>Maintained reps while improving from RIR 1 to RIR 2</x:v>
+      </x:c>
+      <x:c r="M302" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N302" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="303">
-      <x:c r="A303" s="220"/>
-      <x:c r="B303" s="170"/>
-      <x:c r="C303" s="170"/>
-      <x:c r="D303" s="170"/>
-      <x:c r="E303" s="170"/>
-      <x:c r="F303" s="170"/>
-      <x:c r="G303" s="170"/>
-      <x:c r="H303" s="170"/>
-      <x:c r="I303" s="170"/>
-      <x:c r="J303" s="170"/>
-      <x:c r="K303" s="170"/>
+      <x:c r="A303" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B303" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C303" s="170" t="str">
+        <x:v>Concentration Curl</x:v>
+      </x:c>
+      <x:c r="D303" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E303" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F303" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G303" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H303" s="170" t="str">
+        <x:v>Clean and controlled; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I303" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J303" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K303" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L303" s="170"/>
-      <x:c r="M303" s="170"/>
-      <x:c r="N303" s="170"/>
+      <x:c r="M303" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N303" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="304">
-      <x:c r="A304" s="220"/>
-      <x:c r="B304" s="170"/>
-      <x:c r="C304" s="170"/>
-      <x:c r="D304" s="170"/>
-      <x:c r="E304" s="170"/>
-      <x:c r="F304" s="170"/>
-      <x:c r="G304" s="170"/>
-      <x:c r="H304" s="170"/>
-      <x:c r="I304" s="170"/>
-      <x:c r="J304" s="170"/>
-      <x:c r="K304" s="170"/>
+      <x:c r="A304" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B304" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C304" s="170" t="str">
+        <x:v>Concentration Curl</x:v>
+      </x:c>
+      <x:c r="D304" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E304" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F304" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G304" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H304" s="170" t="str">
+        <x:v>Clean and controlled; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I304" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J304" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K304" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L304" s="170"/>
-      <x:c r="M304" s="170"/>
-      <x:c r="N304" s="170"/>
+      <x:c r="M304" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N304" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="305">
-      <x:c r="A305" s="220"/>
-      <x:c r="B305" s="170"/>
-      <x:c r="C305" s="170"/>
-      <x:c r="D305" s="170"/>
-      <x:c r="E305" s="170"/>
-      <x:c r="F305" s="170"/>
-      <x:c r="G305" s="170"/>
-      <x:c r="H305" s="170"/>
-      <x:c r="I305" s="170"/>
-      <x:c r="J305" s="170"/>
-      <x:c r="K305" s="170"/>
-      <x:c r="L305" s="170"/>
-      <x:c r="M305" s="170"/>
-      <x:c r="N305" s="170"/>
+      <x:c r="A305" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B305" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C305" s="170" t="str">
+        <x:v>Concentration Curl</x:v>
+      </x:c>
+      <x:c r="D305" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E305" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F305" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G305" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H305" s="170" t="str">
+        <x:v>Clean and controlled; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I305" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J305" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K305" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L305" s="170" t="str">
+        <x:v>Unplanned third set; progressed from 9 to 10 reps without failure</x:v>
+      </x:c>
+      <x:c r="M305" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N305" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="306">
-      <x:c r="A306" s="220"/>
-      <x:c r="B306" s="170"/>
-      <x:c r="C306" s="170"/>
-      <x:c r="D306" s="170"/>
-      <x:c r="E306" s="170"/>
-      <x:c r="F306" s="170"/>
-      <x:c r="G306" s="170"/>
-      <x:c r="H306" s="170"/>
-      <x:c r="I306" s="170"/>
-      <x:c r="J306" s="170"/>
-      <x:c r="K306" s="170"/>
-      <x:c r="L306" s="170"/>
-      <x:c r="M306" s="170"/>
-      <x:c r="N306" s="170"/>
+      <x:c r="A306" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B306" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C306" s="170" t="str">
+        <x:v>Reverse EZ-Bar Curl</x:v>
+      </x:c>
+      <x:c r="D306" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E306" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F306" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G306" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H306" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I306" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J306" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K306" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L306" s="170" t="str">
+        <x:v>Rep target met but one RIR harder than planned</x:v>
+      </x:c>
+      <x:c r="M306" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N306" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="307">
-      <x:c r="A307" s="220"/>
-      <x:c r="B307" s="170"/>
-      <x:c r="C307" s="170"/>
-      <x:c r="D307" s="170"/>
-      <x:c r="E307" s="170"/>
-      <x:c r="F307" s="170"/>
-      <x:c r="G307" s="170"/>
-      <x:c r="H307" s="170"/>
-      <x:c r="I307" s="170"/>
-      <x:c r="J307" s="170"/>
-      <x:c r="K307" s="170"/>
-      <x:c r="L307" s="170"/>
-      <x:c r="M307" s="170"/>
-      <x:c r="N307" s="170"/>
+      <x:c r="A307" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B307" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C307" s="170" t="str">
+        <x:v>Reverse EZ-Bar Curl</x:v>
+      </x:c>
+      <x:c r="D307" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E307" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F307" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G307" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H307" s="170" t="str">
+        <x:v>Clean; no assistance or body swing</x:v>
+      </x:c>
+      <x:c r="I307" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
+      <x:c r="J307" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K307" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L307" s="170" t="str">
+        <x:v>Only two sets used to preserve the 18-set cap</x:v>
+      </x:c>
+      <x:c r="M307" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N307" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="308">
       <x:c r="A308" s="220"/>
@@ -16909,7 +17413,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbac0593a15924b20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74db20631d204888"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17309,25 +17813,25 @@
         <x:v>Hammer Curl</x:v>
       </x:c>
       <x:c r="C15" s="222" t="str">
-        <x:v>17.5 kg each x 11 @ RIR 1</x:v>
+        <x:v>17.5 kg each x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="D15" s="222" t="str">
-        <x:v>15-17.5 kg</x:v>
+        <x:v>12.5-17.5 kg each</x:v>
       </x:c>
       <x:c r="E15" s="222" t="str">
-        <x:v>17.5 kg x 12 @ RIR 2</x:v>
+        <x:v>17.5 kg each x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F15" s="222" t="str">
         <x:v>Add reps with reserve</x:v>
       </x:c>
       <x:c r="G15" s="222" t="str">
-        <x:v>Neutral wrists</x:v>
+        <x:v>Neutral wrists; no swing</x:v>
       </x:c>
       <x:c r="H15" s="222" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I15" s="222" t="str">
-        <x:v>Each dumbbell</x:v>
+        <x:v>12.5 kg reached 17 reps at RIR 2</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -17338,13 +17842,13 @@
         <x:v>Plate Curl Machine</x:v>
       </x:c>
       <x:c r="C16" s="222" t="str">
-        <x:v>12.5 kg/side x 9 @ RIR 1</x:v>
+        <x:v>12.5 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D16" s="222" t="str">
         <x:v>7.5-12.5 kg/side</x:v>
       </x:c>
       <x:c r="E16" s="222" t="str">
-        <x:v>12.5 kg/side x 10 @ RIR 2</x:v>
+        <x:v>12.5 kg/side x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F16" s="222" t="str">
         <x:v>Add clean rep</x:v>
@@ -17356,7 +17860,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I16" s="222" t="str">
-        <x:v>12.5 kg/side verified; historical 10.25 preserved</x:v>
+        <x:v>Plates each side</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -17370,22 +17874,22 @@
         <x:v>40 kg x 10 @ RIR 1</x:v>
       </x:c>
       <x:c r="D17" s="222" t="str">
-        <x:v>35-40 kg</x:v>
+        <x:v>Historical baseline</x:v>
       </x:c>
       <x:c r="E17" s="222" t="str">
-        <x:v>40 kg x 10-11 @ RIR 2</x:v>
+        <x:v>Not in active sequence</x:v>
       </x:c>
       <x:c r="F17" s="222" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Preserve history</x:v>
       </x:c>
       <x:c r="G17" s="222" t="str">
         <x:v>Elbows close</x:v>
       </x:c>
       <x:c r="H17" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Replaced</x:v>
       </x:c>
       <x:c r="I17" s="222" t="str">
-        <x:v>No load increase</x:v>
+        <x:v>Incline Dumbbell Curl now occupies this active slot</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -17396,24 +17900,26 @@
         <x:v>Reverse EZ Curl</x:v>
       </x:c>
       <x:c r="C18" s="222" t="str">
-        <x:v>10 kg/side x 10 @ RIR 1</x:v>
+        <x:v>10 kg/side x 11 @ RIR 1</x:v>
       </x:c>
       <x:c r="D18" s="222" t="str">
-        <x:v>7.5-10 kg/side</x:v>
+        <x:v>5-10 kg/side</x:v>
       </x:c>
       <x:c r="E18" s="222" t="str">
         <x:v>10 kg/side x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F18" s="222" t="str">
-        <x:v>Add reps with reserve</x:v>
+        <x:v>Improve reserve</x:v>
       </x:c>
       <x:c r="G18" s="222" t="str">
         <x:v>Wrists neutral</x:v>
       </x:c>
       <x:c r="H18" s="222" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="I18" s="222"/>
+        <x:v>Modify effort</x:v>
+      </x:c>
+      <x:c r="I18" s="222" t="str">
+        <x:v>Bar excluded; only 2 sets used to preserve session cap</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="222" t="str">
@@ -17423,16 +17929,16 @@
         <x:v>Concentration Curl</x:v>
       </x:c>
       <x:c r="C19" s="222" t="str">
-        <x:v>12.5 kg x 9 @ RIR 1</x:v>
+        <x:v>12.5 kg each x 10 @ RIR 1</x:v>
       </x:c>
       <x:c r="D19" s="222" t="str">
-        <x:v>7.5-10 kg strict</x:v>
+        <x:v>7.5-12.5 kg each</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>10 kg x 12 @ RIR 2</x:v>
+        <x:v>12.5 kg each x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>Avoid failure</x:v>
+        <x:v>Improve reserve; no failure</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
         <x:v>Elbow fixed; no swing</x:v>
@@ -17441,7 +17947,7 @@
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>10 kg reached RIR 0; 12.5 kg is history, not next load</x:v>
+        <x:v>Clean and controlled; exactly 3 sets next time</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -18087,7 +18593,7 @@
         <x:v>Use instead of extra fly volume</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="34" customHeight="1">
+    <x:row r="43" ht="38" customHeight="1">
       <x:c r="A43" s="170" t="str">
         <x:v>Biceps</x:v>
       </x:c>
@@ -18095,16 +18601,16 @@
         <x:v>Straight Bar Curl</x:v>
       </x:c>
       <x:c r="C43" s="170" t="str">
-        <x:v>15 kg/side x 7 @ RIR 1</x:v>
+        <x:v>15 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="D43" s="170" t="str">
         <x:v>10-15 kg/side</x:v>
       </x:c>
       <x:c r="E43" s="170" t="str">
-        <x:v>15 kg/side x 8 @ RIR 2</x:v>
+        <x:v>15 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F43" s="170" t="str">
-        <x:v>Add reps with reserve</x:v>
+        <x:v>Exactly 3 working sets; add rep before load</x:v>
       </x:c>
       <x:c r="G43" s="170" t="str">
         <x:v>No body swing</x:v>
@@ -18113,10 +18619,10 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I43" s="170" t="str">
-        <x:v>Bar excluded; separate from EZ-bar curl</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="34" customHeight="1">
+        <x:v>Bar excluded; use genuine preparation separately</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="38" customHeight="1">
       <x:c r="A44" s="170" t="str">
         <x:v>Shoulders</x:v>
       </x:c>
@@ -18145,7 +18651,7 @@
         <x:v>Reported loaded-set count remains To verify</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="34" customHeight="1">
+    <x:row r="45" ht="38" customHeight="1">
       <x:c r="A45" s="170" t="str">
         <x:v>Shoulders</x:v>
       </x:c>
@@ -18174,7 +18680,7 @@
         <x:v>Grip and exact effective stack To verify</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="36" customHeight="1">
+    <x:row r="46" ht="38" customHeight="1">
       <x:c r="A46" s="170" t="str">
         <x:v>Core</x:v>
       </x:c>
@@ -18201,6 +18707,35 @@
       </x:c>
       <x:c r="I46" s="170" t="str">
         <x:v>No lower-back discomfort reported</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="38" customHeight="1">
+      <x:c r="A47" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="B47" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="C47" s="170" t="str">
+        <x:v>12.5 kg each x 9 @ RIR 2</x:v>
+      </x:c>
+      <x:c r="D47" s="170" t="str">
+        <x:v>7.5-12.5 kg each</x:v>
+      </x:c>
+      <x:c r="E47" s="170" t="str">
+        <x:v>12.5 kg each x 10 @ RIR 2</x:v>
+      </x:c>
+      <x:c r="F47" s="170" t="str">
+        <x:v>Add clean rep before load</x:v>
+      </x:c>
+      <x:c r="G47" s="170" t="str">
+        <x:v>Bench 45-60 degrees; shoulders back; do not force stretch</x:v>
+      </x:c>
+      <x:c r="H47" s="170" t="str">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I47" s="170" t="str">
+        <x:v>New clean baseline; replaces Cable Curl in active sequence</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18228,7 +18763,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fce9c7079fd4d07"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R063d414910984bcd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18531,19 +19066,25 @@
       <x:c r="L8" s="153" t="str">
         <x:v>Week 2</x:v>
       </x:c>
-      <x:c r="M8" s="154"/>
-      <x:c r="N8" s="155" t="str">
-        <x:f>IF(M8="","",IFERROR(AVERAGEIFS($B$5:$B$200,$A$5:$A$200,"&gt;="&amp;M8-6,$A$5:$A$200,"&lt;="&amp;M8),""))</x:f>
-      </x:c>
-      <x:c r="O8" s="155"/>
-      <x:c r="P8" s="155" t="str">
-        <x:f>IF(O8="","",IFERROR(O8-$O$6,""))</x:f>
+      <x:c r="M8" s="154" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="N8" s="155" t="n">
+        <x:v>88.3</x:v>
+      </x:c>
+      <x:c r="O8" s="155" t="n">
+        <x:v>96.5</x:v>
+      </x:c>
+      <x:c r="P8" s="155" t="n">
+        <x:v>-2.6</x:v>
       </x:c>
       <x:c r="Q8" s="156"/>
       <x:c r="R8" s="157" t="str">
         <x:f>IF(M8="","",IFERROR(AVERAGEIFS($I$5:$I$200,$A$5:$A$200,"&gt;="&amp;M8-6,$A$5:$A$200,"&lt;="&amp;M8),""))</x:f>
       </x:c>
-      <x:c r="S8" s="158"/>
+      <x:c r="S8" s="158" t="str">
+        <x:v>Second standardized Sunday point. Single morning reading, not a weekly average. After bathroom and before food/drink; abdomen relaxed; tape at navel. Change versus 2026-08-09: -0.5 kg and -2.6 cm. Use the multi-week trend before attributing the full change to fat loss.</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="264" hidden="0" customHeight="1">
       <x:c r="A9" s="220" t="n">
@@ -18880,16 +19421,26 @@
       <x:c r="Q18" s="59" t="n"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="220"/>
-      <x:c r="B19" s="170"/>
-      <x:c r="C19" s="170"/>
+      <x:c r="A19" s="220" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="B19" s="170" t="n">
+        <x:v>88.3</x:v>
+      </x:c>
+      <x:c r="C19" s="170" t="n">
+        <x:v>96.5</x:v>
+      </x:c>
       <x:c r="D19" s="170"/>
       <x:c r="E19" s="170"/>
       <x:c r="F19" s="170"/>
       <x:c r="G19" s="170"/>
       <x:c r="H19" s="170"/>
-      <x:c r="I19" s="170"/>
-      <x:c r="J19" s="170"/>
+      <x:c r="I19" s="170" t="str">
+        <x:v>Standardized Sunday measurement check-in</x:v>
+      </x:c>
+      <x:c r="J19" s="170" t="str">
+        <x:v>After bathroom and before food/drink; abdomen relaxed; tape at navel level; verified; photos not supplied</x:v>
+      </x:c>
       <x:c r="K19" s="59" t="n"/>
       <x:c r="L19" s="59" t="n"/>
       <x:c r="M19" s="59" t="n"/>
@@ -18899,16 +19450,28 @@
       <x:c r="Q19" s="59" t="n"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="220"/>
+      <x:c r="A20" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
       <x:c r="B20" s="170"/>
       <x:c r="C20" s="170"/>
-      <x:c r="D20" s="170"/>
-      <x:c r="E20" s="170"/>
-      <x:c r="F20" s="170"/>
+      <x:c r="D20" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E20" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F20" s="170" t="str">
+        <x:v>Usual overall biceps sensation; no unusual lower-biceps symptom; no elbow, wrist or shoulder pain</x:v>
+      </x:c>
       <x:c r="G20" s="170"/>
       <x:c r="H20" s="170"/>
-      <x:c r="I20" s="170"/>
-      <x:c r="J20" s="170"/>
+      <x:c r="I20" s="170" t="str">
+        <x:v>Biceps workout - 90 min; medium-high pump</x:v>
+      </x:c>
+      <x:c r="J20" s="170" t="str">
+        <x:v>Started Medium-High; full EAA+ scoop (100 mg caffeine); no black coffee; no assistance or body swing; incline and concentration curls clean and controlled</x:v>
+      </x:c>
       <x:c r="K20" s="59" t="n"/>
       <x:c r="L20" s="59" t="n"/>
       <x:c r="M20" s="59" t="n"/>
@@ -22393,7 +22956,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cd96f6502da4a20"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc911a8c4399b4753"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23072,13 +23635,55 @@
         <x:v>Retain the 15-set chest cap, improve RIR before load, and keep core work separate</x:v>
       </x:c>
     </x:row>
+    <x:row r="44" ht="48" customHeight="1">
+      <x:c r="A44" s="170" t="str">
+        <x:v>Second standardized Sunday check-in</x:v>
+      </x:c>
+      <x:c r="B44" s="170" t="str">
+        <x:v>2026-08-16: 88.3 kg and 96.5 cm waist, measured after bathroom and before food/drink with abdomen relaxed and tape at navel</x:v>
+      </x:c>
+      <x:c r="C44" s="170" t="str">
+        <x:v>Versus 2026-08-09: -0.5 kg and -2.6 cm; direction is favorable but one week is insufficient to attribute all change to fat loss</x:v>
+      </x:c>
+      <x:c r="D44" s="170" t="str">
+        <x:v>Repeat identical protocol weekly and assess the multi-week trend</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="48" customHeight="1">
+      <x:c r="A45" s="170" t="str">
+        <x:v>Biceps effort distribution improved</x:v>
+      </x:c>
+      <x:c r="B45" s="170" t="str">
+        <x:v>2026-08-19 used exactly 18 working sets: 3 at RIR 3, 12 at RIR 2 and 3 at RIR 1; no RIR 0, assistance or body swing</x:v>
+      </x:c>
+      <x:c r="C45" s="170" t="str">
+        <x:v>This is materially better controlled than the 2026-08-12 session, which had 20 sets, 16 at RIR 1 and one at RIR 0</x:v>
+      </x:c>
+      <x:c r="D45" s="170" t="str">
+        <x:v>Keep the 18-set ceiling and use exactly three sets per exercise next time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="48" customHeight="1">
+      <x:c r="A46" s="170" t="str">
+        <x:v>Incline curl substitution</x:v>
+      </x:c>
+      <x:c r="B46" s="170" t="str">
+        <x:v>Incline Dumbbell Curl replaced Cable Curl and established a clean 7.5-12.5 kg-each baseline without shoulder pain</x:v>
+      </x:c>
+      <x:c r="C46" s="170" t="str">
+        <x:v>The lengthened-position curl was tolerated, while historical cable-curl performance remains preserved</x:v>
+      </x:c>
+      <x:c r="D46" s="170" t="str">
+        <x:v>Keep incline curl in the active sequence; do not force the bottom stretch</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R021c79b3fe284834"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad9f46752b564c0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23566,14 +24171,30 @@
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="220"/>
-      <x:c r="B19" s="170"/>
-      <x:c r="C19" s="170"/>
-      <x:c r="D19" s="170"/>
-      <x:c r="E19" s="170"/>
-      <x:c r="F19" s="170"/>
-      <x:c r="G19" s="170"/>
-      <x:c r="H19" s="170"/>
+      <x:c r="A19" s="220" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="B19" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C19" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D19" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E19" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F19" s="170" t="str">
+        <x:v>Good sleep; Medium-High start and Low final energy; usual overall biceps sensation; no joint pain; medium-high pump; 90 min; no assistance or body swing; full EAA+; no coffee</x:v>
+      </x:c>
+      <x:c r="G19" s="170" t="str">
+        <x:v>Clear improvement over 2026-08-12: volume reduced from 20 to 18, no RIR 0 sets, only three RIR 1 sets, and multiple rep/reserve progressions. Incline dumbbell curl replaced cable curl and established a clean baseline.</x:v>
+      </x:c>
+      <x:c r="H19" s="170" t="str">
+        <x:v>Retain exactly 18 sets and 3 per exercise; keep loads; improve reserve before progression; active sequence uses incline dumbbell curl instead of cable curl</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="220"/>
@@ -23647,7 +24268,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6e29a6a9e26496c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1efd438a3e04901"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23756,13 +24377,13 @@
         <x:v>Current body weight</x:v>
       </x:c>
       <x:c r="C6" s="170" t="str">
-        <x:v>88.8 kg on 2026-08-09, measured after using the bathroom and before any food or drink. The separate 91.5 kg gym reading was post-workout at night and is non-comparable.</x:v>
+        <x:v>88.3 kg on 2026-08-16, measured after using the bathroom and before food or drink. Abdomen relaxed and waist tape at navel level. The historical 91.5 kg post-workout gym reading remains non-comparable.</x:v>
       </x:c>
       <x:c r="D6" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E6" s="170" t="str">
-        <x:v>Use the same standardized morning protocol for trend readings</x:v>
+        <x:v>Continue identical morning protocol and assess weekly trend</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -23824,13 +24445,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>No joint pain reported through 2026-08-18. A little lower-biceps pump followed the final cable-fly set; exact side and resolution remain To verify.</x:v>
+        <x:v>No joint pain reported through 2026-08-19. The lower-biceps pump after the 2026-08-18 Chest session resolved before Biceps training; 2026-08-19 ended with only the usual overall biceps sensation.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Check that the lower-biceps pump resolved before Biceps training</x:v>
+        <x:v>Continue pain checks; stop for sharp or localized distal-biceps pain</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -24012,13 +24633,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Completed Chest on 2026-08-18 in the retained one-body-part split. Biceps is next, subject to fresh readiness and confirmation that the lower-biceps pump resolved.</x:v>
+        <x:v>Completed Biceps on 2026-08-19 in the retained one-body-part split. Legs is next, subject to fresh readiness.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Collect fresh readiness before Biceps</x:v>
+        <x:v>Collect fresh sleep, energy, soreness and knee/hip/lower-back check before Legs</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -24167,13 +24788,13 @@
         <x:v>Waist and verified morning weight</x:v>
       </x:c>
       <x:c r="C30" s="170" t="str">
-        <x:v>2026-08-09 standardized baseline: 88.8 kg and 39 in at the navel (99.1 cm), after bathroom and before food or drink.</x:v>
+        <x:v>2026-08-16 standardized check-in: 88.3 kg and 38 in at the navel (96.5 cm), after bathroom and before food or drink, abdomen relaxed. Change from 2026-08-09: -0.5 kg and -2.6 cm.</x:v>
       </x:c>
       <x:c r="D30" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E30" s="170" t="str">
-        <x:v>Repeat weekly under identical conditions; take two waist readings and verify if they differ by more than 0.5 cm</x:v>
+        <x:v>Repeat weekly under identical conditions; use multi-week trend</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -24218,7 +24839,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8cfdcf5bf5645ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8eb5250e1bb42f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25321,10 +25942,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R682b7c492aa34733"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2ff5ff7e7924666"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dc8801c9e59463d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R010627ed54b64ea0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red42d8c1db2549b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2bc9c86ac3b4f85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77a05e1466bb4eaa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cfc705222a54ccf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 20 legs workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra92fbd93b1654c74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R3b0a901b44974167"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rc74109d616184261"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rd4a1850083ed4aab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rf614fde1278e47df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Reb512a2733a2429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rd5487c6d211f48c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R06cfe3edd064486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R74ab6b3ad2ec4fb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R0886202db97e489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rb4aa6ceadcc24db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R61df015f813d4cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc6a3550a76f341c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rbce06624c8c04a51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Raf6c4ab25b8d4e6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R4b00cc6ad16141ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Re2b80adfaf484025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R3101ed04a912447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R5826c174d2c44d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Raf23db2981af4149"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R548dcf368da34396"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Re7adbc22484845ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf91945eabb754020"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1a683b2447f4679"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N307" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N325" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1803,7 +1803,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2523,7 +2523,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1e8f822aed143b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R416b9c2858bb4dc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3926,7 +3926,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6336d8963d3a4b8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51561240eea94c71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4054,11 +4054,11 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="inlineStr">
@@ -4072,8 +4072,7 @@
         <x:v>Legs</x:v>
       </x:c>
       <x:c r="L5" s="140" t="n">
-        <x:f>SUMIF('Session Summary'!$B$5:$B$200,K5,'Session Summary'!$C$5:$C$200)</x:f>
-        <x:v>14</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4519,22 +4518,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Straight Bar Curl</x:v>
+        <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>15 kg/side x 8 @ RIR 2</x:v>
+        <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>15 kg/side x 9 @ RIR 2</x:v>
+        <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Bar excluded; exactly 3 working sets</x:v>
+        <x:v>No load increase; verify hip</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4545,22 +4544,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Hammer Curl</x:v>
+        <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>17.5 kg each x 11 @ RIR 2</x:v>
+        <x:v>150 kg x 7 total; approx. 2-3 assisted</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>17.5 kg each x 12 @ RIR 2</x:v>
+        <x:v>130 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>No body swing</x:v>
+        <x:v>Omit 150 kg; clean reps only</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4571,22 +4570,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Concentration Curl</x:v>
+        <x:v>Dumbbell Romanian Deadlift</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>12.5 kg each x 10 @ RIR 1</x:v>
+        <x:v>15 kg each x 12 @ RIR 2; back dominant</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>12.5 kg each x 10 @ RIR 2</x:v>
+        <x:v>10 kg each x 10-12 @ RIR 3-4</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>Verify technique</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>No assistance or body swing</x:v>
+        <x:v>Wall-hinge reset; stop if back/hip symptoms</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4597,22 +4596,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Reverse EZ Curl</x:v>
+        <x:v>Leg Curl</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>10 kg/side x 11 @ RIR 1</x:v>
+        <x:v>35 kg x 9 @ RIR 0</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>10 kg/side x 11 @ RIR 2</x:v>
+        <x:v>30 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Bar excluded; preserve the 18-set cap</x:v>
+        <x:v>Full range; no failure</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4641,7 +4640,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R469c0637645e445d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1ebf07ccd34278"/>
 </x:worksheet>
 </file>
 
@@ -17174,212 +17173,772 @@
       </x:c>
     </x:row>
     <x:row r="308">
-      <x:c r="A308" s="220"/>
-      <x:c r="B308" s="170"/>
-      <x:c r="C308" s="170"/>
-      <x:c r="D308" s="170"/>
-      <x:c r="E308" s="170"/>
-      <x:c r="F308" s="170"/>
-      <x:c r="G308" s="170"/>
-      <x:c r="H308" s="170"/>
-      <x:c r="I308" s="170"/>
-      <x:c r="J308" s="170"/>
-      <x:c r="K308" s="170"/>
+      <x:c r="A308" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B308" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C308" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D308" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E308" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F308" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G308" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H308" s="170" t="str">
+        <x:v>Hamstrings felt, but lower-back involvement dominant; technique baseline only</x:v>
+      </x:c>
+      <x:c r="I308" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J308" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K308" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L308" s="170"/>
-      <x:c r="M308" s="170"/>
-      <x:c r="N308" s="170"/>
+      <x:c r="M308" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N308" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="309">
-      <x:c r="A309" s="220"/>
-      <x:c r="B309" s="170"/>
-      <x:c r="C309" s="170"/>
-      <x:c r="D309" s="170"/>
-      <x:c r="E309" s="170"/>
-      <x:c r="F309" s="170"/>
-      <x:c r="G309" s="170"/>
-      <x:c r="H309" s="170"/>
-      <x:c r="I309" s="170"/>
-      <x:c r="J309" s="170"/>
-      <x:c r="K309" s="170"/>
+      <x:c r="A309" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B309" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C309" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D309" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E309" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F309" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G309" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H309" s="170" t="str">
+        <x:v>Hamstrings felt, but lower-back involvement dominant; technique baseline only</x:v>
+      </x:c>
+      <x:c r="I309" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J309" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K309" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L309" s="170"/>
-      <x:c r="M309" s="170"/>
-      <x:c r="N309" s="170"/>
+      <x:c r="M309" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N309" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="310">
-      <x:c r="A310" s="220"/>
-      <x:c r="B310" s="170"/>
-      <x:c r="C310" s="170"/>
-      <x:c r="D310" s="170"/>
-      <x:c r="E310" s="170"/>
-      <x:c r="F310" s="170"/>
-      <x:c r="G310" s="170"/>
-      <x:c r="H310" s="170"/>
-      <x:c r="I310" s="170"/>
-      <x:c r="J310" s="170"/>
-      <x:c r="K310" s="170"/>
-      <x:c r="L310" s="170"/>
-      <x:c r="M310" s="170"/>
-      <x:c r="N310" s="170"/>
+      <x:c r="A310" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B310" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C310" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D310" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E310" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F310" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G310" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H310" s="170" t="str">
+        <x:v>Hamstrings felt, but lower-back involvement dominant; technique baseline only</x:v>
+      </x:c>
+      <x:c r="I310" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J310" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K310" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L310" s="170" t="str">
+        <x:v>Do not add load; reset hinge technique next Legs session</x:v>
+      </x:c>
+      <x:c r="M310" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N310" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="311">
-      <x:c r="A311" s="220"/>
-      <x:c r="B311" s="170"/>
-      <x:c r="C311" s="170"/>
-      <x:c r="D311" s="170"/>
-      <x:c r="E311" s="170"/>
-      <x:c r="F311" s="170"/>
-      <x:c r="G311" s="170"/>
-      <x:c r="H311" s="170"/>
-      <x:c r="I311" s="170"/>
-      <x:c r="J311" s="170"/>
-      <x:c r="K311" s="170"/>
+      <x:c r="A311" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B311" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C311" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D311" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E311" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F311" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G311" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H311" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I311" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J311" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K311" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L311" s="170"/>
-      <x:c r="M311" s="170"/>
-      <x:c r="N311" s="170"/>
+      <x:c r="M311" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N311" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="312">
-      <x:c r="A312" s="220"/>
-      <x:c r="B312" s="170"/>
-      <x:c r="C312" s="170"/>
-      <x:c r="D312" s="170"/>
-      <x:c r="E312" s="170"/>
-      <x:c r="F312" s="170"/>
-      <x:c r="G312" s="170"/>
-      <x:c r="H312" s="170"/>
-      <x:c r="I312" s="170"/>
-      <x:c r="J312" s="170"/>
-      <x:c r="K312" s="170"/>
+      <x:c r="A312" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B312" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C312" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D312" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E312" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F312" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G312" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H312" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I312" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J312" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K312" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L312" s="170"/>
-      <x:c r="M312" s="170"/>
-      <x:c r="N312" s="170"/>
+      <x:c r="M312" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N312" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="313">
-      <x:c r="A313" s="220"/>
-      <x:c r="B313" s="170"/>
-      <x:c r="C313" s="170"/>
-      <x:c r="D313" s="170"/>
-      <x:c r="E313" s="170"/>
-      <x:c r="F313" s="170"/>
-      <x:c r="G313" s="170"/>
-      <x:c r="H313" s="170"/>
-      <x:c r="I313" s="170"/>
-      <x:c r="J313" s="170"/>
-      <x:c r="K313" s="170"/>
+      <x:c r="A313" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B313" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C313" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D313" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E313" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F313" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G313" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H313" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I313" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J313" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K313" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L313" s="170"/>
-      <x:c r="M313" s="170"/>
-      <x:c r="N313" s="170"/>
+      <x:c r="M313" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N313" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="314">
-      <x:c r="A314" s="220"/>
-      <x:c r="B314" s="170"/>
-      <x:c r="C314" s="170"/>
-      <x:c r="D314" s="170"/>
-      <x:c r="E314" s="170"/>
-      <x:c r="F314" s="170"/>
-      <x:c r="G314" s="170"/>
-      <x:c r="H314" s="170"/>
-      <x:c r="I314" s="170"/>
-      <x:c r="J314" s="170"/>
-      <x:c r="K314" s="170"/>
-      <x:c r="L314" s="170"/>
-      <x:c r="M314" s="170"/>
-      <x:c r="N314" s="170"/>
+      <x:c r="A314" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B314" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C314" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D314" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E314" s="170" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F314" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G314" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H314" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I314" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J314" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K314" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L314" s="170" t="str">
+        <x:v>Progressed load while retaining RIR 2; do not add load next time</x:v>
+      </x:c>
+      <x:c r="M314" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N314" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="315">
-      <x:c r="A315" s="220"/>
-      <x:c r="B315" s="170"/>
-      <x:c r="C315" s="170"/>
-      <x:c r="D315" s="170"/>
-      <x:c r="E315" s="170"/>
-      <x:c r="F315" s="170"/>
-      <x:c r="G315" s="170"/>
-      <x:c r="H315" s="170"/>
-      <x:c r="I315" s="170"/>
-      <x:c r="J315" s="170"/>
-      <x:c r="K315" s="170"/>
+      <x:c r="A315" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B315" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C315" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D315" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E315" s="170" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F315" s="170" t="str">
+        <x:v>kg total load</x:v>
+      </x:c>
+      <x:c r="G315" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H315" s="170" t="str">
+        <x:v>Clean; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I315" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J315" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K315" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L315" s="170"/>
-      <x:c r="M315" s="170"/>
-      <x:c r="N315" s="170"/>
+      <x:c r="M315" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N315" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="316">
-      <x:c r="A316" s="220"/>
-      <x:c r="B316" s="170"/>
-      <x:c r="C316" s="170"/>
-      <x:c r="D316" s="170"/>
-      <x:c r="E316" s="170"/>
-      <x:c r="F316" s="170"/>
-      <x:c r="G316" s="170"/>
-      <x:c r="H316" s="170"/>
-      <x:c r="I316" s="170"/>
-      <x:c r="J316" s="170"/>
-      <x:c r="K316" s="170"/>
+      <x:c r="A316" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B316" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C316" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D316" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E316" s="170" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F316" s="170" t="str">
+        <x:v>kg total load</x:v>
+      </x:c>
+      <x:c r="G316" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H316" s="170" t="str">
+        <x:v>Clean; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I316" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J316" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K316" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L316" s="170"/>
-      <x:c r="M316" s="170"/>
-      <x:c r="N316" s="170"/>
+      <x:c r="M316" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N316" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="317">
-      <x:c r="A317" s="220"/>
-      <x:c r="B317" s="170"/>
-      <x:c r="C317" s="170"/>
-      <x:c r="D317" s="170"/>
-      <x:c r="E317" s="170"/>
-      <x:c r="F317" s="170"/>
-      <x:c r="G317" s="170"/>
-      <x:c r="H317" s="170"/>
-      <x:c r="I317" s="170"/>
-      <x:c r="J317" s="170"/>
-      <x:c r="K317" s="170"/>
+      <x:c r="A317" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B317" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C317" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D317" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E317" s="170" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="F317" s="170" t="str">
+        <x:v>kg total load</x:v>
+      </x:c>
+      <x:c r="G317" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H317" s="170" t="str">
+        <x:v>Clean; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I317" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J317" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K317" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L317" s="170"/>
-      <x:c r="M317" s="170"/>
-      <x:c r="N317" s="170"/>
+      <x:c r="M317" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N317" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="318">
-      <x:c r="A318" s="220"/>
-      <x:c r="B318" s="170"/>
-      <x:c r="C318" s="170"/>
-      <x:c r="D318" s="170"/>
-      <x:c r="E318" s="170"/>
-      <x:c r="F318" s="170"/>
-      <x:c r="G318" s="170"/>
-      <x:c r="H318" s="170"/>
-      <x:c r="I318" s="170"/>
-      <x:c r="J318" s="170"/>
-      <x:c r="K318" s="170"/>
-      <x:c r="L318" s="170"/>
-      <x:c r="M318" s="170"/>
-      <x:c r="N318" s="170"/>
+      <x:c r="A318" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B318" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C318" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D318" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E318" s="170" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="F318" s="170" t="str">
+        <x:v>kg total load</x:v>
+      </x:c>
+      <x:c r="G318" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H318" s="170" t="str">
+        <x:v>7 total; approximately 2-3 hand-assisted; approximately 4-5 clean To verify; do not treat as 7 clean</x:v>
+      </x:c>
+      <x:c r="I318" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J318" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K318" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L318" s="170" t="str">
+        <x:v>Omit 150 kg until 130 kg is clean at target reserve and hip pain is absent</x:v>
+      </x:c>
+      <x:c r="M318" s="170" t="str">
+        <x:v>Assisted</x:v>
+      </x:c>
+      <x:c r="N318" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="319">
-      <x:c r="A319" s="220"/>
-      <x:c r="B319" s="170"/>
-      <x:c r="C319" s="170"/>
-      <x:c r="D319" s="170"/>
-      <x:c r="E319" s="170"/>
-      <x:c r="F319" s="170"/>
-      <x:c r="G319" s="170"/>
-      <x:c r="H319" s="170"/>
-      <x:c r="I319" s="170"/>
-      <x:c r="J319" s="170"/>
-      <x:c r="K319" s="170"/>
+      <x:c r="A319" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B319" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C319" s="170" t="str">
+        <x:v>Leg Curl</x:v>
+      </x:c>
+      <x:c r="D319" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E319" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F319" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G319" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H319" s="170" t="str">
+        <x:v>Controlled; full range To verify</x:v>
+      </x:c>
+      <x:c r="I319" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J319" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K319" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
       <x:c r="L319" s="170"/>
-      <x:c r="M319" s="170"/>
-      <x:c r="N319" s="170"/>
+      <x:c r="M319" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N319" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="320">
-      <x:c r="A320" s="220"/>
-      <x:c r="B320" s="170"/>
-      <x:c r="C320" s="170"/>
-      <x:c r="D320" s="170"/>
-      <x:c r="E320" s="170"/>
-      <x:c r="F320" s="170"/>
-      <x:c r="G320" s="170"/>
-      <x:c r="H320" s="170"/>
-      <x:c r="I320" s="170"/>
-      <x:c r="J320" s="170"/>
-      <x:c r="K320" s="170"/>
-      <x:c r="L320" s="170"/>
-      <x:c r="M320" s="170"/>
-      <x:c r="N320" s="170"/>
+      <x:c r="A320" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B320" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C320" s="170" t="str">
+        <x:v>Leg Curl</x:v>
+      </x:c>
+      <x:c r="D320" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E320" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F320" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G320" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H320" s="170" t="str">
+        <x:v>Reached failure reserve; full range To verify</x:v>
+      </x:c>
+      <x:c r="I320" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J320" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K320" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L320" s="170" t="str">
+        <x:v>Reduce load/effort next time; no RIR 0 target</x:v>
+      </x:c>
+      <x:c r="M320" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N320" s="170" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="321">
+      <x:c r="A321" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B321" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C321" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D321" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E321" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F321" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G321" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H321" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I321" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J321" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K321" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L321" s="170"/>
+      <x:c r="M321" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N321" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="322">
+      <x:c r="A322" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B322" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C322" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D322" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E322" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F322" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G322" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H322" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I322" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J322" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K322" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L322" s="170"/>
+      <x:c r="M322" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N322" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="323">
+      <x:c r="A323" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B323" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C323" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D323" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E323" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F323" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G323" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H323" s="170" t="str">
+        <x:v>Controlled; no assistance reported</x:v>
+      </x:c>
+      <x:c r="I323" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J323" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K323" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L323" s="170" t="str">
+        <x:v>Progressed reps; improve reserve before load</x:v>
+      </x:c>
+      <x:c r="M323" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N323" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="324">
+      <x:c r="A324" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B324" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C324" s="170" t="str">
+        <x:v>Standing Calf Raise</x:v>
+      </x:c>
+      <x:c r="D324" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E324" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F324" s="170" t="str">
+        <x:v>kg plates each side; guided bar excluded</x:v>
+      </x:c>
+      <x:c r="G324" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H324" s="170" t="str">
+        <x:v>Controlled; full stretch and top pause To verify</x:v>
+      </x:c>
+      <x:c r="I324" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J324" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K324" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L324" s="170"/>
+      <x:c r="M324" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N324" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="325">
+      <x:c r="A325" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B325" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C325" s="170" t="str">
+        <x:v>Standing Calf Raise</x:v>
+      </x:c>
+      <x:c r="D325" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E325" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F325" s="170" t="str">
+        <x:v>kg plates each side; guided bar excluded</x:v>
+      </x:c>
+      <x:c r="G325" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H325" s="170" t="str">
+        <x:v>Controlled; full stretch and top pause To verify</x:v>
+      </x:c>
+      <x:c r="I325" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
+      <x:c r="J325" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K325" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L325" s="170" t="str">
+        <x:v>Add one clean rep before load</x:v>
+      </x:c>
+      <x:c r="M325" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N325" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -17413,7 +17972,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74db20631d204888"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0549962d73ff49bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17950,7 +18509,7 @@
         <x:v>Clean and controlled; exactly 3 sets next time</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+    <x:row r="20" ht="48" hidden="0" customHeight="1">
       <x:c r="A20" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -17958,26 +18517,28 @@
         <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="C20" s="169" t="str">
-        <x:v>60 kg/side x 10 @ RIR 1</x:v>
+        <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D20" s="169" t="str">
-        <x:v>50-60 kg/side</x:v>
+        <x:v>35-65 kg/side</x:v>
       </x:c>
       <x:c r="E20" s="169" t="str">
-        <x:v>60 kg/side x 10 @ RIR 2</x:v>
+        <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F20" s="169" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Improve reserve; no load increase</x:v>
       </x:c>
       <x:c r="G20" s="169" t="str">
-        <x:v>Back on pad; full-foot pressure</x:v>
+        <x:v>Controlled depth; knees track toes</x:v>
       </x:c>
       <x:c r="H20" s="169" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I20" s="169"/>
-    </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="I20" s="169" t="str">
+        <x:v>Check hip before loading; progressed cleanly on 2026-08-20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" hidden="0" customHeight="1">
       <x:c r="A21" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -17985,28 +18546,28 @@
         <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="C21" s="169" t="str">
-        <x:v>150 kg: 4 clean + 4 assisted</x:v>
+        <x:v>150 kg x 7 total @ RIR 1; approx. 2-3 assisted</x:v>
       </x:c>
       <x:c r="D21" s="169" t="str">
-        <x:v>110-130 kg</x:v>
+        <x:v>100-130 kg total</x:v>
       </x:c>
       <x:c r="E21" s="169" t="str">
-        <x:v>130 kg x 11-12 @ RIR 2</x:v>
+        <x:v>130 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F21" s="169" t="str">
-        <x:v>Clean reps before load</x:v>
+        <x:v>Clean reps only; omit 150 kg</x:v>
       </x:c>
       <x:c r="G21" s="169" t="str">
-        <x:v>No hand assistance</x:v>
+        <x:v>No hand assistance; controlled depth</x:v>
       </x:c>
       <x:c r="H21" s="169" t="str">
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I21" s="169" t="str">
-        <x:v>150 kg is not an 8-clean-rep result</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
+        <x:v>Approx. 4-5 clean reps at 150 kg To verify; hip pain follow-up required</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" hidden="0" customHeight="1">
       <x:c r="A22" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -18014,26 +18575,28 @@
         <x:v>Leg Extension</x:v>
       </x:c>
       <x:c r="C22" s="169" t="str">
-        <x:v>45 kg x 12 @ RIR 1</x:v>
+        <x:v>50 kg x 11 @ RIR 1</x:v>
       </x:c>
       <x:c r="D22" s="169" t="str">
-        <x:v>35-45 kg</x:v>
+        <x:v>40-50 kg</x:v>
       </x:c>
       <x:c r="E22" s="169" t="str">
-        <x:v>45 kg x 12 @ RIR 2</x:v>
+        <x:v>50 kg x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F22" s="169" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Improve reserve before load</x:v>
       </x:c>
       <x:c r="G22" s="169" t="str">
-        <x:v>Pause at top</x:v>
+        <x:v>Controlled lockout; no momentum</x:v>
       </x:c>
       <x:c r="H22" s="169" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I22" s="169"/>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="I22" s="169" t="str">
+        <x:v>Progressed reps on 2026-08-20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="48" hidden="0" customHeight="1">
       <x:c r="A23" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -18041,28 +18604,28 @@
         <x:v>Leg Curl</x:v>
       </x:c>
       <x:c r="C23" s="169" t="str">
-        <x:v>40 kg x 8 @ RIR 1; form To verify</x:v>
+        <x:v>35 kg x 9 @ RIR 0</x:v>
       </x:c>
       <x:c r="D23" s="169" t="str">
-        <x:v>35-40 kg</x:v>
+        <x:v>30-35 kg</x:v>
       </x:c>
       <x:c r="E23" s="169" t="str">
-        <x:v>35 kg x 12-15 strict @ RIR 2</x:v>
+        <x:v>30 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F23" s="169" t="str">
-        <x:v>Verify range before load</x:v>
+        <x:v>Reduce failure exposure</x:v>
       </x:c>
       <x:c r="G23" s="169" t="str">
-        <x:v>Hips stable; full controlled range</x:v>
+        <x:v>Full range; hips down</x:v>
       </x:c>
       <x:c r="H23" s="169" t="str">
-        <x:v>Verify</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I23" s="169" t="str">
-        <x:v>40 kg sets may have shortened range or hip movement</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
+        <x:v>Full range at 35 kg remains To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="48" hidden="0" customHeight="1">
       <x:c r="A24" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -18089,7 +18652,7 @@
       </x:c>
       <x:c r="I24" s="169"/>
     </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
+    <x:row r="25" ht="48" hidden="0" customHeight="1">
       <x:c r="A25" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -18116,7 +18679,7 @@
       </x:c>
       <x:c r="I25" s="169"/>
     </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
+    <x:row r="26" ht="48" hidden="0" customHeight="1">
       <x:c r="A26" s="169" t="str">
         <x:v>Legs</x:v>
       </x:c>
@@ -18124,25 +18687,25 @@
         <x:v>Standing Calf Raise</x:v>
       </x:c>
       <x:c r="C26" s="169" t="str">
-        <x:v>Bar +20 kg/side x 16 @ RIR 2</x:v>
+        <x:v>+20 kg/side x 16 @ RIR 2</x:v>
       </x:c>
       <x:c r="D26" s="169" t="str">
-        <x:v>Bar +20 kg/side</x:v>
+        <x:v>+10 to +20 kg/side</x:v>
       </x:c>
       <x:c r="E26" s="169" t="str">
-        <x:v>17-18 reps @ RIR 2</x:v>
+        <x:v>+20 kg/side x 17 @ RIR 2</x:v>
       </x:c>
       <x:c r="F26" s="169" t="str">
-        <x:v>Add reps first</x:v>
+        <x:v>Add clean rep</x:v>
       </x:c>
       <x:c r="G26" s="169" t="str">
-        <x:v>Full stretch; top pause</x:v>
+        <x:v>Full stretch and top pause</x:v>
       </x:c>
       <x:c r="H26" s="169" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I26" s="169" t="str">
-        <x:v>Guided bar machine</x:v>
+        <x:v>Guided bar excluded from recorded load</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18622,7 +19185,7 @@
         <x:v>Bar excluded; use genuine preparation separately</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="38" customHeight="1">
+    <x:row r="44" ht="48" customHeight="1">
       <x:c r="A44" s="170" t="str">
         <x:v>Shoulders</x:v>
       </x:c>
@@ -18651,7 +19214,7 @@
         <x:v>Reported loaded-set count remains To verify</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="38" customHeight="1">
+    <x:row r="45" ht="48" customHeight="1">
       <x:c r="A45" s="170" t="str">
         <x:v>Shoulders</x:v>
       </x:c>
@@ -18680,7 +19243,7 @@
         <x:v>Grip and exact effective stack To verify</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="38" customHeight="1">
+    <x:row r="46" ht="48" customHeight="1">
       <x:c r="A46" s="170" t="str">
         <x:v>Core</x:v>
       </x:c>
@@ -18709,7 +19272,7 @@
         <x:v>No lower-back discomfort reported</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="38" customHeight="1">
+    <x:row r="47" ht="48" customHeight="1">
       <x:c r="A47" s="170" t="str">
         <x:v>Biceps</x:v>
       </x:c>
@@ -18736,6 +19299,35 @@
       </x:c>
       <x:c r="I47" s="170" t="str">
         <x:v>New clean baseline; replaces Cable Curl in active sequence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="48" customHeight="1">
+      <x:c r="A48" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="B48" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="C48" s="170" t="str">
+        <x:v>15 kg each x 12 @ RIR 2; lower-back dominant</x:v>
+      </x:c>
+      <x:c r="D48" s="170" t="str">
+        <x:v>10 kg each technique only</x:v>
+      </x:c>
+      <x:c r="E48" s="170" t="str">
+        <x:v>10 kg each x 10-12 @ RIR 3-4</x:v>
+      </x:c>
+      <x:c r="F48" s="170" t="str">
+        <x:v>Technique reset; do not add load</x:v>
+      </x:c>
+      <x:c r="G48" s="170" t="str">
+        <x:v>Wall hinge; dumbbells close; hamstring-controlled depth</x:v>
+      </x:c>
+      <x:c r="H48" s="170" t="str">
+        <x:v>Verify technique</x:v>
+      </x:c>
+      <x:c r="I48" s="170" t="str">
+        <x:v>Lower-back dominant; little post-session hip pain; stop if either persists</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18763,7 +19355,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R063d414910984bcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a7daaa3155e41d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19481,16 +20073,28 @@
       <x:c r="Q20" s="59" t="n"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="220"/>
+      <x:c r="A21" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
       <x:c r="B21" s="170"/>
       <x:c r="C21" s="170"/>
-      <x:c r="D21" s="170"/>
-      <x:c r="E21" s="170"/>
-      <x:c r="F21" s="170"/>
+      <x:c r="D21" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E21" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F21" s="170" t="str">
+        <x:v>Post: normal lower-back pump; little hip pain (side, location, trigger and 0-10 severity To verify); no knee pain reported</x:v>
+      </x:c>
       <x:c r="G21" s="170"/>
       <x:c r="H21" s="170"/>
-      <x:c r="I21" s="170"/>
-      <x:c r="J21" s="170"/>
+      <x:c r="I21" s="170" t="str">
+        <x:v>Leg workout - 100 min; stairs/walking better than last Legs session</x:v>
+      </x:c>
+      <x:c r="J21" s="170" t="str">
+        <x:v>Started Medium; full EAA+ scoop (100 mg caffeine); no coffee; approximately 2-3 assisted reps on 150 kg leg press, all other sets unassisted; pre-session soreness and pre-session knee/hip/lower-back status To verify</x:v>
+      </x:c>
       <x:c r="K21" s="59" t="n"/>
       <x:c r="L21" s="59" t="n"/>
       <x:c r="M21" s="59" t="n"/>
@@ -22956,7 +23560,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc911a8c4399b4753"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0322b9f25b744875"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23677,13 +24281,55 @@
         <x:v>Keep incline curl in the active sequence; do not force the bottom stretch</x:v>
       </x:c>
     </x:row>
+    <x:row r="47" ht="52" customHeight="1">
+      <x:c r="A47" s="170" t="str">
+        <x:v>Legs effort and fatigue</x:v>
+      </x:c>
+      <x:c r="B47" s="170" t="str">
+        <x:v>2026-08-20 used exactly 18 sets: 13 at RIR 2, four at RIR 1 and one at RIR 0; final energy Low; duration 100 min</x:v>
+      </x:c>
+      <x:c r="C47" s="170" t="str">
+        <x:v>Volume cap was respected, but one failure set and one assisted set kept effort too high</x:v>
+      </x:c>
+      <x:c r="D47" s="170" t="str">
+        <x:v>Next Legs: no assisted repetitions, no RIR 0 work, and retain the 18-set ceiling</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="52" customHeight="1">
+      <x:c r="A48" s="170" t="str">
+        <x:v>RDL technique baseline</x:v>
+      </x:c>
+      <x:c r="B48" s="170" t="str">
+        <x:v>Dumbbell RDL at 12.5-15 kg each produced more lower-back sensation than hamstring tension; post-session back feeling was a normal pump, not pain</x:v>
+      </x:c>
+      <x:c r="C48" s="170" t="str">
+        <x:v>This is not a load-progression baseline because the intended muscle did not dominate</x:v>
+      </x:c>
+      <x:c r="D48" s="170" t="str">
+        <x:v>Reset to 10 kg each after a wall-hinge drill; stop if the back dominates or hip pain appears</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="52" customHeight="1">
+      <x:c r="A49" s="170" t="str">
+        <x:v>Hip pain follow-up</x:v>
+      </x:c>
+      <x:c r="B49" s="170" t="str">
+        <x:v>A little hip pain was reported after the 2026-08-20 Legs workout; side, exact location, trigger and 0-10 severity remain To verify</x:v>
+      </x:c>
+      <x:c r="C49" s="170" t="str">
+        <x:v>Do not infer a diagnosis or progress hip-loaded work until the symptom is characterized</x:v>
+      </x:c>
+      <x:c r="D49" s="170" t="str">
+        <x:v>Collect details before Shoulders; modify or stop training if pain persists, worsens or affects walking</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad9f46752b564c0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R444ede792397401f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24197,14 +24843,30 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="220"/>
-      <x:c r="B20" s="170"/>
-      <x:c r="C20" s="170"/>
-      <x:c r="D20" s="170"/>
-      <x:c r="E20" s="170"/>
-      <x:c r="F20" s="170"/>
-      <x:c r="G20" s="170"/>
-      <x:c r="H20" s="170"/>
+      <x:c r="A20" s="220" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="B20" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C20" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D20" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E20" s="170" t="str">
+        <x:v>Yellow</x:v>
+      </x:c>
+      <x:c r="F20" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; 100 min; normal lower-back pump without pain; little hip pain with details To verify; no knee pain reported; stairs/walking better than last Legs session; full EAA+; no coffee; only the 150 kg leg-press set included assistance</x:v>
+      </x:c>
+      <x:c r="G20" s="170" t="str">
+        <x:v>Hack squat, leg extension and calf work progressed, and post-session walking/stairs improved. However, the RDL remained lower-back dominant, leg curl reached RIR 0, the top leg-press set again needed assistance, final energy was low, and hip pain requires verification.</x:v>
+      </x:c>
+      <x:c r="H20" s="170" t="str">
+        <x:v>Keep the 18-set cap; no assisted reps or failure; reset RDL technique at 10 kg each; omit 150 kg leg press; verify hip pain before Shoulders</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="220"/>
@@ -24268,7 +24930,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1efd438a3e04901"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24e4216281e4def"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24445,13 +25107,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>No joint pain reported through 2026-08-19. The lower-biceps pump after the 2026-08-18 Chest session resolved before Biceps training; 2026-08-19 ended with only the usual overall biceps sensation.</x:v>
+        <x:v>After Legs on 2026-08-20: little hip pain (side, exact location, trigger and 0-10 severity To verify); normal lower-back muscular pump without pain; no knee pain reported.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Continue pain checks; stop for sharp or localized distal-biceps pain</x:v>
+        <x:v>Clarify hip details before next workout; stop or modify if pain persists, worsens or alters movement</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -24633,13 +25295,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Completed Biceps on 2026-08-19 in the retained one-body-part split. Legs is next, subject to fresh readiness.</x:v>
+        <x:v>Completed Legs on 2026-08-20 in the retained one-body-part split. Shoulders is next, subject to fresh readiness and resolution/clarification of hip pain.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Collect fresh sleep, energy, soreness and knee/hip/lower-back check before Legs</x:v>
+        <x:v>Collect sleep, energy, shoulder soreness/pain and hip status before Shoulders</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -24839,7 +25501,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8eb5250e1bb42f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e4b6d29a2554207"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25942,10 +26604,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red42d8c1db2549b6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2bc9c86ac3b4f85"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77a05e1466bb4eaa"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5cfc705222a54ccf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra11dfd6a54ad4a14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40e75c93aeb84e2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R433d1a0e960c49e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R298e2f93a00f467a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 21 shoulder workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R61df015f813d4cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc6a3550a76f341c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rbce06624c8c04a51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Raf6c4ab25b8d4e6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R4b00cc6ad16141ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Re2b80adfaf484025"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R3101ed04a912447b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R5826c174d2c44d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Raf23db2981af4149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R548dcf368da34396"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Re7adbc22484845ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc37c47c3c06a459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4d09564027604157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rf030130178b946af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rf55f9a4b9bcf4487"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R43a1ee41aa6c4396"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rd190999bdf644252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R2ddb02957a6d4f0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R0996b787be6d4e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R605e75056c6d4fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R5aaa8e8652a44fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R6a5aa5d1e56e460a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1a683b2447f4679"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4dd6d9471c5b4a1f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N325" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N350" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1803,7 +1803,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2523,7 +2523,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R416b9c2858bb4dc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4c81b3f03742f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3926,7 +3926,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51561240eea94c71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ff582cd690f4edd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4054,11 +4054,11 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="inlineStr">
@@ -4096,8 +4096,7 @@
         <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="L6" s="140" t="n">
-        <x:f>SUMIF('Session Summary'!$B$5:$B$200,K6,'Session Summary'!$C$5:$C$200)</x:f>
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4518,22 +4517,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Hack Squat</x:v>
+        <x:v>Dumbbell Shoulder Press</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>65 kg/side x 10 @ RIR 2</x:v>
+        <x:v>22.5 kg each x 8 @ RIR 1</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>65 kg/side x 10 @ RIR 2</x:v>
+        <x:v>22.5 kg x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>No load increase; verify hip</x:v>
+        <x:v>Improve reserve; no load increase</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4544,22 +4543,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Leg Press</x:v>
+        <x:v>Reverse Pec Deck</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>150 kg x 7 total; approx. 2-3 assisted</x:v>
+        <x:v>35 kg x 10 @ RIR 3</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>130 kg x 9-10 @ RIR 2</x:v>
+        <x:v>35 kg x 11-12 @ RIR 2-3</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Omit 150 kg; clean reps only</x:v>
+        <x:v>Add controlled reps</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4570,22 +4569,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Dumbbell Romanian Deadlift</x:v>
+        <x:v>Single-Arm Cable Lateral Raise</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>15 kg each x 12 @ RIR 2; back dominant</x:v>
+        <x:v>10 kg x 15/arm @ RIR 2</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>10 kg each x 10-12 @ RIR 3-4</x:v>
+        <x:v>10 kg x 16/arm @ RIR 2</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Verify technique</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Wall-hinge reset; stop if back/hip symptoms</x:v>
+        <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4596,22 +4595,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Leg Curl</x:v>
+        <x:v>Dumbbell Shrug</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>35 kg x 9 @ RIR 0</x:v>
+        <x:v>40 kg each x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>30 kg x 12 @ RIR 2</x:v>
+        <x:v>40 kg each x 11-12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>Active / Preferred</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Full range; no failure</x:v>
+        <x:v>Replace low-pulley cable shrug</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4640,7 +4639,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1ebf07ccd34278"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcceaea6088af4b64"/>
 </x:worksheet>
 </file>
 
@@ -17938,6 +17937,1100 @@
       </x:c>
       <x:c r="N325" s="170" t="n">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="326">
+      <x:c r="A326" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B326" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C326" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D326" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E326" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F326" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G326" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H326" s="170" t="str">
+        <x:v>Preparation set; clean; no assistance</x:v>
+      </x:c>
+      <x:c r="I326" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J326" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K326" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L326" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M326" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N326" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="327">
+      <x:c r="A327" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B327" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C327" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D327" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E327" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F327" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G327" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H327" s="170" t="str">
+        <x:v>Clean; no assistance</x:v>
+      </x:c>
+      <x:c r="I327" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J327" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K327" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L327" s="170" t="str">
+        <x:v>Added one rep from prior session</x:v>
+      </x:c>
+      <x:c r="M327" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N327" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="328">
+      <x:c r="A328" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B328" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C328" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D328" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E328" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F328" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G328" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H328" s="170" t="str">
+        <x:v>Clean; no assistance</x:v>
+      </x:c>
+      <x:c r="I328" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J328" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K328" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L328" s="170" t="str">
+        <x:v>Matched reps with improved reserve</x:v>
+      </x:c>
+      <x:c r="M328" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N328" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="329">
+      <x:c r="A329" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B329" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C329" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D329" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E329" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F329" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G329" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H329" s="170" t="str">
+        <x:v>Clean; no assistance</x:v>
+      </x:c>
+      <x:c r="I329" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J329" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K329" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L329" s="170" t="str">
+        <x:v>Matched top set; improve reserve before load</x:v>
+      </x:c>
+      <x:c r="M329" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N329" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="330">
+      <x:c r="A330" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B330" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C330" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D330" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E330" s="170" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F330" s="170" t="str">
+        <x:v>kg plates each side; unloaded resistance excluded</x:v>
+      </x:c>
+      <x:c r="G330" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H330" s="170" t="str">
+        <x:v>Controlled; no shrug reported</x:v>
+      </x:c>
+      <x:c r="I330" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J330" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K330" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L330" s="170"/>
+      <x:c r="M330" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N330" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="331">
+      <x:c r="A331" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B331" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C331" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D331" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E331" s="170" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F331" s="170" t="str">
+        <x:v>kg plates each side; unloaded resistance excluded</x:v>
+      </x:c>
+      <x:c r="G331" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H331" s="170" t="str">
+        <x:v>Controlled; no shrug reported</x:v>
+      </x:c>
+      <x:c r="I331" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J331" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K331" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L331" s="170"/>
+      <x:c r="M331" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N331" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="332">
+      <x:c r="A332" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B332" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C332" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D332" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E332" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F332" s="170" t="str">
+        <x:v>kg plates each side; unloaded resistance excluded</x:v>
+      </x:c>
+      <x:c r="G332" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H332" s="170" t="str">
+        <x:v>Controlled; no shrug reported</x:v>
+      </x:c>
+      <x:c r="I332" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J332" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K332" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L332" s="170" t="str">
+        <x:v>New 5 kg/side baseline; machine resistance To verify</x:v>
+      </x:c>
+      <x:c r="M332" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N332" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="333">
+      <x:c r="A333" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B333" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C333" s="170" t="str">
+        <x:v>Experimental Rear-Delt Lateral-Raise Machine</x:v>
+      </x:c>
+      <x:c r="D333" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E333" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F333" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G333" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H333" s="170" t="str">
+        <x:v>Experimental rear-delt movement performed facing away from machine; exact setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I333" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J333" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K333" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L333" s="170" t="str">
+        <x:v>Counts toward fatigue; exclude from next active sequence</x:v>
+      </x:c>
+      <x:c r="M333" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N333" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="334">
+      <x:c r="A334" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B334" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C334" s="170" t="str">
+        <x:v>Experimental Rear-Delt Lateral-Raise Machine</x:v>
+      </x:c>
+      <x:c r="D334" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E334" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F334" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G334" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H334" s="170" t="str">
+        <x:v>Experimental rear-delt movement performed facing away from machine; exact setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I334" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J334" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K334" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L334" s="170" t="str">
+        <x:v>Counts toward fatigue; exclude from next active sequence</x:v>
+      </x:c>
+      <x:c r="M334" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N334" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="335">
+      <x:c r="A335" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B335" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C335" s="170" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D335" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E335" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F335" s="170" t="str">
+        <x:v>kg total machine load</x:v>
+      </x:c>
+      <x:c r="G335" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H335" s="170" t="str">
+        <x:v>Controlled; no assistance</x:v>
+      </x:c>
+      <x:c r="I335" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J335" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K335" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L335" s="170" t="str">
+        <x:v>Reserve improved</x:v>
+      </x:c>
+      <x:c r="M335" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N335" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="336">
+      <x:c r="A336" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B336" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C336" s="170" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D336" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E336" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F336" s="170" t="str">
+        <x:v>kg total machine load</x:v>
+      </x:c>
+      <x:c r="G336" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H336" s="170" t="str">
+        <x:v>Controlled; no assistance</x:v>
+      </x:c>
+      <x:c r="I336" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J336" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K336" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L336" s="170" t="str">
+        <x:v>Added one rep with better reserve</x:v>
+      </x:c>
+      <x:c r="M336" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N336" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="337">
+      <x:c r="A337" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B337" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C337" s="170" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D337" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E337" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F337" s="170" t="str">
+        <x:v>kg total machine load</x:v>
+      </x:c>
+      <x:c r="G337" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H337" s="170" t="str">
+        <x:v>Controlled; no assistance</x:v>
+      </x:c>
+      <x:c r="I337" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J337" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K337" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L337" s="170" t="str">
+        <x:v>Matched reps with substantially better reserve</x:v>
+      </x:c>
+      <x:c r="M337" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N337" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="338">
+      <x:c r="A338" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B338" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C338" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D338" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E338" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F338" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G338" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H338" s="170" t="str">
+        <x:v>Controlled; comfortable height</x:v>
+      </x:c>
+      <x:c r="I338" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J338" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K338" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L338" s="170" t="str">
+        <x:v>Clear rep/reserve progression</x:v>
+      </x:c>
+      <x:c r="M338" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N338" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="339">
+      <x:c r="A339" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B339" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C339" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D339" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E339" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F339" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G339" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H339" s="170" t="str">
+        <x:v>Controlled; comfortable height</x:v>
+      </x:c>
+      <x:c r="I339" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J339" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K339" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L339" s="170"/>
+      <x:c r="M339" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N339" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="340">
+      <x:c r="A340" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B340" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C340" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D340" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E340" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F340" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G340" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H340" s="170" t="str">
+        <x:v>Controlled; comfortable height</x:v>
+      </x:c>
+      <x:c r="I340" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J340" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K340" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L340" s="170" t="str">
+        <x:v>Keep load and improve final-set reserve</x:v>
+      </x:c>
+      <x:c r="M340" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N340" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="341">
+      <x:c r="A341" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B341" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C341" s="170" t="str">
+        <x:v>Single-Arm Cable Lateral Raise</x:v>
+      </x:c>
+      <x:c r="D341" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E341" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F341" s="170" t="str">
+        <x:v>kg stack; reps each arm</x:v>
+      </x:c>
+      <x:c r="G341" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H341" s="170" t="str">
+        <x:v>Controlled; both arms completed</x:v>
+      </x:c>
+      <x:c r="I341" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J341" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K341" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L341" s="170" t="str">
+        <x:v>Progressed from 15 reps</x:v>
+      </x:c>
+      <x:c r="M341" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N341" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="342">
+      <x:c r="A342" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B342" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C342" s="170" t="str">
+        <x:v>Single-Arm Cable Lateral Raise</x:v>
+      </x:c>
+      <x:c r="D342" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E342" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F342" s="170" t="str">
+        <x:v>kg stack; reps each arm</x:v>
+      </x:c>
+      <x:c r="G342" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H342" s="170" t="str">
+        <x:v>Controlled; both arms completed</x:v>
+      </x:c>
+      <x:c r="I342" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J342" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K342" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L342" s="170" t="str">
+        <x:v>Progressed from 12 reps</x:v>
+      </x:c>
+      <x:c r="M342" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N342" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="343">
+      <x:c r="A343" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B343" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C343" s="170" t="str">
+        <x:v>Single-Arm Cable Lateral Raise</x:v>
+      </x:c>
+      <x:c r="D343" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E343" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F343" s="170" t="str">
+        <x:v>kg stack; reps each arm</x:v>
+      </x:c>
+      <x:c r="G343" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H343" s="170" t="str">
+        <x:v>Controlled; both arms completed</x:v>
+      </x:c>
+      <x:c r="I343" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J343" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K343" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L343" s="170" t="str">
+        <x:v>Progressed from 12 reps</x:v>
+      </x:c>
+      <x:c r="M343" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N343" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="344">
+      <x:c r="A344" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B344" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C344" s="170" t="str">
+        <x:v>Cable Shrug</x:v>
+      </x:c>
+      <x:c r="D344" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E344" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F344" s="170" t="str">
+        <x:v>kg total stack; straight bar on low pulley</x:v>
+      </x:c>
+      <x:c r="G344" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H344" s="170" t="str">
+        <x:v>Elbows tended to bend but were consciously controlled; low trap sensation</x:v>
+      </x:c>
+      <x:c r="I344" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J344" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K344" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L344" s="170" t="str">
+        <x:v>Experimental substitution; poor stimulus; effective cable resistance To verify</x:v>
+      </x:c>
+      <x:c r="M344" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N344" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="345">
+      <x:c r="A345" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B345" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C345" s="170" t="str">
+        <x:v>Cable Shrug</x:v>
+      </x:c>
+      <x:c r="D345" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E345" s="170" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="F345" s="170" t="str">
+        <x:v>kg total stack; straight bar on low pulley</x:v>
+      </x:c>
+      <x:c r="G345" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H345" s="170" t="str">
+        <x:v>Elbows tended to bend but were consciously controlled; low trap sensation</x:v>
+      </x:c>
+      <x:c r="I345" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J345" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K345" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L345" s="170" t="str">
+        <x:v>Experimental substitution; poor stimulus; effective cable resistance To verify</x:v>
+      </x:c>
+      <x:c r="M345" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N345" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="346">
+      <x:c r="A346" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B346" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C346" s="170" t="str">
+        <x:v>Cable Shrug</x:v>
+      </x:c>
+      <x:c r="D346" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E346" s="170" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="F346" s="170" t="str">
+        <x:v>kg total stack; straight bar on low pulley</x:v>
+      </x:c>
+      <x:c r="G346" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H346" s="170" t="str">
+        <x:v>Elbows tended to bend but were consciously controlled; low trap sensation</x:v>
+      </x:c>
+      <x:c r="I346" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J346" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K346" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L346" s="170" t="str">
+        <x:v>Replace with dumbbell or dedicated shrug next time</x:v>
+      </x:c>
+      <x:c r="M346" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N346" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="347">
+      <x:c r="A347" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B347" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C347" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="D347" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E347" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="F347" s="170" t="str">
+        <x:v>60 seconds</x:v>
+      </x:c>
+      <x:c r="G347" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H347" s="170" t="str">
+        <x:v>No form breakdown or lower-back pain reported; detailed alignment To verify</x:v>
+      </x:c>
+      <x:c r="I347" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J347" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K347" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L347" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="M347" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="N347" s="170" t="str">
+        <x:v>To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="348">
+      <x:c r="A348" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B348" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C348" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="D348" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E348" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="F348" s="170" t="str">
+        <x:v>60 seconds</x:v>
+      </x:c>
+      <x:c r="G348" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H348" s="170" t="str">
+        <x:v>No form breakdown or lower-back pain reported; detailed alignment To verify</x:v>
+      </x:c>
+      <x:c r="I348" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J348" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K348" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L348" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="M348" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="N348" s="170" t="str">
+        <x:v>To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="349">
+      <x:c r="A349" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B349" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C349" s="170" t="str">
+        <x:v>Front Plank</x:v>
+      </x:c>
+      <x:c r="D349" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E349" s="170" t="str">
+        <x:v>Body weight</x:v>
+      </x:c>
+      <x:c r="F349" s="170" t="str">
+        <x:v>60 seconds</x:v>
+      </x:c>
+      <x:c r="G349" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="H349" s="170" t="str">
+        <x:v>No form breakdown or lower-back pain reported; detailed alignment To verify</x:v>
+      </x:c>
+      <x:c r="I349" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J349" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K349" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L349" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="M349" s="170" t="str">
+        <x:v>Core finisher</x:v>
+      </x:c>
+      <x:c r="N349" s="170" t="str">
+        <x:v>To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="350">
+      <x:c r="A350" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B350" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C350" s="170" t="str">
+        <x:v>Treadmill Incline Walk</x:v>
+      </x:c>
+      <x:c r="D350" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E350" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F350" s="170" t="str">
+        <x:v>% incline; displayed speed 4 (unit To verify)</x:v>
+      </x:c>
+      <x:c r="G350" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H350" s="170" t="str">
+        <x:v>Completed 10 minutes; no hip or other pain</x:v>
+      </x:c>
+      <x:c r="I350" s="170" t="str">
+        <x:v>No shoulder, neck, elbow, wrist, hip or lower-back pain reported during or after session</x:v>
+      </x:c>
+      <x:c r="J350" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="K350" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L350" s="170" t="str">
+        <x:v>Steep conditioning finisher after Legs; use easier incline for recovery cardio</x:v>
+      </x:c>
+      <x:c r="M350" s="170" t="str">
+        <x:v>Cardio finisher</x:v>
+      </x:c>
+      <x:c r="N350" s="170" t="str">
+        <x:v>Not applicable</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17972,7 +19065,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0549962d73ff49bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cacc35ed2fc43cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18722,10 +19815,10 @@
         <x:v>17.5-22.5 kg each</x:v>
       </x:c>
       <x:c r="E27" s="170" t="str">
-        <x:v>22.5 kg x 9 @ RIR 1-2</x:v>
+        <x:v>22.5 kg each x 8 @ RIR 2 or 9 @ RIR 1-2</x:v>
       </x:c>
       <x:c r="F27" s="170" t="str">
-        <x:v>Add rep before load</x:v>
+        <x:v>Improve reserve before load</x:v>
       </x:c>
       <x:c r="G27" s="170" t="str">
         <x:v>Neutral wrist; controlled path</x:v>
@@ -18733,7 +19826,9 @@
       <x:c r="H27" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I27" s="170"/>
+      <x:c r="I27" s="170" t="str">
+        <x:v>15 kg set is preparation only; 17.5 kg reps and 20 kg reserve improved</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A28" s="170" t="str">
@@ -18801,13 +19896,13 @@
         <x:v>Reverse Pec Deck</x:v>
       </x:c>
       <x:c r="C30" s="170" t="str">
-        <x:v>35 kg x 10 @ RIR 1</x:v>
+        <x:v>35 kg x 10 @ RIR 3</x:v>
       </x:c>
       <x:c r="D30" s="170" t="str">
         <x:v>25-35 kg</x:v>
       </x:c>
       <x:c r="E30" s="170" t="str">
-        <x:v>35 kg x 11-12 @ RIR 2</x:v>
+        <x:v>35 kg x 11-12 @ RIR 2-3</x:v>
       </x:c>
       <x:c r="F30" s="170" t="str">
         <x:v>Add reps with reserve</x:v>
@@ -18818,7 +19913,9 @@
       <x:c r="H30" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I30" s="170"/>
+      <x:c r="I30" s="170" t="str">
+        <x:v>Reserve improved markedly on 2026-08-21</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A31" s="170" t="str">
@@ -18828,13 +19925,13 @@
         <x:v>Single-Arm Cable Lateral Raise</x:v>
       </x:c>
       <x:c r="C31" s="170" t="str">
-        <x:v>10 kg x 12 each arm @ RIR 2</x:v>
+        <x:v>10 kg x 15 each arm @ RIR 2</x:v>
       </x:c>
       <x:c r="D31" s="170" t="str">
         <x:v>5-10 kg stack</x:v>
       </x:c>
       <x:c r="E31" s="170" t="str">
-        <x:v>10 kg x 13-15 @ RIR 2</x:v>
+        <x:v>10 kg x 16 each arm @ RIR 2</x:v>
       </x:c>
       <x:c r="F31" s="170" t="str">
         <x:v>Add reps first</x:v>
@@ -18845,7 +19942,9 @@
       <x:c r="H31" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I31" s="170"/>
+      <x:c r="I31" s="170" t="str">
+        <x:v>Both 10 kg sets progressed from 12 to 15 reps</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A32" s="170" t="str">
@@ -18861,18 +19960,20 @@
         <x:v>30-40 kg each</x:v>
       </x:c>
       <x:c r="E32" s="170" t="str">
-        <x:v>40 kg x 11-12 @ RIR 2</x:v>
+        <x:v>40 kg each x 11-12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F32" s="170" t="str">
         <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G32" s="170" t="str">
-        <x:v>Vertical shrug; top pause</x:v>
+        <x:v>Vertical shrug; top pause; straight arms</x:v>
       </x:c>
       <x:c r="H32" s="170" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="I32" s="170"/>
+        <x:v>Active / Preferred</x:v>
+      </x:c>
+      <x:c r="I32" s="170" t="str">
+        <x:v>Use dumbbells or dedicated shrug machine; low-pulley cable shrug produced poor stimulus</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="170" t="str">
@@ -19193,25 +20294,25 @@
         <x:v>Plate-Loaded Lateral Raise Machine</x:v>
       </x:c>
       <x:c r="C44" s="170" t="str">
-        <x:v>2.5 kg/side x 15 @ RIR 2</x:v>
+        <x:v>5 kg/side x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D44" s="170" t="str">
-        <x:v>Free to 2.5 kg/side</x:v>
+        <x:v>2.5-5 kg/side</x:v>
       </x:c>
       <x:c r="E44" s="170" t="str">
-        <x:v>2.5 kg/side x 16-18 @ RIR 2</x:v>
+        <x:v>5 kg/side x 13-15 @ RIR 2</x:v>
       </x:c>
       <x:c r="F44" s="170" t="str">
-        <x:v>Add reps; cap sets</x:v>
+        <x:v>Add reps; maximum 3 sets</x:v>
       </x:c>
       <x:c r="G44" s="170" t="str">
         <x:v>No shrug; controlled eccentric</x:v>
       </x:c>
       <x:c r="H44" s="170" t="str">
-        <x:v>Verify set count</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I44" s="170" t="str">
-        <x:v>Reported loaded-set count remains To verify</x:v>
+        <x:v>Unloaded machine resistance excluded and To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
@@ -19222,16 +20323,16 @@
         <x:v>Cable Upright Row</x:v>
       </x:c>
       <x:c r="C45" s="170" t="str">
-        <x:v>50 kg x 14 @ RIR 1</x:v>
+        <x:v>50 kg x 10 @ RIR 1 after 50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D45" s="170" t="str">
-        <x:v>30-50 kg stack</x:v>
+        <x:v>40-50 kg stack</x:v>
       </x:c>
       <x:c r="E45" s="170" t="str">
-        <x:v>50 kg x 14 @ RIR 2</x:v>
+        <x:v>50 kg x 12-14 @ RIR 2</x:v>
       </x:c>
       <x:c r="F45" s="170" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Improve final-set reserve</x:v>
       </x:c>
       <x:c r="G45" s="170" t="str">
         <x:v>Pull only to comfortable height</x:v>
@@ -19240,7 +20341,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I45" s="170" t="str">
-        <x:v>Grip and exact effective stack To verify</x:v>
+        <x:v>40 kg set progressed; exact effective stack To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
@@ -19251,7 +20352,7 @@
         <x:v>Front Plank</x:v>
       </x:c>
       <x:c r="C46" s="170" t="str">
-        <x:v>3 x 60 sec strict</x:v>
+        <x:v>3 x 60 sec; form detail To verify</x:v>
       </x:c>
       <x:c r="D46" s="170" t="str">
         <x:v>Body weight</x:v>
@@ -19260,7 +20361,7 @@
         <x:v>3 x 60 sec strict</x:v>
       </x:c>
       <x:c r="F46" s="170" t="str">
-        <x:v>Add time only after perfect sets</x:v>
+        <x:v>Maintain before adding time</x:v>
       </x:c>
       <x:c r="G46" s="170" t="str">
         <x:v>Glutes tight; ribs down; no hip sag</x:v>
@@ -19269,7 +20370,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I46" s="170" t="str">
-        <x:v>No lower-back discomfort reported</x:v>
+        <x:v>No lower-back pain or breakdown reported on 2026-08-21</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="48" customHeight="1">
@@ -19328,6 +20429,64 @@
       </x:c>
       <x:c r="I48" s="170" t="str">
         <x:v>Lower-back dominant; little post-session hip pain; stop if either persists</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="52" customHeight="1">
+      <x:c r="A49" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="B49" s="170" t="str">
+        <x:v>Experimental Rear-Delt Lateral-Raise Machine</x:v>
+      </x:c>
+      <x:c r="C49" s="170" t="str">
+        <x:v>5 kg/side x 8 @ RIR 1</x:v>
+      </x:c>
+      <x:c r="D49" s="170" t="str">
+        <x:v>Historical experiment only</x:v>
+      </x:c>
+      <x:c r="E49" s="170" t="str">
+        <x:v>Do not repeat in active sequence</x:v>
+      </x:c>
+      <x:c r="F49" s="170" t="str">
+        <x:v>Use Reverse Pec Deck instead</x:v>
+      </x:c>
+      <x:c r="G49" s="170" t="str">
+        <x:v>Exact setup/path To verify</x:v>
+      </x:c>
+      <x:c r="H49" s="170" t="str">
+        <x:v>Experimental / Replaced</x:v>
+      </x:c>
+      <x:c r="I49" s="170" t="str">
+        <x:v>Two sets retained as working fatigue; not deleted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="52" customHeight="1">
+      <x:c r="A50" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="B50" s="170" t="str">
+        <x:v>Cable Shrug</x:v>
+      </x:c>
+      <x:c r="C50" s="170" t="str">
+        <x:v>80 kg x 13 @ RIR 2; poor trap sensation</x:v>
+      </x:c>
+      <x:c r="D50" s="170" t="str">
+        <x:v>Historical experiment only</x:v>
+      </x:c>
+      <x:c r="E50" s="170" t="str">
+        <x:v>Use Dumbbell Shrug target</x:v>
+      </x:c>
+      <x:c r="F50" s="170" t="str">
+        <x:v>Replace; do not progress cable load</x:v>
+      </x:c>
+      <x:c r="G50" s="170" t="str">
+        <x:v>Straight arms; dedicated shrug path</x:v>
+      </x:c>
+      <x:c r="H50" s="170" t="str">
+        <x:v>Poor stimulus / Replaced</x:v>
+      </x:c>
+      <x:c r="I50" s="170" t="str">
+        <x:v>Elbows tended to bend; effective cable resistance To verify</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19355,7 +20514,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a7daaa3155e41d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R967527592b7144ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20104,16 +21263,28 @@
       <x:c r="Q21" s="59" t="n"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="220"/>
+      <x:c r="A22" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
       <x:c r="B22" s="170"/>
       <x:c r="C22" s="170"/>
-      <x:c r="D22" s="170"/>
-      <x:c r="E22" s="170"/>
-      <x:c r="F22" s="170"/>
+      <x:c r="D22" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E22" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="F22" s="170" t="str">
+        <x:v>No pain; low-medium shoulder pump; delayed shoulder soreness To verify the following morning</x:v>
+      </x:c>
       <x:c r="G22" s="170"/>
       <x:c r="H22" s="170"/>
-      <x:c r="I22" s="170"/>
-      <x:c r="J22" s="170"/>
+      <x:c r="I22" s="170" t="str">
+        <x:v>Shoulders + 3 x 60-sec plank + 10-min treadmill - 100 min</x:v>
+      </x:c>
+      <x:c r="J22" s="170" t="str">
+        <x:v>Started Medium-High; full EAA+ scoop (100 mg caffeine); no coffee; no assistance; treadmill 12% incline at displayed speed 4 (unit To verify); cable shrug had poor trap sensation and elbow-bend tendency</x:v>
+      </x:c>
       <x:c r="K22" s="59" t="n"/>
       <x:c r="L22" s="59" t="n"/>
       <x:c r="M22" s="59" t="n"/>
@@ -23560,7 +24731,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0322b9f25b744875"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re07baeff5e124a9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24323,13 +25494,83 @@
         <x:v>Collect details before Shoulders; modify or stop training if pain persists, worsens or affects walking</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" ht="52" customHeight="1">
+      <x:c r="A50" s="170" t="str">
+        <x:v>Shoulder performance progression</x:v>
+      </x:c>
+      <x:c r="B50" s="170" t="str">
+        <x:v>2026-08-21 had 20 shoulder working sets: 5 at RIR 3, 11 at RIR 2 and 4 at RIR 1; no pain or assistance</x:v>
+      </x:c>
+      <x:c r="C50" s="170" t="str">
+        <x:v>Press, reverse pec deck and lateral raises objectively progressed</x:v>
+      </x:c>
+      <x:c r="D50" s="170" t="str">
+        <x:v>Keep loads; improve reserve before adding weight</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="52" customHeight="1">
+      <x:c r="A51" s="170" t="str">
+        <x:v>Shoulder volume over cap</x:v>
+      </x:c>
+      <x:c r="B51" s="170" t="str">
+        <x:v>Two experimental rear-delt sets raised direct shoulder volume from the planned 18 to 20 sets</x:v>
+      </x:c>
+      <x:c r="C51" s="170" t="str">
+        <x:v>The experiment still counts as fatigue even though it is not in the active sequence</x:v>
+      </x:c>
+      <x:c r="D51" s="170" t="str">
+        <x:v>Next Shoulders: exactly 18 working sets and no experimental extras</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="52" customHeight="1">
+      <x:c r="A52" s="170" t="str">
+        <x:v>Cable shrug poor stimulus</x:v>
+      </x:c>
+      <x:c r="B52" s="170" t="str">
+        <x:v>60-80 kg total-stack low-pulley cable shrugs produced low trap sensation; elbows tended to bend but were controlled</x:v>
+      </x:c>
+      <x:c r="C52" s="170" t="str">
+        <x:v>Recorded numbers are not a useful progression target; cable geometry/effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="D52" s="170" t="str">
+        <x:v>Return to dumbbell shrugs or a dedicated shrug machine</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="52" customHeight="1">
+      <x:c r="A53" s="170" t="str">
+        <x:v>Shoulder core and cardio finishers</x:v>
+      </x:c>
+      <x:c r="B53" s="170" t="str">
+        <x:v>Completed 3 x 60-sec planks and 10 min at displayed speed 4 and 12% incline without pain</x:v>
+      </x:c>
+      <x:c r="C53" s="170" t="str">
+        <x:v>The steep incline was conditioning, not easy recovery cardio, one day after Legs</x:v>
+      </x:c>
+      <x:c r="D53" s="170" t="str">
+        <x:v>When recovery is the goal use an easier 3-4% incline; speed unit To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="52" customHeight="1">
+      <x:c r="A54" s="170" t="str">
+        <x:v>Delayed soreness follow-up</x:v>
+      </x:c>
+      <x:c r="B54" s="170" t="str">
+        <x:v>Immediate shoulder pump was Low-Medium; delayed shoulder soreness remains To verify</x:v>
+      </x:c>
+      <x:c r="C54" s="170" t="str">
+        <x:v>Immediate pump does not establish recovery readiness</x:v>
+      </x:c>
+      <x:c r="D54" s="170" t="str">
+        <x:v>Check shoulder, hip and leg response the following morning before Triceps</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R444ede792397401f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R564d1acb3f494287"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24869,14 +26110,30 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="220"/>
-      <x:c r="B21" s="170"/>
-      <x:c r="C21" s="170"/>
-      <x:c r="D21" s="170"/>
-      <x:c r="E21" s="170"/>
-      <x:c r="F21" s="170"/>
-      <x:c r="G21" s="170"/>
-      <x:c r="H21" s="170"/>
+      <x:c r="A21" s="220" t="n">
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="B21" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C21" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D21" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E21" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F21" s="170" t="str">
+        <x:v>Good sleep; Medium-High start and Medium final energy; no shoulder, neck, elbow, wrist, hip or lower-back pain; 100 min; no assistance; low-medium shoulder pump; full EAA+; no coffee; delayed soreness To verify</x:v>
+      </x:c>
+      <x:c r="G21" s="170" t="str">
+        <x:v>Pressing reserve, reverse-pec-deck reserve and lateral-raise performance progressed without pain. However, 20 shoulder working sets exceeded the 18-set cap, the cable shrug produced poor trap stimulus, and the 12% incline finisher added unnecessary fatigue after Legs.</x:v>
+      </x:c>
+      <x:c r="H21" s="170" t="str">
+        <x:v>Return to exactly 18 shoulder working sets; no experimental extras; keep loads and improve reserve; replace cable shrug with dumbbell/dedicated shrug; check delayed soreness before Triceps</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="220"/>
@@ -24930,7 +26187,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd24e4216281e4def"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91c53d21f9884b57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25107,13 +26364,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Legs on 2026-08-20: little hip pain (side, exact location, trigger and 0-10 severity To verify); normal lower-back muscular pump without pain; no knee pain reported.</x:v>
+        <x:v>After Shoulders on 2026-08-21: no shoulder, neck, elbow, wrist, hip or lower-back pain. Low-medium immediate shoulder pump; delayed soreness remains To verify.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Clarify hip details before next workout; stop or modify if pain persists, worsens or alters movement</x:v>
+        <x:v>Check next-morning shoulder, hip and leg response before Triceps</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -25295,13 +26552,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Completed Legs on 2026-08-20 in the retained one-body-part split. Shoulders is next, subject to fresh readiness and resolution/clarification of hip pain.</x:v>
+        <x:v>Completed Shoulders on 2026-08-21. Triceps is next in the retained one-body-part split, subject to fresh readiness and delayed-soreness checks.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Collect sleep, energy, shoulder soreness/pain and hip status before Shoulders</x:v>
+        <x:v>Collect sleep, energy, shoulder soreness and joint pain before Triceps</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -25501,7 +26758,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e4b6d29a2554207"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1054a22a7924ce5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26604,10 +27861,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra11dfd6a54ad4a14"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40e75c93aeb84e2a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R433d1a0e960c49e3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R298e2f93a00f467a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff2d2deb8cbe43e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44a20160a524903"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f6f0c21a7db44fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29a59995b8d4d69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 22 triceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc37c47c3c06a459b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4d09564027604157"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rf030130178b946af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rf55f9a4b9bcf4487"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R43a1ee41aa6c4396"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rd190999bdf644252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R2ddb02957a6d4f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R0996b787be6d4e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R605e75056c6d4fd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R5aaa8e8652a44fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R6a5aa5d1e56e460a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R28f3aae7031d404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R8036e5f1fed54fd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R9e52479cd8a74783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R4972e4c0f18c4f39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rde71f2db43ca4f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R1de8e34b109842d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rc8a63917148745ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Re2a57659ae0c4f77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R73a990ecbfa642a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R7085d429fef34559"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R4fc0d84c25004fb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4dd6d9471c5b4a1f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb54775ee8f494ec2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N350" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N370" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D54" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2523,7 +2523,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4c81b3f03742f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc70219399d9e43a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3926,7 +3926,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ff582cd690f4edd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf34c30b9df434337"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4054,7 +4054,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4122,8 +4122,7 @@
         <x:v>Triceps</x:v>
       </x:c>
       <x:c r="L7" s="146" t="n">
-        <x:f>SUMIF('Session Summary'!$B$5:$B$200,K7,'Session Summary'!$C$5:$C$200)</x:f>
-        <x:v>14</x:v>
+        <x:v>33</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4517,22 +4516,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Dumbbell Shoulder Press</x:v>
+        <x:v>Straight-Bar Pushdown</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>22.5 kg each x 8 @ RIR 1</x:v>
+        <x:v>60 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>22.5 kg x 8 @ RIR 2</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Improve reserve; no load increase</x:v>
+        <x:v>Preparation separate; improve reserve</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4543,22 +4542,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Reverse Pec Deck</x:v>
+        <x:v>Rope Pushdown</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>35 kg x 10 @ RIR 3</x:v>
+        <x:v>40 kg x 11 @ RIR 1</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>35 kg x 11-12 @ RIR 2-3</x:v>
+        <x:v>40 kg x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify volume</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Add controlled reps</x:v>
+        <x:v>Exactly 3 sets; no repeat set</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4569,22 +4568,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Single-Arm Cable Lateral Raise</x:v>
+        <x:v>Overhead DB Extension</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>10 kg x 15/arm @ RIR 2</x:v>
+        <x:v>25 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>10 kg x 16/arm @ RIR 2</x:v>
+        <x:v>25 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Add reps before load</x:v>
+        <x:v>Add clean rep before load</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4595,22 +4594,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Dumbbell Shrug</x:v>
+        <x:v>Assisted Dip Machine</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>40 kg each x 10 @ RIR 2</x:v>
+        <x:v>50 kg assist x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>40 kg each x 11-12 @ RIR 2</x:v>
+        <x:v>50 kg assist x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>Active / Preferred</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Replace low-pulley cable shrug</x:v>
+        <x:v>Higher assistance is easier</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4639,7 +4638,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcceaea6088af4b64"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca77882f9964ee8"/>
 </x:worksheet>
 </file>
 
@@ -19031,6 +19030,866 @@
       </x:c>
       <x:c r="N350" s="170" t="str">
         <x:v>Not applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="351">
+      <x:c r="A351" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B351" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C351" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D351" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E351" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F351" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G351" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H351" s="170" t="str">
+        <x:v>Preparation set; controlled; no assistance</x:v>
+      </x:c>
+      <x:c r="I351" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J351" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K351" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L351" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M351" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N351" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="352">
+      <x:c r="A352" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B352" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C352" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D352" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E352" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F352" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G352" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H352" s="170" t="str">
+        <x:v>Elbows fixed; no forced reps</x:v>
+      </x:c>
+      <x:c r="I352" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J352" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K352" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L352" s="170"/>
+      <x:c r="M352" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N352" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="353">
+      <x:c r="A353" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B353" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C353" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D353" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E353" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F353" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G353" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H353" s="170" t="str">
+        <x:v>Elbows fixed; no forced reps</x:v>
+      </x:c>
+      <x:c r="I353" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J353" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K353" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L353" s="170" t="str">
+        <x:v>Added one rep from prior baseline</x:v>
+      </x:c>
+      <x:c r="M353" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N353" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="354">
+      <x:c r="A354" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B354" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C354" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D354" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E354" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F354" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G354" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H354" s="170" t="str">
+        <x:v>Elbows fixed; no forced reps</x:v>
+      </x:c>
+      <x:c r="I354" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J354" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K354" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L354" s="170" t="str">
+        <x:v>Reached rep target; improve reserve before load</x:v>
+      </x:c>
+      <x:c r="M354" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N354" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="355">
+      <x:c r="A355" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B355" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C355" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D355" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E355" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F355" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G355" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H355" s="170" t="str">
+        <x:v>Controlled; rope spread; no forced reps</x:v>
+      </x:c>
+      <x:c r="I355" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J355" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K355" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L355" s="170"/>
+      <x:c r="M355" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N355" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="356">
+      <x:c r="A356" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B356" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C356" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D356" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E356" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F356" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G356" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H356" s="170" t="str">
+        <x:v>Controlled; rope spread; no forced reps</x:v>
+      </x:c>
+      <x:c r="I356" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J356" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K356" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L356" s="170"/>
+      <x:c r="M356" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N356" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="357">
+      <x:c r="A357" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B357" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C357" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D357" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E357" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F357" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G357" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H357" s="170" t="str">
+        <x:v>Controlled; rope spread; no forced reps</x:v>
+      </x:c>
+      <x:c r="I357" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J357" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K357" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L357" s="170"/>
+      <x:c r="M357" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N357" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="358">
+      <x:c r="A358" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B358" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C358" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D358" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E358" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F358" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G358" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H358" s="170" t="str">
+        <x:v>Controlled; rope spread; no forced reps</x:v>
+      </x:c>
+      <x:c r="I358" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J358" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K358" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L358" s="170" t="str">
+        <x:v>Fourth working set exceeded plan; do not progress load</x:v>
+      </x:c>
+      <x:c r="M358" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N358" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="359">
+      <x:c r="A359" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B359" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C359" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D359" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E359" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F359" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G359" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H359" s="170" t="str">
+        <x:v>Ribs down; elbows stable; shoulder soreness did not increase</x:v>
+      </x:c>
+      <x:c r="I359" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J359" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K359" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L359" s="170"/>
+      <x:c r="M359" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N359" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="360">
+      <x:c r="A360" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B360" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C360" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D360" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E360" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F360" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G360" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H360" s="170" t="str">
+        <x:v>Ribs down; elbows stable; shoulder soreness did not increase</x:v>
+      </x:c>
+      <x:c r="I360" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J360" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K360" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L360" s="170"/>
+      <x:c r="M360" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N360" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="361">
+      <x:c r="A361" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B361" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C361" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D361" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E361" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F361" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G361" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H361" s="170" t="str">
+        <x:v>Ribs down; elbows stable; shoulder soreness did not increase</x:v>
+      </x:c>
+      <x:c r="I361" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J361" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K361" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L361" s="170" t="str">
+        <x:v>Keep load and add one clean rep</x:v>
+      </x:c>
+      <x:c r="M361" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N361" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="362">
+      <x:c r="A362" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B362" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C362" s="170" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D362" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E362" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F362" s="170" t="str">
+        <x:v>kg stack; reps each arm</x:v>
+      </x:c>
+      <x:c r="G362" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H362" s="170" t="str">
+        <x:v>Both arms completed; side-to-side difference To verify</x:v>
+      </x:c>
+      <x:c r="I362" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J362" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K362" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L362" s="170"/>
+      <x:c r="M362" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N362" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="363">
+      <x:c r="A363" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B363" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C363" s="170" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D363" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E363" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F363" s="170" t="str">
+        <x:v>kg stack; reps each arm</x:v>
+      </x:c>
+      <x:c r="G363" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H363" s="170" t="str">
+        <x:v>Both arms completed; side-to-side difference To verify</x:v>
+      </x:c>
+      <x:c r="I363" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J363" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K363" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L363" s="170" t="str">
+        <x:v>Better reserve than prior RIR-1 baseline</x:v>
+      </x:c>
+      <x:c r="M363" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N363" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="364">
+      <x:c r="A364" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B364" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C364" s="170" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D364" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E364" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F364" s="170" t="str">
+        <x:v>kg stack; reps each arm</x:v>
+      </x:c>
+      <x:c r="G364" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H364" s="170" t="str">
+        <x:v>Both arms completed; side-to-side difference To verify</x:v>
+      </x:c>
+      <x:c r="I364" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J364" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K364" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L364" s="170" t="str">
+        <x:v>Better reserve than prior RIR-1 baseline</x:v>
+      </x:c>
+      <x:c r="M364" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N364" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="365">
+      <x:c r="A365" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B365" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C365" s="170" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D365" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E365" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F365" s="170" t="str">
+        <x:v>kg one dumbbell total</x:v>
+      </x:c>
+      <x:c r="G365" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H365" s="170" t="str">
+        <x:v>Back supported; ribs down; no forced reps</x:v>
+      </x:c>
+      <x:c r="I365" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J365" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K365" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L365" s="170"/>
+      <x:c r="M365" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N365" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="366">
+      <x:c r="A366" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B366" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C366" s="170" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D366" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E366" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F366" s="170" t="str">
+        <x:v>kg one dumbbell total</x:v>
+      </x:c>
+      <x:c r="G366" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H366" s="170" t="str">
+        <x:v>Back supported; ribs down; no forced reps</x:v>
+      </x:c>
+      <x:c r="I366" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J366" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K366" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L366" s="170" t="str">
+        <x:v>Added one rep</x:v>
+      </x:c>
+      <x:c r="M366" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N366" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="367">
+      <x:c r="A367" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B367" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C367" s="170" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D367" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E367" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F367" s="170" t="str">
+        <x:v>kg one dumbbell total</x:v>
+      </x:c>
+      <x:c r="G367" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H367" s="170" t="str">
+        <x:v>Back supported; ribs down; no forced reps</x:v>
+      </x:c>
+      <x:c r="I367" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J367" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K367" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L367" s="170" t="str">
+        <x:v>Third set completed despite live reduction to two; retained as fatigue</x:v>
+      </x:c>
+      <x:c r="M367" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N367" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="368">
+      <x:c r="A368" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B368" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C368" s="170" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="D368" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E368" s="170" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="F368" s="170" t="str">
+        <x:v>kg machine assistance; higher is easier</x:v>
+      </x:c>
+      <x:c r="G368" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H368" s="170" t="str">
+        <x:v>Controlled depth; no forced human assistance</x:v>
+      </x:c>
+      <x:c r="I368" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J368" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K368" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L368" s="170"/>
+      <x:c r="M368" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N368" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="369">
+      <x:c r="A369" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B369" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C369" s="170" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="D369" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E369" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F369" s="170" t="str">
+        <x:v>kg machine assistance; higher is easier</x:v>
+      </x:c>
+      <x:c r="G369" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H369" s="170" t="str">
+        <x:v>Controlled depth; no forced human assistance</x:v>
+      </x:c>
+      <x:c r="I369" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J369" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K369" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L369" s="170"/>
+      <x:c r="M369" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N369" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="370">
+      <x:c r="A370" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B370" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C370" s="170" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="D370" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E370" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F370" s="170" t="str">
+        <x:v>kg machine assistance; higher is easier</x:v>
+      </x:c>
+      <x:c r="G370" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H370" s="170" t="str">
+        <x:v>Controlled depth; no forced human assistance</x:v>
+      </x:c>
+      <x:c r="I370" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
+      <x:c r="J370" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K370" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L370" s="170" t="str">
+        <x:v>Third set completed despite live reduction to two; improve reserve before reducing assistance</x:v>
+      </x:c>
+      <x:c r="M370" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N370" s="170" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19065,7 +19924,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cacc35ed2fc43cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23affba764aa48b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19975,7 +20834,7 @@
         <x:v>Use dumbbells or dedicated shrug machine; low-pulley cable shrug produced poor stimulus</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
+    <x:row r="33" ht="48" hidden="0" customHeight="1">
       <x:c r="A33" s="170" t="str">
         <x:v>Triceps</x:v>
       </x:c>
@@ -19983,28 +20842,28 @@
         <x:v>Straight-Bar Pushdown</x:v>
       </x:c>
       <x:c r="C33" s="170" t="str">
-        <x:v>60 kg x 8 @ RIR 1 after rope work</x:v>
+        <x:v>60 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="D33" s="170" t="str">
         <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E33" s="170" t="str">
-        <x:v>60 kg x 9 @ RIR 1-2</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F33" s="170" t="str">
-        <x:v>Use only 3 working sets</x:v>
+        <x:v>Exactly 3 working sets; improve reserve</x:v>
       </x:c>
       <x:c r="G33" s="170" t="str">
         <x:v>Elbows fixed; torso still</x:v>
       </x:c>
       <x:c r="H33" s="170" t="str">
-        <x:v>Modify volume</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I33" s="170" t="str">
-        <x:v>Exercise order affected comparison</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>45 kg x 16 was preparation only; 55 and 60 kg reps progressed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="48" hidden="0" customHeight="1">
       <x:c r="A34" s="170" t="str">
         <x:v>Triceps</x:v>
       </x:c>
@@ -20012,26 +20871,28 @@
         <x:v>Rope Pushdown</x:v>
       </x:c>
       <x:c r="C34" s="170" t="str">
-        <x:v>40 kg x 10 @ RIR 2</x:v>
+        <x:v>40 kg x 11 @ RIR 1 after prior 40 kg set</x:v>
       </x:c>
       <x:c r="D34" s="170" t="str">
         <x:v>30-40 kg</x:v>
       </x:c>
       <x:c r="E34" s="170" t="str">
-        <x:v>40 kg x 11 @ RIR 2</x:v>
+        <x:v>40 kg x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F34" s="170" t="str">
-        <x:v>Add rep; no fourth set</x:v>
+        <x:v>Exactly 3 sets; no repeated 40 kg set</x:v>
       </x:c>
       <x:c r="G34" s="170" t="str">
         <x:v>Spread rope; slow return</x:v>
       </x:c>
       <x:c r="H34" s="170" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="I34" s="170"/>
-    </x:row>
-    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Modify volume</x:v>
+      </x:c>
+      <x:c r="I34" s="170" t="str">
+        <x:v>Fourth set exceeded plan; repetition gain does not justify load</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="48" hidden="0" customHeight="1">
       <x:c r="A35" s="170" t="str">
         <x:v>Triceps</x:v>
       </x:c>
@@ -20045,10 +20906,10 @@
         <x:v>30-40 kg</x:v>
       </x:c>
       <x:c r="E35" s="170" t="str">
-        <x:v>40 kg x 11-12 @ RIR 2</x:v>
+        <x:v>40 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F35" s="170" t="str">
-        <x:v>Add controlled reps</x:v>
+        <x:v>Add controlled rep</x:v>
       </x:c>
       <x:c r="G35" s="170" t="str">
         <x:v>Ribs down; elbows stable</x:v>
@@ -20056,9 +20917,11 @@
       <x:c r="H35" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I35" s="170"/>
-    </x:row>
-    <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="I35" s="170" t="str">
+        <x:v>30 and 35 kg sets progressed without increasing shoulder soreness</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="48" hidden="0" customHeight="1">
       <x:c r="A36" s="170" t="str">
         <x:v>Triceps</x:v>
       </x:c>
@@ -20066,26 +20929,28 @@
         <x:v>Single-Arm Cable Pushdown</x:v>
       </x:c>
       <x:c r="C36" s="170" t="str">
-        <x:v>15 kg x 10 each @ RIR 1</x:v>
+        <x:v>15 kg x 10 each @ RIR 2</x:v>
       </x:c>
       <x:c r="D36" s="170" t="str">
         <x:v>10-15 kg</x:v>
       </x:c>
       <x:c r="E36" s="170" t="str">
-        <x:v>15 kg x 10 @ RIR 2</x:v>
+        <x:v>15 kg x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F36" s="170" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Match both arms; add rep</x:v>
       </x:c>
       <x:c r="G36" s="170" t="str">
-        <x:v>Match weaker side</x:v>
+        <x:v>Elbow fixed; match weaker side</x:v>
       </x:c>
       <x:c r="H36" s="170" t="str">
-        <x:v>Modify effort</x:v>
-      </x:c>
-      <x:c r="I36" s="170"/>
-    </x:row>
-    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>In progress</x:v>
+      </x:c>
+      <x:c r="I36" s="170" t="str">
+        <x:v>Side-to-side difference To verify; reserve improved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="48" hidden="0" customHeight="1">
       <x:c r="A37" s="170" t="str">
         <x:v>Triceps</x:v>
       </x:c>
@@ -20099,10 +20964,10 @@
         <x:v>20-25 kg</x:v>
       </x:c>
       <x:c r="E37" s="170" t="str">
-        <x:v>25 kg x 11-12 @ RIR 2</x:v>
+        <x:v>25 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F37" s="170" t="str">
-        <x:v>Add reps before load</x:v>
+        <x:v>Exactly 3 sets; add rep before load</x:v>
       </x:c>
       <x:c r="G37" s="170" t="str">
         <x:v>Back supported; ribs down</x:v>
@@ -20110,9 +20975,11 @@
       <x:c r="H37" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
-      <x:c r="I37" s="170"/>
-    </x:row>
-    <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="I37" s="170" t="str">
+        <x:v>22.5 kg progressed to 13 reps; completed third set despite live reduction</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="48" hidden="0" customHeight="1">
       <x:c r="A38" s="170" t="str">
         <x:v>Triceps</x:v>
       </x:c>
@@ -20120,25 +20987,25 @@
         <x:v>Assisted Dip Machine</x:v>
       </x:c>
       <x:c r="C38" s="170" t="str">
-        <x:v>50 kg assistance x 8 @ RIR 1</x:v>
+        <x:v>50 kg assistance x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="D38" s="170" t="str">
         <x:v>50-70 kg assistance</x:v>
       </x:c>
       <x:c r="E38" s="170" t="str">
-        <x:v>50 kg assistance x 9-10 @ RIR 2</x:v>
+        <x:v>50 kg assistance x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F38" s="170" t="str">
-        <x:v>Earn reps before less support</x:v>
+        <x:v>Improve reserve before less support</x:v>
       </x:c>
       <x:c r="G38" s="170" t="str">
-        <x:v>Controlled depth</x:v>
+        <x:v>Controlled depth; no forced reps</x:v>
       </x:c>
       <x:c r="H38" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I38" s="170" t="str">
-        <x:v>Higher support weight is easier</x:v>
+        <x:v>Higher support weight is easier; completed third set despite live reduction</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
@@ -20514,7 +21381,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R967527592b7144ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87908f6f3bda421b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21294,16 +22161,28 @@
       <x:c r="Q22" s="59" t="n"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="220"/>
+      <x:c r="A23" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
       <x:c r="B23" s="170"/>
       <x:c r="C23" s="170"/>
-      <x:c r="D23" s="170"/>
-      <x:c r="E23" s="170"/>
-      <x:c r="F23" s="170"/>
+      <x:c r="D23" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E23" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F23" s="170" t="str">
+        <x:v>Very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain</x:v>
+      </x:c>
       <x:c r="G23" s="170"/>
       <x:c r="H23" s="170"/>
-      <x:c r="I23" s="170"/>
-      <x:c r="J23" s="170"/>
+      <x:c r="I23" s="170" t="str">
+        <x:v>Triceps workout - 75 min; 19 working sets; medium pump; no formal cardio/core</x:v>
+      </x:c>
+      <x:c r="J23" s="170" t="str">
+        <x:v>Started Medium; full EAA+ scoop (100 mg caffeine); no coffee; no forced reps; machine-assisted dips were working sets, not forced repetitions; cardio omitted due Low final energy</x:v>
+      </x:c>
       <x:c r="K23" s="59" t="n"/>
       <x:c r="L23" s="59" t="n"/>
       <x:c r="M23" s="59" t="n"/>
@@ -24731,7 +25610,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re07baeff5e124a9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41f3b94032a04fdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25564,13 +26443,83 @@
         <x:v>Check shoulder, hip and leg response the following morning before Triceps</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="52" customHeight="1">
+      <x:c r="A55" s="170" t="str">
+        <x:v>Triceps performance and effort</x:v>
+      </x:c>
+      <x:c r="B55" s="170" t="str">
+        <x:v>2026-08-22 used 19 working sets: 4 at RIR 3, 12 at RIR 2 and 3 at RIR 1; no failure, pain, forced reps or breakdown; duration 75 min</x:v>
+      </x:c>
+      <x:c r="C55" s="170" t="str">
+        <x:v>Performance and time efficiency improved while direct volume fell from 20 to 19</x:v>
+      </x:c>
+      <x:c r="D55" s="170" t="str">
+        <x:v>Keep loads; improve reserve; next session exactly 18 sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="52" customHeight="1">
+      <x:c r="A56" s="170" t="str">
+        <x:v>Live volume adjustment</x:v>
+      </x:c>
+      <x:c r="B56" s="170" t="str">
+        <x:v>A fourth rope set was followed by instructions to reduce overhead-dumbbell and dip work, but all three sets of each were completed</x:v>
+      </x:c>
+      <x:c r="C56" s="170" t="str">
+        <x:v>All completed sets count toward fatigue and remain preserved; session finished one set above cap</x:v>
+      </x:c>
+      <x:c r="D56" s="170" t="str">
+        <x:v>Follow live reductions; no fourth sets or replacement extras</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="52" customHeight="1">
+      <x:c r="A57" s="170" t="str">
+        <x:v>Post-Triceps cardio decision</x:v>
+      </x:c>
+      <x:c r="B57" s="170" t="str">
+        <x:v>Final energy was Low after 19 working sets; formal cardio and core were omitted</x:v>
+      </x:c>
+      <x:c r="C57" s="170" t="str">
+        <x:v>Additional conditioning was unlikely to add useful benefit in this recovery state</x:v>
+      </x:c>
+      <x:c r="D57" s="170" t="str">
+        <x:v>Resume cardio only when readiness and final energy support it</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="52" customHeight="1">
+      <x:c r="A58" s="170" t="str">
+        <x:v>Temporary four-day training week</x:v>
+      </x:c>
+      <x:c r="B58" s="170" t="str">
+        <x:v>Next week has only four available training days; exact days remain To verify</x:v>
+      </x:c>
+      <x:c r="C58" s="170" t="str">
+        <x:v>Consolidate upper-body work while preserving Legs as a standalone priority session</x:v>
+      </x:c>
+      <x:c r="D58" s="170" t="str">
+        <x:v>Provisional: Back+Biceps, Chest+Triceps, Legs, Shoulders+small arm finishers; confirm day spacing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="52" customHeight="1">
+      <x:c r="A59" s="170" t="str">
+        <x:v>Upcoming abdominal-fat phase</x:v>
+      </x:c>
+      <x:c r="B59" s="170" t="str">
+        <x:v>From the following week, add structured core, progressive cardio, step tracking and quantified diet management while retaining resistance training</x:v>
+      </x:c>
+      <x:c r="C59" s="170" t="str">
+        <x:v>Abdominal exercises strengthen the core, while waist reduction requires overall energy management and sustainable activity</x:v>
+      </x:c>
+      <x:c r="D59" s="170" t="str">
+        <x:v>Collect exact day schedule, average steps and quantified meal portions before final calorie target</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R564d1acb3f494287"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf288e7698ff1400d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26136,14 +27085,30 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="220"/>
-      <x:c r="B22" s="170"/>
-      <x:c r="C22" s="170"/>
-      <x:c r="D22" s="170"/>
-      <x:c r="E22" s="170"/>
-      <x:c r="F22" s="170"/>
-      <x:c r="G22" s="170"/>
-      <x:c r="H22" s="170"/>
+      <x:c r="A22" s="220" t="n">
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="B22" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C22" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D22" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E22" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F22" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; very little shoulder soreness unchanged; no shoulder, elbow or wrist pain; 75 min; no forced reps or technique breakdown; medium pump; full EAA+; no coffee; no formal cardio/core</x:v>
+      </x:c>
+      <x:c r="G22" s="170" t="str">
+        <x:v>Multiple rep/reserve progressions were pain-free and duration improved to 75 min. Direct work decreased from 20 to 19 sets, but the 18-set ceiling was still exceeded after live set reductions were not followed; Low final energy supported omitting cardio.</x:v>
+      </x:c>
+      <x:c r="H22" s="170" t="str">
+        <x:v>Exactly 18 direct sets next time: three per exercise, no fourth rope set and no extra sets after live adjustment; keep loads and improve reserve; temporary four-day week pending exact days</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="220"/>
@@ -26187,7 +27152,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91c53d21f9884b57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R769b8a6d31bd458e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26364,13 +27329,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Shoulders on 2026-08-21: no shoulder, neck, elbow, wrist, hip or lower-back pain. Low-medium immediate shoulder pump; delayed soreness remains To verify.</x:v>
+        <x:v>After Triceps on 2026-08-22: very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain; no forced reps or reported technique breakdown.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Check next-morning shoulder, hip and leg response before Triceps</x:v>
+        <x:v>Check next-morning shoulder, elbow and triceps soreness before the next training week</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -26552,13 +27517,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Completed Shoulders on 2026-08-21. Triceps is next in the retained one-body-part split, subject to fresh readiness and delayed-soreness checks.</x:v>
+        <x:v>Completed Triceps on 2026-08-22. Next week is a temporary four-day consolidation with Legs retained standalone; exact available days remain To verify.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Collect sleep, energy, shoulder soreness and joint pain before Triceps</x:v>
+        <x:v>Confirm the four available days before finalizing sequence and recovery spacing</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -26758,7 +27723,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1054a22a7924ce5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e5eea86bb724ef4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27861,10 +28826,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff2d2deb8cbe43e3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd44a20160a524903"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f6f0c21a7db44fd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29a59995b8d4d69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd412a89726594236"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R236db1d65f8b4b92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5e9807e41424faf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9076f84ec592491d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 24 back and biceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R28f3aae7031d404d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R8036e5f1fed54fd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R9e52479cd8a74783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R4972e4c0f18c4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rde71f2db43ca4f27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R1de8e34b109842d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rc8a63917148745ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Re2a57659ae0c4f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R73a990ecbfa642a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R7085d429fef34559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R4fc0d84c25004fb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Raf0d472a8dc64425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R27b2c64b0a1f4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R1597fa5be17741b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rc6647855ba6c460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R336929d0158b4936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R963d330cd5fe409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rfad17dcfe846403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R30bd16f4078e48cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R1f4755a5918a4902"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R958fad1d1bde4060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R3f89de10166c4c79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb54775ee8f494ec2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a351d62d4b3417d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N370" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N390" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1767,7 +1767,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="PhotoMeasurementTable" displayName="PhotoMeasurementTable" ref="A4:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="34" name="PhotoMeasurementTable" displayName="PhotoMeasurementTable" ref="A4:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D59" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2508,6 +2508,35 @@
         <x:v>Missing photos</x:v>
       </x:c>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="220" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="B8" s="170" t="n">
+        <x:v>87.7</x:v>
+      </x:c>
+      <x:c r="C8" s="170" t="n">
+        <x:v>96.5</x:v>
+      </x:c>
+      <x:c r="D8" s="170"/>
+      <x:c r="E8" s="170"/>
+      <x:c r="F8" s="170"/>
+      <x:c r="G8" s="170" t="str">
+        <x:v>To link</x:v>
+      </x:c>
+      <x:c r="H8" s="170" t="str">
+        <x:v>To link</x:v>
+      </x:c>
+      <x:c r="I8" s="170" t="str">
+        <x:v>To link</x:v>
+      </x:c>
+      <x:c r="J8" s="170" t="str">
+        <x:v>Repeated morning readings 87.6-87.7 kg before food/drink; no morning bowel movement because bowel movement occurred around midnight. Abdomen relaxed and tape at navel. Previous-day 88.7 kg conditions To verify; photos not supplied.</x:v>
+      </x:c>
+      <x:c r="K8" s="170" t="str">
+        <x:v>Partial / missing photos</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K2"/>
@@ -2523,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc70219399d9e43a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6351cd62e8574a42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3926,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf34c30b9df434337"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceaf8f2fdb174a78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4054,17 +4083,15 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
         <x:v>56</x:v>
       </x:c>
       <x:c r="G5" s="53" t="n"/>
-      <x:c r="H5" s="93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6-day</x:t>
-        </x:is>
+      <x:c r="H5" s="93" t="str">
+        <x:v>4-day temporary</x:v>
       </x:c>
       <x:c r="I5" s="53" t="n"/>
       <x:c r="J5" s="59" t="n"/>
@@ -4082,7 +4109,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="59" t="str">
-        <x:v>88.3 kg (2026-08-16)</x:v>
+        <x:v>87.7 kg (2026-08-23)</x:v>
       </x:c>
       <x:c r="C6" s="59" t="n"/>
       <x:c r="D6" s="53" t="n"/>
@@ -4252,15 +4279,11 @@
       <x:c r="L12" s="59" t="n"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Monday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Back</x:t>
-        </x:is>
+      <x:c r="A13" s="92" t="str">
+        <x:v>Day 1</x:v>
+      </x:c>
+      <x:c r="B13" s="59" t="str">
+        <x:v>Back + Biceps - completed 2026-08-24</x:v>
       </x:c>
       <x:c r="C13" s="59" t="n"/>
       <x:c r="D13" s="94" t="inlineStr">
@@ -4282,15 +4305,11 @@
       <x:c r="L13" s="59" t="n"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Tuesday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chest</x:t>
-        </x:is>
+      <x:c r="A14" s="92" t="str">
+        <x:v>Day 2</x:v>
+      </x:c>
+      <x:c r="B14" s="59" t="str">
+        <x:v>Chest + Triceps</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4304,15 +4323,11 @@
       <x:c r="L14" s="59" t="n"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Wednesday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Biceps</x:t>
-        </x:is>
+      <x:c r="A15" s="92" t="str">
+        <x:v>Day 3</x:v>
+      </x:c>
+      <x:c r="B15" s="59" t="str">
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4330,15 +4345,11 @@
       <x:c r="L15" s="59" t="n"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Thursday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Legs</x:t>
-        </x:is>
+      <x:c r="A16" s="92" t="str">
+        <x:v>Day 4</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="str">
+        <x:v>Shoulders + core / optional arm finishers</x:v>
       </x:c>
       <x:c r="C16" s="59" t="n"/>
       <x:c r="D16" s="94" t="inlineStr">
@@ -4376,15 +4387,11 @@
       <x:c r="L16" s="59" t="n"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Friday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shoulders</x:t>
-        </x:is>
+      <x:c r="A17" s="92" t="str">
+        <x:v>Other days</x:v>
+      </x:c>
+      <x:c r="B17" s="59" t="str">
+        <x:v>Rest / walking</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="inlineStr">
@@ -4412,15 +4419,11 @@
       <x:c r="L17" s="59" t="n"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Saturday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Triceps</x:t>
-        </x:is>
+      <x:c r="A18" s="92" t="str">
+        <x:v>Spacing</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="str">
+        <x:v>Exact remaining days To verify</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="inlineStr">
@@ -4448,16 +4451,8 @@
       <x:c r="L18" s="59" t="n"/>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sunday</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B19" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rest / Swimming / Cardio</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A19" s="92"/>
+      <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="inlineStr">
         <x:is>
@@ -4516,22 +4511,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Back</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Straight-Bar Pushdown</x:v>
+        <x:v>Lat Pulldown</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>60 kg x 9 @ RIR 1</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>60 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Preparation separate; improve reserve</x:v>
+        <x:v>Improve reserve; no load increase</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4542,22 +4537,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Back</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Rope Pushdown</x:v>
+        <x:v>Seated Cable Row</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>40 kg x 11 @ RIR 1</x:v>
+        <x:v>60 kg x 10 @ RIR 1</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>40 kg x 10-11 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>Modify volume</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Exactly 3 sets; no repeat set</x:v>
+        <x:v>Match reps with reserve</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4568,22 +4563,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Overhead DB Extension</x:v>
+        <x:v>Incline DB Curl</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>25 kg x 10 @ RIR 2</x:v>
+        <x:v>12.5 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>25 kg x 11 @ RIR 2</x:v>
+        <x:v>12.5 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Add clean rep before load</x:v>
+        <x:v>No extra sets</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4594,22 +4589,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Assisted Dip Machine</x:v>
+        <x:v>Hammer Curl</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>50 kg assist x 9 @ RIR 1</x:v>
+        <x:v>17.5 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>50 kg assist x 9 @ RIR 2</x:v>
+        <x:v>17.5 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Higher assistance is easier</x:v>
+        <x:v>Add one clean rep</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4638,7 +4633,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca77882f9964ee8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd3c0bcb61d45ec"/>
 </x:worksheet>
 </file>
 
@@ -19890,6 +19885,878 @@
       </x:c>
       <x:c r="N370" s="170" t="n">
         <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="371">
+      <x:c r="A371" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B371" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C371" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D371" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E371" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F371" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G371" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H371" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I371" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J371" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K371" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L371" s="170" t="str">
+        <x:v>Preparation set but RIR 3 and high repetitions created working-level fatigue</x:v>
+      </x:c>
+      <x:c r="M371" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N371" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="372">
+      <x:c r="A372" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B372" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C372" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D372" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E372" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F372" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G372" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H372" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I372" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J372" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K372" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L372" s="170"/>
+      <x:c r="M372" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N372" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="373">
+      <x:c r="A373" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B373" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C373" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D373" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E373" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F373" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G373" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H373" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I373" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J373" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K373" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L373" s="170" t="str">
+        <x:v>Reached target</x:v>
+      </x:c>
+      <x:c r="M373" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N373" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="374">
+      <x:c r="A374" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B374" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C374" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D374" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E374" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F374" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G374" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H374" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I374" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J374" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K374" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L374" s="170" t="str">
+        <x:v>Added one rep while improving reserve</x:v>
+      </x:c>
+      <x:c r="M374" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N374" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="375">
+      <x:c r="A375" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B375" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C375" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D375" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E375" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F375" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G375" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H375" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I375" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J375" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K375" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L375" s="170" t="str">
+        <x:v>Preparation set but RIR 3 and high repetitions created working-level fatigue</x:v>
+      </x:c>
+      <x:c r="M375" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N375" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="376">
+      <x:c r="A376" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B376" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C376" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D376" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E376" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F376" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G376" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H376" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I376" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J376" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K376" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L376" s="170"/>
+      <x:c r="M376" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N376" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="377">
+      <x:c r="A377" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B377" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C377" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D377" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E377" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F377" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G377" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H377" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I377" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J377" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K377" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L377" s="170" t="str">
+        <x:v>Reserve improved</x:v>
+      </x:c>
+      <x:c r="M377" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N377" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="378">
+      <x:c r="A378" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B378" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C378" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D378" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E378" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F378" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G378" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H378" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I378" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J378" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K378" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L378" s="170" t="str">
+        <x:v>Added one rep but missed RIR-2 target; keep load</x:v>
+      </x:c>
+      <x:c r="M378" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N378" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="379">
+      <x:c r="A379" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B379" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C379" s="170" t="str">
+        <x:v>Chest-Supported Row</x:v>
+      </x:c>
+      <x:c r="D379" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E379" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F379" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G379" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H379" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I379" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J379" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K379" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L379" s="170" t="str">
+        <x:v>Added one rep</x:v>
+      </x:c>
+      <x:c r="M379" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N379" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="380">
+      <x:c r="A380" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B380" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C380" s="170" t="str">
+        <x:v>Chest-Supported Row</x:v>
+      </x:c>
+      <x:c r="D380" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E380" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F380" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G380" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H380" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I380" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J380" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K380" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L380" s="170" t="str">
+        <x:v>Reserve improved</x:v>
+      </x:c>
+      <x:c r="M380" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N380" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="381">
+      <x:c r="A381" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B381" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C381" s="170" t="str">
+        <x:v>Chest-Supported Row</x:v>
+      </x:c>
+      <x:c r="D381" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E381" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F381" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G381" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H381" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I381" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J381" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K381" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L381" s="170" t="str">
+        <x:v>Quality progression through improved reserve</x:v>
+      </x:c>
+      <x:c r="M381" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N381" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="382">
+      <x:c r="A382" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B382" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C382" s="170" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D382" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E382" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F382" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G382" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H382" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I382" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J382" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K382" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L382" s="170"/>
+      <x:c r="M382" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N382" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="383">
+      <x:c r="A383" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B383" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C383" s="170" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D383" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E383" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F383" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G383" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H383" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I383" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J383" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K383" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L383" s="170" t="str">
+        <x:v>Reached target</x:v>
+      </x:c>
+      <x:c r="M383" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N383" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="384">
+      <x:c r="A384" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B384" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C384" s="170" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D384" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E384" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F384" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G384" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H384" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I384" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J384" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K384" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L384" s="170" t="str">
+        <x:v>Unplanned third set; retained as fatigue; no progression credit</x:v>
+      </x:c>
+      <x:c r="M384" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N384" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="385">
+      <x:c r="A385" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B385" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C385" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D385" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E385" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F385" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G385" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H385" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I385" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J385" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K385" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L385" s="170" t="str">
+        <x:v>Completed after live reduction to two sets</x:v>
+      </x:c>
+      <x:c r="M385" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N385" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="386">
+      <x:c r="A386" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B386" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C386" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D386" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E386" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F386" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G386" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H386" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I386" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J386" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K386" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L386" s="170"/>
+      <x:c r="M386" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N386" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="387">
+      <x:c r="A387" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B387" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C387" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D387" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E387" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F387" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G387" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H387" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I387" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J387" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K387" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L387" s="170" t="str">
+        <x:v>Third set completed despite live reduction; keep load</x:v>
+      </x:c>
+      <x:c r="M387" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N387" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="388">
+      <x:c r="A388" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B388" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C388" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D388" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E388" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F388" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G388" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H388" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I388" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J388" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K388" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L388" s="170" t="str">
+        <x:v>Only one set was prescribed after live volume adjustment</x:v>
+      </x:c>
+      <x:c r="M388" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N388" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="389">
+      <x:c r="A389" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B389" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C389" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D389" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E389" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F389" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G389" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H389" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I389" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J389" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K389" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L389" s="170" t="str">
+        <x:v>Unplanned after live one-set limit; retained as fatigue</x:v>
+      </x:c>
+      <x:c r="M389" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N389" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="390">
+      <x:c r="A390" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B390" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C390" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D390" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E390" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F390" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G390" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H390" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I390" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
+      <x:c r="J390" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K390" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L390" s="170" t="str">
+        <x:v>Unplanned after live one-set limit; keep load until 12 reps at RIR 2</x:v>
+      </x:c>
+      <x:c r="M390" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N390" s="170" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19924,7 +20791,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23affba764aa48b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04aca3356fc545b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20036,16 +20903,16 @@
         <x:v>Lat Pulldown</x:v>
       </x:c>
       <x:c r="C5" s="222" t="str">
-        <x:v>60 kg x 8 @ RIR 1</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D5" s="222" t="str">
         <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E5" s="222" t="str">
-        <x:v>60 kg x 8 @ RIR 2</x:v>
+        <x:v>60 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F5" s="222" t="str">
-        <x:v>Repeat with better reserve</x:v>
+        <x:v>Improve reserve before load</x:v>
       </x:c>
       <x:c r="G5" s="222" t="str">
         <x:v>Elbows down; no swinging</x:v>
@@ -20054,7 +20921,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I5" s="222" t="str">
-        <x:v>Do not add load</x:v>
+        <x:v>45 kg preparation reached RIR 3; 50-60 kg progressed</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -20065,25 +20932,25 @@
         <x:v>Seated Cable Row</x:v>
       </x:c>
       <x:c r="C6" s="222" t="str">
-        <x:v>60 kg x 9 @ RIR 1</x:v>
+        <x:v>60 kg x 10 @ RIR 1</x:v>
       </x:c>
       <x:c r="D6" s="222" t="str">
-        <x:v>55-60 kg</x:v>
+        <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E6" s="222" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F6" s="222" t="str">
-        <x:v>Recover prior reps with reserve</x:v>
+        <x:v>Match reps with better reserve</x:v>
       </x:c>
       <x:c r="G6" s="222" t="str">
         <x:v>Torso stable</x:v>
       </x:c>
       <x:c r="H6" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I6" s="222" t="str">
-        <x:v>Latest 60 kg set was 8 reps</x:v>
+        <x:v>55 kg reserve improved; top set too close to failure</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -20094,13 +20961,13 @@
         <x:v>Chest-Supported Row</x:v>
       </x:c>
       <x:c r="C7" s="222" t="str">
-        <x:v>60 kg/side x 11 @ RIR 2</x:v>
+        <x:v>60 kg/side x 11 @ RIR 3</x:v>
       </x:c>
       <x:c r="D7" s="222" t="str">
-        <x:v>50-60 kg/side</x:v>
+        <x:v>40-60 kg/side</x:v>
       </x:c>
       <x:c r="E7" s="222" t="str">
-        <x:v>60 kg/side x 12 @ RIR 2</x:v>
+        <x:v>60 kg/side x 12 @ RIR 2-3</x:v>
       </x:c>
       <x:c r="F7" s="222" t="str">
         <x:v>Add one clean rep</x:v>
@@ -20112,7 +20979,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I7" s="222" t="str">
-        <x:v>50 kg/side reached 13 reps</x:v>
+        <x:v>40 kg reps and reserve across top sets improved</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -20123,25 +20990,25 @@
         <x:v>Straight-Arm Pulldown</x:v>
       </x:c>
       <x:c r="C8" s="222" t="str">
-        <x:v>50 kg x 10 @ RIR 2</x:v>
+        <x:v>50 kg x 12 @ RIR 2; extra 55 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="D8" s="222" t="str">
-        <x:v>40-50 kg</x:v>
+        <x:v>45-50 kg</x:v>
       </x:c>
       <x:c r="E8" s="222" t="str">
-        <x:v>50 kg x 11-12 @ RIR 2</x:v>
+        <x:v>50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F8" s="222" t="str">
-        <x:v>Add reps before load</x:v>
+        <x:v>Exactly 2 sets; no 55 kg</x:v>
       </x:c>
       <x:c r="G8" s="222" t="str">
         <x:v>Elbows fixed</x:v>
       </x:c>
       <x:c r="H8" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify volume</x:v>
       </x:c>
       <x:c r="I8" s="222" t="str">
-        <x:v>Do not use 55 kg yet</x:v>
+        <x:v>55 kg was unplanned fatigue and receives no progression credit</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" hidden="0" customHeight="1">
@@ -20333,7 +21200,7 @@
         <x:v>17.5 kg each x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F15" s="222" t="str">
-        <x:v>Add reps with reserve</x:v>
+        <x:v>Add one rep; no extra sets</x:v>
       </x:c>
       <x:c r="G15" s="222" t="str">
         <x:v>Neutral wrists; no swing</x:v>
@@ -20342,7 +21209,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I15" s="222" t="str">
-        <x:v>12.5 kg reached 17 reps at RIR 2</x:v>
+        <x:v>All 3 sets controlled but last 2 exceeded live one-set limit</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -21248,25 +22115,25 @@
         <x:v>Incline Dumbbell Curl</x:v>
       </x:c>
       <x:c r="C47" s="170" t="str">
-        <x:v>12.5 kg each x 9 @ RIR 2</x:v>
+        <x:v>12.5 kg each x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="D47" s="170" t="str">
         <x:v>7.5-12.5 kg each</x:v>
       </x:c>
       <x:c r="E47" s="170" t="str">
-        <x:v>12.5 kg each x 10 @ RIR 2</x:v>
+        <x:v>12.5 kg each x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F47" s="170" t="str">
-        <x:v>Add clean rep before load</x:v>
+        <x:v>Keep load; improve reserve</x:v>
       </x:c>
       <x:c r="G47" s="170" t="str">
-        <x:v>Bench 45-60 degrees; shoulders back; do not force stretch</x:v>
+        <x:v>Bench 45-60 deg; no forced stretch</x:v>
       </x:c>
       <x:c r="H47" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I47" s="170" t="str">
-        <x:v>New clean baseline; replaces Cable Curl in active sequence</x:v>
+        <x:v>Third set completed despite live reduction; detailed form To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
@@ -21381,7 +22248,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87908f6f3bda421b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6db857ad961d47a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22192,16 +23059,26 @@
       <x:c r="Q23" s="59" t="n"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="220"/>
-      <x:c r="B24" s="170"/>
-      <x:c r="C24" s="170"/>
+      <x:c r="A24" s="220" t="n">
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="B24" s="170" t="n">
+        <x:v>87.7</x:v>
+      </x:c>
+      <x:c r="C24" s="170" t="n">
+        <x:v>96.5</x:v>
+      </x:c>
       <x:c r="D24" s="170"/>
       <x:c r="E24" s="170"/>
       <x:c r="F24" s="170"/>
       <x:c r="G24" s="170"/>
       <x:c r="H24" s="170"/>
-      <x:c r="I24" s="170"/>
-      <x:c r="J24" s="170"/>
+      <x:c r="I24" s="170" t="str">
+        <x:v>Standardized morning body check-in</x:v>
+      </x:c>
+      <x:c r="J24" s="170" t="str">
+        <x:v>Before food/drink; no morning bowel movement because bowel movement occurred around midnight; repeated scale readings 87.6-87.7 kg; 88.7 kg previous-day conditions To verify; abdomen relaxed at navel</x:v>
+      </x:c>
       <x:c r="K24" s="59" t="n"/>
       <x:c r="L24" s="59" t="n"/>
       <x:c r="M24" s="59" t="n"/>
@@ -22211,16 +23088,28 @@
       <x:c r="Q24" s="59" t="n"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="220"/>
+      <x:c r="A25" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
       <x:c r="B25" s="170"/>
       <x:c r="C25" s="170"/>
-      <x:c r="D25" s="170"/>
-      <x:c r="E25" s="170"/>
-      <x:c r="F25" s="170"/>
+      <x:c r="D25" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E25" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F25" s="170" t="str">
+        <x:v>No back, biceps, elbow, shoulder or lower-back pain; no unusual sensation reported</x:v>
+      </x:c>
       <x:c r="G25" s="170"/>
       <x:c r="H25" s="170"/>
-      <x:c r="I25" s="170"/>
-      <x:c r="J25" s="170"/>
+      <x:c r="I25" s="170" t="str">
+        <x:v>Back + Biceps workout - 75 min; 20 entries; no cardio/core</x:v>
+      </x:c>
+      <x:c r="J25" s="170" t="str">
+        <x:v>Started Medium-High; full EAA+ scoop (100 mg caffeine); coffee consumed in morning, amount/time To verify; no assistance or breakdown; pre-existing muscular soreness To verify</x:v>
+      </x:c>
       <x:c r="K25" s="59" t="n"/>
       <x:c r="L25" s="59" t="n"/>
       <x:c r="M25" s="59" t="n"/>
@@ -25610,7 +26499,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41f3b94032a04fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94c3add0753e4568"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26513,13 +27402,83 @@
         <x:v>Collect exact day schedule, average steps and quantified meal portions before final calorie target</x:v>
       </x:c>
     </x:row>
+    <x:row r="60" ht="52" customHeight="1">
+      <x:c r="A60" s="170" t="str">
+        <x:v>2026-08-23 body check-in</x:v>
+      </x:c>
+      <x:c r="B60" s="170" t="str">
+        <x:v>87.7 kg and 38 in navel waist; repeated scale readings 87.6-87.7 before food/drink; bowel movement occurred around midnight rather than morning</x:v>
+      </x:c>
+      <x:c r="C60" s="170" t="str">
+        <x:v>Current reading is reliable, but overnight change is not equivalent fat loss; protocol difference retained</x:v>
+      </x:c>
+      <x:c r="D60" s="170" t="str">
+        <x:v>Use daily readings and seven-day average; do not change calories from one result</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="52" customHeight="1">
+      <x:c r="A61" s="170" t="str">
+        <x:v>Egg introduction</x:v>
+      </x:c>
+      <x:c r="B61" s="170" t="str">
+        <x:v>Vipin started eating eggs; exact amount, preparation and adherence To verify</x:v>
+      </x:c>
+      <x:c r="C61" s="170" t="str">
+        <x:v>Recommended 2 whole eggs + 2 whites replacing the tofu sandwich, not added to every meal</x:v>
+      </x:c>
+      <x:c r="D61" s="170" t="str">
+        <x:v>Keep quantified protein minimum unchanged until actual intake is confirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="52" customHeight="1">
+      <x:c r="A62" s="170" t="str">
+        <x:v>Back + Biceps performance</x:v>
+      </x:c>
+      <x:c r="B62" s="170" t="str">
+        <x:v>2026-08-24 completed 20 entries in 75 min; no pain, assistance or breakdown; most loads progressed or improved reserve</x:v>
+      </x:c>
+      <x:c r="C62" s="170" t="str">
+        <x:v>Two RIR-3 preparation sets plus 18 working sets created about 20 meaningful sets</x:v>
+      </x:c>
+      <x:c r="D62" s="170" t="str">
+        <x:v>Keep loads; improve reserve; combined-session ceiling is 18 meaningful sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="52" customHeight="1">
+      <x:c r="A63" s="170" t="str">
+        <x:v>Combined-session volume adherence</x:v>
+      </x:c>
+      <x:c r="B63" s="170" t="str">
+        <x:v>Extra 55 kg straight-arm set and unreduced incline/hammer sets were completed after live set reductions</x:v>
+      </x:c>
+      <x:c r="C63" s="170" t="str">
+        <x:v>All work remains recorded, but unplanned sets do not justify progression and final energy fell to Low</x:v>
+      </x:c>
+      <x:c r="D63" s="170" t="str">
+        <x:v>A live reduction replaces the earlier plan; stop when the revised set count is reached</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="52" customHeight="1">
+      <x:c r="A64" s="170" t="str">
+        <x:v>Morning coffee plus EAA+</x:v>
+      </x:c>
+      <x:c r="B64" s="170" t="str">
+        <x:v>Morning coffee was consumed and a full EAA+ scoop added 100 mg caffeine; coffee amount and time To verify</x:v>
+      </x:c>
+      <x:c r="C64" s="170" t="str">
+        <x:v>Total daily caffeine cannot yet be quantified; timing may still affect sleep</x:v>
+      </x:c>
+      <x:c r="D64" s="170" t="str">
+        <x:v>Record coffee amount/time and next-morning sleep quality</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf288e7698ff1400d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0155eb8706d74ff4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27111,14 +28070,30 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="220"/>
-      <x:c r="B23" s="170"/>
-      <x:c r="C23" s="170"/>
-      <x:c r="D23" s="170"/>
-      <x:c r="E23" s="170"/>
-      <x:c r="F23" s="170"/>
-      <x:c r="G23" s="170"/>
-      <x:c r="H23" s="170"/>
+      <x:c r="A23" s="220" t="n">
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="B23" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C23" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D23" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E23" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F23" s="170" t="str">
+        <x:v>Good sleep; Medium-High start and Low final energy; no back, biceps, elbow, shoulder or lower-back pain; no unusual sensation; 75 min; no assistance or technique breakdown; full EAA+; morning coffee amount/time To verify; no cardio/core</x:v>
+      </x:c>
+      <x:c r="G23" s="170" t="str">
+        <x:v>Back performance improved without pain, but 20 meaningful sets were accumulated after three live volume reductions were not followed. Two sets were classified as preparation, yet both ended at RIR 3 and contributed material fatigue. Low final energy confirmed that the extra volume was unnecessary.</x:v>
+      </x:c>
+      <x:c r="H23" s="170" t="str">
+        <x:v>Next immediate session Chest + Triceps, fresh readiness required; combined sessions capped at 18 meaningful sets; follow live reductions; keep loads and improve reserve</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="220"/>
@@ -27152,7 +28127,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R769b8a6d31bd458e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14eeab497f6a489a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27261,13 +28236,13 @@
         <x:v>Current body weight</x:v>
       </x:c>
       <x:c r="C6" s="170" t="str">
-        <x:v>88.3 kg on 2026-08-16, measured after using the bathroom and before food or drink. Abdomen relaxed and waist tape at navel level. The historical 91.5 kg post-workout gym reading remains non-comparable.</x:v>
+        <x:v>87.7 kg on 2026-08-23; repeated 87.6-87.7 kg before food/drink. No morning bowel movement because bowel movement occurred around midnight. Previous-day 88.7 kg conditions To verify.</x:v>
       </x:c>
       <x:c r="D6" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Known with protocol note</x:v>
       </x:c>
       <x:c r="E6" s="170" t="str">
-        <x:v>Continue identical morning protocol and assess weekly trend</x:v>
+        <x:v>Continue daily readings and compare seven-day averages</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -27329,13 +28304,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Triceps on 2026-08-22: very little shoulder soreness, unchanged from pre-workout; no shoulder, elbow or wrist pain; no forced reps or reported technique breakdown.</x:v>
+        <x:v>After Back + Biceps on 2026-08-24: no back, biceps, elbow, shoulder or lower-back pain; no unusual sensation; no assistance or reported breakdown.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
-        <x:v>Partial / To verify</x:v>
+        <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Check next-morning shoulder, elbow and triceps soreness before the next training week</x:v>
+        <x:v>Check next-morning back, biceps and elbow soreness before Chest + Triceps</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -27517,13 +28492,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Completed Triceps on 2026-08-22. Next week is a temporary four-day consolidation with Legs retained standalone; exact available days remain To verify.</x:v>
+        <x:v>Temporary four-day week: Day 1 Back + Biceps completed 2026-08-24; Chest + Triceps is next; Legs remains standalone; exact remaining days To verify.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Confirm the four available days before finalizing sequence and recovery spacing</x:v>
+        <x:v>Confirm day spacing before each remaining session</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -27551,14 +28526,13 @@
         <x:v>Dietary pattern</x:v>
       </x:c>
       <x:c r="C23" s="170" t="str">
-        <x:v>Lacto-vegetarian: no eggs; milk/dairy used; avoids non-vegetarian food.
-Fish-oil capsule is an animal-derived exception to verify.</x:v>
+        <x:v>Eggs introduced on 2026-08-24 after prior lacto-vegetarian pattern; exact intake and preparation To verify. Milk, yogurt and whey remain in use; other non-vegetarian foods avoided.</x:v>
       </x:c>
       <x:c r="D23" s="170" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E23" s="170" t="str">
-        <x:v>Confirm whether fish oil is an intentional exception</x:v>
+        <x:v>Confirm whether 2 whole + 2 whites replaces the tofu sandwich and how often</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -27586,13 +28560,13 @@
         <x:v>Foods avoided</x:v>
       </x:c>
       <x:c r="C25" s="170" t="str">
-        <x:v>Non-vegetarian foods; no added sugar; tea stopped; black coffee only</x:v>
+        <x:v>Non-vegetarian foods other than newly introduced eggs; no added sugar; tea stopped; black coffee used selectively</x:v>
       </x:c>
       <x:c r="D25" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="E25" s="170" t="str">
-        <x:v>Meal-plan boundaries</x:v>
+        <x:v>Confirm egg frequency and preparation</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -27672,13 +28646,13 @@
         <x:v>Waist and verified morning weight</x:v>
       </x:c>
       <x:c r="C30" s="170" t="str">
-        <x:v>2026-08-16 standardized check-in: 88.3 kg and 38 in at the navel (96.5 cm), after bathroom and before food or drink, abdomen relaxed. Change from 2026-08-09: -0.5 kg and -2.6 cm.</x:v>
+        <x:v>2026-08-23 check-in: 87.7 kg and 38 in at navel (96.5 cm), before food/drink; no morning bowel movement because bowel movement occurred around midnight. Repeated scale readings 87.6-87.7 kg.</x:v>
       </x:c>
       <x:c r="D30" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Known with protocol note</x:v>
       </x:c>
       <x:c r="E30" s="170" t="str">
-        <x:v>Repeat weekly under identical conditions; use multi-week trend</x:v>
+        <x:v>Use seven-day weight average and repeat Sunday waist under matching conditions</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -27723,7 +28697,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e5eea86bb724ef4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc9fbf298bbb4b61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27857,19 +28831,19 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="D6" s="150" t="str">
-        <x:v>113.60 g/day quantified minimum after the reported yogurt update; several meal components remain incomplete</x:v>
+        <x:v>113.60 g/day quantified minimum; eggs introduced but actual intake is not yet confirmed</x:v>
       </x:c>
       <x:c r="E6" s="150" t="str">
-        <x:v>Protein from sabji, fruit, lentils and salad; ghee calories</x:v>
+        <x:v>Protein from eggs, sabji, fruit, lentils and salad; ghee calories</x:v>
       </x:c>
       <x:c r="F6" s="150" t="str">
-        <x:v>Quantify the cooked lentil bowl next, then sabji in Protein Calculator</x:v>
+        <x:v>Confirm actual egg intake, then quantify cooked lentils and sabji</x:v>
       </x:c>
       <x:c r="G6" s="150" t="str">
         <x:v>7-day intake log plus Sunday trend</x:v>
       </x:c>
       <x:c r="H6" s="152" t="str">
-        <x:v>Milk, rotis, tofu and bread are now included; do not count EAA grams as dietary protein</x:v>
+        <x:v>Do not count EAA grams as dietary protein; do not add provisional egg protein until confirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -27903,25 +28877,25 @@
         <x:v>Diet pattern</x:v>
       </x:c>
       <x:c r="B8" s="156" t="str">
-        <x:v>Lacto-vegetarian; no eggs</x:v>
+        <x:v>Eggs introduced; prior lacto-vegetarian pattern updated</x:v>
       </x:c>
       <x:c r="C8" s="156" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="D8" s="156" t="str">
-        <x:v>Milk, yogurt and whey are used; non-vegetarian foods avoided</x:v>
+        <x:v>Vipin reported starting eggs on 2026-08-24; milk, yogurt and whey remain in use</x:v>
       </x:c>
       <x:c r="E8" s="156" t="str">
-        <x:v>Whether fish oil is an intentional animal-derived exception</x:v>
+        <x:v>Exact egg count, whole/white split, preparation, frequency and whether sandwich is replaced</x:v>
       </x:c>
       <x:c r="F8" s="156" t="str">
-        <x:v>Confirm preference; strict vegetarian alternative can be discussed if needed</x:v>
+        <x:v>Recommended 2 whole eggs + 2 whites replacing the tofu sandwich; do not add eggs to every meal</x:v>
       </x:c>
       <x:c r="G8" s="156" t="str">
-        <x:v>Supplement-label review</x:v>
+        <x:v>Confirm actual intake before changing protein subtotal</x:v>
       </x:c>
       <x:c r="H8" s="158" t="str">
-        <x:v>No allergy or intolerance reported</x:v>
+        <x:v>Alternative: 3 whole eggs when separating whites is inconvenient</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -28188,10 +29162,10 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G19" s="170" t="str">
-        <x:v>Spreads/oil and fruit frequency</x:v>
+        <x:v>Whether egg option replaces sandwich; exact egg count/preparation; spreads/oil and fruit frequency</x:v>
       </x:c>
       <x:c r="H19" s="170" t="str">
-        <x:v>Confirmed sandwich protein: 8.99 g (29 g tofu = 4.12 g; two bread slices/50 g = 4.87 g).</x:v>
+        <x:v>Current confirmed sandwich remains quantified at 8.99 g protein. Proposed cutting substitution is 2 whole eggs + 2 whites; do not count until actual intake is confirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -28826,10 +29800,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd412a89726594236"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R236db1d65f8b4b92"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5e9807e41424faf"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9076f84ec592491d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec8b2b12183d4115"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98290730334a4e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b0773a0bc14e88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda807d9d0d4745ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 25 chest and triceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Raf0d472a8dc64425"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R27b2c64b0a1f4810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R1597fa5be17741b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rc6647855ba6c460c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R336929d0158b4936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R963d330cd5fe409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rfad17dcfe846403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R30bd16f4078e48cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R1f4755a5918a4902"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R958fad1d1bde4060"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R3f89de10166c4c79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re0cde04628134b03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R140da18b767c4366"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R50527aae56844435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R6bf577d86c94435a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R702626e600374bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rab872a5d47ee457e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Re9139ba429644171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Ree903bcbcf5543a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R7e437f2730204ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R3a5f96ba6e2a4fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rc6499a85b19b4b90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a351d62d4b3417d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R99ebb4b0e4ec46d6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N390" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N410" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6351cd62e8574a42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a87173320a4051"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rceaf8f2fdb174a78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b7228f2ed44653"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4083,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4309,7 +4309,7 @@
         <x:v>Day 2</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Chest + Triceps - completed 2026-08-25</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4327,7 +4327,7 @@
         <x:v>Day 3</x:v>
       </x:c>
       <x:c r="B15" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Legs - next; fresh readiness required</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4394,25 +4394,23 @@
         <x:v>Rest / walking</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
-      <x:c r="D17" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Back</x:t>
-        </x:is>
+      <x:c r="D17" s="59" t="str">
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E17" s="59" t="str">
-        <x:v>Lat Pulldown</x:v>
+        <x:v>Flat Bench Press</x:v>
       </x:c>
       <x:c r="F17" s="59" t="str">
-        <x:v>60 kg x 8 @ RIR 1</x:v>
+        <x:v>22.5 kg/side x 8 @ RIR 0</x:v>
       </x:c>
       <x:c r="G17" s="59" t="str">
-        <x:v>60 kg x 8 @ RIR 2</x:v>
+        <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
       </x:c>
       <x:c r="H17" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I17" s="59" t="str">
-        <x:v>Repeat with better reserve</x:v>
+        <x:v>No RIR 0; bar excluded</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
@@ -4426,25 +4424,23 @@
         <x:v>Exact remaining days To verify</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
-      <x:c r="D18" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Back</x:t>
-        </x:is>
+      <x:c r="D18" s="59" t="str">
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E18" s="59" t="str">
-        <x:v>Seated Cable Row</x:v>
+        <x:v>Incline Barbell Bench</x:v>
       </x:c>
       <x:c r="F18" s="59" t="str">
-        <x:v>60 kg x 9 @ RIR 1</x:v>
+        <x:v>15 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G18" s="59" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>Repeat with RIR 2</x:v>
       </x:c>
       <x:c r="H18" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I18" s="59" t="str">
-        <x:v>Recover best reps cleanly</x:v>
+        <x:v>Keep load</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
@@ -4454,25 +4450,23 @@
       <x:c r="A19" s="92"/>
       <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
-      <x:c r="D19" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chest</x:t>
-        </x:is>
+      <x:c r="D19" s="59" t="str">
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Flat Bench Press</x:v>
+        <x:v>Plate Chest Press</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>22.5 kg/side x 7 @ RIR 1</x:v>
+        <x:v>50 kg/side x 8 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
+        <x:v>45 kg/side x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify load</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>Bar excluded; improve reserve</x:v>
+        <x:v>No 50 kg yet</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
@@ -4482,25 +4476,23 @@
       <x:c r="A20" s="59" t="n"/>
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
-      <x:c r="D20" s="59" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Chest</x:t>
-        </x:is>
+      <x:c r="D20" s="59" t="str">
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Incline Barbell Bench</x:v>
+        <x:v>Pec Deck Fly</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>15 kg/side x 9 @ RIR 1 clean</x:v>
+        <x:v>60 kg x 11 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>15 kg/side x 9 @ RIR 2</x:v>
+        <x:v>55 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify technique</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>No assistance; do not add load</x:v>
+        <x:v>Monitor biceps pump; no 60 kg</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4511,22 +4503,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Back</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Lat Pulldown</x:v>
+        <x:v>Straight-Bar Pushdown</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
+        <x:v>60 kg x 9 @ RIR 1</x:v>
+      </x:c>
+      <x:c r="G21" s="59" t="str">
         <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
-      <x:c r="G21" s="59" t="str">
-        <x:v>60 kg x 9-10 @ RIR 2</x:v>
-      </x:c>
       <x:c r="H21" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Improve reserve; no load increase</x:v>
+        <x:v>Exactly 3 working sets</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4537,22 +4529,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Back</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Seated Cable Row</x:v>
+        <x:v>Overhead Rope Extension</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>60 kg x 10 @ RIR 1</x:v>
+        <x:v>45 kg x 7 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>60 kg x 10 @ RIR 2</x:v>
+        <x:v>40 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>Modify load</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Match reps with reserve</x:v>
+        <x:v>No 45 kg</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4563,22 +4555,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Incline DB Curl</x:v>
+        <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>12.5 kg x 9 @ RIR 1</x:v>
+        <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>12.5 kg x 9-10 @ RIR 2</x:v>
+        <x:v>Repeat after readiness</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>No extra sets</x:v>
+        <x:v>Check hip and biceps pump</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4589,22 +4581,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Hammer Curl</x:v>
+        <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>17.5 kg x 11 @ RIR 2</x:v>
+        <x:v>130 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>17.5 kg x 12 @ RIR 2</x:v>
+        <x:v>130 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Add one clean rep</x:v>
+        <x:v>No assisted 150 kg</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4633,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd3c0bcb61d45ec"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7dcc2d5c7984048"/>
 </x:worksheet>
 </file>
 
@@ -20757,6 +20749,872 @@
       </x:c>
       <x:c r="N390" s="170" t="n">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="391">
+      <x:c r="A391" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B391" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C391" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D391" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E391" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F391" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G391" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H391" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I391" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J391" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K391" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L391" s="170" t="str">
+        <x:v>RIR-3 high-repetition set counted as meaningful fatigue, not preparation</x:v>
+      </x:c>
+      <x:c r="M391" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N391" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="392">
+      <x:c r="A392" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B392" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C392" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D392" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E392" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F392" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G392" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H392" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I392" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J392" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K392" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L392" s="170"/>
+      <x:c r="M392" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N392" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="393">
+      <x:c r="A393" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B393" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C393" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D393" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E393" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F393" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G393" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H393" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I393" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J393" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K393" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L393" s="170" t="str">
+        <x:v>Repeated 20 kg set at target reserve</x:v>
+      </x:c>
+      <x:c r="M393" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N393" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="394">
+      <x:c r="A394" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B394" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C394" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D394" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E394" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F394" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G394" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H394" s="170" t="str">
+        <x:v>Clean and unassisted; reached failure-level effort</x:v>
+      </x:c>
+      <x:c r="I394" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J394" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K394" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L394" s="170" t="str">
+        <x:v>Rep target reached at RIR 0; no progression credit and no load increase</x:v>
+      </x:c>
+      <x:c r="M394" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N394" s="170" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="395">
+      <x:c r="A395" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B395" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C395" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D395" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E395" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F395" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G395" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H395" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I395" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J395" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K395" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L395" s="170"/>
+      <x:c r="M395" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N395" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="396">
+      <x:c r="A396" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B396" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C396" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D396" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E396" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F396" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G396" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H396" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I396" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J396" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K396" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L396" s="170"/>
+      <x:c r="M396" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N396" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="397">
+      <x:c r="A397" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B397" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C397" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D397" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E397" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F397" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G397" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H397" s="170" t="str">
+        <x:v>Clean and unassisted; controlled bar path To verify</x:v>
+      </x:c>
+      <x:c r="I397" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J397" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K397" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L397" s="170" t="str">
+        <x:v>Rep progression achieved; keep load and improve reserve across session</x:v>
+      </x:c>
+      <x:c r="M397" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N397" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="398">
+      <x:c r="A398" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B398" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C398" s="170" t="str">
+        <x:v>Plate Chest Press</x:v>
+      </x:c>
+      <x:c r="D398" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E398" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F398" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G398" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H398" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I398" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J398" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K398" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L398" s="170"/>
+      <x:c r="M398" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N398" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="399">
+      <x:c r="A399" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B399" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C399" s="170" t="str">
+        <x:v>Plate Chest Press</x:v>
+      </x:c>
+      <x:c r="D399" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E399" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F399" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G399" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H399" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I399" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J399" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K399" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L399" s="170" t="str">
+        <x:v>Exceeded repetition target</x:v>
+      </x:c>
+      <x:c r="M399" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N399" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="400">
+      <x:c r="A400" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B400" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C400" s="170" t="str">
+        <x:v>Plate Chest Press</x:v>
+      </x:c>
+      <x:c r="D400" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E400" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F400" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G400" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H400" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I400" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J400" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K400" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L400" s="170" t="str">
+        <x:v>Unplanned third set and load jump; retained as fatigue; no progression credit</x:v>
+      </x:c>
+      <x:c r="M400" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N400" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="401">
+      <x:c r="A401" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B401" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C401" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D401" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E401" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F401" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G401" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H401" s="170" t="str">
+        <x:v>Strong upper-biceps/arm pump later attributed to pec deck; non-painful; exact side To verify</x:v>
+      </x:c>
+      <x:c r="I401" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J401" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K401" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L401" s="170" t="str">
+        <x:v>Use relaxed grip and elbow-driven arc next time</x:v>
+      </x:c>
+      <x:c r="M401" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N401" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="402">
+      <x:c r="A402" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B402" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C402" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D402" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E402" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F402" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G402" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H402" s="170" t="str">
+        <x:v>Strong upper-biceps/arm pump later attributed to pec deck; non-painful; exact side To verify</x:v>
+      </x:c>
+      <x:c r="I402" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J402" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K402" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L402" s="170"/>
+      <x:c r="M402" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N402" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="403">
+      <x:c r="A403" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B403" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C403" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D403" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E403" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F403" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G403" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H403" s="170" t="str">
+        <x:v>Strong upper-biceps/arm pump later attributed to pec deck; non-painful; exact side To verify</x:v>
+      </x:c>
+      <x:c r="I403" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J403" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K403" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L403" s="170" t="str">
+        <x:v>Unplanned third set; omit 60 kg next time; no progression credit</x:v>
+      </x:c>
+      <x:c r="M403" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N403" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="404">
+      <x:c r="A404" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B404" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C404" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D404" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E404" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F404" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G404" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H404" s="170" t="str">
+        <x:v>Genuine preparation set; elbows fixed; no assistance</x:v>
+      </x:c>
+      <x:c r="I404" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J404" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K404" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L404" s="170" t="str">
+        <x:v>Excluded from meaningful-set total</x:v>
+      </x:c>
+      <x:c r="M404" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N404" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="405">
+      <x:c r="A405" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B405" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C405" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D405" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E405" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F405" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G405" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H405" s="170" t="str">
+        <x:v>No assistance or technique breakdown reported; detailed form To verify</x:v>
+      </x:c>
+      <x:c r="I405" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J405" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K405" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L405" s="170"/>
+      <x:c r="M405" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N405" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="406">
+      <x:c r="A406" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B406" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C406" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D406" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E406" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F406" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G406" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H406" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I406" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J406" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K406" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L406" s="170" t="str">
+        <x:v>Harder than RIR-2 target; keep load</x:v>
+      </x:c>
+      <x:c r="M406" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N406" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="407">
+      <x:c r="A407" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B407" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C407" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D407" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E407" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F407" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G407" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H407" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I407" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J407" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K407" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L407" s="170" t="str">
+        <x:v>Matched reps but missed RIR-2 target; keep load</x:v>
+      </x:c>
+      <x:c r="M407" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N407" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="408">
+      <x:c r="A408" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B408" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C408" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D408" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E408" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F408" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G408" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H408" s="170" t="str">
+        <x:v>Reported clean; no assistance or technique breakdown</x:v>
+      </x:c>
+      <x:c r="I408" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J408" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K408" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L408" s="170"/>
+      <x:c r="M408" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N408" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="409">
+      <x:c r="A409" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B409" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C409" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D409" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E409" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F409" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G409" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H409" s="170" t="str">
+        <x:v>Reported clean; no assistance or technique breakdown</x:v>
+      </x:c>
+      <x:c r="I409" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J409" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K409" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L409" s="170" t="str">
+        <x:v>40 kg used instead of prescribed 35 kg</x:v>
+      </x:c>
+      <x:c r="M409" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N409" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="410">
+      <x:c r="A410" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B410" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C410" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D410" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E410" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F410" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G410" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H410" s="170" t="str">
+        <x:v>Reported clean; no assistance or technique breakdown</x:v>
+      </x:c>
+      <x:c r="I410" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
+      <x:c r="J410" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K410" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L410" s="170" t="str">
+        <x:v>Unplanned third set after explicit two-set limit; no progression credit</x:v>
+      </x:c>
+      <x:c r="M410" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N410" s="170" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -20791,7 +21649,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04aca3356fc545b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdce32aa422314668"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21019,7 +21877,7 @@
         <x:v>Flat Bench Press</x:v>
       </x:c>
       <x:c r="C9" s="222" t="str">
-        <x:v>22.5 kg/side x 7 @ RIR 1</x:v>
+        <x:v>22.5 kg/side x 8 @ RIR 0</x:v>
       </x:c>
       <x:c r="D9" s="222" t="str">
         <x:v>17.5-22.5 kg/side</x:v>
@@ -21028,16 +21886,16 @@
         <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
       </x:c>
       <x:c r="F9" s="222" t="str">
-        <x:v>Improve reserve; add rep before load</x:v>
+        <x:v>No failure; improve reserve</x:v>
       </x:c>
       <x:c r="G9" s="222" t="str">
-        <x:v>Shoulder blades set</x:v>
+        <x:v>Shoulder blades set; genuine prep near RIR 5</x:v>
       </x:c>
       <x:c r="H9" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I9" s="222" t="str">
-        <x:v>20 kg/side x 10 reached only RIR 1; bar excluded</x:v>
+        <x:v>15 kg x 15 counted as fatigue; top set reached RIR 0; bar excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" hidden="0" customHeight="1">
@@ -21077,25 +21935,25 @@
         <x:v>Plate Chest Press</x:v>
       </x:c>
       <x:c r="C11" s="222" t="str">
-        <x:v>45 kg/side x 8 @ RIR 1 clean</x:v>
+        <x:v>50 kg/side x 8 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="D11" s="222" t="str">
         <x:v>30-45 kg/side</x:v>
       </x:c>
       <x:c r="E11" s="222" t="str">
-        <x:v>45 kg/side x 9 @ RIR 2</x:v>
+        <x:v>45 kg/side x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F11" s="222" t="str">
-        <x:v>Add clean rep with reserve</x:v>
+        <x:v>Do not use 50 kg yet</x:v>
       </x:c>
       <x:c r="G11" s="222" t="str">
         <x:v>Controlled eccentric</x:v>
       </x:c>
       <x:c r="H11" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify load/volume</x:v>
       </x:c>
       <x:c r="I11" s="222" t="str">
-        <x:v>New 45 kg/side baseline; clean and unassisted</x:v>
+        <x:v>50 kg was an unplanned third set and receives no progression credit</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" hidden="0" customHeight="1">
@@ -21135,7 +21993,7 @@
         <x:v>Pec Deck Fly</x:v>
       </x:c>
       <x:c r="C13" s="222" t="str">
-        <x:v>55 kg x 12 @ RIR 1</x:v>
+        <x:v>60 kg x 11 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="D13" s="222" t="str">
         <x:v>45-55 kg</x:v>
@@ -21144,16 +22002,16 @@
         <x:v>55 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F13" s="222" t="str">
-        <x:v>Improve reserve; no load increase</x:v>
+        <x:v>Omit 60 kg; monitor biceps pump</x:v>
       </x:c>
       <x:c r="G13" s="222" t="str">
-        <x:v>Slow stretch; shoulders controlled</x:v>
+        <x:v>Relax grip; fixed soft elbow; drive elbows</x:v>
       </x:c>
       <x:c r="H13" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify technique/volume</x:v>
       </x:c>
       <x:c r="I13" s="222" t="str">
-        <x:v>Build reserve before load</x:v>
+        <x:v>Strong non-painful upper-biceps pump likely related; exact side To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -21724,10 +22582,10 @@
         <x:v>Elbows fixed; torso still</x:v>
       </x:c>
       <x:c r="H33" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I33" s="170" t="str">
-        <x:v>45 kg x 16 was preparation only; 55 and 60 kg reps progressed</x:v>
+        <x:v>45 kg x 12 @ RIR 4 was preparation; working sets were harder than targets</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="48" hidden="0" customHeight="1">
@@ -21767,25 +22625,25 @@
         <x:v>Overhead Rope Extension</x:v>
       </x:c>
       <x:c r="C35" s="170" t="str">
-        <x:v>40 kg x 10 @ RIR 2</x:v>
+        <x:v>45 kg x 7 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="D35" s="170" t="str">
         <x:v>30-40 kg</x:v>
       </x:c>
       <x:c r="E35" s="170" t="str">
-        <x:v>40 kg x 11 @ RIR 2</x:v>
+        <x:v>40 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F35" s="170" t="str">
-        <x:v>Add controlled rep</x:v>
+        <x:v>Exactly 3 sets; no 45 kg</x:v>
       </x:c>
       <x:c r="G35" s="170" t="str">
         <x:v>Ribs down; elbows stable</x:v>
       </x:c>
       <x:c r="H35" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify load/volume</x:v>
       </x:c>
       <x:c r="I35" s="170" t="str">
-        <x:v>30 and 35 kg sets progressed without increasing shoulder soreness</x:v>
+        <x:v>Third set exceeded live two-set limit and receives no progression credit</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="48" hidden="0" customHeight="1">
@@ -21941,16 +22799,16 @@
         <x:v>Incline Barbell Bench Press</x:v>
       </x:c>
       <x:c r="C41" s="170" t="str">
-        <x:v>15 kg/side x 9 @ RIR 1; unassisted</x:v>
+        <x:v>15 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D41" s="170" t="str">
         <x:v>10-15 kg/side</x:v>
       </x:c>
       <x:c r="E41" s="170" t="str">
-        <x:v>15 kg/side x 9 @ RIR 2</x:v>
+        <x:v>15 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F41" s="170" t="str">
-        <x:v>Improve reserve before load</x:v>
+        <x:v>Keep reps; improve first-set reserve</x:v>
       </x:c>
       <x:c r="G41" s="170" t="str">
         <x:v>Controlled bar path</x:v>
@@ -21959,7 +22817,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I41" s="170" t="str">
-        <x:v>Bar excluded; 12.5 kg/side target remains 12 reps</x:v>
+        <x:v>All three loads progressed; bar excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -22248,7 +23106,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6db857ad961d47a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1082d0a745844226"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23119,16 +23977,28 @@
       <x:c r="Q25" s="59" t="n"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="220"/>
+      <x:c r="A26" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
       <x:c r="B26" s="170"/>
       <x:c r="C26" s="170"/>
-      <x:c r="D26" s="170"/>
-      <x:c r="E26" s="170"/>
-      <x:c r="F26" s="170"/>
+      <x:c r="D26" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E26" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F26" s="170" t="str">
+        <x:v>No chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely pec-deck-related; exact side To verify</x:v>
+      </x:c>
       <x:c r="G26" s="170"/>
       <x:c r="H26" s="170"/>
-      <x:c r="I26" s="170"/>
-      <x:c r="J26" s="170"/>
+      <x:c r="I26" s="170" t="str">
+        <x:v>Chest + Triceps workout - 75 min; 20 entries; 19 meaningful sets; no cardio/core</x:v>
+      </x:c>
+      <x:c r="J26" s="170" t="str">
+        <x:v>Started Medium; medium chest/triceps pump; full EAA+ scoop (100 mg caffeine); no coffee; no assistance or breakdown; all overhead-rope sets clean; upper-biceps pump felt strongly but not painful</x:v>
+      </x:c>
       <x:c r="K26" s="59" t="n"/>
       <x:c r="L26" s="59" t="n"/>
       <x:c r="M26" s="59" t="n"/>
@@ -26499,7 +27369,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94c3add0753e4568"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b0533ba26e4437b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27472,13 +28342,69 @@
         <x:v>Record coffee amount/time and next-morning sleep quality</x:v>
       </x:c>
     </x:row>
+    <x:row r="65" ht="52" customHeight="1">
+      <x:c r="A65" s="170" t="str">
+        <x:v>Chest + Triceps performance</x:v>
+      </x:c>
+      <x:c r="B65" s="170" t="str">
+        <x:v>2026-08-25 completed 20 entries in 75 min; incline and established loads progressed; no pain, assistance or breakdown</x:v>
+      </x:c>
+      <x:c r="C65" s="170" t="str">
+        <x:v>One RIR-0 flat-bench set and Low final energy limit progression credit</x:v>
+      </x:c>
+      <x:c r="D65" s="170" t="str">
+        <x:v>Keep loads; next combined session exactly 18 meaningful sets and no failure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="52" customHeight="1">
+      <x:c r="A66" s="170" t="str">
+        <x:v>Repeated live-volume non-adherence</x:v>
+      </x:c>
+      <x:c r="B66" s="170" t="str">
+        <x:v>Plate press, pec deck and overhead rope exceeded revised live limits; session reached 19 meaningful sets</x:v>
+      </x:c>
+      <x:c r="C66" s="170" t="str">
+        <x:v>All completed work remains in history, but unplanned sets and loads do not justify progression</x:v>
+      </x:c>
+      <x:c r="D66" s="170" t="str">
+        <x:v>A live reduction replaces the earlier plan; stop at the revised count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="52" customHeight="1">
+      <x:c r="A67" s="170" t="str">
+        <x:v>Pec-deck upper-biceps pump</x:v>
+      </x:c>
+      <x:c r="B67" s="170" t="str">
+        <x:v>Strong upper-biceps/upper-arm pump likely triggered by pec deck; explicitly not painful; exact side To verify</x:v>
+      </x:c>
+      <x:c r="C67" s="170" t="str">
+        <x:v>Likely technique/fatigue signal rather than injury based on current report</x:v>
+      </x:c>
+      <x:c r="D67" s="170" t="str">
+        <x:v>Relax grip, drive elbows, omit 60 kg; confirm resolution before next upper session</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="52" customHeight="1">
+      <x:c r="A68" s="170" t="str">
+        <x:v>Failure exposure</x:v>
+      </x:c>
+      <x:c r="B68" s="170" t="str">
+        <x:v>Flat bench 22.5 kg/side x 8 reached RIR 0</x:v>
+      </x:c>
+      <x:c r="C68" s="170" t="str">
+        <x:v>Rep target was reached without assistance but reserve target was missed</x:v>
+      </x:c>
+      <x:c r="D68" s="170" t="str">
+        <x:v>Keep load; require RIR 1-2 and no assisted repetition before progression</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0155eb8706d74ff4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf44478e3a9de4d50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28096,14 +29022,30 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="220"/>
-      <x:c r="B24" s="170"/>
-      <x:c r="C24" s="170"/>
-      <x:c r="D24" s="170"/>
-      <x:c r="E24" s="170"/>
-      <x:c r="F24" s="170"/>
-      <x:c r="G24" s="170"/>
-      <x:c r="H24" s="170"/>
+      <x:c r="A24" s="220" t="n">
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="B24" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C24" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D24" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E24" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F24" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; no chest, shoulder, elbow or wrist pain; strong non-painful upper-biceps/arm pump likely from pec deck, exact side To verify; 75 min; medium chest/triceps pump; no assistance or breakdown; full EAA+; no coffee; no cardio/core</x:v>
+      </x:c>
+      <x:c r="G24" s="170" t="str">
+        <x:v>Performance improved across incline pressing and several established loads without pain or assistance, but 19 meaningful sets exceeded the 18-set cap. Flat bench reached RIR 0 and three live volume reductions were not followed. Low final energy confirmed the extra work was unnecessary.</x:v>
+      </x:c>
+      <x:c r="H24" s="170" t="str">
+        <x:v>Legs next after fresh readiness and biceps-pump resolution; next combined Chest + Triceps exactly 18 meaningful sets; no RIR 0; follow live reductions; omit unplanned 50 kg plate press, 60 kg pec deck and 45 kg overhead rope</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="220"/>
@@ -28127,7 +29069,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14eeab497f6a489a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R763c8925571846f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28304,13 +29246,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Back + Biceps on 2026-08-24: no back, biceps, elbow, shoulder or lower-back pain; no unusual sensation; no assistance or reported breakdown.</x:v>
+        <x:v>After Chest + Triceps on 2026-08-25: no chest, shoulder, elbow or wrist pain. Strong upper-biceps/upper-arm pump likely from pec deck was not painful; exact side To verify.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Known with verification flag</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Check next-morning back, biceps and elbow soreness before Chest + Triceps</x:v>
+        <x:v>Confirm pump resolves; pause direct upper-body loading if pain, bruising or weakness develops</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -28492,13 +29434,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Temporary four-day week: Day 1 Back + Biceps completed 2026-08-24; Chest + Triceps is next; Legs remains standalone; exact remaining days To verify.</x:v>
+        <x:v>Temporary four-day week: Day 1 Back + Biceps completed 2026-08-24; Day 2 Chest + Triceps completed 2026-08-25; Legs is next; Day 4 Shoulders + core; exact spacing To verify.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Confirm day spacing before each remaining session</x:v>
+        <x:v>Confirm readiness and day spacing before Legs</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -28697,7 +29639,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc9fbf298bbb4b61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58fd9f2406014922"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29800,10 +30742,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec8b2b12183d4115"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98290730334a4e74"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b0773a0bc14e88"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda807d9d0d4745ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e5ccbce0a2e48de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf164dd7f2fc64593"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc83f777712a041ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re35b06aa6fc14d2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 26 shoulders and biceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re0cde04628134b03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R140da18b767c4366"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R50527aae56844435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R6bf577d86c94435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R702626e600374bce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rab872a5d47ee457e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Re9139ba429644171"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Ree903bcbcf5543a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R7e437f2730204ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R3a5f96ba6e2a4fa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rc6499a85b19b4b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8093760176c743b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb4dde22ba9c7407a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rfb432a5f20db4478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R82a35bb9ab89423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R07efffaa975a42f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R7340f1e6983240a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R70d26c83bbc44f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R4c932b342f454833"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R3dd3291087f14334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc5a695c94b2e4806"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R892844fa43e4485f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R99ebb4b0e4ec46d6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08613bcf59e5403a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N410" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N429" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D68" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a87173320a4051"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R085db3d201e2400d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2b7228f2ed44653"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5453c2d7148741d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4083,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4327,7 +4327,7 @@
         <x:v>Day 3</x:v>
       </x:c>
       <x:c r="B15" s="59" t="str">
-        <x:v>Legs - next; fresh readiness required</x:v>
+        <x:v>Shoulders + Biceps - completed 2026-08-26</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4349,7 +4349,7 @@
         <x:v>Day 4</x:v>
       </x:c>
       <x:c r="B16" s="59" t="str">
-        <x:v>Shoulders + core / optional arm finishers</x:v>
+        <x:v>Legs - next; fresh lower-body readiness required</x:v>
       </x:c>
       <x:c r="C16" s="59" t="n"/>
       <x:c r="D16" s="94" t="inlineStr">
@@ -4395,22 +4395,22 @@
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E17" s="59" t="str">
-        <x:v>Flat Bench Press</x:v>
+        <x:v>Dumbbell Shoulder Press</x:v>
       </x:c>
       <x:c r="F17" s="59" t="str">
-        <x:v>22.5 kg/side x 8 @ RIR 0</x:v>
+        <x:v>25 kg each x 8 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="G17" s="59" t="str">
-        <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
+        <x:v>22.5 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H17" s="59" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>Modify volume</x:v>
       </x:c>
       <x:c r="I17" s="59" t="str">
-        <x:v>No RIR 0; bar excluded</x:v>
+        <x:v>Exactly 3 working sets; no 25 kg yet</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
@@ -4421,26 +4421,26 @@
         <x:v>Spacing</x:v>
       </x:c>
       <x:c r="B18" s="59" t="str">
-        <x:v>Exact remaining days To verify</x:v>
+        <x:v>Equipment-driven order swap preserved</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E18" s="59" t="str">
-        <x:v>Incline Barbell Bench</x:v>
+        <x:v>Plate Lateral Raise</x:v>
       </x:c>
       <x:c r="F18" s="59" t="str">
-        <x:v>15 kg/side x 10 @ RIR 2</x:v>
+        <x:v>5 kg/side x 15 x2 @ RIR 2</x:v>
       </x:c>
       <x:c r="G18" s="59" t="str">
-        <x:v>Repeat with RIR 2</x:v>
+        <x:v>5 kg/side x 16 @ RIR 2</x:v>
       </x:c>
       <x:c r="H18" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I18" s="59" t="str">
-        <x:v>Keep load</x:v>
+        <x:v>Unloaded resistance To verify</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
@@ -4451,22 +4451,22 @@
       <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Plate Chest Press</x:v>
+        <x:v>Cable Upright Row</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>50 kg/side x 8 @ RIR 1 unplanned</x:v>
+        <x:v>60 kg x 9 @ RIR 2 unplanned</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>45 kg/side x 9-10 @ RIR 2</x:v>
+        <x:v>50 kg x 11-12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
         <x:v>Modify load</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>No 50 kg yet</x:v>
+        <x:v>No 60 kg yet</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
@@ -4477,22 +4477,22 @@
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Shoulders</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Pec Deck Fly</x:v>
+        <x:v>Dumbbell Shrug</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>60 kg x 11 @ RIR 1 unplanned</x:v>
+        <x:v>40 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>55 kg x 12 @ RIR 2</x:v>
+        <x:v>40 kg each x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>Modify technique</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>Monitor biceps pump; no 60 kg</x:v>
+        <x:v>Keep load; top pause</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4503,22 +4503,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Straight-Bar Pushdown</x:v>
+        <x:v>Plate Curl Machine</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>60 kg x 9 @ RIR 1</x:v>
+        <x:v>12.5 kg/side x 11 @ RIR 3</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>12.5 kg/side x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Exactly 3 working sets</x:v>
+        <x:v>No extra 15 kg set</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4529,22 +4529,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Overhead Rope Extension</x:v>
+        <x:v>Dumbbell RDL</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>45 kg x 7 @ RIR 1 unplanned</x:v>
+        <x:v>15 kg each x 12; back dominant</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>40 kg x 9-10 @ RIR 2</x:v>
+        <x:v>10 kg each technique sets</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>Modify load</x:v>
+        <x:v>Verify technique</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>No 45 kg</x:v>
+        <x:v>Stop if back or hip dominates</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4570,7 +4570,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Check hip and biceps pump</x:v>
+        <x:v>No load increase</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4587,7 +4587,7 @@
         <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>130 kg x 9 @ RIR 1</x:v>
+        <x:v>150 kg x 7 with assistance</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
         <x:v>130 kg x 9-10 @ RIR 2</x:v>
@@ -4625,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7dcc2d5c7984048"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58cc489811d84211"/>
 </x:worksheet>
 </file>
 
@@ -21615,6 +21615,842 @@
       </x:c>
       <x:c r="N410" s="170" t="n">
         <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="411">
+      <x:c r="A411" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B411" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C411" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D411" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E411" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F411" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G411" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H411" s="170" t="str">
+        <x:v>Reported very easy; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I411" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J411" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K411" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L411" s="170" t="str">
+        <x:v>Genuine warm-up; excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M411" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N411" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="412">
+      <x:c r="A412" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B412" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C412" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D412" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E412" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F412" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G412" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H412" s="170" t="str">
+        <x:v>Clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I412" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J412" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K412" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L412" s="170" t="str">
+        <x:v>Rep progression achieved</x:v>
+      </x:c>
+      <x:c r="M412" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N412" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="413">
+      <x:c r="A413" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B413" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C413" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D413" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E413" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F413" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G413" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H413" s="170" t="str">
+        <x:v>Clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I413" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J413" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K413" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L413" s="170" t="str">
+        <x:v>Two-repetition progression at matched reserve</x:v>
+      </x:c>
+      <x:c r="M413" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N413" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="414">
+      <x:c r="A414" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B414" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C414" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D414" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E414" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F414" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G414" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H414" s="170" t="str">
+        <x:v>Clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I414" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J414" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K414" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L414" s="170" t="str">
+        <x:v>One-repetition progression with improved reserve</x:v>
+      </x:c>
+      <x:c r="M414" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N414" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="415">
+      <x:c r="A415" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B415" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C415" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D415" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E415" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F415" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G415" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H415" s="170" t="str">
+        <x:v>Confirmed clean and pain-free; no assistance or breakdown</x:v>
+      </x:c>
+      <x:c r="I415" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J415" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K415" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L415" s="170" t="str">
+        <x:v>Unplanned fourth working set; retained as fatigue; no independent progression credit</x:v>
+      </x:c>
+      <x:c r="M415" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N415" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="416">
+      <x:c r="A416" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B416" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C416" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D416" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E416" s="170" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F416" s="170" t="str">
+        <x:v>kg plates each side; unloaded resistance excluded and To verify</x:v>
+      </x:c>
+      <x:c r="G416" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H416" s="170" t="str">
+        <x:v>No assistance or breakdown; detailed arm path To verify</x:v>
+      </x:c>
+      <x:c r="I416" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J416" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K416" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L416" s="170" t="str">
+        <x:v>Easy working set; counts toward the 18-set ceiling</x:v>
+      </x:c>
+      <x:c r="M416" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N416" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="417">
+      <x:c r="A417" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B417" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C417" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D417" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E417" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F417" s="170" t="str">
+        <x:v>kg plates each side; unloaded resistance excluded and To verify</x:v>
+      </x:c>
+      <x:c r="G417" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H417" s="170" t="str">
+        <x:v>No assistance or breakdown; detailed arm path To verify</x:v>
+      </x:c>
+      <x:c r="I417" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J417" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K417" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L417" s="170" t="str">
+        <x:v>Rep progression from prior 12-rep baseline</x:v>
+      </x:c>
+      <x:c r="M417" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N417" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="418">
+      <x:c r="A418" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B418" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C418" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D418" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E418" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F418" s="170" t="str">
+        <x:v>kg plates each side; unloaded resistance excluded and To verify</x:v>
+      </x:c>
+      <x:c r="G418" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H418" s="170" t="str">
+        <x:v>No assistance or breakdown; detailed arm path To verify</x:v>
+      </x:c>
+      <x:c r="I418" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J418" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K418" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L418" s="170" t="str">
+        <x:v>Repeated progressed set cleanly</x:v>
+      </x:c>
+      <x:c r="M418" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N418" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="419">
+      <x:c r="A419" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B419" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C419" s="170" t="str">
+        <x:v>Experimental Rear-Delt Lateral-Raise Machine</x:v>
+      </x:c>
+      <x:c r="D419" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E419" s="170" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F419" s="170" t="str">
+        <x:v>kg plates each side; exact reverse-facing setup/path To verify</x:v>
+      </x:c>
+      <x:c r="G419" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H419" s="170" t="str">
+        <x:v>Reverse-facing rear-delt variation; no pain or breakdown; exact setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I419" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J419" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K419" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L419" s="170" t="str">
+        <x:v>Replaced reverse pec deck today; counts as rear-delt working fatigue</x:v>
+      </x:c>
+      <x:c r="M419" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N419" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="420">
+      <x:c r="A420" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B420" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C420" s="170" t="str">
+        <x:v>Experimental Rear-Delt Lateral-Raise Machine</x:v>
+      </x:c>
+      <x:c r="D420" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E420" s="170" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F420" s="170" t="str">
+        <x:v>kg plates each side; exact reverse-facing setup/path To verify</x:v>
+      </x:c>
+      <x:c r="G420" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H420" s="170" t="str">
+        <x:v>Reverse-facing rear-delt variation; no pain or breakdown; exact setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I420" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J420" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K420" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L420" s="170" t="str">
+        <x:v>Do not combine with reverse pec deck in the active sequence</x:v>
+      </x:c>
+      <x:c r="M420" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N420" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="421">
+      <x:c r="A421" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B421" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C421" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D421" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E421" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F421" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G421" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H421" s="170" t="str">
+        <x:v>Clean and pain-free; no assistance or breakdown</x:v>
+      </x:c>
+      <x:c r="I421" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J421" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K421" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L421" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M421" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N421" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="422">
+      <x:c r="A422" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B422" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C422" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D422" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E422" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F422" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G422" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H422" s="170" t="str">
+        <x:v>Clean and pain-free; no assistance or breakdown</x:v>
+      </x:c>
+      <x:c r="I422" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J422" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K422" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L422" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M422" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N422" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="423">
+      <x:c r="A423" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B423" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C423" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D423" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E423" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F423" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G423" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H423" s="170" t="str">
+        <x:v>Confirmed clean and pain-free; no assistance or breakdown</x:v>
+      </x:c>
+      <x:c r="I423" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J423" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K423" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L423" s="170" t="str">
+        <x:v>Above prescribed range; retained without progression credit; return to 50 kg target</x:v>
+      </x:c>
+      <x:c r="M423" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N423" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="424">
+      <x:c r="A424" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B424" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C424" s="170" t="str">
+        <x:v>Dumbbell Shrugs</x:v>
+      </x:c>
+      <x:c r="D424" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E424" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F424" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G424" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H424" s="170" t="str">
+        <x:v>Clean and unassisted; top-pause detail To verify</x:v>
+      </x:c>
+      <x:c r="I424" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J424" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K424" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L424" s="170" t="str">
+        <x:v>Reserve was one rep harder than target</x:v>
+      </x:c>
+      <x:c r="M424" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N424" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="425">
+      <x:c r="A425" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B425" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C425" s="170" t="str">
+        <x:v>Dumbbell Shrugs</x:v>
+      </x:c>
+      <x:c r="D425" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E425" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F425" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G425" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H425" s="170" t="str">
+        <x:v>Clean and unassisted; top-pause detail To verify</x:v>
+      </x:c>
+      <x:c r="I425" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J425" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K425" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L425" s="170" t="str">
+        <x:v>Below rep target; keep load</x:v>
+      </x:c>
+      <x:c r="M425" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N425" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="426">
+      <x:c r="A426" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B426" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C426" s="170" t="str">
+        <x:v>Dumbbell Shrugs</x:v>
+      </x:c>
+      <x:c r="D426" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E426" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F426" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G426" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H426" s="170" t="str">
+        <x:v>Clean and unassisted; top-pause detail To verify</x:v>
+      </x:c>
+      <x:c r="I426" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J426" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K426" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L426" s="170" t="str">
+        <x:v>Below rep target; keep load</x:v>
+      </x:c>
+      <x:c r="M426" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N426" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="427">
+      <x:c r="A427" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B427" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C427" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D427" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E427" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F427" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G427" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H427" s="170" t="str">
+        <x:v>Clean and unassisted; upper arms supported</x:v>
+      </x:c>
+      <x:c r="I427" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J427" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K427" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L427" s="170" t="str">
+        <x:v>Replaced incline curl, not added to it</x:v>
+      </x:c>
+      <x:c r="M427" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N427" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="428">
+      <x:c r="A428" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B428" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C428" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D428" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E428" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F428" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G428" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H428" s="170" t="str">
+        <x:v>Clean and unassisted; upper arms supported</x:v>
+      </x:c>
+      <x:c r="I428" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J428" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K428" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L428" s="170" t="str">
+        <x:v>Improved reserve</x:v>
+      </x:c>
+      <x:c r="M428" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N428" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="429">
+      <x:c r="A429" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B429" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C429" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D429" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E429" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F429" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G429" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H429" s="170" t="str">
+        <x:v>Clean and unassisted; upper arms supported</x:v>
+      </x:c>
+      <x:c r="I429" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
+      <x:c r="J429" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K429" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L429" s="170" t="str">
+        <x:v>Improved reserve; requested 15 kg set correctly omitted</x:v>
+      </x:c>
+      <x:c r="M429" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N429" s="170" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21649,7 +22485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdce32aa422314668"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R090187bf579842fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22078,25 +22914,25 @@
         <x:v>Plate Curl Machine</x:v>
       </x:c>
       <x:c r="C16" s="222" t="str">
-        <x:v>12.5 kg/side x 10 @ RIR 2</x:v>
+        <x:v>12.5 kg/side x 11 @ RIR 3</x:v>
       </x:c>
       <x:c r="D16" s="222" t="str">
         <x:v>7.5-12.5 kg/side</x:v>
       </x:c>
       <x:c r="E16" s="222" t="str">
-        <x:v>12.5 kg/side x 11 @ RIR 2</x:v>
+        <x:v>12.5 kg/side x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F16" s="222" t="str">
-        <x:v>Add clean rep</x:v>
+        <x:v>No 15 kg until target is earned</x:v>
       </x:c>
       <x:c r="G16" s="222" t="str">
-        <x:v>Upper arm fixed</x:v>
+        <x:v>Upper arms fixed</x:v>
       </x:c>
       <x:c r="H16" s="222" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I16" s="222" t="str">
-        <x:v>Plates each side</x:v>
+        <x:v>All three sets improved reserve; machine replaced incline curl in this combined session</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -22393,25 +23229,25 @@
         <x:v>Dumbbell Shoulder Press</x:v>
       </x:c>
       <x:c r="C27" s="170" t="str">
-        <x:v>22.5 kg each x 8 @ RIR 1</x:v>
+        <x:v>25 kg each x 8 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="D27" s="170" t="str">
         <x:v>17.5-22.5 kg each</x:v>
       </x:c>
       <x:c r="E27" s="170" t="str">
-        <x:v>22.5 kg each x 8 @ RIR 2 or 9 @ RIR 1-2</x:v>
+        <x:v>22.5 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F27" s="170" t="str">
-        <x:v>Improve reserve before load</x:v>
+        <x:v>Exactly 3 working sets; no 25 kg yet</x:v>
       </x:c>
       <x:c r="G27" s="170" t="str">
         <x:v>Neutral wrist; controlled path</x:v>
       </x:c>
       <x:c r="H27" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify volume/load</x:v>
       </x:c>
       <x:c r="I27" s="170" t="str">
-        <x:v>15 kg set is preparation only; 17.5 kg reps and 20 kg reserve improved</x:v>
+        <x:v>15 kg was warm-up; 17.5-22.5 kg progressed; unplanned 25 kg retained without progression credit</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -22538,13 +23374,13 @@
         <x:v>Dumbbell Shrugs</x:v>
       </x:c>
       <x:c r="C32" s="170" t="str">
-        <x:v>40 kg each x 10 @ RIR 2</x:v>
+        <x:v>40 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D32" s="170" t="str">
         <x:v>30-40 kg each</x:v>
       </x:c>
       <x:c r="E32" s="170" t="str">
-        <x:v>40 kg each x 11-12 @ RIR 2</x:v>
+        <x:v>40 kg each x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F32" s="170" t="str">
         <x:v>Add reps before load</x:v>
@@ -22556,7 +23392,7 @@
         <x:v>Active / Preferred</x:v>
       </x:c>
       <x:c r="I32" s="170" t="str">
-        <x:v>Use dumbbells or dedicated shrug machine; low-pulley cable shrug produced poor stimulus</x:v>
+        <x:v>35 kg and 40 kg finished below repetition targets; keep loads</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="48" hidden="0" customHeight="1">
@@ -22886,16 +23722,16 @@
         <x:v>Plate-Loaded Lateral Raise Machine</x:v>
       </x:c>
       <x:c r="C44" s="170" t="str">
-        <x:v>5 kg/side x 12 @ RIR 2</x:v>
+        <x:v>5 kg/side x 15 for 2 sets @ RIR 2</x:v>
       </x:c>
       <x:c r="D44" s="170" t="str">
         <x:v>2.5-5 kg/side</x:v>
       </x:c>
       <x:c r="E44" s="170" t="str">
-        <x:v>5 kg/side x 13-15 @ RIR 2</x:v>
+        <x:v>5 kg/side x 16 @ RIR 2</x:v>
       </x:c>
       <x:c r="F44" s="170" t="str">
-        <x:v>Add reps; maximum 3 sets</x:v>
+        <x:v>Maximum 3 sets; add one rep</x:v>
       </x:c>
       <x:c r="G44" s="170" t="str">
         <x:v>No shrug; controlled eccentric</x:v>
@@ -22915,25 +23751,25 @@
         <x:v>Cable Upright Row</x:v>
       </x:c>
       <x:c r="C45" s="170" t="str">
-        <x:v>50 kg x 10 @ RIR 1 after 50 kg x 12 @ RIR 2</x:v>
+        <x:v>60 kg x 9 @ RIR 2 unplanned</x:v>
       </x:c>
       <x:c r="D45" s="170" t="str">
         <x:v>40-50 kg stack</x:v>
       </x:c>
       <x:c r="E45" s="170" t="str">
-        <x:v>50 kg x 12-14 @ RIR 2</x:v>
+        <x:v>50 kg x 11-12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F45" s="170" t="str">
-        <x:v>Improve final-set reserve</x:v>
+        <x:v>No 60 kg until both 50 kg sets qualify</x:v>
       </x:c>
       <x:c r="G45" s="170" t="str">
         <x:v>Pull only to comfortable height</x:v>
       </x:c>
       <x:c r="H45" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify load</x:v>
       </x:c>
       <x:c r="I45" s="170" t="str">
-        <x:v>40 kg set progressed; exact effective stack To verify</x:v>
+        <x:v>60 kg was clean but above plan; effective stack resistance To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
@@ -23031,16 +23867,16 @@
         <x:v>Experimental Rear-Delt Lateral-Raise Machine</x:v>
       </x:c>
       <x:c r="C49" s="170" t="str">
-        <x:v>5 kg/side x 8 @ RIR 1</x:v>
+        <x:v>2.5 kg/side x 14 for 2 sets @ RIR 2</x:v>
       </x:c>
       <x:c r="D49" s="170" t="str">
         <x:v>Historical experiment only</x:v>
       </x:c>
       <x:c r="E49" s="170" t="str">
-        <x:v>Do not repeat in active sequence</x:v>
+        <x:v>Use Reverse Pec Deck in active sequence</x:v>
       </x:c>
       <x:c r="F49" s="170" t="str">
-        <x:v>Use Reverse Pec Deck instead</x:v>
+        <x:v>Do not combine both movements</x:v>
       </x:c>
       <x:c r="G49" s="170" t="str">
         <x:v>Exact setup/path To verify</x:v>
@@ -23049,7 +23885,7 @@
         <x:v>Experimental / Replaced</x:v>
       </x:c>
       <x:c r="I49" s="170" t="str">
-        <x:v>Two sets retained as working fatigue; not deleted</x:v>
+        <x:v>Repeated due equipment/order choice; two sets retained as working fatigue; exact geometry To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="52" customHeight="1">
@@ -23106,7 +23942,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1082d0a745844226"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6f398bff5cc42f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24008,16 +24844,28 @@
       <x:c r="Q26" s="59" t="n"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="220"/>
+      <x:c r="A27" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
       <x:c r="B27" s="170"/>
       <x:c r="C27" s="170"/>
-      <x:c r="D27" s="170"/>
-      <x:c r="E27" s="170"/>
-      <x:c r="F27" s="170"/>
+      <x:c r="D27" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E27" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F27" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, biceps or other pain; prior upper-biceps pump resolved</x:v>
+      </x:c>
       <x:c r="G27" s="170"/>
       <x:c r="H27" s="170"/>
-      <x:c r="I27" s="170"/>
-      <x:c r="J27" s="170"/>
+      <x:c r="I27" s="170" t="str">
+        <x:v>Shoulders + Biceps workout - 75 min; 19 entries; 18 working sets; no core/cardio</x:v>
+      </x:c>
+      <x:c r="J27" s="170" t="str">
+        <x:v>Started Medium; medium shoulder/trap pump; full EAA+ scoop (100 mg caffeine); no coffee; no assistance or breakdown; 25 kg press and 60 kg upright row clean; no extra 15 kg curl</x:v>
+      </x:c>
       <x:c r="K27" s="59" t="n"/>
       <x:c r="L27" s="59" t="n"/>
       <x:c r="M27" s="59" t="n"/>
@@ -27369,7 +28217,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b0533ba26e4437b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bf5887a337743f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28398,13 +29246,83 @@
         <x:v>Keep load; require RIR 1-2 and no assisted repetition before progression</x:v>
       </x:c>
     </x:row>
+    <x:row r="69" ht="52" customHeight="1">
+      <x:c r="A69" s="170" t="str">
+        <x:v>Shoulders + Biceps performance</x:v>
+      </x:c>
+      <x:c r="B69" s="170" t="str">
+        <x:v>2026-08-26 completed one warm-up plus exactly 18 working sets in 75 min; no pain, assistance, breakdown or RIR 0</x:v>
+      </x:c>
+      <x:c r="C69" s="170" t="str">
+        <x:v>Press, lateral raise and curl performance improved, but final energy fell from Medium to Low</x:v>
+      </x:c>
+      <x:c r="D69" s="170" t="str">
+        <x:v>Keep volume fixed; no load expansion from unplanned sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="52" customHeight="1">
+      <x:c r="A70" s="170" t="str">
+        <x:v>Equipment-driven schedule swap</x:v>
+      </x:c>
+      <x:c r="B70" s="170" t="str">
+        <x:v>Leg machines were busy, so Day 3 changed from Legs to Shoulders + Biceps</x:v>
+      </x:c>
+      <x:c r="C70" s="170" t="str">
+        <x:v>The swap preserved the four available training days without waiting or mixing body-part sessions</x:v>
+      </x:c>
+      <x:c r="D70" s="170" t="str">
+        <x:v>Legs becomes Day 4 after fresh lower-body readiness</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="52" customHeight="1">
+      <x:c r="A71" s="170" t="str">
+        <x:v>Live volume correction followed</x:v>
+      </x:c>
+      <x:c r="B71" s="170" t="str">
+        <x:v>Two reverse-facing rear-delt sets replaced reverse pec deck, and the requested extra 15 kg curl was omitted</x:v>
+      </x:c>
+      <x:c r="C71" s="170" t="str">
+        <x:v>The unplanned fourth shoulder-press set did not push the session above 18 working sets</x:v>
+      </x:c>
+      <x:c r="D71" s="170" t="str">
+        <x:v>Continue treating live reductions as final</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="52" customHeight="1">
+      <x:c r="A72" s="170" t="str">
+        <x:v>Unplanned upper-body loads</x:v>
+      </x:c>
+      <x:c r="B72" s="170" t="str">
+        <x:v>25 kg shoulder press x 8 @ RIR 1 and 60 kg upright row x 9 @ RIR 2 were clean but above plan</x:v>
+      </x:c>
+      <x:c r="C72" s="170" t="str">
+        <x:v>Low final energy and prior volume pattern make these insufficient progression evidence</x:v>
+      </x:c>
+      <x:c r="D72" s="170" t="str">
+        <x:v>Return to the prescribed ranges next time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="52" customHeight="1">
+      <x:c r="A73" s="170" t="str">
+        <x:v>Third consecutive Low final energy</x:v>
+      </x:c>
+      <x:c r="B73" s="170" t="str">
+        <x:v>2026-08-24, 2026-08-25 and 2026-08-26 resistance sessions all ended with Low energy</x:v>
+      </x:c>
+      <x:c r="C73" s="170" t="str">
+        <x:v>Performance is improving, but accumulated fatigue is becoming consistent</x:v>
+      </x:c>
+      <x:c r="D73" s="170" t="str">
+        <x:v>Keep Legs at 18 sets, avoid RIR 0/assistance, then schedule recovery</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf44478e3a9de4d50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898137546536421d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29048,14 +29966,30 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="220"/>
-      <x:c r="B25" s="170"/>
-      <x:c r="C25" s="170"/>
-      <x:c r="D25" s="170"/>
-      <x:c r="E25" s="170"/>
-      <x:c r="F25" s="170"/>
-      <x:c r="G25" s="170"/>
-      <x:c r="H25" s="170"/>
+      <x:c r="A25" s="220" t="n">
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="B25" s="170" t="str">
+        <x:v>Shoulders + Biceps</x:v>
+      </x:c>
+      <x:c r="C25" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D25" s="170" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E25" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F25" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; no soreness or pain; prior upper-biceps pump resolved; 75 min; medium shoulder/trap pump; no assistance or form breakdown; 25 kg shoulder press and 60 kg upright row confirmed clean; full EAA+; no coffee; no core/cardio; no additional 15 kg curl</x:v>
+      </x:c>
+      <x:c r="G25" s="170" t="str">
+        <x:v>Exactly 18 working sets plus one genuine warm-up were completed without pain, assistance or RIR 0. Pressing, lateral raises and curl reserve progressed. Live substitution preserved the set ceiling, but Low final energy means the unplanned 25 kg press and 60 kg upright row do not justify expanding load or volume.</x:v>
+      </x:c>
+      <x:c r="H25" s="170" t="str">
+        <x:v>Legs next after fresh hip, knee and lower-back readiness; keep exactly 18 working sets, no failure or hand assistance; RDL technique reset at 10 kg each; next Shoulders use three planned press sets and no 60 kg upright row</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -29069,7 +30003,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R763c8925571846f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6293a6220d5c4b7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29246,13 +30180,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Chest + Triceps on 2026-08-25: no chest, shoulder, elbow or wrist pain. Strong upper-biceps/upper-arm pump likely from pec deck was not painful; exact side To verify.</x:v>
+        <x:v>After Shoulders + Biceps on 2026-08-26: no shoulder, elbow, wrist, biceps or other pain; prior pec-deck-related upper-biceps pump resolved.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
-        <x:v>Known with verification flag</x:v>
+        <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Confirm pump resolves; pause direct upper-body loading if pain, bruising or weakness develops</x:v>
+        <x:v>Recheck hip, knee and lower back before Legs</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -29434,13 +30368,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Temporary four-day week: Day 1 Back + Biceps completed 2026-08-24; Day 2 Chest + Triceps completed 2026-08-25; Legs is next; Day 4 Shoulders + core; exact spacing To verify.</x:v>
+        <x:v>Temporary four-day week: Back + Biceps completed 2026-08-24; Chest + Triceps completed 2026-08-25; Shoulders + Biceps completed 2026-08-26 after leg-equipment congestion; Legs is Day 4 next.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
-        <x:v>Partial / To verify</x:v>
+        <x:v>Known for current week</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Confirm readiness and day spacing before Legs</x:v>
+        <x:v>Complete Legs only after fresh lower-body readiness</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -29639,7 +30573,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58fd9f2406014922"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85520e9dbd454f23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30742,10 +31676,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e5ccbce0a2e48de"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf164dd7f2fc64593"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc83f777712a041ac"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re35b06aa6fc14d2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5b2a97ed4274adc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R066845464844409f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbafaa5f3690341ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287312e5f7924810"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 27 legs workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8093760176c743b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb4dde22ba9c7407a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rfb432a5f20db4478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R82a35bb9ab89423d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R07efffaa975a42f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R7340f1e6983240a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R70d26c83bbc44f33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R4c932b342f454833"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R3dd3291087f14334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc5a695c94b2e4806"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R892844fa43e4485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R93498e34581c4992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb862d47c44454c3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R22977a1eab6d4de6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rf29b31b4ef474299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R238f63c7d4d545a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rb625f0bea5d04f7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rdd997a41c12e400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Rc12033eae7da45a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R795441e263f64630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R88243cd8ff024119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R462eb484e93341dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08613bcf59e5403a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfeab76a10df44eac"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N429" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N447" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R085db3d201e2400d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R843456876d34492d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5453c2d7148741d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98d5cf0e00b143f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4083,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4349,7 +4349,7 @@
         <x:v>Day 4</x:v>
       </x:c>
       <x:c r="B16" s="59" t="str">
-        <x:v>Legs - next; fresh lower-body readiness required</x:v>
+        <x:v>Legs - completed 2026-08-27</x:v>
       </x:c>
       <x:c r="C16" s="59" t="n"/>
       <x:c r="D16" s="94" t="inlineStr">
@@ -4388,29 +4388,29 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="92" t="str">
-        <x:v>Other days</x:v>
+        <x:v>Next</x:v>
       </x:c>
       <x:c r="B17" s="59" t="str">
-        <x:v>Rest / walking</x:v>
+        <x:v>Recovery / rest; easy walking only if desired</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E17" s="59" t="str">
-        <x:v>Dumbbell Shoulder Press</x:v>
+        <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="F17" s="59" t="str">
-        <x:v>25 kg each x 8 @ RIR 1 unplanned</x:v>
+        <x:v>65 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="G17" s="59" t="str">
-        <x:v>22.5 kg each x 9 @ RIR 2</x:v>
+        <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H17" s="59" t="str">
-        <x:v>Modify volume</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I17" s="59" t="str">
-        <x:v>Exactly 3 working sets; no 25 kg yet</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
@@ -4418,29 +4418,29 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="92" t="str">
-        <x:v>Spacing</x:v>
+        <x:v>Reason</x:v>
       </x:c>
       <x:c r="B18" s="59" t="str">
-        <x:v>Equipment-driven order swap preserved</x:v>
+        <x:v>Four consecutive sessions ended with Low energy</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E18" s="59" t="str">
-        <x:v>Plate Lateral Raise</x:v>
+        <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="F18" s="59" t="str">
-        <x:v>5 kg/side x 15 x2 @ RIR 2</x:v>
+        <x:v>160 kg x 5 clean + 2 assisted</x:v>
       </x:c>
       <x:c r="G18" s="59" t="str">
-        <x:v>5 kg/side x 16 @ RIR 2</x:v>
+        <x:v>140 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H18" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify / Verify</x:v>
       </x:c>
       <x:c r="I18" s="59" t="str">
-        <x:v>Unloaded resistance To verify</x:v>
+        <x:v>No assisted 160; old load discrepancy To verify</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
@@ -4451,22 +4451,22 @@
       <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Cable Upright Row</x:v>
+        <x:v>Dumbbell RDL</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>60 kg x 9 @ RIR 2 unplanned</x:v>
+        <x:v>15 kg each x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>50 kg x 11-12 @ RIR 2</x:v>
+        <x:v>15 kg each x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>Modify load</x:v>
+        <x:v>Technique improving</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>No 60 kg yet</x:v>
+        <x:v>Hamstrings dominant; keep pain-free</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
@@ -4477,22 +4477,22 @@
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="59" t="str">
-        <x:v>Shoulders</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Dumbbell Shrug</x:v>
+        <x:v>Leg Curl</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>40 kg each x 9 @ RIR 2</x:v>
+        <x:v>35 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>40 kg each x 10 @ RIR 2</x:v>
+        <x:v>35 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>Keep load; top pause</x:v>
+        <x:v>No failure</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4503,22 +4503,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Plate Curl Machine</x:v>
+        <x:v>Leg Extension</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>12.5 kg/side x 11 @ RIR 3</x:v>
+        <x:v>50 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>12.5 kg/side x 12 @ RIR 2</x:v>
+        <x:v>50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>No extra 15 kg set</x:v>
+        <x:v>Add one rep</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4532,19 +4532,19 @@
         <x:v>Legs</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Dumbbell RDL</x:v>
+        <x:v>Standing Calf Raise</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>15 kg each x 12; back dominant</x:v>
+        <x:v>20 kg/side x 16 @ RIR 3</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>10 kg each technique sets</x:v>
+        <x:v>20 kg/side x 17 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>Verify technique</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Stop if back or hip dominates</x:v>
+        <x:v>Return to 3 planned sets</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4555,22 +4555,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Recovery</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Hack Squat</x:v>
+        <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>65 kg/side x 10 @ RIR 2</x:v>
+        <x:v>Low after 4 consecutive sessions</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Repeat after readiness</x:v>
+        <x:v>Rest / easy walking</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Recovery due</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>No load increase</x:v>
+        <x:v>No compensatory cardio</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4581,22 +4581,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Program</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Leg Press</x:v>
+        <x:v>Working-set ceiling</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>150 kg x 7 with assistance</x:v>
+        <x:v>18 sets achieved</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>130 kg x 9-10 @ RIR 2</x:v>
+        <x:v>Maintain 18</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>On target</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>No assisted 150 kg</x:v>
+        <x:v>Pre-plan 3 leg-press sets</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4625,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58cc489811d84211"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b3f221b10c64188"/>
 </x:worksheet>
 </file>
 
@@ -22450,6 +22450,798 @@
         <x:v>Working</x:v>
       </x:c>
       <x:c r="N429" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430">
+      <x:c r="A430" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B430" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C430" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D430" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E430" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F430" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G430" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H430" s="170" t="str">
+        <x:v>Clean and unassisted; controlled depth To verify</x:v>
+      </x:c>
+      <x:c r="I430" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J430" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K430" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L430" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M430" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N430" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="431">
+      <x:c r="A431" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B431" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C431" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D431" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E431" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F431" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G431" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H431" s="170" t="str">
+        <x:v>Clean and unassisted; controlled depth To verify</x:v>
+      </x:c>
+      <x:c r="I431" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J431" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K431" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L431" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M431" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N431" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432">
+      <x:c r="A432" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B432" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C432" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D432" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E432" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F432" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G432" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H432" s="170" t="str">
+        <x:v>Clean and unassisted; controlled depth To verify</x:v>
+      </x:c>
+      <x:c r="I432" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J432" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K432" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L432" s="170" t="str">
+        <x:v>Reserve improved</x:v>
+      </x:c>
+      <x:c r="M432" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N432" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433">
+      <x:c r="A433" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B433" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C433" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D433" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E433" s="170" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F433" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G433" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H433" s="170" t="str">
+        <x:v>Clean and unassisted; controlled depth To verify</x:v>
+      </x:c>
+      <x:c r="I433" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J433" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K433" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L433" s="170" t="str">
+        <x:v>One rep below target; keep load</x:v>
+      </x:c>
+      <x:c r="M433" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N433" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434">
+      <x:c r="A434" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B434" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C434" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D434" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E434" s="170" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F434" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G434" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H434" s="170" t="str">
+        <x:v>Clean and unassisted; depth and sled resistance To verify</x:v>
+      </x:c>
+      <x:c r="I434" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J434" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K434" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L434" s="170" t="str">
+        <x:v>Exceeded prescribed rep range; keep load and improve reserve</x:v>
+      </x:c>
+      <x:c r="M434" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N434" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="435">
+      <x:c r="A435" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B435" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C435" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D435" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E435" s="170" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F435" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G435" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H435" s="170" t="str">
+        <x:v>Clean and unassisted; depth and sled resistance To verify</x:v>
+      </x:c>
+      <x:c r="I435" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J435" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K435" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L435" s="170" t="str">
+        <x:v>Exceeded prescribed rep range; keep load</x:v>
+      </x:c>
+      <x:c r="M435" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N435" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="436">
+      <x:c r="A436" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B436" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C436" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D436" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E436" s="170" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F436" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G436" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H436" s="170" t="str">
+        <x:v>Clean and unassisted; depth and sled resistance To verify</x:v>
+      </x:c>
+      <x:c r="I436" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J436" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K436" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L436" s="170" t="str">
+        <x:v>Harder than target; historical 130/150 versus 140/160 load discrepancy To verify</x:v>
+      </x:c>
+      <x:c r="M436" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N436" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="437">
+      <x:c r="A437" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B437" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C437" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D437" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E437" s="170" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F437" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G437" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H437" s="170" t="str">
+        <x:v>Five clean reps plus two human hand-assisted reps; assistance source To verify</x:v>
+      </x:c>
+      <x:c r="I437" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J437" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K437" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L437" s="170" t="str">
+        <x:v>Unplanned assisted top set; no progression credit; omit next time; historical load discrepancy To verify</x:v>
+      </x:c>
+      <x:c r="M437" s="170" t="str">
+        <x:v>Assisted</x:v>
+      </x:c>
+      <x:c r="N437" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="438">
+      <x:c r="A438" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B438" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C438" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D438" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E438" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F438" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G438" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H438" s="170" t="str">
+        <x:v>Pain-free; hamstrings dominant with a little non-painful lower-back involvement; detailed hinge depth To verify</x:v>
+      </x:c>
+      <x:c r="I438" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J438" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K438" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L438" s="170" t="str">
+        <x:v>Technique improved from prior lower-back-dominant session</x:v>
+      </x:c>
+      <x:c r="M438" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N438" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="439">
+      <x:c r="A439" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B439" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C439" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D439" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E439" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F439" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G439" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H439" s="170" t="str">
+        <x:v>Pain-free; hamstrings dominant with a little non-painful lower-back involvement; detailed hinge depth To verify</x:v>
+      </x:c>
+      <x:c r="I439" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J439" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K439" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L439" s="170" t="str">
+        <x:v>Pain-free progression; keep load controlled</x:v>
+      </x:c>
+      <x:c r="M439" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N439" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="440">
+      <x:c r="A440" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B440" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C440" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D440" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E440" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F440" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G440" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H440" s="170" t="str">
+        <x:v>Pain-free; hamstrings dominant with a little non-painful lower-back involvement; detailed hinge depth To verify</x:v>
+      </x:c>
+      <x:c r="I440" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J440" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K440" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L440" s="170" t="str">
+        <x:v>Third set completed after leg press; no load increase yet</x:v>
+      </x:c>
+      <x:c r="M440" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N440" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="441">
+      <x:c r="A441" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B441" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C441" s="170" t="str">
+        <x:v>Leg Curl</x:v>
+      </x:c>
+      <x:c r="D441" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E441" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F441" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G441" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H441" s="170" t="str">
+        <x:v>Clean and unassisted; full range To verify</x:v>
+      </x:c>
+      <x:c r="I441" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J441" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K441" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L441" s="170" t="str">
+        <x:v>One reserve harder than target</x:v>
+      </x:c>
+      <x:c r="M441" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N441" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="442">
+      <x:c r="A442" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B442" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C442" s="170" t="str">
+        <x:v>Leg Curl</x:v>
+      </x:c>
+      <x:c r="D442" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E442" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F442" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G442" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H442" s="170" t="str">
+        <x:v>Clean and unassisted; full range To verify</x:v>
+      </x:c>
+      <x:c r="I442" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J442" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K442" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L442" s="170" t="str">
+        <x:v>Below 10-12 rep target and harder than target; keep load</x:v>
+      </x:c>
+      <x:c r="M442" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N442" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="443">
+      <x:c r="A443" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B443" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C443" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D443" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E443" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F443" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G443" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H443" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I443" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J443" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K443" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L443" s="170" t="str">
+        <x:v>Target met exactly</x:v>
+      </x:c>
+      <x:c r="M443" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N443" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="444">
+      <x:c r="A444" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B444" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C444" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D444" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E444" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F444" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G444" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H444" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I444" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J444" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K444" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L444" s="170" t="str">
+        <x:v>Target met exactly</x:v>
+      </x:c>
+      <x:c r="M444" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N444" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="445">
+      <x:c r="A445" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B445" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C445" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D445" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E445" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F445" s="170" t="str">
+        <x:v>kg total stack; effective resistance To verify</x:v>
+      </x:c>
+      <x:c r="G445" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H445" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I445" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J445" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K445" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L445" s="170" t="str">
+        <x:v>Target met exactly</x:v>
+      </x:c>
+      <x:c r="M445" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N445" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="446">
+      <x:c r="A446" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B446" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C446" s="170" t="str">
+        <x:v>Standing Calf Raise</x:v>
+      </x:c>
+      <x:c r="D446" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E446" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F446" s="170" t="str">
+        <x:v>kg plates each side on guided bar; bar excluded</x:v>
+      </x:c>
+      <x:c r="G446" s="170" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H446" s="170" t="str">
+        <x:v>Clean and unassisted; pause and stretch detail To verify</x:v>
+      </x:c>
+      <x:c r="I446" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J446" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K446" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L446" s="170" t="str">
+        <x:v>Rep progression with reserve</x:v>
+      </x:c>
+      <x:c r="M446" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N446" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="447">
+      <x:c r="A447" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B447" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C447" s="170" t="str">
+        <x:v>Standing Calf Raise</x:v>
+      </x:c>
+      <x:c r="D447" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E447" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F447" s="170" t="str">
+        <x:v>kg plates each side on guided bar; bar excluded</x:v>
+      </x:c>
+      <x:c r="G447" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H447" s="170" t="str">
+        <x:v>Clean and unassisted; pause and stretch detail To verify</x:v>
+      </x:c>
+      <x:c r="I447" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
+      <x:c r="J447" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K447" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L447" s="170" t="str">
+        <x:v>Reserve improved; only two sets used to preserve 18-set ceiling</x:v>
+      </x:c>
+      <x:c r="M447" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N447" s="170" t="n">
         <x:v>3</x:v>
       </x:c>
     </x:row>
@@ -22485,7 +23277,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R090187bf579842fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c2e4f45a34f4d08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23030,7 +23822,7 @@
         <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="C20" s="169" t="str">
-        <x:v>65 kg/side x 10 @ RIR 2</x:v>
+        <x:v>65 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D20" s="169" t="str">
         <x:v>35-65 kg/side</x:v>
@@ -23039,7 +23831,7 @@
         <x:v>65 kg/side x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F20" s="169" t="str">
-        <x:v>Improve reserve; no load increase</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="G20" s="169" t="str">
         <x:v>Controlled depth; knees track toes</x:v>
@@ -23048,7 +23840,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I20" s="169" t="str">
-        <x:v>Check hip before loading; progressed cleanly on 2026-08-20</x:v>
+        <x:v>35-55 kg reserve improved; machine carriage excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" hidden="0" customHeight="1">
@@ -23059,25 +23851,25 @@
         <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="C21" s="169" t="str">
-        <x:v>150 kg x 7 total @ RIR 1; approx. 2-3 assisted</x:v>
+        <x:v>160 kg x 5 clean + 2 assisted @ RIR 1</x:v>
       </x:c>
       <x:c r="D21" s="169" t="str">
-        <x:v>100-130 kg total</x:v>
+        <x:v>100-140 kg total</x:v>
       </x:c>
       <x:c r="E21" s="169" t="str">
-        <x:v>130 kg x 9-10 @ RIR 2</x:v>
+        <x:v>140 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F21" s="169" t="str">
-        <x:v>Clean reps only; omit 150 kg</x:v>
+        <x:v>Exactly 3 sets; no assisted 160 kg</x:v>
       </x:c>
       <x:c r="G21" s="169" t="str">
-        <x:v>No hand assistance; controlled depth</x:v>
+        <x:v>Hips stay on pad; controlled depth</x:v>
       </x:c>
       <x:c r="H21" s="169" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>Modify load/effort / To verify</x:v>
       </x:c>
       <x:c r="I21" s="169" t="str">
-        <x:v>Approx. 4-5 clean reps at 150 kg To verify; hip pain follow-up required</x:v>
+        <x:v>Earlier 130/150 entry conflicts with reported 140/160 machine increments; preserve both and verify before rewriting history</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" hidden="0" customHeight="1">
@@ -23088,25 +23880,25 @@
         <x:v>Leg Extension</x:v>
       </x:c>
       <x:c r="C22" s="169" t="str">
-        <x:v>50 kg x 11 @ RIR 1</x:v>
+        <x:v>50 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="D22" s="169" t="str">
         <x:v>40-50 kg</x:v>
       </x:c>
       <x:c r="E22" s="169" t="str">
-        <x:v>50 kg x 10-11 @ RIR 2</x:v>
+        <x:v>50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F22" s="169" t="str">
-        <x:v>Improve reserve before load</x:v>
+        <x:v>Add one clean rep</x:v>
       </x:c>
       <x:c r="G22" s="169" t="str">
-        <x:v>Controlled lockout; no momentum</x:v>
+        <x:v>Controlled eccentric; no forceful lockout</x:v>
       </x:c>
       <x:c r="H22" s="169" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="169" t="str">
-        <x:v>Progressed reps on 2026-08-20</x:v>
+        <x:v>All three targets met exactly</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" hidden="0" customHeight="1">
@@ -23117,25 +23909,25 @@
         <x:v>Leg Curl</x:v>
       </x:c>
       <x:c r="C23" s="169" t="str">
-        <x:v>35 kg x 9 @ RIR 0</x:v>
+        <x:v>35 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="D23" s="169" t="str">
         <x:v>30-35 kg</x:v>
       </x:c>
       <x:c r="E23" s="169" t="str">
-        <x:v>30 kg x 12 @ RIR 2</x:v>
+        <x:v>35 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F23" s="169" t="str">
-        <x:v>Reduce failure exposure</x:v>
+        <x:v>Add rep and reserve before load</x:v>
       </x:c>
       <x:c r="G23" s="169" t="str">
-        <x:v>Full range; hips down</x:v>
+        <x:v>Full range; controlled eccentric</x:v>
       </x:c>
       <x:c r="H23" s="169" t="str">
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I23" s="169" t="str">
-        <x:v>Full range at 35 kg remains To verify</x:v>
+        <x:v>30 kg was RIR 2; 35 kg remains too close to failure</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" hidden="0" customHeight="1">
@@ -23200,25 +23992,25 @@
         <x:v>Standing Calf Raise</x:v>
       </x:c>
       <x:c r="C26" s="169" t="str">
-        <x:v>+20 kg/side x 16 @ RIR 2</x:v>
+        <x:v>20 kg/side x 16 @ RIR 3</x:v>
       </x:c>
       <x:c r="D26" s="169" t="str">
-        <x:v>+10 to +20 kg/side</x:v>
+        <x:v>10-20 kg/side</x:v>
       </x:c>
       <x:c r="E26" s="169" t="str">
-        <x:v>+20 kg/side x 17 @ RIR 2</x:v>
+        <x:v>20 kg/side x 17 @ RIR 2</x:v>
       </x:c>
       <x:c r="F26" s="169" t="str">
-        <x:v>Add clean rep</x:v>
+        <x:v>Return to 3 sets within 18-set plan</x:v>
       </x:c>
       <x:c r="G26" s="169" t="str">
-        <x:v>Full stretch and top pause</x:v>
+        <x:v>Full stretch; pause at top</x:v>
       </x:c>
       <x:c r="H26" s="169" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I26" s="169" t="str">
-        <x:v>Guided bar excluded from recorded load</x:v>
+        <x:v>Two sets only today because extra leg-press set consumed the set budget; bar excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -23838,25 +24630,25 @@
         <x:v>Dumbbell Romanian Deadlift</x:v>
       </x:c>
       <x:c r="C48" s="170" t="str">
-        <x:v>15 kg each x 12 @ RIR 2; lower-back dominant</x:v>
+        <x:v>15 kg each x 10 @ RIR 2; pain-free</x:v>
       </x:c>
       <x:c r="D48" s="170" t="str">
-        <x:v>10 kg each technique only</x:v>
+        <x:v>10-15 kg each</x:v>
       </x:c>
       <x:c r="E48" s="170" t="str">
-        <x:v>10 kg each x 10-12 @ RIR 3-4</x:v>
+        <x:v>15 kg each x 10-11 @ RIR 2 with hamstrings dominant</x:v>
       </x:c>
       <x:c r="F48" s="170" t="str">
-        <x:v>Technique reset; do not add load</x:v>
+        <x:v>Keep load; technique before progression</x:v>
       </x:c>
       <x:c r="G48" s="170" t="str">
-        <x:v>Wall hinge; dumbbells close; hamstring-controlled depth</x:v>
+        <x:v>Brace; hips back; dumbbells close; hamstring-controlled depth</x:v>
       </x:c>
       <x:c r="H48" s="170" t="str">
-        <x:v>Verify technique</x:v>
+        <x:v>Technique improving</x:v>
       </x:c>
       <x:c r="I48" s="170" t="str">
-        <x:v>Lower-back dominant; little post-session hip pain; stop if either persists</x:v>
+        <x:v>Hamstrings dominated with only a little non-painful back involvement</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="52" customHeight="1">
@@ -23942,7 +24734,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6f398bff5cc42f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a5ae830445f4f0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24874,17 +25666,29 @@
       <x:c r="P27" s="59" t="n"/>
       <x:c r="Q27" s="59" t="n"/>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="220"/>
+    <x:row r="28" ht="72" customHeight="1">
+      <x:c r="A28" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
       <x:c r="B28" s="170"/>
       <x:c r="C28" s="170"/>
-      <x:c r="D28" s="170"/>
-      <x:c r="E28" s="170"/>
-      <x:c r="F28" s="170"/>
+      <x:c r="D28" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E28" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F28" s="170" t="str">
+        <x:v>No lower-back, knee or hip pain; RDL felt mainly in hamstrings with a little non-painful lower-back involvement</x:v>
+      </x:c>
       <x:c r="G28" s="170"/>
       <x:c r="H28" s="170"/>
-      <x:c r="I28" s="170"/>
-      <x:c r="J28" s="170"/>
+      <x:c r="I28" s="170" t="str">
+        <x:v>Leg workout - 90 min; exactly 18 working sets; medium leg/lower-back pump; no cardio/core</x:v>
+      </x:c>
+      <x:c r="J28" s="170" t="str">
+        <x:v>Started Medium; full EAA+ scoop (100 mg caffeine); no coffee; only two final repetitions at 160 kg leg press were human-assisted; no other assistance or form breakdown</x:v>
+      </x:c>
       <x:c r="K28" s="59" t="n"/>
       <x:c r="L28" s="59" t="n"/>
       <x:c r="M28" s="59" t="n"/>
@@ -28217,7 +29021,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bf5887a337743f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48a6d2b6c1e04587"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29316,13 +30120,97 @@
         <x:v>Keep Legs at 18 sets, avoid RIR 0/assistance, then schedule recovery</x:v>
       </x:c>
     </x:row>
+    <x:row r="74" ht="52" customHeight="1">
+      <x:c r="A74" s="170" t="str">
+        <x:v>Legs performance</x:v>
+      </x:c>
+      <x:c r="B74" s="170" t="str">
+        <x:v>2026-08-27 completed exactly 18 working sets in 90 min; no pain or RIR 0; final energy Low</x:v>
+      </x:c>
+      <x:c r="C74" s="170" t="str">
+        <x:v>Hack squat reserve, RDL targeting, leg extension and calf reserve improved</x:v>
+      </x:c>
+      <x:c r="D74" s="170" t="str">
+        <x:v>Keep loads controlled; recovery/rest next</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="52" customHeight="1">
+      <x:c r="A75" s="170" t="str">
+        <x:v>RDL technique improvement</x:v>
+      </x:c>
+      <x:c r="B75" s="170" t="str">
+        <x:v>10-15 kg each for 15/12/10 reps at RIR 2; hamstrings dominated and no pain occurred</x:v>
+      </x:c>
+      <x:c r="C75" s="170" t="str">
+        <x:v>This is a meaningful improvement from the prior lower-back-dominant baseline</x:v>
+      </x:c>
+      <x:c r="D75" s="170" t="str">
+        <x:v>Keep the same range; stop if the lower back or hip becomes dominant</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="52" customHeight="1">
+      <x:c r="A76" s="170" t="str">
+        <x:v>Leg-press assistance</x:v>
+      </x:c>
+      <x:c r="B76" s="170" t="str">
+        <x:v>160 kg produced five clean plus two human-assisted reps at RIR 1</x:v>
+      </x:c>
+      <x:c r="C76" s="170" t="str">
+        <x:v>Assisted repetitions do not earn progression and added fatigue</x:v>
+      </x:c>
+      <x:c r="D76" s="170" t="str">
+        <x:v>Next Legs use 100, 120 and 140 kg only; require 140 kg x 10 @ RIR 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="52" customHeight="1">
+      <x:c r="A77" s="170" t="str">
+        <x:v>Historical leg-press load discrepancy</x:v>
+      </x:c>
+      <x:c r="B77" s="170" t="str">
+        <x:v>Vipin reported that the prior leg-press loads were 140/160 kg, while the canonical 2026-08-20 entry records 130/150 kg</x:v>
+      </x:c>
+      <x:c r="C77" s="170" t="str">
+        <x:v>History must not be silently rewritten when the two reports conflict</x:v>
+      </x:c>
+      <x:c r="D77" s="170" t="str">
+        <x:v>Preserve the old entry and mark the discrepancy To verify against the machine increments or contemporaneous evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="52" customHeight="1">
+      <x:c r="A78" s="170" t="str">
+        <x:v>Temporary four-day week complete</x:v>
+      </x:c>
+      <x:c r="B78" s="170" t="str">
+        <x:v>Back+Biceps, Chest+Triceps, Shoulders+Biceps and Legs were completed on 2026-08-24 through 2026-08-27</x:v>
+      </x:c>
+      <x:c r="C78" s="170" t="str">
+        <x:v>Four consecutive resistance sessions ended with Low final energy</x:v>
+      </x:c>
+      <x:c r="D78" s="170" t="str">
+        <x:v>Use immediate recovery/rest before the next resistance session; do not add compensatory cardio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="52" customHeight="1">
+      <x:c r="A79" s="170" t="str">
+        <x:v>Live set-ceiling adjustment followed</x:v>
+      </x:c>
+      <x:c r="B79" s="170" t="str">
+        <x:v>Four leg-press sets and three RDL sets were completed; calf work was reduced to two sets</x:v>
+      </x:c>
+      <x:c r="C79" s="170" t="str">
+        <x:v>The adjustment preserved exactly 18 working sets without deleting completed work</x:v>
+      </x:c>
+      <x:c r="D79" s="170" t="str">
+        <x:v>Next Legs pre-plan three leg-press and three calf sets</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898137546536421d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R647f86a178db48fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29991,6 +30879,32 @@
         <x:v>Legs next after fresh hip, knee and lower-back readiness; keep exactly 18 working sets, no failure or hand assistance; RDL technique reset at 10 kg each; next Shoulders use three planned press sets and no 60 kg upright row</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="84" customHeight="1">
+      <x:c r="A26" s="220" t="n">
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="B26" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C26" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D26" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E26" s="170" t="str">
+        <x:v>Yellow</x:v>
+      </x:c>
+      <x:c r="F26" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; no soreness or pre-session pain; no post-session lower-back, knee or hip pain; 90 min; medium leg/lower-back pump; RDL hamstrings dominant with a little back involvement; full EAA+; no coffee; only the final two repetitions at 160 kg leg press were human-assisted</x:v>
+      </x:c>
+      <x:c r="G26" s="170" t="str">
+        <x:v>Exactly 18 working sets were completed with no RIR 0 or pain. Hack squat reserve, RDL targeting, leg-extension execution and calf reserve improved. The assisted 160 kg leg-press set and fourth consecutive Low final-energy session prevent load progression and support immediate recovery.</x:v>
+      </x:c>
+      <x:c r="H26" s="170" t="str">
+        <x:v>Recovery/rest next; next Legs use three unassisted leg-press sets, keep RDL pain-free and hamstring-led, improve leg-curl reserve, and retain exactly 18 working sets</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -30003,7 +30917,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6293a6220d5c4b7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1106a282119498d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30180,13 +31094,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Shoulders + Biceps on 2026-08-26: no shoulder, elbow, wrist, biceps or other pain; prior pec-deck-related upper-biceps pump resolved.</x:v>
+        <x:v>After Legs on 2026-08-27: no lower-back, knee or hip pain. RDL was hamstring-dominant with a little non-painful back involvement.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Recheck hip, knee and lower back before Legs</x:v>
+        <x:v>Recheck delayed leg/back soreness and energy before the next resistance session</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -30368,13 +31282,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Temporary four-day week: Back + Biceps completed 2026-08-24; Chest + Triceps completed 2026-08-25; Shoulders + Biceps completed 2026-08-26 after leg-equipment congestion; Legs is Day 4 next.</x:v>
+        <x:v>Temporary four-day week completed: Back + Biceps 2026-08-24; Chest + Triceps 2026-08-25; Shoulders + Biceps 2026-08-26; Legs 2026-08-27.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known for current week</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Complete Legs only after fresh lower-body readiness</x:v>
+        <x:v>Recovery/rest next because four consecutive sessions ended with Low final energy</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -30573,7 +31487,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85520e9dbd454f23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112ee6676fca4956"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31676,10 +32590,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5b2a97ed4274adc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R066845464844409f"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbafaa5f3690341ca"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R287312e5f7924810"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc773ad4a4db4f2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f69ce31d5e4032"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d671af1ec63410e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R522fc9d783fe42ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log August 31 chest and triceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R93498e34581c4992"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb862d47c44454c3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R22977a1eab6d4de6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rf29b31b4ef474299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R238f63c7d4d545a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rb625f0bea5d04f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rdd997a41c12e400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Rc12033eae7da45a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R795441e263f64630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R88243cd8ff024119"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R462eb484e93341dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R772ffc799e594d4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rdcfdc6d3278140c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rd1c9bec3c528494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Re4c8ede6b98a4937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Ra4fd2bca4ab8432d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rf7a8e964afb74128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R73eea8372fea4531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Rf38bd190b0d04804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R266fddb1b0d34285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R84a32a4d22e245ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R6c61d431267349b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfeab76a10df44eac"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re74ee2b478ac461b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N447" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N465" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R843456876d34492d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bbef083e0394d39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98d5cf0e00b143f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab955d759f8343df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4083,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4280,10 +4280,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="92" t="str">
-        <x:v>Day 1</x:v>
+        <x:v>Monday</x:v>
       </x:c>
       <x:c r="B13" s="59" t="str">
-        <x:v>Back + Biceps - completed 2026-08-24</x:v>
+        <x:v>Chest + Triceps - completed 2026-08-31</x:v>
       </x:c>
       <x:c r="C13" s="59" t="n"/>
       <x:c r="D13" s="94" t="inlineStr">
@@ -4306,10 +4306,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="92" t="str">
-        <x:v>Day 2</x:v>
+        <x:v>Tuesday</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
-        <x:v>Chest + Triceps - completed 2026-08-25</x:v>
+        <x:v>Back + Biceps - next after readiness</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4324,10 +4324,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="92" t="str">
-        <x:v>Day 3</x:v>
+        <x:v>Wednesday</x:v>
       </x:c>
       <x:c r="B15" s="59" t="str">
-        <x:v>Shoulders + Biceps - completed 2026-08-26</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4346,10 +4346,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="92" t="str">
-        <x:v>Day 4</x:v>
+        <x:v>Thursday</x:v>
       </x:c>
       <x:c r="B16" s="59" t="str">
-        <x:v>Legs - completed 2026-08-27</x:v>
+        <x:v>Legs + Calves</x:v>
       </x:c>
       <x:c r="C16" s="59" t="n"/>
       <x:c r="D16" s="94" t="inlineStr">
@@ -4388,29 +4388,29 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="92" t="str">
-        <x:v>Next</x:v>
+        <x:v>Friday</x:v>
       </x:c>
       <x:c r="B17" s="59" t="str">
-        <x:v>Recovery / rest; easy walking only if desired</x:v>
+        <x:v>Chest + Shoulders</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E17" s="59" t="str">
-        <x:v>Hack Squat</x:v>
+        <x:v>Flat Bench Press</x:v>
       </x:c>
       <x:c r="F17" s="59" t="str">
-        <x:v>65 kg/side x 9 @ RIR 2</x:v>
+        <x:v>22.5 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="G17" s="59" t="str">
-        <x:v>65 kg/side x 10 @ RIR 2</x:v>
+        <x:v>22.5 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H17" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I17" s="59" t="str">
-        <x:v>Add rep before load</x:v>
+        <x:v>Add rep; bar excluded</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
@@ -4418,29 +4418,29 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="92" t="str">
-        <x:v>Reason</x:v>
+        <x:v>Saturday</x:v>
       </x:c>
       <x:c r="B18" s="59" t="str">
-        <x:v>Four consecutive sessions ended with Low energy</x:v>
+        <x:v>Back + Biceps; Sunday rest</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E18" s="59" t="str">
-        <x:v>Leg Press</x:v>
+        <x:v>Incline Barbell Bench</x:v>
       </x:c>
       <x:c r="F18" s="59" t="str">
-        <x:v>160 kg x 5 clean + 2 assisted</x:v>
+        <x:v>17.5 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="G18" s="59" t="str">
-        <x:v>140 kg x 10 @ RIR 2</x:v>
+        <x:v>17.5 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H18" s="59" t="str">
-        <x:v>Modify / Verify</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I18" s="59" t="str">
-        <x:v>No assisted 160; old load discrepancy To verify</x:v>
+        <x:v>New baseline; add rep</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
@@ -4451,22 +4451,22 @@
       <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Chest</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Dumbbell RDL</x:v>
+        <x:v>Pec Deck Fly</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>15 kg each x 10 @ RIR 2</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>15 kg each x 10-11 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>Technique improving</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>Hamstrings dominant; keep pain-free</x:v>
+        <x:v>Monitor upper-biceps response</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
@@ -4477,22 +4477,22 @@
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Leg Curl</x:v>
+        <x:v>Straight-Bar Pushdown</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>35 kg x 9 @ RIR 1</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>35 kg x 10 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>No failure</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4503,22 +4503,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Leg Extension</x:v>
+        <x:v>Overhead Rope Extension</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>50 kg x 11 @ RIR 2</x:v>
+        <x:v>45 kg x 8 @ RIR 1 extra</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>50 kg x 12 @ RIR 2</x:v>
+        <x:v>45 kg x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify volume</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Add one rep</x:v>
+        <x:v>Exactly 2 sets next time</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4529,22 +4529,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Legs</x:v>
+        <x:v>Triceps</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Standing Calf Raise</x:v>
+        <x:v>Assisted Dip</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>20 kg/side x 16 @ RIR 3</x:v>
+        <x:v>50 kg assist x 8 @ RIR 1</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>20 kg/side x 17 @ RIR 2</x:v>
+        <x:v>50 kg assist x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Return to 3 planned sets</x:v>
+        <x:v>Keep machine assistance</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4555,22 +4555,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Recovery</x:v>
+        <x:v>Cardio</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Final energy</x:v>
+        <x:v>Incline treadmill</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>Low after 4 consecutive sessions</x:v>
+        <x:v>15 min; 12%; 3-4 mph reported</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Rest / easy walking</x:v>
+        <x:v>Repeat only if energy Medium+</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Recovery due</x:v>
+        <x:v>Hold</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>No compensatory cardio</x:v>
+        <x:v>Exact speed/calibration To verify</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4581,22 +4581,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Program</x:v>
+        <x:v>Recovery</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Working-set ceiling</x:v>
+        <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>18 sets achieved</x:v>
+        <x:v>Low after 100 min</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>Maintain 18</x:v>
+        <x:v>Back+Biceps after fresh readiness</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>On target</x:v>
+        <x:v>Monitor</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Pre-plan 3 leg-press sets</x:v>
+        <x:v>No added volume</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4625,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b3f221b10c64188"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039a955038124c4c"/>
 </x:worksheet>
 </file>
 
@@ -23243,6 +23243,798 @@
       </x:c>
       <x:c r="N447" s="170" t="n">
         <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="448">
+      <x:c r="A448" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B448" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C448" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D448" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E448" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F448" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G448" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H448" s="170" t="str">
+        <x:v>Genuine preparation set; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I448" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J448" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K448" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L448" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M448" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N448" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="449">
+      <x:c r="A449" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B449" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C449" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D449" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E449" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F449" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G449" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H449" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I449" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J449" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K449" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L449" s="170" t="str">
+        <x:v>Target met with better reserve</x:v>
+      </x:c>
+      <x:c r="M449" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N449" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="450">
+      <x:c r="A450" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B450" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C450" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D450" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E450" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F450" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G450" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H450" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I450" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J450" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K450" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L450" s="170" t="str">
+        <x:v>Reserve exceeded target</x:v>
+      </x:c>
+      <x:c r="M450" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N450" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="451">
+      <x:c r="A451" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B451" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C451" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D451" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E451" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F451" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G451" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H451" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I451" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J451" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K451" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L451" s="170" t="str">
+        <x:v>Previous RIR-0 exposure corrected; progression-quality set</x:v>
+      </x:c>
+      <x:c r="M451" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N451" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="452">
+      <x:c r="A452" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B452" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C452" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D452" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E452" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F452" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G452" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H452" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I452" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J452" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K452" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L452" s="170" t="str">
+        <x:v>10 kg preparation/working target was skipped; completed load retained</x:v>
+      </x:c>
+      <x:c r="M452" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N452" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="453">
+      <x:c r="A453" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B453" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C453" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D453" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E453" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F453" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G453" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H453" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I453" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J453" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K453" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L453" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M453" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N453" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="454">
+      <x:c r="A454" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B454" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C454" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D454" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E454" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F454" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G454" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H454" s="170" t="str">
+        <x:v>Clean and unassisted; detailed bar path To verify</x:v>
+      </x:c>
+      <x:c r="I454" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J454" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K454" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L454" s="170" t="str">
+        <x:v>New higher-load baseline at target reserve; no immediate load increase</x:v>
+      </x:c>
+      <x:c r="M454" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N454" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="455">
+      <x:c r="A455" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B455" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C455" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D455" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E455" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F455" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G455" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H455" s="170" t="str">
+        <x:v>Clean and unassisted; relaxed-grip detail To verify; no upper-biceps pain</x:v>
+      </x:c>
+      <x:c r="I455" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J455" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K455" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L455" s="170" t="str">
+        <x:v>Reserve improved</x:v>
+      </x:c>
+      <x:c r="M455" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N455" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="456">
+      <x:c r="A456" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B456" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C456" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D456" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E456" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F456" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G456" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H456" s="170" t="str">
+        <x:v>Clean and unassisted; relaxed-grip detail To verify; no upper-biceps pain</x:v>
+      </x:c>
+      <x:c r="I456" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J456" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K456" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L456" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M456" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N456" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="457">
+      <x:c r="A457" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B457" s="170" t="str">
+        <x:v>Chest</x:v>
+      </x:c>
+      <x:c r="C457" s="170" t="str">
+        <x:v>Pec Deck Fly</x:v>
+      </x:c>
+      <x:c r="D457" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E457" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F457" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G457" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H457" s="170" t="str">
+        <x:v>Clean and unassisted; relaxed-grip detail To verify; no upper-biceps pain</x:v>
+      </x:c>
+      <x:c r="I457" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J457" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K457" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L457" s="170" t="str">
+        <x:v>Reserve improved from prior RIR 1; add rep before load</x:v>
+      </x:c>
+      <x:c r="M457" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N457" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="458">
+      <x:c r="A458" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B458" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C458" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D458" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E458" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F458" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G458" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H458" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I458" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J458" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K458" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L458" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M458" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N458" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="459">
+      <x:c r="A459" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B459" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C459" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D459" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E459" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F459" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G459" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H459" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I459" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J459" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K459" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L459" s="170" t="str">
+        <x:v>Reserve improved</x:v>
+      </x:c>
+      <x:c r="M459" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N459" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="460">
+      <x:c r="A460" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B460" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C460" s="170" t="str">
+        <x:v>Straight-Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D460" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E460" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F460" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G460" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H460" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I460" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J460" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K460" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L460" s="170" t="str">
+        <x:v>Previous RIR-1 result corrected; add rep before load</x:v>
+      </x:c>
+      <x:c r="M460" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N460" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="461">
+      <x:c r="A461" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B461" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C461" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D461" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E461" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F461" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G461" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H461" s="170" t="str">
+        <x:v>Clean and unassisted; elbow/rib position To verify</x:v>
+      </x:c>
+      <x:c r="I461" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J461" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K461" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L461" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M461" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N461" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="462">
+      <x:c r="A462" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B462" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C462" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D462" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E462" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F462" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G462" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H462" s="170" t="str">
+        <x:v>Clean and unassisted; elbow/rib position To verify</x:v>
+      </x:c>
+      <x:c r="I462" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J462" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K462" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L462" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M462" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N462" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="463">
+      <x:c r="A463" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B463" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C463" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D463" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E463" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F463" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G463" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H463" s="170" t="str">
+        <x:v>Clean and unassisted; elbow/rib position To verify</x:v>
+      </x:c>
+      <x:c r="I463" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J463" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K463" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L463" s="170" t="str">
+        <x:v>Unplanned third set beyond two-set prescription; retained without progression credit</x:v>
+      </x:c>
+      <x:c r="M463" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N463" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="464">
+      <x:c r="A464" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B464" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C464" s="170" t="str">
+        <x:v>Assisted Dip</x:v>
+      </x:c>
+      <x:c r="D464" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E464" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F464" s="170" t="str">
+        <x:v>kg machine assistance/support; effective resistance and machine model To verify</x:v>
+      </x:c>
+      <x:c r="G464" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H464" s="170" t="str">
+        <x:v>Machine-assisted only; no human assistance; controlled depth To verify</x:v>
+      </x:c>
+      <x:c r="I464" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J464" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K464" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L464" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M464" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N464" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="465">
+      <x:c r="A465" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B465" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C465" s="170" t="str">
+        <x:v>Assisted Dip</x:v>
+      </x:c>
+      <x:c r="D465" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E465" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F465" s="170" t="str">
+        <x:v>kg machine assistance/support; effective resistance and machine model To verify</x:v>
+      </x:c>
+      <x:c r="G465" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H465" s="170" t="str">
+        <x:v>Machine-assisted only; no human assistance; controlled depth To verify</x:v>
+      </x:c>
+      <x:c r="I465" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J465" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K465" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L465" s="170" t="str">
+        <x:v>Harder than target; keep assistance level and improve reserve</x:v>
+      </x:c>
+      <x:c r="M465" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N465" s="170" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23277,7 +24069,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c2e4f45a34f4d08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb41ab8d121874774"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23505,25 +24297,25 @@
         <x:v>Flat Bench Press</x:v>
       </x:c>
       <x:c r="C9" s="222" t="str">
-        <x:v>22.5 kg/side x 8 @ RIR 0</x:v>
+        <x:v>22.5 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="D9" s="222" t="str">
         <x:v>17.5-22.5 kg/side</x:v>
       </x:c>
       <x:c r="E9" s="222" t="str">
-        <x:v>22.5 kg/side x 8 @ RIR 1-2</x:v>
+        <x:v>22.5 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F9" s="222" t="str">
-        <x:v>No failure; improve reserve</x:v>
+        <x:v>Add one clean rep before load</x:v>
       </x:c>
       <x:c r="G9" s="222" t="str">
-        <x:v>Shoulder blades set; genuine prep near RIR 5</x:v>
+        <x:v>Shoulder blades set; genuine preparation near RIR 5</x:v>
       </x:c>
       <x:c r="H9" s="222" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I9" s="222" t="str">
-        <x:v>15 kg x 15 counted as fatigue; top set reached RIR 0; bar excluded</x:v>
+        <x:v>15 kg x 8 was warm-up; all working sets unassisted; bar excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="40" hidden="0" customHeight="1">
@@ -23621,25 +24413,25 @@
         <x:v>Pec Deck Fly</x:v>
       </x:c>
       <x:c r="C13" s="222" t="str">
-        <x:v>60 kg x 11 @ RIR 1 unplanned</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D13" s="222" t="str">
-        <x:v>45-55 kg</x:v>
+        <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E13" s="222" t="str">
-        <x:v>55 kg x 12 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F13" s="222" t="str">
-        <x:v>Omit 60 kg; monitor biceps pump</x:v>
+        <x:v>Add rep; monitor upper-biceps response</x:v>
       </x:c>
       <x:c r="G13" s="222" t="str">
         <x:v>Relax grip; fixed soft elbow; drive elbows</x:v>
       </x:c>
       <x:c r="H13" s="222" t="str">
-        <x:v>Modify technique/volume</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I13" s="222" t="str">
-        <x:v>Strong non-painful upper-biceps pump likely related; exact side To verify</x:v>
+        <x:v>No pain or upper-biceps issue reported today</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -24195,25 +24987,25 @@
         <x:v>Straight-Bar Pushdown</x:v>
       </x:c>
       <x:c r="C33" s="170" t="str">
-        <x:v>60 kg x 9 @ RIR 1</x:v>
+        <x:v>60 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D33" s="170" t="str">
         <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E33" s="170" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F33" s="170" t="str">
-        <x:v>Exactly 3 working sets; improve reserve</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="G33" s="170" t="str">
         <x:v>Elbows fixed; torso still</x:v>
       </x:c>
       <x:c r="H33" s="170" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I33" s="170" t="str">
-        <x:v>45 kg x 12 @ RIR 4 was preparation; working sets were harder than targets</x:v>
+        <x:v>All three sets stayed at RIR 2</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="48" hidden="0" customHeight="1">
@@ -24253,25 +25045,25 @@
         <x:v>Overhead Rope Extension</x:v>
       </x:c>
       <x:c r="C35" s="170" t="str">
-        <x:v>45 kg x 7 @ RIR 1 unplanned</x:v>
+        <x:v>45 kg x 8 @ RIR 1 unplanned</x:v>
       </x:c>
       <x:c r="D35" s="170" t="str">
-        <x:v>30-40 kg</x:v>
+        <x:v>35-45 kg</x:v>
       </x:c>
       <x:c r="E35" s="170" t="str">
-        <x:v>40 kg x 9-10 @ RIR 2</x:v>
+        <x:v>45 kg x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="F35" s="170" t="str">
-        <x:v>Exactly 3 sets; no 45 kg</x:v>
+        <x:v>Exactly 2 sets; no additional third set</x:v>
       </x:c>
       <x:c r="G35" s="170" t="str">
         <x:v>Ribs down; elbows stable</x:v>
       </x:c>
       <x:c r="H35" s="170" t="str">
-        <x:v>Modify load/volume</x:v>
+        <x:v>Modify volume/effort</x:v>
       </x:c>
       <x:c r="I35" s="170" t="str">
-        <x:v>Third set exceeded live two-set limit and receives no progression credit</x:v>
+        <x:v>35 and 40 kg met targets; 45 kg was an extra third set and earns no progression credit</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="48" hidden="0" customHeight="1">
@@ -24427,25 +25219,25 @@
         <x:v>Incline Barbell Bench Press</x:v>
       </x:c>
       <x:c r="C41" s="170" t="str">
-        <x:v>15 kg/side x 10 @ RIR 2</x:v>
+        <x:v>17.5 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="D41" s="170" t="str">
-        <x:v>10-15 kg/side</x:v>
+        <x:v>12.5-17.5 kg/side</x:v>
       </x:c>
       <x:c r="E41" s="170" t="str">
-        <x:v>15 kg/side x 10 @ RIR 2</x:v>
+        <x:v>17.5 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F41" s="170" t="str">
-        <x:v>Keep reps; improve first-set reserve</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="G41" s="170" t="str">
-        <x:v>Controlled bar path</x:v>
+        <x:v>Controlled bar path; no assisted finish</x:v>
       </x:c>
       <x:c r="H41" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I41" s="170" t="str">
-        <x:v>All three loads progressed; bar excluded</x:v>
+        <x:v>New clean higher-load baseline; bar excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
@@ -24734,7 +25526,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a5ae830445f4f0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0278436f96f48ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25697,17 +26489,29 @@
       <x:c r="P28" s="59" t="n"/>
       <x:c r="Q28" s="59" t="n"/>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="220"/>
+    <x:row r="29" ht="76" customHeight="1">
+      <x:c r="A29" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
       <x:c r="B29" s="170"/>
       <x:c r="C29" s="170"/>
-      <x:c r="D29" s="170"/>
-      <x:c r="E29" s="170"/>
-      <x:c r="F29" s="170"/>
+      <x:c r="D29" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E29" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F29" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no pre-session soreness</x:v>
+      </x:c>
       <x:c r="G29" s="170"/>
       <x:c r="H29" s="170"/>
-      <x:c r="I29" s="170"/>
-      <x:c r="J29" s="170"/>
+      <x:c r="I29" s="170" t="str">
+        <x:v>Chest + Triceps workout - 100 min total; 17 working sets plus one warm-up; 15 min treadmill at 12% incline; speed reported as 3-4 mph range</x:v>
+      </x:c>
+      <x:c r="J29" s="170" t="str">
+        <x:v>Started Medium; medium chest/triceps pump; full EAA+ scoop (100 mg caffeine); no coffee; creatine not started; no human assistance or form breakdown; no pain during cardio</x:v>
+      </x:c>
       <x:c r="K29" s="59" t="n"/>
       <x:c r="L29" s="59" t="n"/>
       <x:c r="M29" s="59" t="n"/>
@@ -29021,7 +29825,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48a6d2b6c1e04587"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re16d392bc2954322"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30204,13 +31008,83 @@
         <x:v>Next Legs pre-plan three leg-press and three calf sets</x:v>
       </x:c>
     </x:row>
+    <x:row r="80" ht="56" customHeight="1">
+      <x:c r="A80" s="170" t="str">
+        <x:v>Six-day two-body-part split adopted</x:v>
+      </x:c>
+      <x:c r="B80" s="170" t="str">
+        <x:v>Active sequence from 2026-08-31: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest</x:v>
+      </x:c>
+      <x:c r="C80" s="170" t="str">
+        <x:v>Upper body and arms receive two weekly exposures; Legs remains one dedicated high-quality day by user preference</x:v>
+      </x:c>
+      <x:c r="D80" s="170" t="str">
+        <x:v>Run the block for four weeks; keep daily resistance volume at or below 18 working sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="56" customHeight="1">
+      <x:c r="A81" s="170" t="str">
+        <x:v>Chest + Triceps performance</x:v>
+      </x:c>
+      <x:c r="B81" s="170" t="str">
+        <x:v>2026-08-31 completed 17 working sets plus one warm-up with no pain, RIR 0, human assistance or form breakdown</x:v>
+      </x:c>
+      <x:c r="C81" s="170" t="str">
+        <x:v>Flat, incline, pec deck and pushdown reserve improved after the travel break</x:v>
+      </x:c>
+      <x:c r="D81" s="170" t="str">
+        <x:v>Keep progression rep-led and preserve RIR 2 before adding load</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="56" customHeight="1">
+      <x:c r="A82" s="170" t="str">
+        <x:v>Overhead-rope volume deviation</x:v>
+      </x:c>
+      <x:c r="B82" s="170" t="str">
+        <x:v>35 x13 @2, 40 x10 @2 and an extra 45 x8 @1 were completed although only two sets were prescribed</x:v>
+      </x:c>
+      <x:c r="C82" s="170" t="str">
+        <x:v>The third set remains historical work but does not earn progression credit; final energy was Low</x:v>
+      </x:c>
+      <x:c r="D82" s="170" t="str">
+        <x:v>Next Monday use exactly two overhead-rope sets and stop at the revised count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="56" customHeight="1">
+      <x:c r="A83" s="170" t="str">
+        <x:v>Fat-loss cardio baseline</x:v>
+      </x:c>
+      <x:c r="B83" s="170" t="str">
+        <x:v>15 min treadmill at 12% incline; speed reported as 3-4 mph range; no pain; final energy Low</x:v>
+      </x:c>
+      <x:c r="C83" s="170" t="str">
+        <x:v>Useful conditioning dose, but both exact speed and treadmill calibration remain To verify</x:v>
+      </x:c>
+      <x:c r="D83" s="170" t="str">
+        <x:v>Do not increase incline, speed or duration next time; perform post-lift cardio only when final energy is Medium or higher</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="56" customHeight="1">
+      <x:c r="A84" s="170" t="str">
+        <x:v>Creatine status</x:v>
+      </x:c>
+      <x:c r="B84" s="170" t="str">
+        <x:v>Creatine monohydrate had not started as of 2026-08-31</x:v>
+      </x:c>
+      <x:c r="C84" s="170" t="str">
+        <x:v>Current performance and body-weight trends are pre-creatine baselines</x:v>
+      </x:c>
+      <x:c r="D84" s="170" t="str">
+        <x:v>Verify product label and actual start date before attributing any scale change to creatine</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R647f86a178db48fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9180e94968c24a63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30905,6 +31779,32 @@
         <x:v>Recovery/rest next; next Legs use three unassisted leg-press sets, keep RDL pain-free and hamstring-led, improve leg-curl reserve, and retain exactly 18 working sets</x:v>
       </x:c>
     </x:row>
+    <x:row r="27" ht="84" customHeight="1">
+      <x:c r="A27" s="220" t="n">
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="B27" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C27" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D27" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E27" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F27" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; no soreness or pain; 100 min total including cardio; medium chest/triceps pump; no human-assisted repetitions or form breakdown; full EAA+ (100 mg caffeine); no coffee; creatine not started; 15 min treadmill at 12% incline and reported 3-4 mph walking-speed range</x:v>
+      </x:c>
+      <x:c r="G27" s="170" t="str">
+        <x:v>Seventeen working sets plus one genuine warm-up were completed with no pain, RIR 0 or human assistance. Flat-bench reserve improved, incline established a clean 17.5 kg/side baseline, pec deck and pushdown reserve improved. The extra 45 kg overhead-rope set exceeded the two-set prescription, and Low final energy means no additional volume or cardio progression is warranted.</x:v>
+      </x:c>
+      <x:c r="H27" s="170" t="str">
+        <x:v>Back + Biceps next after fresh readiness; use the new six-day split, cap the session at 16 working sets, keep most sets at RIR 2, and add cardio only if final energy remains Medium or higher</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -30917,7 +31817,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1106a282119498d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc0c56f9923b455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31094,13 +31994,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Legs on 2026-08-27: no lower-back, knee or hip pain. RDL was hamstring-dominant with a little non-painful back involvement.</x:v>
+        <x:v>After Chest + Triceps on 2026-08-31: no chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no soreness; no form breakdown.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Recheck delayed leg/back soreness and energy before the next resistance session</x:v>
+        <x:v>Fresh readiness before Back + Biceps; monitor delayed chest/triceps soreness</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -31282,13 +32182,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Temporary four-day week completed: Back + Biceps 2026-08-24; Chest + Triceps 2026-08-25; Shoulders + Biceps 2026-08-26; Legs 2026-08-27.</x:v>
+        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday 2026-08-31 completed.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
-        <x:v>Known for current week</x:v>
+        <x:v>Known / active four-week block</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Recovery/rest next because four consecutive sessions ended with Low final energy</x:v>
+        <x:v>Back + Biceps next after fresh readiness; preserve 18-set ceiling</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -31487,7 +32387,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112ee6676fca4956"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b5e7491bc1e46d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32590,10 +33490,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc773ad4a4db4f2d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49f69ce31d5e4032"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d671af1ec63410e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R522fc9d783fe42ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae9ba9403113484e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ff3d66e2144709"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9725356124e64fa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3c0c252621490d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 1 back and biceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R772ffc799e594d4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rdcfdc6d3278140c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rd1c9bec3c528494e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Re4c8ede6b98a4937"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Ra4fd2bca4ab8432d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Rf7a8e964afb74128"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R73eea8372fea4531"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Rf38bd190b0d04804"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R266fddb1b0d34285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R84a32a4d22e245ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R6c61d431267349b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8bd364b21e78471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4c8a4cfd7af74b22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rc2ac4b7f3da84250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rde3fcb8c1e2049cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R8aa3b002dc824094"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R397b38f24e9643fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R9523795e73cc42a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R4ba25784ec9d4e6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Ra4603ec508bf4a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc1df7d6821f54f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R9f5705a2155e4f22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re74ee2b478ac461b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4efbcfc0aca94cbb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N465" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N484" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1803,7 +1803,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1bbef083e0394d39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R191e0927119d4b96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab955d759f8343df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464b0fbb013247cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,11 +4083,11 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="str">
@@ -4309,7 +4309,7 @@
         <x:v>Tuesday</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
-        <x:v>Back + Biceps - next after readiness</x:v>
+        <x:v>Back + Biceps - completed 2026-09-01</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4327,7 +4327,7 @@
         <x:v>Wednesday</x:v>
       </x:c>
       <x:c r="B15" s="59" t="str">
-        <x:v>Shoulders + Triceps</x:v>
+        <x:v>Shoulders + Triceps - next after readiness</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4395,22 +4395,22 @@
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Back</x:v>
       </x:c>
       <x:c r="E17" s="59" t="str">
-        <x:v>Flat Bench Press</x:v>
+        <x:v>Lat Pulldown</x:v>
       </x:c>
       <x:c r="F17" s="59" t="str">
-        <x:v>22.5 kg/side x 8 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G17" s="59" t="str">
-        <x:v>22.5 kg/side x 9 @ RIR 2</x:v>
+        <x:v>Hold; improve 55 kg reps</x:v>
       </x:c>
       <x:c r="H17" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I17" s="59" t="str">
-        <x:v>Add rep; bar excluded</x:v>
+        <x:v>True preparation achieved</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
@@ -4425,22 +4425,22 @@
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Back</x:v>
       </x:c>
       <x:c r="E18" s="59" t="str">
-        <x:v>Incline Barbell Bench</x:v>
+        <x:v>Seated Cable Row</x:v>
       </x:c>
       <x:c r="F18" s="59" t="str">
-        <x:v>17.5 kg/side x 8 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="G18" s="59" t="str">
-        <x:v>17.5 kg/side x 9 @ RIR 2</x:v>
+        <x:v>60 kg x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="H18" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I18" s="59" t="str">
-        <x:v>New baseline; add rep</x:v>
+        <x:v>Reserve improved</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
@@ -4451,22 +4451,22 @@
       <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="str">
-        <x:v>Chest</x:v>
+        <x:v>Back</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Pec Deck Fly</x:v>
+        <x:v>Chest-Supported T-Bar</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>40 kg x 10 @ RIR 1</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>60 kg x 10 @ RIR 2</x:v>
+        <x:v>40 kg x 8-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>New / verify</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>Monitor upper-biceps response</x:v>
+        <x:v>Load basis To verify</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
@@ -4477,22 +4477,22 @@
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Back</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Straight-Bar Pushdown</x:v>
+        <x:v>Chest-Supported Row</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>55 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>60 kg x 10 @ RIR 2</x:v>
+        <x:v>55 kg x 12-13 @ RIR 2</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify selection</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>Add rep before load</x:v>
+        <x:v>Use one row variation</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4503,22 +4503,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Overhead Rope Extension</x:v>
+        <x:v>Incline DB Curl</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>45 kg x 8 @ RIR 1 extra</x:v>
+        <x:v>15 kg x 8 @ RIR 1</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>45 kg x 8 @ RIR 2</x:v>
+        <x:v>15 kg x 8-9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
-        <x:v>Modify volume</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>Exactly 2 sets next time</x:v>
+        <x:v>No load increase</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4529,22 +4529,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Triceps</x:v>
+        <x:v>Biceps</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Assisted Dip</x:v>
+        <x:v>Hammer Curl</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>50 kg assist x 8 @ RIR 1</x:v>
+        <x:v>17.5 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>50 kg assist x 8 @ RIR 2</x:v>
+        <x:v>17.5 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Keep machine assistance</x:v>
+        <x:v>Exactly two sets</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4561,16 +4561,16 @@
         <x:v>Incline treadmill</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>15 min; 12%; 3-4 mph reported</x:v>
+        <x:v>20 min; 3 km/h; 12%</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Repeat only if energy Medium+</x:v>
+        <x:v>20 min; 3 km/h; 8-10%</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Hold</x:v>
+        <x:v>Progress / moderate</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Exact speed/calibration To verify</x:v>
+        <x:v>200 kcal display To verify</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4587,10 +4587,10 @@
         <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>Low after 100 min</x:v>
+        <x:v>Low after 90 min</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>Back+Biceps after fresh readiness</x:v>
+        <x:v>Shoulders+Triceps after readiness</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
         <x:v>Monitor</x:v>
@@ -4625,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039a955038124c4c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b153402bfb342c1"/>
 </x:worksheet>
 </file>
 
@@ -24035,6 +24035,842 @@
       </x:c>
       <x:c r="N465" s="170" t="n">
         <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="466">
+      <x:c r="A466" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B466" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C466" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D466" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E466" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F466" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G466" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H466" s="170" t="str">
+        <x:v>Genuine low-fatigue preparation; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I466" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J466" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K466" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L466" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M466" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N466" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="467">
+      <x:c r="A467" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B467" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C467" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D467" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E467" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F467" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G467" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H467" s="170" t="str">
+        <x:v>Clean and unassisted; elbow path and torso angle To verify</x:v>
+      </x:c>
+      <x:c r="I467" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J467" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K467" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L467" s="170" t="str">
+        <x:v>One reserve harder than target; keep load</x:v>
+      </x:c>
+      <x:c r="M467" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N467" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="468">
+      <x:c r="A468" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B468" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C468" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D468" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E468" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F468" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G468" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H468" s="170" t="str">
+        <x:v>Clean and unassisted; elbow path and torso angle To verify</x:v>
+      </x:c>
+      <x:c r="I468" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J468" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K468" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L468" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M468" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N468" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="469">
+      <x:c r="A469" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B469" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C469" s="170" t="str">
+        <x:v>Lat Pulldown</x:v>
+      </x:c>
+      <x:c r="D469" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E469" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F469" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G469" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H469" s="170" t="str">
+        <x:v>Clean and unassisted; elbow path and torso angle To verify</x:v>
+      </x:c>
+      <x:c r="I469" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J469" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K469" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L469" s="170" t="str">
+        <x:v>Rep progression at retained reserve</x:v>
+      </x:c>
+      <x:c r="M469" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N469" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="470">
+      <x:c r="A470" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B470" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C470" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D470" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E470" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F470" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G470" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H470" s="170" t="str">
+        <x:v>Genuine low-fatigue preparation; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I470" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J470" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K470" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L470" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M470" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N470" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="471">
+      <x:c r="A471" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B471" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C471" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D471" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E471" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F471" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G471" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H471" s="170" t="str">
+        <x:v>Clean and unassisted; torso stability To verify</x:v>
+      </x:c>
+      <x:c r="I471" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J471" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K471" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L471" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M471" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N471" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="472">
+      <x:c r="A472" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B472" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C472" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D472" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E472" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F472" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G472" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H472" s="170" t="str">
+        <x:v>Clean and unassisted; torso stability To verify</x:v>
+      </x:c>
+      <x:c r="I472" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J472" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K472" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L472" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M472" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N472" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="473">
+      <x:c r="A473" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B473" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C473" s="170" t="str">
+        <x:v>Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D473" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E473" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F473" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G473" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H473" s="170" t="str">
+        <x:v>Clean and unassisted; torso stability To verify</x:v>
+      </x:c>
+      <x:c r="I473" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J473" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K473" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L473" s="170" t="str">
+        <x:v>Previous RIR-1 result corrected</x:v>
+      </x:c>
+      <x:c r="M473" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N473" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="474">
+      <x:c r="A474" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B474" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C474" s="170" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="D474" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E474" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F474" s="170" t="str">
+        <x:v>kg reported machine load; total plates/displayed resistance and starting resistance To verify</x:v>
+      </x:c>
+      <x:c r="G474" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H474" s="170" t="str">
+        <x:v>Chest supported; no reported breakdown; detailed grip/path To verify</x:v>
+      </x:c>
+      <x:c r="I474" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J474" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K474" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L474" s="170" t="str">
+        <x:v>New-machine baseline; load not comparable with established row machine</x:v>
+      </x:c>
+      <x:c r="M474" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N474" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="475">
+      <x:c r="A475" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B475" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C475" s="170" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="D475" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E475" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F475" s="170" t="str">
+        <x:v>kg reported machine load; total plates/displayed resistance and starting resistance To verify</x:v>
+      </x:c>
+      <x:c r="G475" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H475" s="170" t="str">
+        <x:v>Chest supported; no reported breakdown; detailed grip/path To verify</x:v>
+      </x:c>
+      <x:c r="I475" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J475" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K475" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L475" s="170" t="str">
+        <x:v>Too close to failure; reduce intermediate load next time</x:v>
+      </x:c>
+      <x:c r="M475" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N475" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="476">
+      <x:c r="A476" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B476" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C476" s="170" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="D476" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E476" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F476" s="170" t="str">
+        <x:v>kg reported machine load; total plates/displayed resistance and starting resistance To verify</x:v>
+      </x:c>
+      <x:c r="G476" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H476" s="170" t="str">
+        <x:v>Chest supported; no reported breakdown; detailed grip/path To verify</x:v>
+      </x:c>
+      <x:c r="I476" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J476" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K476" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L476" s="170" t="str">
+        <x:v>Repeated RIR-1 exposure; no load progression</x:v>
+      </x:c>
+      <x:c r="M476" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N476" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="477">
+      <x:c r="A477" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B477" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C477" s="170" t="str">
+        <x:v>Chest-Supported Row Machine</x:v>
+      </x:c>
+      <x:c r="D477" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E477" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F477" s="170" t="str">
+        <x:v>kg reported established-machine load; exact plate convention To verify</x:v>
+      </x:c>
+      <x:c r="G477" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H477" s="170" t="str">
+        <x:v>Genuine preparation set; chest supported; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I477" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J477" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K477" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L477" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M477" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N477" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="478">
+      <x:c r="A478" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B478" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C478" s="170" t="str">
+        <x:v>Chest-Supported Row Machine</x:v>
+      </x:c>
+      <x:c r="D478" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E478" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F478" s="170" t="str">
+        <x:v>kg reported established-machine load; exact plate convention To verify</x:v>
+      </x:c>
+      <x:c r="G478" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H478" s="170" t="str">
+        <x:v>Chest supported; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I478" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J478" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K478" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L478" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M478" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N478" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="479">
+      <x:c r="A479" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B479" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C479" s="170" t="str">
+        <x:v>Chest-Supported Row Machine</x:v>
+      </x:c>
+      <x:c r="D479" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E479" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F479" s="170" t="str">
+        <x:v>kg reported established-machine load; exact plate convention To verify</x:v>
+      </x:c>
+      <x:c r="G479" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H479" s="170" t="str">
+        <x:v>Chest supported; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I479" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J479" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K479" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L479" s="170" t="str">
+        <x:v>Performed instead of 50 kg; retain as baseline</x:v>
+      </x:c>
+      <x:c r="M479" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N479" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="480">
+      <x:c r="A480" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B480" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C480" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D480" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E480" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F480" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G480" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H480" s="170" t="str">
+        <x:v>Clean and unassisted; bench angle and bottom stretch To verify</x:v>
+      </x:c>
+      <x:c r="I480" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J480" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K480" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L480" s="170" t="str">
+        <x:v>7.5 kg target skipped</x:v>
+      </x:c>
+      <x:c r="M480" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N480" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="481">
+      <x:c r="A481" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B481" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C481" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D481" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E481" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F481" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G481" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H481" s="170" t="str">
+        <x:v>Clean and unassisted; bench angle and bottom stretch To verify</x:v>
+      </x:c>
+      <x:c r="I481" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J481" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K481" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L481" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M481" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N481" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="482">
+      <x:c r="A482" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B482" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C482" s="170" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D482" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E482" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F482" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G482" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H482" s="170" t="str">
+        <x:v>Clean and unassisted; bench angle and bottom stretch To verify</x:v>
+      </x:c>
+      <x:c r="I482" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J482" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K482" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L482" s="170" t="str">
+        <x:v>New heavier baseline; improve reserve before progression</x:v>
+      </x:c>
+      <x:c r="M482" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N482" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="483">
+      <x:c r="A483" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B483" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C483" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D483" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E483" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F483" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G483" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H483" s="170" t="str">
+        <x:v>Clean and unassisted; neutral wrist To verify</x:v>
+      </x:c>
+      <x:c r="I483" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J483" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K483" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L483" s="170" t="str">
+        <x:v>Below rep target; keep load</x:v>
+      </x:c>
+      <x:c r="M483" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N483" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="484">
+      <x:c r="A484" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B484" s="170" t="str">
+        <x:v>Biceps</x:v>
+      </x:c>
+      <x:c r="C484" s="170" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D484" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E484" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F484" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G484" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H484" s="170" t="str">
+        <x:v>Clean and unassisted; neutral wrist To verify</x:v>
+      </x:c>
+      <x:c r="I484" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
+      <x:c r="J484" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K484" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L484" s="170" t="str">
+        <x:v>One rep below target; keep load</x:v>
+      </x:c>
+      <x:c r="M484" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N484" s="170" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -24069,7 +24905,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb41ab8d121874774"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d19a29add74d16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24181,16 +25017,16 @@
         <x:v>Lat Pulldown</x:v>
       </x:c>
       <x:c r="C5" s="222" t="str">
-        <x:v>60 kg x 9 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D5" s="222" t="str">
         <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E5" s="222" t="str">
-        <x:v>60 kg x 9-10 @ RIR 2</x:v>
+        <x:v>60 kg x 10 @ RIR 2; 55 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F5" s="222" t="str">
-        <x:v>Improve reserve before load</x:v>
+        <x:v>Improve 50 kg reserve and 55 kg reps before load</x:v>
       </x:c>
       <x:c r="G5" s="222" t="str">
         <x:v>Elbows down; no swinging</x:v>
@@ -24199,7 +25035,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I5" s="222" t="str">
-        <x:v>45 kg preparation reached RIR 3; 50-60 kg progressed</x:v>
+        <x:v>45 kg x12 was true preparation; 60 kg gained a rep at RIR 2</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -24210,25 +25046,25 @@
         <x:v>Seated Cable Row</x:v>
       </x:c>
       <x:c r="C6" s="222" t="str">
-        <x:v>60 kg x 10 @ RIR 1</x:v>
+        <x:v>60 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D6" s="222" t="str">
         <x:v>50-60 kg</x:v>
       </x:c>
       <x:c r="E6" s="222" t="str">
-        <x:v>60 kg x 10 @ RIR 2</x:v>
+        <x:v>60 kg x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="F6" s="222" t="str">
-        <x:v>Match reps with better reserve</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="G6" s="222" t="str">
         <x:v>Torso stable</x:v>
       </x:c>
       <x:c r="H6" s="222" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I6" s="222" t="str">
-        <x:v>55 kg reserve improved; top set too close to failure</x:v>
+        <x:v>All targets met; prior top-set RIR 1 improved to RIR 2</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -24239,25 +25075,25 @@
         <x:v>Chest-Supported Row</x:v>
       </x:c>
       <x:c r="C7" s="222" t="str">
-        <x:v>60 kg/side x 11 @ RIR 3</x:v>
+        <x:v>55 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D7" s="222" t="str">
-        <x:v>40-60 kg/side</x:v>
+        <x:v>40-55 kg on established machine</x:v>
       </x:c>
       <x:c r="E7" s="222" t="str">
-        <x:v>60 kg/side x 12 @ RIR 2-3</x:v>
+        <x:v>55 kg x 12-13 @ RIR 2</x:v>
       </x:c>
       <x:c r="F7" s="222" t="str">
-        <x:v>Add one clean rep</x:v>
+        <x:v>Use one row variation only</x:v>
       </x:c>
       <x:c r="G7" s="222" t="str">
         <x:v>Chest stays on pad</x:v>
       </x:c>
       <x:c r="H7" s="222" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify exercise selection</x:v>
       </x:c>
       <x:c r="I7" s="222" t="str">
-        <x:v>40 kg reps and reserve across top sets improved</x:v>
+        <x:v>30 kg prep @4; 40 x15 @3; 55 x12 @2; exact machine load convention To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -24268,7 +25104,7 @@
         <x:v>Straight-Arm Pulldown</x:v>
       </x:c>
       <x:c r="C8" s="222" t="str">
-        <x:v>50 kg x 12 @ RIR 2; extra 55 kg x 9 @ RIR 1</x:v>
+        <x:v>Not performed; replaced by second chest-supported row</x:v>
       </x:c>
       <x:c r="D8" s="222" t="str">
         <x:v>45-50 kg</x:v>
@@ -24277,16 +25113,16 @@
         <x:v>50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F8" s="222" t="str">
-        <x:v>Exactly 2 sets; no 55 kg</x:v>
+        <x:v>Exactly 2 sets when established row machine is used</x:v>
       </x:c>
       <x:c r="G8" s="222" t="str">
         <x:v>Elbows fixed</x:v>
       </x:c>
       <x:c r="H8" s="222" t="str">
-        <x:v>Modify volume</x:v>
+        <x:v>Resume next Back session</x:v>
       </x:c>
       <x:c r="I8" s="222" t="str">
-        <x:v>55 kg was unplanned fatigue and receives no progression credit</x:v>
+        <x:v>Omitted to preserve 16-set ceiling after duplicate row variations</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" hidden="0" customHeight="1">
@@ -24472,13 +25308,13 @@
         <x:v>17.5 kg each x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="D15" s="222" t="str">
-        <x:v>12.5-17.5 kg each</x:v>
+        <x:v>15-17.5 kg each</x:v>
       </x:c>
       <x:c r="E15" s="222" t="str">
         <x:v>17.5 kg each x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="F15" s="222" t="str">
-        <x:v>Add one rep; no extra sets</x:v>
+        <x:v>Add one clean rep</x:v>
       </x:c>
       <x:c r="G15" s="222" t="str">
         <x:v>Neutral wrists; no swing</x:v>
@@ -24487,7 +25323,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I15" s="222" t="str">
-        <x:v>All 3 sets controlled but last 2 exceeded live one-set limit</x:v>
+        <x:v>Exactly two sets; both pain-free and unassisted</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -25393,25 +26229,25 @@
         <x:v>Incline Dumbbell Curl</x:v>
       </x:c>
       <x:c r="C47" s="170" t="str">
-        <x:v>12.5 kg each x 9 @ RIR 1</x:v>
+        <x:v>15 kg each x 8 @ RIR 1</x:v>
       </x:c>
       <x:c r="D47" s="170" t="str">
-        <x:v>7.5-12.5 kg each</x:v>
+        <x:v>10-15 kg each</x:v>
       </x:c>
       <x:c r="E47" s="170" t="str">
-        <x:v>12.5 kg each x 9-10 @ RIR 2</x:v>
+        <x:v>15 kg each x 8-9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F47" s="170" t="str">
-        <x:v>Keep load; improve reserve</x:v>
+        <x:v>Improve reserve before reps/load</x:v>
       </x:c>
       <x:c r="G47" s="170" t="str">
-        <x:v>Bench 45-60 deg; no forced stretch</x:v>
+        <x:v>Bench 45-60 degrees; no forced bottom stretch</x:v>
       </x:c>
       <x:c r="H47" s="170" t="str">
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I47" s="170" t="str">
-        <x:v>Third set completed despite live reduction; detailed form To verify</x:v>
+        <x:v>7.5 kg skipped; 15 kg establishes heavier baseline</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="48" customHeight="1">
@@ -25499,6 +26335,35 @@
       </x:c>
       <x:c r="I50" s="170" t="str">
         <x:v>Elbows tended to bend; effective cable resistance To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>40 kg x 10 @ RIR 1</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>30-40 kg reported machine load; basis To verify</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>30 kg x 12-15 @ RIR 3; approximately 35 kg x 10-12 @ RIR 2; 40 kg x 8-10 @ RIR 2</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Use only when established row machine is unavailable</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>Chest fixed to pad; avoid torso lift</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>New baseline / To verify</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>Different machine; total plates/displayed load and starting resistance To verify; do not compare with established row machine</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -25526,7 +26391,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0278436f96f48ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4ce57c98ffb4593"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26520,17 +27385,29 @@
       <x:c r="P29" s="59" t="n"/>
       <x:c r="Q29" s="59" t="n"/>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="220"/>
+    <x:row r="30" ht="76" customHeight="1">
+      <x:c r="A30" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
       <x:c r="B30" s="170"/>
       <x:c r="C30" s="170"/>
-      <x:c r="D30" s="170"/>
-      <x:c r="E30" s="170"/>
-      <x:c r="F30" s="170"/>
+      <x:c r="D30" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E30" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F30" s="170" t="str">
+        <x:v>No back, lower-back, shoulder, elbow or biceps pain; no pre-session soreness; no pain or adverse symptoms during cardio</x:v>
+      </x:c>
       <x:c r="G30" s="170"/>
       <x:c r="H30" s="170"/>
-      <x:c r="I30" s="170"/>
-      <x:c r="J30" s="170"/>
+      <x:c r="I30" s="170" t="str">
+        <x:v>Back + Biceps workout - 90 min total; 16 working sets plus three preparation sets; medium pump; 20 min treadmill at 3 km/h and 12% incline</x:v>
+      </x:c>
+      <x:c r="J30" s="170" t="str">
+        <x:v>Started Medium; full EAA+ scoop (100 mg caffeine); no coffee; no assistance or reported form breakdown; treadmill showed '200k', provisionally interpreted as approximately 200 kcal machine estimate To verify; rail support and creatine status To verify</x:v>
+      </x:c>
       <x:c r="K30" s="59" t="n"/>
       <x:c r="L30" s="59" t="n"/>
       <x:c r="M30" s="59" t="n"/>
@@ -29825,7 +30702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re16d392bc2954322"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab3cc518f3549e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31078,13 +31955,69 @@
         <x:v>Verify product label and actual start date before attributing any scale change to creatine</x:v>
       </x:c>
     </x:row>
+    <x:row r="85" ht="60" customHeight="1">
+      <x:c r="A85" s="170" t="str">
+        <x:v>Back + Biceps performance</x:v>
+      </x:c>
+      <x:c r="B85" s="170" t="str">
+        <x:v>2026-09-01 completed exactly 16 working sets plus three genuine preparation sets; no pain, RIR 0, assistance or form breakdown</x:v>
+      </x:c>
+      <x:c r="C85" s="170" t="str">
+        <x:v>Lat pulldown and seated cable row progressed cleanly; final energy was Low</x:v>
+      </x:c>
+      <x:c r="D85" s="170" t="str">
+        <x:v>Keep progression rep-led and maintain routine RIR 2-3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="60" customHeight="1">
+      <x:c r="A86" s="170" t="str">
+        <x:v>Duplicate horizontal-row substitution</x:v>
+      </x:c>
+      <x:c r="B86" s="170" t="str">
+        <x:v>Both a new chest-supported T-bar machine and the established chest-supported-row machine were used; straight-arm pulldown was omitted</x:v>
+      </x:c>
+      <x:c r="C86" s="170" t="str">
+        <x:v>Working-set ceiling was preserved, but duplicate rowing displaced shoulder-extension work</x:v>
+      </x:c>
+      <x:c r="D86" s="170" t="str">
+        <x:v>Next Back day use only one chest-supported-row variation and restore straight-arm pulldown</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="60" customHeight="1">
+      <x:c r="A87" s="170" t="str">
+        <x:v>T-bar machine baseline</x:v>
+      </x:c>
+      <x:c r="B87" s="170" t="str">
+        <x:v>30 x12 @2, 40 x10 @1 and 40 x10 @1 on a different chest-supported T-bar machine</x:v>
+      </x:c>
+      <x:c r="C87" s="170" t="str">
+        <x:v>Load basis and machine starting resistance are To verify; two sets were too close to failure</x:v>
+      </x:c>
+      <x:c r="D87" s="170" t="str">
+        <x:v>Next use 30/approximately 35/40 kg at RIR 3/2/2 only if the established machine is unavailable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="60" customHeight="1">
+      <x:c r="A88" s="170" t="str">
+        <x:v>Fat-loss cardio progression</x:v>
+      </x:c>
+      <x:c r="B88" s="170" t="str">
+        <x:v>20 min treadmill at 3 km/h and 12% incline; no pain, dizziness or unusual breathlessness; machine display reported as '200k'</x:v>
+      </x:c>
+      <x:c r="C88" s="170" t="str">
+        <x:v>First full 20-min dose completed; approximately 200 kcal remains only a machine estimate To verify; final energy Low</x:v>
+      </x:c>
+      <x:c r="D88" s="170" t="str">
+        <x:v>Next comparable session use 20 min at 8-10% incline; do not eat back machine calories</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9180e94968c24a63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R093cb86e02404ff9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31805,6 +32738,32 @@
         <x:v>Back + Biceps next after fresh readiness; use the new six-day split, cap the session at 16 working sets, keep most sets at RIR 2, and add cardio only if final energy remains Medium or higher</x:v>
       </x:c>
     </x:row>
+    <x:row r="28" ht="84" customHeight="1">
+      <x:c r="A28" s="220" t="n">
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="B28" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C28" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D28" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E28" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F28" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; no soreness or pain; 90 min total including 20 min treadmill; medium back/biceps pump; no assisted repetitions or form breakdown; full EAA+ (100 mg caffeine); no coffee; creatine status To verify; cardio 3 km/h at 12% incline; machine displayed '200k' interpreted as approximately 200 kcal To verify</x:v>
+      </x:c>
+      <x:c r="G28" s="170" t="str">
+        <x:v>Exactly 16 working sets plus three genuine preparation sets were completed with no pain or RIR 0. Lat pulldown and seated-row performance progressed. A new T-bar machine and the established row machine were both used, duplicating the horizontal-row pattern and displacing straight-arm pulldown; three sets reached RIR 1 and final energy was Low.</x:v>
+      </x:c>
+      <x:c r="H28" s="170" t="str">
+        <x:v>Shoulders + Triceps next after fresh readiness; next Back + Biceps use only one chest-supported-row variation, retain exactly 16 working sets, keep routine work at RIR 2-3, and use 20 min cardio at a moderated 8-10% incline</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -31817,7 +32776,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc0c56f9923b455f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R613c7074036d42b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31994,13 +32953,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Chest + Triceps on 2026-08-31: no chest, shoulder, elbow, upper-biceps, knee, hip or lower-back pain; no soreness; no form breakdown.</x:v>
+        <x:v>After Back + Biceps on 2026-09-01: no back, lower-back, shoulder, elbow or biceps pain; no cardio symptoms; no reported form breakdown.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Fresh readiness before Back + Biceps; monitor delayed chest/triceps soreness</x:v>
+        <x:v>Fresh readiness before Shoulders + Triceps; monitor delayed back/biceps soreness</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -32182,13 +33141,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday 2026-08-31 completed.</x:v>
+        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday and Tuesday completed this week.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known / active four-week block</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Back + Biceps next after fresh readiness; preserve 18-set ceiling</x:v>
+        <x:v>Shoulders + Triceps next; control resistance duration to preserve 20 min cardio</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -32387,7 +33346,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b5e7491bc1e46d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0860414fb498464d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33490,10 +34449,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae9ba9403113484e"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ff3d66e2144709"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9725356124e64fa5"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3c0c252621490d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0190e83935fe4b1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cecf3c5f8ee4aaa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R988750d655cd4bde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0525382dd774da4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 2 and 3 workouts
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8bd364b21e78471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4c8a4cfd7af74b22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rc2ac4b7f3da84250"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rde3fcb8c1e2049cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R8aa3b002dc824094"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R397b38f24e9643fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R9523795e73cc42a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R4ba25784ec9d4e6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Ra4603ec508bf4a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc1df7d6821f54f93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R9f5705a2155e4f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rddc690c893a246a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R310333ca0c2f4393"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R6a046f8988694956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R78d50b8c2ff14bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R6837c83cbdb14e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R9f0536acbea64cb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R34d6bdd3b8464d9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R44e32c925a8449ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rc4eb560cac9f44cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R26c4860149c4497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R924b6455ff9042b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4efbcfc0aca94cbb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R825f029de92843ea"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N484" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N522" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R191e0927119d4b96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62ee4c719247403a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R464b0fbb013247cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a445547f8524075"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4083,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4091,7 +4091,7 @@
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="str">
-        <x:v>4-day temporary</x:v>
+        <x:v>6-day active</x:v>
       </x:c>
       <x:c r="I5" s="53" t="n"/>
       <x:c r="J5" s="59" t="n"/>
@@ -4327,7 +4327,7 @@
         <x:v>Wednesday</x:v>
       </x:c>
       <x:c r="B15" s="59" t="str">
-        <x:v>Shoulders + Triceps - next after readiness</x:v>
+        <x:v>Shoulders + Triceps - completed 2026-09-02</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4349,7 +4349,7 @@
         <x:v>Thursday</x:v>
       </x:c>
       <x:c r="B16" s="59" t="str">
-        <x:v>Legs + Calves</x:v>
+        <x:v>Legs + Calves - completed 2026-09-03</x:v>
       </x:c>
       <x:c r="C16" s="59" t="n"/>
       <x:c r="D16" s="94" t="inlineStr">
@@ -4391,26 +4391,26 @@
         <x:v>Friday</x:v>
       </x:c>
       <x:c r="B17" s="59" t="str">
-        <x:v>Chest + Shoulders</x:v>
+        <x:v>Chest + Shoulders - next after readiness</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="str">
-        <x:v>Back</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E17" s="59" t="str">
-        <x:v>Lat Pulldown</x:v>
+        <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="F17" s="59" t="str">
-        <x:v>60 kg x 10 @ RIR 2</x:v>
+        <x:v>65 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="G17" s="59" t="str">
-        <x:v>Hold; improve 55 kg reps</x:v>
+        <x:v>65 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="H17" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I17" s="59" t="str">
-        <x:v>True preparation achieved</x:v>
+        <x:v>Hold load</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
@@ -4425,22 +4425,22 @@
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="str">
-        <x:v>Back</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E18" s="59" t="str">
-        <x:v>Seated Cable Row</x:v>
+        <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="F18" s="59" t="str">
-        <x:v>60 kg x 10 @ RIR 2</x:v>
+        <x:v>160 kg x 7 unassisted @1</x:v>
       </x:c>
       <x:c r="G18" s="59" t="str">
-        <x:v>60 kg x 10-11 @ RIR 2</x:v>
+        <x:v>140 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H18" s="59" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify volume/effort</x:v>
       </x:c>
       <x:c r="I18" s="59" t="str">
-        <x:v>Reserve improved</x:v>
+        <x:v>Exactly 3 sets; no 160</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
@@ -4451,22 +4451,22 @@
       <x:c r="B19" s="59"/>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="str">
-        <x:v>Back</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Chest-Supported T-Bar</x:v>
+        <x:v>DB Romanian Deadlift</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>40 kg x 10 @ RIR 1</x:v>
+        <x:v>17.5 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>40 kg x 8-10 @ RIR 2</x:v>
+        <x:v>15 kg each x 10-11 @ RIR 2</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>New / verify</x:v>
+        <x:v>Modify technique</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>Load basis To verify</x:v>
+        <x:v>17.5 was substitution</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
@@ -4477,22 +4477,22 @@
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="59" t="str">
-        <x:v>Back</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Chest-Supported Row</x:v>
+        <x:v>Leg Curl</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>55 kg x 12 @ RIR 2</x:v>
+        <x:v>35 kg x 9 @ RIR 1</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>55 kg x 12-13 @ RIR 2</x:v>
+        <x:v>35 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>Modify selection</x:v>
+        <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>Use one row variation</x:v>
+        <x:v>No extra set</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
@@ -4503,22 +4503,22 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="59" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Legs</x:v>
       </x:c>
       <x:c r="E21" s="59" t="str">
-        <x:v>Incline DB Curl</x:v>
+        <x:v>Leg Extension</x:v>
       </x:c>
       <x:c r="F21" s="59" t="str">
-        <x:v>15 kg x 8 @ RIR 1</x:v>
+        <x:v>50 kg x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="G21" s="59" t="str">
-        <x:v>15 kg x 8-9 @ RIR 2</x:v>
+        <x:v>50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="H21" s="59" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I21" s="59" t="str">
-        <x:v>No load increase</x:v>
+        <x:v>Add one rep</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
@@ -4529,22 +4529,22 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="59" t="str">
-        <x:v>Biceps</x:v>
+        <x:v>Calves</x:v>
       </x:c>
       <x:c r="E22" s="59" t="str">
-        <x:v>Hammer Curl</x:v>
+        <x:v>Standing Calf Raise</x:v>
       </x:c>
       <x:c r="F22" s="59" t="str">
-        <x:v>17.5 kg x 11 @ RIR 2</x:v>
+        <x:v>20 kg/side x 17 @ RIR 2</x:v>
       </x:c>
       <x:c r="G22" s="59" t="str">
-        <x:v>17.5 kg x 12 @ RIR 2</x:v>
+        <x:v>Repeat plus third set</x:v>
       </x:c>
       <x:c r="H22" s="59" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="59" t="str">
-        <x:v>Exactly two sets</x:v>
+        <x:v>Three sets next time</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4555,22 +4555,22 @@
       <x:c r="B23" s="50" t="n"/>
       <x:c r="C23" s="50" t="n"/>
       <x:c r="D23" s="50" t="str">
-        <x:v>Cardio</x:v>
+        <x:v>Recovery</x:v>
       </x:c>
       <x:c r="E23" s="50" t="str">
-        <x:v>Incline treadmill</x:v>
+        <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>20 min; 3 km/h; 12%</x:v>
+        <x:v>Low after 80 min</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>20 min; 3 km/h; 8-10%</x:v>
+        <x:v>Fresh readiness required</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Progress / moderate</x:v>
+        <x:v>Monitor</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>200 kcal display To verify</x:v>
+        <x:v>No cardio today</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4581,22 +4581,22 @@
       <x:c r="B24" s="50" t="n"/>
       <x:c r="C24" s="50" t="n"/>
       <x:c r="D24" s="50" t="str">
-        <x:v>Recovery</x:v>
+        <x:v>Next</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Final energy</x:v>
+        <x:v>Chest + Shoulders</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>Low after 90 min</x:v>
+        <x:v>Four days completed</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>Shoulders+Triceps after readiness</x:v>
+        <x:v>No unplanned sets</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>Monitor</x:v>
+        <x:v>Planned</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>No added volume</x:v>
+        <x:v>Cardio only if energy allows</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4625,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b153402bfb342c1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc6905544644101"/>
 </x:worksheet>
 </file>
 
@@ -24870,6 +24870,1678 @@
         <x:v>Working</x:v>
       </x:c>
       <x:c r="N484" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="485">
+      <x:c r="A485" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B485" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C485" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D485" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E485" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F485" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G485" s="170" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H485" s="170" t="str">
+        <x:v>Genuine low-fatigue preparation; clean and unassisted</x:v>
+      </x:c>
+      <x:c r="I485" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J485" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K485" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L485" s="170" t="str">
+        <x:v>Excluded from working-set total</x:v>
+      </x:c>
+      <x:c r="M485" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N485" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="486">
+      <x:c r="A486" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B486" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C486" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D486" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E486" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F486" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G486" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H486" s="170" t="str">
+        <x:v>Clean and unassisted; controlled path reported</x:v>
+      </x:c>
+      <x:c r="I486" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J486" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K486" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L486" s="170" t="str">
+        <x:v>Working-set progression; fourth press set later exceeded plan</x:v>
+      </x:c>
+      <x:c r="M486" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N486" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="487">
+      <x:c r="A487" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B487" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C487" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D487" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E487" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F487" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G487" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H487" s="170" t="str">
+        <x:v>Clean and unassisted; controlled path reported</x:v>
+      </x:c>
+      <x:c r="I487" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J487" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K487" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L487" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M487" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N487" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="488">
+      <x:c r="A488" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B488" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C488" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D488" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E488" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F488" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G488" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H488" s="170" t="str">
+        <x:v>Clean and unassisted; controlled path reported</x:v>
+      </x:c>
+      <x:c r="I488" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J488" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K488" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L488" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M488" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N488" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="489">
+      <x:c r="A489" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B489" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C489" s="170" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D489" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E489" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F489" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G489" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H489" s="170" t="str">
+        <x:v>Clean and unassisted; controlled path reported</x:v>
+      </x:c>
+      <x:c r="I489" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J489" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K489" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L489" s="170" t="str">
+        <x:v>Improved from 8 @ RIR 1; extra fourth working press set, no load progression</x:v>
+      </x:c>
+      <x:c r="M489" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N489" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="490">
+      <x:c r="A490" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B490" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C490" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D490" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E490" s="170" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F490" s="170" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="G490" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H490" s="170" t="str">
+        <x:v>Clean and unassisted; no shrug/form detail To verify</x:v>
+      </x:c>
+      <x:c r="I490" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J490" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K490" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L490" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M490" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N490" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="491">
+      <x:c r="A491" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B491" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C491" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D491" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E491" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F491" s="170" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="G491" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H491" s="170" t="str">
+        <x:v>Clean and unassisted; no shrug/form detail To verify</x:v>
+      </x:c>
+      <x:c r="I491" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J491" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K491" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L491" s="170" t="str">
+        <x:v>Retain load</x:v>
+      </x:c>
+      <x:c r="M491" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N491" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="492">
+      <x:c r="A492" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B492" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C492" s="170" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D492" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E492" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F492" s="170" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="G492" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H492" s="170" t="str">
+        <x:v>Clean and unassisted; no shrug/form detail To verify</x:v>
+      </x:c>
+      <x:c r="I492" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J492" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K492" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L492" s="170" t="str">
+        <x:v>New heavier baseline; no load increase</x:v>
+      </x:c>
+      <x:c r="M492" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N492" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="493">
+      <x:c r="A493" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B493" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C493" s="170" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D493" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E493" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F493" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G493" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H493" s="170" t="str">
+        <x:v>Clean and unassisted; chest contact/path To verify</x:v>
+      </x:c>
+      <x:c r="I493" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J493" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K493" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L493" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M493" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N493" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="494">
+      <x:c r="A494" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B494" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C494" s="170" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D494" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E494" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F494" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G494" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H494" s="170" t="str">
+        <x:v>Clean and unassisted; chest contact/path To verify</x:v>
+      </x:c>
+      <x:c r="I494" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J494" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K494" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L494" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M494" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N494" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="495">
+      <x:c r="A495" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B495" s="170" t="str">
+        <x:v>Shoulders</x:v>
+      </x:c>
+      <x:c r="C495" s="170" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D495" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E495" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F495" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G495" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H495" s="170" t="str">
+        <x:v>Clean and unassisted; chest contact/path To verify</x:v>
+      </x:c>
+      <x:c r="I495" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J495" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K495" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L495" s="170" t="str">
+        <x:v>New higher-load baseline; third set exceeded live two-set reduction</x:v>
+      </x:c>
+      <x:c r="M495" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N495" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="496">
+      <x:c r="A496" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B496" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C496" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D496" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E496" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F496" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G496" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H496" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I496" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J496" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K496" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L496" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M496" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N496" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="497">
+      <x:c r="A497" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B497" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C497" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D497" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E497" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F497" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G497" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H497" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I497" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J497" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K497" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L497" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M497" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N497" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="498">
+      <x:c r="A498" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B498" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C498" s="170" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D498" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E498" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F498" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G498" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H498" s="170" t="str">
+        <x:v>Clean and unassisted; elbows fixed To verify</x:v>
+      </x:c>
+      <x:c r="I498" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J498" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K498" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L498" s="170" t="str">
+        <x:v>Retain load</x:v>
+      </x:c>
+      <x:c r="M498" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N498" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="499">
+      <x:c r="A499" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B499" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C499" s="170" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D499" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E499" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F499" s="170" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="G499" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H499" s="170" t="str">
+        <x:v>Clean and unassisted; both arms completed; side difference To verify</x:v>
+      </x:c>
+      <x:c r="I499" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J499" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K499" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L499" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M499" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N499" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="500">
+      <x:c r="A500" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B500" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C500" s="170" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D500" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E500" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F500" s="170" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="G500" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H500" s="170" t="str">
+        <x:v>Clean and unassisted; both arms completed; side difference To verify</x:v>
+      </x:c>
+      <x:c r="I500" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J500" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K500" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L500" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M500" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N500" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="501">
+      <x:c r="A501" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B501" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C501" s="170" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D501" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E501" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F501" s="170" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="G501" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H501" s="170" t="str">
+        <x:v>Clean and unassisted; both arms completed; side difference To verify</x:v>
+      </x:c>
+      <x:c r="I501" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J501" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K501" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L501" s="170" t="str">
+        <x:v>Rep progression; retain load</x:v>
+      </x:c>
+      <x:c r="M501" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N501" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="502">
+      <x:c r="A502" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B502" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C502" s="170" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D502" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E502" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F502" s="170" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="G502" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H502" s="170" t="str">
+        <x:v>Clean and unassisted; seated setup and elbow path To verify</x:v>
+      </x:c>
+      <x:c r="I502" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J502" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K502" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L502" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M502" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N502" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="503">
+      <x:c r="A503" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B503" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C503" s="170" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D503" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E503" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F503" s="170" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="G503" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H503" s="170" t="str">
+        <x:v>Clean and unassisted; seated setup and elbow path To verify</x:v>
+      </x:c>
+      <x:c r="I503" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J503" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K503" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L503" s="170" t="str">
+        <x:v>Added beyond live one-set instruction</x:v>
+      </x:c>
+      <x:c r="M503" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N503" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="504">
+      <x:c r="A504" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B504" s="170" t="str">
+        <x:v>Triceps</x:v>
+      </x:c>
+      <x:c r="C504" s="170" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D504" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E504" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F504" s="170" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="G504" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H504" s="170" t="str">
+        <x:v>Clean and unassisted; seated setup and elbow path To verify</x:v>
+      </x:c>
+      <x:c r="I504" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="J504" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K504" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L504" s="170" t="str">
+        <x:v>New heavy baseline; extra volume receives no automatic progression credit</x:v>
+      </x:c>
+      <x:c r="M504" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N504" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="505">
+      <x:c r="A505" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B505" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C505" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D505" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E505" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F505" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G505" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H505" s="170" t="str">
+        <x:v>Clean and unassisted; depth and knee tracking To verify</x:v>
+      </x:c>
+      <x:c r="I505" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J505" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K505" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L505" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M505" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N505" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="506">
+      <x:c r="A506" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B506" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C506" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D506" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E506" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F506" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G506" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H506" s="170" t="str">
+        <x:v>Clean and unassisted; depth and knee tracking To verify</x:v>
+      </x:c>
+      <x:c r="I506" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J506" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K506" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L506" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M506" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N506" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="507">
+      <x:c r="A507" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B507" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C507" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D507" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E507" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F507" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G507" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H507" s="170" t="str">
+        <x:v>Clean and unassisted; depth and knee tracking To verify</x:v>
+      </x:c>
+      <x:c r="I507" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J507" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K507" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L507" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M507" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N507" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="508">
+      <x:c r="A508" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B508" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C508" s="170" t="str">
+        <x:v>Hack Squat</x:v>
+      </x:c>
+      <x:c r="D508" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E508" s="170" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F508" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G508" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H508" s="170" t="str">
+        <x:v>Clean and unassisted; depth and knee tracking To verify</x:v>
+      </x:c>
+      <x:c r="I508" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J508" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K508" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L508" s="170" t="str">
+        <x:v>One rep below prior session; hold load</x:v>
+      </x:c>
+      <x:c r="M508" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N508" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="509">
+      <x:c r="A509" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B509" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C509" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D509" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E509" s="170" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="F509" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G509" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H509" s="170" t="str">
+        <x:v>Clean and unassisted; hips and depth To verify</x:v>
+      </x:c>
+      <x:c r="I509" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J509" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K509" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L509" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M509" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N509" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="510">
+      <x:c r="A510" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B510" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C510" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D510" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E510" s="170" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="F510" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G510" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H510" s="170" t="str">
+        <x:v>Clean and unassisted; hips and depth To verify</x:v>
+      </x:c>
+      <x:c r="I510" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J510" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K510" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L510" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M510" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N510" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="511">
+      <x:c r="A511" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B511" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C511" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D511" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E511" s="170" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="F511" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G511" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H511" s="170" t="str">
+        <x:v>Clean and unassisted; hips and depth To verify</x:v>
+      </x:c>
+      <x:c r="I511" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J511" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K511" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L511" s="170" t="str">
+        <x:v>Too close to failure; improve reserve</x:v>
+      </x:c>
+      <x:c r="M511" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N511" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="512">
+      <x:c r="A512" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B512" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C512" s="170" t="str">
+        <x:v>Leg Press</x:v>
+      </x:c>
+      <x:c r="D512" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E512" s="170" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F512" s="170" t="str">
+        <x:v>kg total displayed load</x:v>
+      </x:c>
+      <x:c r="G512" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H512" s="170" t="str">
+        <x:v>All seven reps unassisted; detailed depth To verify</x:v>
+      </x:c>
+      <x:c r="I512" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J512" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K512" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L512" s="170" t="str">
+        <x:v>Improved from five clean plus two assisted; extra fourth set receives no progression credit</x:v>
+      </x:c>
+      <x:c r="M512" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N512" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="513">
+      <x:c r="A513" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B513" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C513" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D513" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E513" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F513" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G513" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H513" s="170" t="str">
+        <x:v>No pain; hamstrings felt but not strongly; hinge detail To verify</x:v>
+      </x:c>
+      <x:c r="I513" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J513" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K513" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L513" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M513" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N513" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="514">
+      <x:c r="A514" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B514" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C514" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D514" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E514" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F514" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G514" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H514" s="170" t="str">
+        <x:v>No pain; hamstrings felt but not strongly; hinge detail To verify</x:v>
+      </x:c>
+      <x:c r="I514" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J514" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K514" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L514" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M514" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N514" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="515">
+      <x:c r="A515" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B515" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C515" s="170" t="str">
+        <x:v>Dumbbell Romanian Deadlift</x:v>
+      </x:c>
+      <x:c r="D515" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E515" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F515" s="170" t="str">
+        <x:v>kg each dumbbell; 15 kg unavailable</x:v>
+      </x:c>
+      <x:c r="G515" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H515" s="170" t="str">
+        <x:v>No pain; hamstrings felt but not strongly; hinge detail To verify</x:v>
+      </x:c>
+      <x:c r="I515" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J515" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K515" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L515" s="170" t="str">
+        <x:v>Equipment-availability substitution; not a progression target</x:v>
+      </x:c>
+      <x:c r="M515" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N515" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="516">
+      <x:c r="A516" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B516" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C516" s="170" t="str">
+        <x:v>Leg Curl</x:v>
+      </x:c>
+      <x:c r="D516" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E516" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F516" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G516" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H516" s="170" t="str">
+        <x:v>Clean and unassisted; range/eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I516" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J516" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K516" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L516" s="170" t="str">
+        <x:v>One reserve harder than target</x:v>
+      </x:c>
+      <x:c r="M516" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N516" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="517">
+      <x:c r="A517" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B517" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C517" s="170" t="str">
+        <x:v>Leg Curl</x:v>
+      </x:c>
+      <x:c r="D517" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E517" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F517" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G517" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H517" s="170" t="str">
+        <x:v>Clean and unassisted; range/eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I517" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J517" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K517" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L517" s="170" t="str">
+        <x:v>Repeated RIR 1; no load or set increase</x:v>
+      </x:c>
+      <x:c r="M517" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N517" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="518">
+      <x:c r="A518" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B518" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C518" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D518" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E518" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F518" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G518" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H518" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I518" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J518" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K518" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L518" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M518" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N518" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="519">
+      <x:c r="A519" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B519" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C519" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D519" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E519" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F519" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G519" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H519" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I519" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J519" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K519" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L519" s="170" t="str">
+        <x:v>Retain load and add rep</x:v>
+      </x:c>
+      <x:c r="M519" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N519" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="520">
+      <x:c r="A520" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B520" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C520" s="170" t="str">
+        <x:v>Leg Extension</x:v>
+      </x:c>
+      <x:c r="D520" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E520" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F520" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G520" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H520" s="170" t="str">
+        <x:v>Clean and unassisted; controlled eccentric To verify</x:v>
+      </x:c>
+      <x:c r="I520" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J520" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K520" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L520" s="170" t="str">
+        <x:v>Retain load and add rep</x:v>
+      </x:c>
+      <x:c r="M520" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N520" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="521">
+      <x:c r="A521" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B521" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C521" s="170" t="str">
+        <x:v>Standing Calf Raise</x:v>
+      </x:c>
+      <x:c r="D521" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E521" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F521" s="170" t="str">
+        <x:v>kg plates each side on guided bar; bar excluded</x:v>
+      </x:c>
+      <x:c r="G521" s="170" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H521" s="170" t="str">
+        <x:v>Clean and unassisted; stretch and top pause To verify</x:v>
+      </x:c>
+      <x:c r="I521" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J521" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K521" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L521" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M521" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N521" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="522">
+      <x:c r="A522" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B522" s="170" t="str">
+        <x:v>Legs</x:v>
+      </x:c>
+      <x:c r="C522" s="170" t="str">
+        <x:v>Standing Calf Raise</x:v>
+      </x:c>
+      <x:c r="D522" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E522" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F522" s="170" t="str">
+        <x:v>kg plates each side on guided bar; bar excluded</x:v>
+      </x:c>
+      <x:c r="G522" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H522" s="170" t="str">
+        <x:v>Clean and unassisted; stretch and top pause To verify</x:v>
+      </x:c>
+      <x:c r="I522" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="J522" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="K522" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L522" s="170" t="str">
+        <x:v>Target met; two sets because fourth leg-press set consumed budget</x:v>
+      </x:c>
+      <x:c r="M522" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N522" s="170" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -24905,7 +26577,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16d19a29add74d16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e00955fc7024f2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25450,13 +27122,13 @@
         <x:v>Hack Squat</x:v>
       </x:c>
       <x:c r="C20" s="169" t="str">
-        <x:v>65 kg/side x 9 @ RIR 2</x:v>
+        <x:v>65 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="D20" s="169" t="str">
         <x:v>35-65 kg/side</x:v>
       </x:c>
       <x:c r="E20" s="169" t="str">
-        <x:v>65 kg/side x 10 @ RIR 2</x:v>
+        <x:v>65 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F20" s="169" t="str">
         <x:v>Add rep before load</x:v>
@@ -25468,7 +27140,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I20" s="169" t="str">
-        <x:v>35-55 kg reserve improved; machine carriage excluded</x:v>
+        <x:v>Machine carriage excluded; one rep below prior session</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" hidden="0" customHeight="1">
@@ -25479,7 +27151,7 @@
         <x:v>Leg Press</x:v>
       </x:c>
       <x:c r="C21" s="169" t="str">
-        <x:v>160 kg x 5 clean + 2 assisted @ RIR 1</x:v>
+        <x:v>160 kg x 7 unassisted @ RIR 1</x:v>
       </x:c>
       <x:c r="D21" s="169" t="str">
         <x:v>100-140 kg total</x:v>
@@ -25488,16 +27160,16 @@
         <x:v>140 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F21" s="169" t="str">
-        <x:v>Exactly 3 sets; no assisted 160 kg</x:v>
+        <x:v>Exactly 3 sets; omit 160 kg</x:v>
       </x:c>
       <x:c r="G21" s="169" t="str">
-        <x:v>Hips stay on pad; controlled depth</x:v>
+        <x:v>Hips on pad; controlled depth</x:v>
       </x:c>
       <x:c r="H21" s="169" t="str">
-        <x:v>Modify load/effort / To verify</x:v>
+        <x:v>Modify volume/effort / To verify</x:v>
       </x:c>
       <x:c r="I21" s="169" t="str">
-        <x:v>Earlier 130/150 entry conflicts with reported 140/160 machine increments; preserve both and verify before rewriting history</x:v>
+        <x:v>160 kg improved to seven unassisted but was extra and RIR 1; historical load discrepancy remains To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" hidden="0" customHeight="1">
@@ -25526,7 +27198,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I22" s="169" t="str">
-        <x:v>All three targets met exactly</x:v>
+        <x:v>Matched prior session at intended reserve</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" hidden="0" customHeight="1">
@@ -25543,10 +27215,10 @@
         <x:v>30-35 kg</x:v>
       </x:c>
       <x:c r="E23" s="169" t="str">
-        <x:v>35 kg x 10 @ RIR 2</x:v>
+        <x:v>35 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F23" s="169" t="str">
-        <x:v>Add rep and reserve before load</x:v>
+        <x:v>Improve reserve; no extra set</x:v>
       </x:c>
       <x:c r="G23" s="169" t="str">
         <x:v>Full range; controlled eccentric</x:v>
@@ -25555,7 +27227,7 @@
         <x:v>Modify effort</x:v>
       </x:c>
       <x:c r="I23" s="169" t="str">
-        <x:v>30 kg was RIR 2; 35 kg remains too close to failure</x:v>
+        <x:v>Repeated prior result; 30 kg set also one reserve harder than target</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" hidden="0" customHeight="1">
@@ -25620,16 +27292,16 @@
         <x:v>Standing Calf Raise</x:v>
       </x:c>
       <x:c r="C26" s="169" t="str">
-        <x:v>20 kg/side x 16 @ RIR 3</x:v>
+        <x:v>20 kg/side x 17 @ RIR 2</x:v>
       </x:c>
       <x:c r="D26" s="169" t="str">
         <x:v>10-20 kg/side</x:v>
       </x:c>
       <x:c r="E26" s="169" t="str">
-        <x:v>20 kg/side x 17 @ RIR 2</x:v>
+        <x:v>20 kg/side x 17 then 15-17 @ RIR 2</x:v>
       </x:c>
       <x:c r="F26" s="169" t="str">
-        <x:v>Return to 3 sets within 18-set plan</x:v>
+        <x:v>Use 3 sets when leg press is 3 sets</x:v>
       </x:c>
       <x:c r="G26" s="169" t="str">
         <x:v>Full stretch; pause at top</x:v>
@@ -25638,7 +27310,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I26" s="169" t="str">
-        <x:v>Two sets only today because extra leg-press set consumed the set budget; bar excluded</x:v>
+        <x:v>Both targets met; two sets used to preserve 18-set ceiling</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -25649,25 +27321,25 @@
         <x:v>Dumbbell Shoulder Press</x:v>
       </x:c>
       <x:c r="C27" s="170" t="str">
-        <x:v>25 kg each x 8 @ RIR 1 unplanned</x:v>
+        <x:v>25 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D27" s="170" t="str">
-        <x:v>17.5-22.5 kg each</x:v>
+        <x:v>20-25 kg each</x:v>
       </x:c>
       <x:c r="E27" s="170" t="str">
-        <x:v>22.5 kg each x 9 @ RIR 2</x:v>
+        <x:v>25 kg each x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F27" s="170" t="str">
-        <x:v>Exactly 3 working sets; no 25 kg yet</x:v>
+        <x:v>Exactly 3 working sets; omit 17.5 kg working set</x:v>
       </x:c>
       <x:c r="G27" s="170" t="str">
         <x:v>Neutral wrist; controlled path</x:v>
       </x:c>
       <x:c r="H27" s="170" t="str">
-        <x:v>Modify volume/load</x:v>
+        <x:v>Modify volume</x:v>
       </x:c>
       <x:c r="I27" s="170" t="str">
-        <x:v>15 kg was warm-up; 17.5-22.5 kg progressed; unplanned 25 kg retained without progression credit</x:v>
+        <x:v>15 kg preparation; 25 kg progressed cleanly but was extra fourth working set</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -25736,16 +27408,16 @@
         <x:v>Reverse Pec Deck</x:v>
       </x:c>
       <x:c r="C30" s="170" t="str">
-        <x:v>35 kg x 10 @ RIR 3</x:v>
+        <x:v>40 kg x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D30" s="170" t="str">
-        <x:v>25-35 kg</x:v>
+        <x:v>30-40 kg</x:v>
       </x:c>
       <x:c r="E30" s="170" t="str">
-        <x:v>35 kg x 11-12 @ RIR 2-3</x:v>
+        <x:v>40 kg x 9-10 @ RIR 2</x:v>
       </x:c>
       <x:c r="F30" s="170" t="str">
-        <x:v>Add reps with reserve</x:v>
+        <x:v>Add rep before load</x:v>
       </x:c>
       <x:c r="G30" s="170" t="str">
         <x:v>Chest on pad; lead elbows</x:v>
@@ -25754,7 +27426,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I30" s="170" t="str">
-        <x:v>Reserve improved markedly on 2026-08-21</x:v>
+        <x:v>All sets RIR 2; third set exceeded live two-set reduction</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -25852,16 +27524,16 @@
         <x:v>Rope Pushdown</x:v>
       </x:c>
       <x:c r="C34" s="170" t="str">
-        <x:v>40 kg x 11 @ RIR 1 after prior 40 kg set</x:v>
+        <x:v>40 kg x 10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D34" s="170" t="str">
         <x:v>30-40 kg</x:v>
       </x:c>
       <x:c r="E34" s="170" t="str">
-        <x:v>40 kg x 10-11 @ RIR 2</x:v>
+        <x:v>35 kg x 13-14 @ RIR 2</x:v>
       </x:c>
       <x:c r="F34" s="170" t="str">
-        <x:v>Exactly 3 sets; no repeated 40 kg set</x:v>
+        <x:v>Exactly 2 sets; no third set</x:v>
       </x:c>
       <x:c r="G34" s="170" t="str">
         <x:v>Spread rope; slow return</x:v>
@@ -25870,7 +27542,7 @@
         <x:v>Modify volume</x:v>
       </x:c>
       <x:c r="I34" s="170" t="str">
-        <x:v>Fourth set exceeded plan; repetition gain does not justify load</x:v>
+        <x:v>Use 30 and 35 kg only next time to control total volume</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="48" hidden="0" customHeight="1">
@@ -25910,16 +27582,16 @@
         <x:v>Single-Arm Cable Pushdown</x:v>
       </x:c>
       <x:c r="C36" s="170" t="str">
-        <x:v>15 kg x 10 each @ RIR 2</x:v>
+        <x:v>15 kg each arm x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D36" s="170" t="str">
         <x:v>10-15 kg</x:v>
       </x:c>
       <x:c r="E36" s="170" t="str">
-        <x:v>15 kg x 10-11 @ RIR 2</x:v>
+        <x:v>15 kg each x 12-13 @ RIR 2</x:v>
       </x:c>
       <x:c r="F36" s="170" t="str">
-        <x:v>Match both arms; add rep</x:v>
+        <x:v>Exactly 2 sets; match both arms</x:v>
       </x:c>
       <x:c r="G36" s="170" t="str">
         <x:v>Elbow fixed; match weaker side</x:v>
@@ -25928,7 +27600,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I36" s="170" t="str">
-        <x:v>Side-to-side difference To verify; reserve improved</x:v>
+        <x:v>Use 10 and 15 kg only; side-to-side difference To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="48" hidden="0" customHeight="1">
@@ -25939,25 +27611,25 @@
         <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
       </x:c>
       <x:c r="C37" s="170" t="str">
-        <x:v>25 kg x 10 @ RIR 2</x:v>
+        <x:v>30 kg x 7 @ RIR 2 unplanned</x:v>
       </x:c>
       <x:c r="D37" s="170" t="str">
         <x:v>20-25 kg</x:v>
       </x:c>
       <x:c r="E37" s="170" t="str">
-        <x:v>25 kg x 11 @ RIR 2</x:v>
+        <x:v>25 kg x 12-13 @ RIR 2</x:v>
       </x:c>
       <x:c r="F37" s="170" t="str">
-        <x:v>Exactly 3 sets; add rep before load</x:v>
+        <x:v>Exactly 2 sets; no 30 kg next time</x:v>
       </x:c>
       <x:c r="G37" s="170" t="str">
         <x:v>Back supported; ribs down</x:v>
       </x:c>
       <x:c r="H37" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Modify volume/load</x:v>
       </x:c>
       <x:c r="I37" s="170" t="str">
-        <x:v>22.5 kg progressed to 13 reps; completed third set despite live reduction</x:v>
+        <x:v>25 and 30 kg were added beyond live one-set instruction; no automatic progression credit</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="48" hidden="0" customHeight="1">
@@ -26142,16 +27814,16 @@
         <x:v>Plate-Loaded Lateral Raise Machine</x:v>
       </x:c>
       <x:c r="C44" s="170" t="str">
-        <x:v>5 kg/side x 15 for 2 sets @ RIR 2</x:v>
+        <x:v>7.5 kg/side x 8 @ RIR 2</x:v>
       </x:c>
       <x:c r="D44" s="170" t="str">
-        <x:v>2.5-5 kg/side</x:v>
+        <x:v>2.5-7.5 kg/side</x:v>
       </x:c>
       <x:c r="E44" s="170" t="str">
-        <x:v>5 kg/side x 16 @ RIR 2</x:v>
+        <x:v>7.5 kg/side x 8-9 @ RIR 2</x:v>
       </x:c>
       <x:c r="F44" s="170" t="str">
-        <x:v>Maximum 3 sets; add one rep</x:v>
+        <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G44" s="170" t="str">
         <x:v>No shrug; controlled eccentric</x:v>
@@ -26160,7 +27832,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I44" s="170" t="str">
-        <x:v>Unloaded machine resistance excluded and To verify</x:v>
+        <x:v>New 7.5 kg baseline; unloaded machine resistance To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="48" customHeight="1">
@@ -26258,7 +27930,7 @@
         <x:v>Dumbbell Romanian Deadlift</x:v>
       </x:c>
       <x:c r="C48" s="170" t="str">
-        <x:v>15 kg each x 10 @ RIR 2; pain-free</x:v>
+        <x:v>17.5 kg each x 9 @ RIR 2 substitution</x:v>
       </x:c>
       <x:c r="D48" s="170" t="str">
         <x:v>10-15 kg each</x:v>
@@ -26267,16 +27939,16 @@
         <x:v>15 kg each x 10-11 @ RIR 2 with hamstrings dominant</x:v>
       </x:c>
       <x:c r="F48" s="170" t="str">
-        <x:v>Keep load; technique before progression</x:v>
+        <x:v>Technique and stimulus before load</x:v>
       </x:c>
       <x:c r="G48" s="170" t="str">
-        <x:v>Brace; hips back; dumbbells close; hamstring-controlled depth</x:v>
+        <x:v>Brace; hips back; dumbbells close</x:v>
       </x:c>
       <x:c r="H48" s="170" t="str">
-        <x:v>Technique improving</x:v>
+        <x:v>Modify load/technique</x:v>
       </x:c>
       <x:c r="I48" s="170" t="str">
-        <x:v>Hamstrings dominated with only a little non-painful back involvement</x:v>
+        <x:v>15 kg unavailable; 17.5 kg substitution was pain-free but hamstring sensation was limited</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="52" customHeight="1">
@@ -26391,7 +28063,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4ce57c98ffb4593"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfd47d7feb13407a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27416,17 +29088,29 @@
       <x:c r="P30" s="59" t="n"/>
       <x:c r="Q30" s="59" t="n"/>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31"/>
-      <x:c r="B31"/>
-      <x:c r="C31"/>
-      <x:c r="D31"/>
-      <x:c r="E31"/>
-      <x:c r="F31"/>
-      <x:c r="G31"/>
-      <x:c r="H31"/>
-      <x:c r="I31"/>
-      <x:c r="J31"/>
+    <x:row r="31" ht="76" customHeight="1">
+      <x:c r="A31" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B31" s="170"/>
+      <x:c r="C31" s="170"/>
+      <x:c r="D31" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E31" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="F31" s="170" t="str">
+        <x:v>No shoulder, elbow, wrist, back or lower-back pain; no pre-session soreness; no cardio symptoms</x:v>
+      </x:c>
+      <x:c r="G31" s="170"/>
+      <x:c r="H31" s="170"/>
+      <x:c r="I31" s="170" t="str">
+        <x:v>Shoulders + Triceps workout - 90 min total; 19 working sets plus one preparation set; medium pump; 20 min treadmill at 3.5 km/h and 12% incline</x:v>
+      </x:c>
+      <x:c r="J31" s="170" t="str">
+        <x:v>Started Medium; full EAA+ scoop (100 mg caffeine); no coffee; no assistance or reported form breakdown; no rail support or cardio symptoms; creatine status To verify</x:v>
+      </x:c>
       <x:c r="K31" s="59" t="n"/>
       <x:c r="L31" s="59" t="n"/>
       <x:c r="M31" s="59" t="n"/>
@@ -27435,17 +29119,29 @@
       <x:c r="P31" s="59" t="n"/>
       <x:c r="Q31" s="59" t="n"/>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32"/>
-      <x:c r="B32"/>
-      <x:c r="C32"/>
-      <x:c r="D32"/>
-      <x:c r="E32"/>
-      <x:c r="F32"/>
-      <x:c r="G32"/>
-      <x:c r="H32"/>
-      <x:c r="I32"/>
-      <x:c r="J32"/>
+    <x:row r="32" ht="76" customHeight="1">
+      <x:c r="A32" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B32" s="170"/>
+      <x:c r="C32" s="170"/>
+      <x:c r="D32" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E32" s="170" t="str">
+        <x:v>Low final</x:v>
+      </x:c>
+      <x:c r="F32" s="170" t="str">
+        <x:v>No hip, knee, lower-back or other pain; no pre-session soreness</x:v>
+      </x:c>
+      <x:c r="G32" s="170"/>
+      <x:c r="H32" s="170"/>
+      <x:c r="I32" s="170" t="str">
+        <x:v>Legs + Calves workout - 80 min; exactly 18 working sets; medium leg pump; no cardio/core</x:v>
+      </x:c>
+      <x:c r="J32" s="170" t="str">
+        <x:v>Started Medium; full EAA+ scoop (100 mg caffeine); no coffee; no assistance or reported form breakdown; 160 kg leg press all seven reps unassisted; creatine status To verify</x:v>
+      </x:c>
       <x:c r="K32" s="59" t="n"/>
       <x:c r="L32" s="59" t="n"/>
       <x:c r="M32" s="59" t="n"/>
@@ -30702,7 +32398,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab3cc518f3549e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ede55c7f20c4c52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32011,13 +33707,125 @@
         <x:v>Next comparable session use 20 min at 8-10% incline; do not eat back machine calories</x:v>
       </x:c>
     </x:row>
+    <x:row r="89" ht="60" customHeight="1">
+      <x:c r="A89" s="170" t="str">
+        <x:v>Shoulders + Triceps performance</x:v>
+      </x:c>
+      <x:c r="B89" s="170" t="str">
+        <x:v>2026-09-02 completed 19 working sets plus one genuine preparation set; all working sets ended at RIR 2-3 with no pain, assistance or form breakdown</x:v>
+      </x:c>
+      <x:c r="C89" s="170" t="str">
+        <x:v>Strength and reserve progressed without failure exposure</x:v>
+      </x:c>
+      <x:c r="D89" s="170" t="str">
+        <x:v>Retain loads and make the next session exactly 15 working sets</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="60" customHeight="1">
+      <x:c r="A90" s="170" t="str">
+        <x:v>Resistance-volume ceiling exceeded</x:v>
+      </x:c>
+      <x:c r="B90" s="170" t="str">
+        <x:v>The session exceeded the planned 15 working sets by four and the absolute 18-set ceiling by one</x:v>
+      </x:c>
+      <x:c r="C90" s="170" t="str">
+        <x:v>This was the third consecutive training day and final energy fell to Medium-Low</x:v>
+      </x:c>
+      <x:c r="D90" s="170" t="str">
+        <x:v>Completed sets remain historical fatigue but do not earn automatic load or volume progression</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="60" customHeight="1">
+      <x:c r="A91" s="170" t="str">
+        <x:v>Shoulder progression baselines</x:v>
+      </x:c>
+      <x:c r="B91" s="170" t="str">
+        <x:v>25 kg shoulder press x9 @2, 7.5 kg/side lateral raise x8 @2 and 40 kg reverse pec deck x9 @2</x:v>
+      </x:c>
+      <x:c r="C91" s="170" t="str">
+        <x:v>All were pain-free, but some occurred beyond live volume reductions</x:v>
+      </x:c>
+      <x:c r="D91" s="170" t="str">
+        <x:v>Build reps at the same loads within the 15-set structure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="60" customHeight="1">
+      <x:c r="A92" s="170" t="str">
+        <x:v>Shoulders-day cardio</x:v>
+      </x:c>
+      <x:c r="B92" s="170" t="str">
+        <x:v>20 min treadmill at 3.5 km/h and 12% incline without rail support or symptoms</x:v>
+      </x:c>
+      <x:c r="C92" s="170" t="str">
+        <x:v>The cardio dose was completed, but the incline exceeded the 6-8% prescription and Legs follows</x:v>
+      </x:c>
+      <x:c r="D92" s="170" t="str">
+        <x:v>No cardio progression; after Legs use only 5-10 min easy walking or omit it</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="60" customHeight="1">
+      <x:c r="A93" s="170" t="str">
+        <x:v>Legs + Calves performance</x:v>
+      </x:c>
+      <x:c r="B93" s="170" t="str">
+        <x:v>2026-09-03 completed exactly 18 working sets in 80 min with no pain, assistance, form breakdown or RIR 0</x:v>
+      </x:c>
+      <x:c r="C93" s="170" t="str">
+        <x:v>The session preserved the absolute set ceiling and remained pain-free</x:v>
+      </x:c>
+      <x:c r="D93" s="170" t="str">
+        <x:v>Keep loads stable and progress reps/reserve rather than adding load</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="60" customHeight="1">
+      <x:c r="A94" s="170" t="str">
+        <x:v>Unassisted 160 kg leg press</x:v>
+      </x:c>
+      <x:c r="B94" s="170" t="str">
+        <x:v>Seven repetitions at RIR 1 were completed without assistance after the prior five clean plus two assisted result</x:v>
+      </x:c>
+      <x:c r="C94" s="170" t="str">
+        <x:v>Execution improved, but the set was an unplanned fourth press set and too close to failure</x:v>
+      </x:c>
+      <x:c r="D94" s="170" t="str">
+        <x:v>Next Legs omit 160 kg and require 140 kg x10 @ RIR 2 before reconsidering it</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="60" customHeight="1">
+      <x:c r="A95" s="170" t="str">
+        <x:v>RDL equipment substitution</x:v>
+      </x:c>
+      <x:c r="B95" s="170" t="str">
+        <x:v>15 kg dumbbells were unavailable, so 17.5 kg each x9 @ RIR 2 was used; no pain but limited hamstring sensation</x:v>
+      </x:c>
+      <x:c r="C95" s="170" t="str">
+        <x:v>The heavier load may reduce the intended hinge stimulus even when pain-free</x:v>
+      </x:c>
+      <x:c r="D95" s="170" t="str">
+        <x:v>Return to 15 kg when available and verify hinge mechanics before progressing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="60" customHeight="1">
+      <x:c r="A96" s="170" t="str">
+        <x:v>Low final energy trend</x:v>
+      </x:c>
+      <x:c r="B96" s="170" t="str">
+        <x:v>2026-09-03 ended Low after three earlier consecutive sessions ended Low or Medium-Low</x:v>
+      </x:c>
+      <x:c r="C96" s="170" t="str">
+        <x:v>Accumulated fatigue can reduce performance quality despite pain-free sessions</x:v>
+      </x:c>
+      <x:c r="D96" s="170" t="str">
+        <x:v>No compensatory cardio; require fresh readiness and no unplanned sets for Chest + Shoulders</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R093cb86e02404ff9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd23a4e59f3845bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32764,6 +34572,58 @@
         <x:v>Shoulders + Triceps next after fresh readiness; next Back + Biceps use only one chest-supported-row variation, retain exactly 16 working sets, keep routine work at RIR 2-3, and use 20 min cardio at a moderated 8-10% incline</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="84" customHeight="1">
+      <x:c r="A29" s="220" t="n">
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="B29" s="170" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C29" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D29" s="170" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E29" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F29" s="170" t="str">
+        <x:v>Good sleep; Medium start and Medium-to-Low final energy; no soreness or pain; 90 min total including 20 min treadmill; medium shoulder/triceps pump; no assisted repetitions or form breakdown; full EAA+ (100 mg caffeine); no coffee; creatine status To verify; cardio 3.5 km/h at 12% incline without rail support or symptoms</x:v>
+      </x:c>
+      <x:c r="G29" s="170" t="str">
+        <x:v>Nineteen working sets plus one genuine preparation set were completed pain-free, with five sets at RIR 3 and fourteen at RIR 2. Performance and reserve progressed, but the session exceeded the planned 15 working sets by four and the absolute 18-set ceiling by one during the third consecutive training day.</x:v>
+      </x:c>
+      <x:c r="H29" s="170" t="str">
+        <x:v>Legs + Calves next after fresh readiness; next Shoulders + Triceps exactly 15 working sets, no load increases, and post-leg cardio limited to 5-10 min easy or omitted</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="84" customHeight="1">
+      <x:c r="A30" s="220" t="n">
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="B30" s="170" t="str">
+        <x:v>Legs + Calves</x:v>
+      </x:c>
+      <x:c r="C30" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D30" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E30" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F30" s="170" t="str">
+        <x:v>Good sleep; Medium start and Low final energy; no soreness or pain; 80 min; medium leg pump; no assistance or form breakdown; full EAA+ (100 mg caffeine); no coffee; creatine status To verify; no cardio/core</x:v>
+      </x:c>
+      <x:c r="G30" s="170" t="str">
+        <x:v>Exactly 18 working sets were completed without pain or RIR 0. The 160 kg leg press improved from five clean plus two assisted repetitions to seven unassisted. Calf targets were met. However, three sets reached RIR 1, the fourth leg-press set exceeded prescription, and the 17.5 kg RDL substitution produced only limited hamstring sensation.</x:v>
+      </x:c>
+      <x:c r="H30" s="170" t="str">
+        <x:v>Chest + Shoulders next after fresh readiness; next Legs exactly three leg-press sets, planned RDL top load returns to 15 kg each, improve leg-curl reserve, and use three calf sets within the 18-set ceiling</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -32776,7 +34636,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R613c7074036d42b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f72309f3f14a60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32953,13 +34813,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Back + Biceps on 2026-09-01: no back, lower-back, shoulder, elbow or biceps pain; no cardio symptoms; no reported form breakdown.</x:v>
+        <x:v>After Legs + Calves on 2026-09-03: no hip, knee, lower-back or other pain; no assistance or reported form breakdown.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
         <x:v>Known</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Fresh readiness before Shoulders + Triceps; monitor delayed back/biceps soreness</x:v>
+        <x:v>Fresh chest, shoulder and joint readiness before Chest + Shoulders; monitor delayed leg soreness</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -33141,13 +35001,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday and Tuesday completed this week.</x:v>
+        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday through Thursday completed this week.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known / active four-week block</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Shoulders + Triceps next; control resistance duration to preserve 20 min cardio</x:v>
+        <x:v>Chest + Shoulders next; no unplanned sets and cardio only if final energy remains Medium or higher</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -33346,7 +35206,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0860414fb498464d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb57474d248f4531"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34449,10 +36309,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0190e83935fe4b1f"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cecf3c5f8ee4aaa"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R988750d655cd4bde"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0525382dd774da4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb77180a5124e85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ba31e2bd6944c48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25134b61f8ec4cf9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f9dd789cb6c45fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 4 chest and shoulders workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rddc690c893a246a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R310333ca0c2f4393"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R6a046f8988694956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R78d50b8c2ff14bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R6837c83cbdb14e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R9f0536acbea64cb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R34d6bdd3b8464d9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R44e32c925a8449ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rc4eb560cac9f44cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R26c4860149c4497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R924b6455ff9042b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R25bde1780882414a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Re7908410721d4f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R3b455d177ab64146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rb7a24c0890044062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R51bb39bd551b4431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R7c90d73a2799405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R2e360cde33dd40b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R48bb77fa33a243ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R21954db5f6ec4f86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rb4611fc9255e4ec8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R5145d3d85b474ca6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R825f029de92843ea"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc246d21dce34e74"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62ee4c719247403a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7c092a1ca724cae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a445547f8524075"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0aa34563b20425b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4391,7 +4391,7 @@
         <x:v>Friday</x:v>
       </x:c>
       <x:c r="B17" s="59" t="str">
-        <x:v>Chest + Shoulders - next after readiness</x:v>
+        <x:v>Chest + Shoulders - completed 2026-09-04</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="59" t="str">
@@ -4584,19 +4584,19 @@
         <x:v>Next</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Chest + Shoulders</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>Four days completed</x:v>
+        <x:v>Five days completed</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>No unplanned sets</x:v>
+        <x:v>16 working sets; no cardio</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Conditional</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Cardio only if energy allows</x:v>
+        <x:v>Train only after fresh readiness</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4625,7 +4625,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc6905544644101"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R505cd8568a5b4cb9"/>
 </x:worksheet>
 </file>
 
@@ -26542,6 +26542,886 @@
         <x:v>Working</x:v>
       </x:c>
       <x:c r="N522" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="523" ht="42" customHeight="1">
+      <x:c r="A523" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B523" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C523" s="170" t="str">
+        <x:v>Plate-Loaded Chest Press</x:v>
+      </x:c>
+      <x:c r="D523" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E523" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F523" s="170" t="str">
+        <x:v>kg reported plate load; total vs per side To verify</x:v>
+      </x:c>
+      <x:c r="G523" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H523" s="170" t="str">
+        <x:v>No reported form breakdown; machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I523" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J523" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K523" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L523" s="170" t="str">
+        <x:v>Low-fatigue preparation</x:v>
+      </x:c>
+      <x:c r="M523" s="170" t="str">
+        <x:v>Preparation</x:v>
+      </x:c>
+      <x:c r="N523" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="524" ht="42" customHeight="1">
+      <x:c r="A524" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B524" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C524" s="170" t="str">
+        <x:v>Plate-Loaded Chest Press</x:v>
+      </x:c>
+      <x:c r="D524" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E524" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F524" s="170" t="str">
+        <x:v>kg reported plate load; total vs per side To verify</x:v>
+      </x:c>
+      <x:c r="G524" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H524" s="170" t="str">
+        <x:v>Clean and unassisted; machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I524" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J524" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K524" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L524" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M524" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N524" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="525" ht="42" customHeight="1">
+      <x:c r="A525" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B525" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C525" s="170" t="str">
+        <x:v>Plate-Loaded Chest Press</x:v>
+      </x:c>
+      <x:c r="D525" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E525" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F525" s="170" t="str">
+        <x:v>kg reported plate load; total vs per side To verify</x:v>
+      </x:c>
+      <x:c r="G525" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H525" s="170" t="str">
+        <x:v>Clean and unassisted; machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I525" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J525" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K525" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L525" s="170" t="str">
+        <x:v>Improved reserve; add reps before load</x:v>
+      </x:c>
+      <x:c r="M525" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N525" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="526" ht="42" customHeight="1">
+      <x:c r="A526" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B526" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C526" s="170" t="str">
+        <x:v>Plate-Loaded Chest Press</x:v>
+      </x:c>
+      <x:c r="D526" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E526" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F526" s="170" t="str">
+        <x:v>kg reported plate load; total vs per side To verify</x:v>
+      </x:c>
+      <x:c r="G526" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H526" s="170" t="str">
+        <x:v>Clean and unassisted; machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I526" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J526" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K526" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L526" s="170" t="str">
+        <x:v>Current top-set baseline; verify load basis</x:v>
+      </x:c>
+      <x:c r="M526" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N526" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="527" ht="42" customHeight="1">
+      <x:c r="A527" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B527" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C527" s="170" t="str">
+        <x:v>Incline Dumbbell Press</x:v>
+      </x:c>
+      <x:c r="D527" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E527" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F527" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G527" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H527" s="170" t="str">
+        <x:v>Clean and unassisted; bench angle To verify</x:v>
+      </x:c>
+      <x:c r="I527" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J527" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K527" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L527" s="170" t="str">
+        <x:v>Refreshed working baseline</x:v>
+      </x:c>
+      <x:c r="M527" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N527" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="528" ht="42" customHeight="1">
+      <x:c r="A528" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B528" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C528" s="170" t="str">
+        <x:v>Incline Dumbbell Press</x:v>
+      </x:c>
+      <x:c r="D528" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E528" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F528" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G528" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H528" s="170" t="str">
+        <x:v>Clean and unassisted; bench angle To verify</x:v>
+      </x:c>
+      <x:c r="I528" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J528" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K528" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L528" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M528" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N528" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="529" ht="42" customHeight="1">
+      <x:c r="A529" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B529" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C529" s="170" t="str">
+        <x:v>Incline Dumbbell Press</x:v>
+      </x:c>
+      <x:c r="D529" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E529" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F529" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G529" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H529" s="170" t="str">
+        <x:v>Clean and unassisted; bench angle To verify</x:v>
+      </x:c>
+      <x:c r="I529" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J529" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K529" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L529" s="170" t="str">
+        <x:v>Current top-set baseline; add rep before load</x:v>
+      </x:c>
+      <x:c r="M529" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N529" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="530" ht="42" customHeight="1">
+      <x:c r="A530" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B530" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C530" s="170" t="str">
+        <x:v>Low-to-High Cable Fly</x:v>
+      </x:c>
+      <x:c r="D530" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E530" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F530" s="170" t="str">
+        <x:v>kg reported stack setting; per-side basis To verify</x:v>
+      </x:c>
+      <x:c r="G530" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="H530" s="170" t="str">
+        <x:v>No meaningful stimulus reported; exact cable setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I530" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J530" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K530" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L530" s="170" t="str">
+        <x:v>Preparation; do not repeat as working volume</x:v>
+      </x:c>
+      <x:c r="M530" s="170" t="str">
+        <x:v>Preparation</x:v>
+      </x:c>
+      <x:c r="N530" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="531" ht="42" customHeight="1">
+      <x:c r="A531" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B531" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C531" s="170" t="str">
+        <x:v>Low-to-High Cable Fly</x:v>
+      </x:c>
+      <x:c r="D531" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E531" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F531" s="170" t="str">
+        <x:v>kg reported stack setting; per-side basis To verify</x:v>
+      </x:c>
+      <x:c r="G531" s="170" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H531" s="170" t="str">
+        <x:v>No meaningful stimulus reported; exact cable setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I531" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J531" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K531" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L531" s="170" t="str">
+        <x:v>Preparation; use only one prep set next time</x:v>
+      </x:c>
+      <x:c r="M531" s="170" t="str">
+        <x:v>Preparation</x:v>
+      </x:c>
+      <x:c r="N531" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="532" ht="42" customHeight="1">
+      <x:c r="A532" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B532" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C532" s="170" t="str">
+        <x:v>Low-to-High Cable Fly</x:v>
+      </x:c>
+      <x:c r="D532" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E532" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F532" s="170" t="str">
+        <x:v>kg reported stack setting; per-side basis To verify</x:v>
+      </x:c>
+      <x:c r="G532" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H532" s="170" t="str">
+        <x:v>No reported form breakdown; exact cable setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I532" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J532" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K532" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L532" s="170" t="str">
+        <x:v>Refreshed working baseline</x:v>
+      </x:c>
+      <x:c r="M532" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N532" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="533" ht="42" customHeight="1">
+      <x:c r="A533" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B533" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C533" s="170" t="str">
+        <x:v>Low-to-High Cable Fly</x:v>
+      </x:c>
+      <x:c r="D533" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E533" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F533" s="170" t="str">
+        <x:v>kg reported stack setting; per-side basis To verify</x:v>
+      </x:c>
+      <x:c r="G533" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H533" s="170" t="str">
+        <x:v>No reported form breakdown; exact cable setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I533" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J533" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K533" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L533" s="170" t="str">
+        <x:v>Target-quality set</x:v>
+      </x:c>
+      <x:c r="M533" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N533" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="534" ht="42" customHeight="1">
+      <x:c r="A534" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B534" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C534" s="170" t="str">
+        <x:v>Low-to-High Cable Fly</x:v>
+      </x:c>
+      <x:c r="D534" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E534" s="170" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F534" s="170" t="str">
+        <x:v>kg reported stack setting; per-side basis To verify</x:v>
+      </x:c>
+      <x:c r="G534" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H534" s="170" t="str">
+        <x:v>No reported form breakdown; exact cable setup/path To verify</x:v>
+      </x:c>
+      <x:c r="I534" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J534" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K534" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L534" s="170" t="str">
+        <x:v>Current top-set baseline; add rep before load</x:v>
+      </x:c>
+      <x:c r="M534" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N534" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="535" ht="42" customHeight="1">
+      <x:c r="A535" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B535" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C535" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D535" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E535" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F535" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G535" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H535" s="170" t="str">
+        <x:v>No reported form breakdown or shoulder pinching; pull height To verify</x:v>
+      </x:c>
+      <x:c r="I535" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J535" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K535" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L535" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M535" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N535" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="536" ht="42" customHeight="1">
+      <x:c r="A536" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B536" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C536" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D536" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E536" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F536" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G536" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H536" s="170" t="str">
+        <x:v>No reported form breakdown or shoulder pinching; pull height To verify</x:v>
+      </x:c>
+      <x:c r="I536" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J536" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K536" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L536" s="170" t="str">
+        <x:v>Improved reserve</x:v>
+      </x:c>
+      <x:c r="M536" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N536" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="537" ht="42" customHeight="1">
+      <x:c r="A537" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B537" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C537" s="170" t="str">
+        <x:v>Cable Upright Row</x:v>
+      </x:c>
+      <x:c r="D537" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E537" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F537" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G537" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H537" s="170" t="str">
+        <x:v>No reported form breakdown or shoulder pinching; pull height To verify</x:v>
+      </x:c>
+      <x:c r="I537" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J537" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K537" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L537" s="170" t="str">
+        <x:v>Rep progression at RIR 2</x:v>
+      </x:c>
+      <x:c r="M537" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N537" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="538" ht="42" customHeight="1">
+      <x:c r="A538" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B538" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C538" s="170" t="str">
+        <x:v>Face Pull</x:v>
+      </x:c>
+      <x:c r="D538" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E538" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F538" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G538" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H538" s="170" t="str">
+        <x:v>No reported form breakdown; rope path and lean-back To verify</x:v>
+      </x:c>
+      <x:c r="I538" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J538" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K538" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L538" s="170" t="str">
+        <x:v>Comfortably below failure</x:v>
+      </x:c>
+      <x:c r="M538" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N538" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="539" ht="42" customHeight="1">
+      <x:c r="A539" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B539" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C539" s="170" t="str">
+        <x:v>Face Pull</x:v>
+      </x:c>
+      <x:c r="D539" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E539" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F539" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G539" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H539" s="170" t="str">
+        <x:v>No reported form breakdown; rope path and lean-back To verify</x:v>
+      </x:c>
+      <x:c r="I539" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J539" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K539" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L539" s="170" t="str">
+        <x:v>Improved reserve</x:v>
+      </x:c>
+      <x:c r="M539" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N539" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="540" ht="42" customHeight="1">
+      <x:c r="A540" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B540" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C540" s="170" t="str">
+        <x:v>Face Pull</x:v>
+      </x:c>
+      <x:c r="D540" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E540" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F540" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G540" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H540" s="170" t="str">
+        <x:v>No reported form breakdown; rope path and lean-back To verify</x:v>
+      </x:c>
+      <x:c r="I540" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J540" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K540" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L540" s="170" t="str">
+        <x:v>Extra third set retained; no volume increase</x:v>
+      </x:c>
+      <x:c r="M540" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N540" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="541" ht="42" customHeight="1">
+      <x:c r="A541" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B541" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C541" s="170" t="str">
+        <x:v>Dumbbell Shrug</x:v>
+      </x:c>
+      <x:c r="D541" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E541" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F541" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G541" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H541" s="170" t="str">
+        <x:v>Clean and unassisted; top-pause duration/range To verify</x:v>
+      </x:c>
+      <x:c r="I541" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J541" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K541" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L541" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M541" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N541" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="542" ht="42" customHeight="1">
+      <x:c r="A542" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B542" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C542" s="170" t="str">
+        <x:v>Dumbbell Shrug</x:v>
+      </x:c>
+      <x:c r="D542" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E542" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F542" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G542" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H542" s="170" t="str">
+        <x:v>Clean and unassisted; top-pause duration/range To verify</x:v>
+      </x:c>
+      <x:c r="I542" s="170" t="str">
+        <x:v>No post-session chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="J542" s="170" t="str">
+        <x:v>Medium to Low final; starting energy To verify</x:v>
+      </x:c>
+      <x:c r="K542" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L542" s="170" t="str">
+        <x:v>Target met; add rep before load</x:v>
+      </x:c>
+      <x:c r="M542" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N542" s="170" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -26577,7 +27457,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e00955fc7024f2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R225780325b944d78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26834,25 +27714,25 @@
         <x:v>Incline DB Press</x:v>
       </x:c>
       <x:c r="C10" s="222" t="str">
-        <x:v>22.5 kg × 8</x:v>
+        <x:v>25 kg each x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D10" s="222" t="str">
-        <x:v>20–22.5 kg</x:v>
+        <x:v>20-25 kg each</x:v>
       </x:c>
       <x:c r="E10" s="222" t="str">
-        <x:v>22.5 kg × 9–10</x:v>
+        <x:v>20 kg x15 @3; 22.5 kg x13 @2; 25 kg x10 @2</x:v>
       </x:c>
       <x:c r="F10" s="222" t="str">
-        <x:v>Add reps first</x:v>
+        <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G10" s="222" t="str">
-        <x:v>Bench 30–45°</x:v>
+        <x:v>Moderate incline; shoulder blades set</x:v>
       </x:c>
       <x:c r="H10" s="222" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I10" s="222" t="str">
-        <x:v>Each dumbbell</x:v>
+        <x:v>Current baseline refreshed 2026-09-04; no assistance or pain</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="40" hidden="0" customHeight="1">
@@ -26863,25 +27743,25 @@
         <x:v>Plate Chest Press</x:v>
       </x:c>
       <x:c r="C11" s="222" t="str">
-        <x:v>50 kg/side x 8 @ RIR 1 unplanned</x:v>
+        <x:v>50 kg reported x9 @ RIR 2; load basis To verify</x:v>
       </x:c>
       <x:c r="D11" s="222" t="str">
-        <x:v>30-45 kg/side</x:v>
+        <x:v>30-50 kg reported; total vs per side To verify</x:v>
       </x:c>
       <x:c r="E11" s="222" t="str">
-        <x:v>45 kg/side x 9-10 @ RIR 2</x:v>
+        <x:v>Prep 20 kg x10-12 @5; 30 x15 @3; 40 x14-15 @3; 50 x10 @2</x:v>
       </x:c>
       <x:c r="F11" s="222" t="str">
-        <x:v>Do not use 50 kg yet</x:v>
+        <x:v>Verify load basis, then add reps</x:v>
       </x:c>
       <x:c r="G11" s="222" t="str">
-        <x:v>Controlled eccentric</x:v>
+        <x:v>Shoulder blades against pad; controlled depth</x:v>
       </x:c>
       <x:c r="H11" s="222" t="str">
-        <x:v>Modify load/volume</x:v>
+        <x:v>In progress / To verify</x:v>
       </x:c>
       <x:c r="I11" s="222" t="str">
-        <x:v>50 kg was an unplanned third set and receives no progression credit</x:v>
+        <x:v>Prior per-side convention conflicts with unreconfirmed current basis; preserve uncertainty</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="40" hidden="0" customHeight="1">
@@ -27379,16 +28259,16 @@
         <x:v>Face Pull</x:v>
       </x:c>
       <x:c r="C29" s="170" t="str">
-        <x:v>40 kg x 12 @ RIR 1</x:v>
+        <x:v>45 kg x10 @ RIR 3</x:v>
       </x:c>
       <x:c r="D29" s="170" t="str">
-        <x:v>30-40 kg total stack</x:v>
+        <x:v>40-45 kg total stack</x:v>
       </x:c>
       <x:c r="E29" s="170" t="str">
-        <x:v>40 kg x 13-15 @ RIR 2</x:v>
+        <x:v>Exactly 2 sets: 40 kg x12-13 @3; 45 kg x10-11 @2-3</x:v>
       </x:c>
       <x:c r="F29" s="170" t="str">
-        <x:v>Add controlled reps before load</x:v>
+        <x:v>No third set; add controlled reps</x:v>
       </x:c>
       <x:c r="G29" s="170" t="str">
         <x:v>Rope to eye/forehead; no lean-back</x:v>
@@ -27397,7 +28277,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I29" s="170" t="str">
-        <x:v>45 kg x 10 @ RIR 2 only if the path stays clean</x:v>
+        <x:v>35 kg x15 @4 was extra low-fatigue work; 3 sets completed despite 2-set plan</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -27466,25 +28346,25 @@
         <x:v>Dumbbell Shrugs</x:v>
       </x:c>
       <x:c r="C32" s="170" t="str">
-        <x:v>40 kg each x 9 @ RIR 2</x:v>
+        <x:v>40 kg each x12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D32" s="170" t="str">
-        <x:v>30-40 kg each</x:v>
+        <x:v>35-40 kg each</x:v>
       </x:c>
       <x:c r="E32" s="170" t="str">
-        <x:v>40 kg each x 10 @ RIR 2</x:v>
+        <x:v>35 kg each x15-16 @3; 40 kg each x13 @2</x:v>
       </x:c>
       <x:c r="F32" s="170" t="str">
         <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G32" s="170" t="str">
-        <x:v>Vertical shrug; top pause; straight arms</x:v>
+        <x:v>Vertical shrug; one-second top pause; straight arms</x:v>
       </x:c>
       <x:c r="H32" s="170" t="str">
         <x:v>Active / Preferred</x:v>
       </x:c>
       <x:c r="I32" s="170" t="str">
-        <x:v>35 kg and 40 kg finished below repetition targets; keep loads</x:v>
+        <x:v>Both planned sets achieved; exact top pause To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="48" hidden="0" customHeight="1">
@@ -27756,25 +28636,25 @@
         <x:v>Low-to-High Cable Fly</x:v>
       </x:c>
       <x:c r="C42" s="170" t="str">
-        <x:v>10 kg/side x 15 @ RIR 3</x:v>
+        <x:v>30 kg reported x8 @ RIR 2; load basis To verify</x:v>
       </x:c>
       <x:c r="D42" s="170" t="str">
-        <x:v>5-10 kg/side</x:v>
+        <x:v>20-30 kg reported; per-side basis To verify</x:v>
       </x:c>
       <x:c r="E42" s="170" t="str">
-        <x:v>10 kg/side x 16-18 @ RIR 2-3</x:v>
+        <x:v>One 15 kg prep; 20 x15-16 @3; 25 x13 @2; 30 x9 @2</x:v>
       </x:c>
       <x:c r="F42" s="170" t="str">
-        <x:v>Add reps first</x:v>
+        <x:v>Add reps before load; remove redundant prep</x:v>
       </x:c>
       <x:c r="G42" s="170" t="str">
         <x:v>Soft elbow bend; low-to-high arc</x:v>
       </x:c>
       <x:c r="H42" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>In progress / To verify</x:v>
       </x:c>
       <x:c r="I42" s="170" t="str">
-        <x:v>Use instead of extra fly volume</x:v>
+        <x:v>10 and 15 kg produced no meaningful stimulus; exact cable load basis To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="38" customHeight="1">
@@ -27843,25 +28723,25 @@
         <x:v>Cable Upright Row</x:v>
       </x:c>
       <x:c r="C45" s="170" t="str">
-        <x:v>60 kg x 9 @ RIR 2 unplanned</x:v>
+        <x:v>60 kg x10 @ RIR 2</x:v>
       </x:c>
       <x:c r="D45" s="170" t="str">
-        <x:v>40-50 kg stack</x:v>
+        <x:v>40-60 kg total stack</x:v>
       </x:c>
       <x:c r="E45" s="170" t="str">
-        <x:v>50 kg x 11-12 @ RIR 2</x:v>
+        <x:v>40 kg x15 @3; 50 kg x13 @3; 60 kg x11 @2</x:v>
       </x:c>
       <x:c r="F45" s="170" t="str">
-        <x:v>No 60 kg until both 50 kg sets qualify</x:v>
+        <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G45" s="170" t="str">
-        <x:v>Pull only to comfortable height</x:v>
+        <x:v>Pull only to comfortable height; elbows no higher than shoulders</x:v>
       </x:c>
       <x:c r="H45" s="170" t="str">
-        <x:v>Modify load</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I45" s="170" t="str">
-        <x:v>60 kg was clean but above plan; effective stack resistance To verify</x:v>
+        <x:v>No shoulder pinching; 50 kg reserve and 60 kg reps improved</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="48" customHeight="1">
@@ -28063,7 +28943,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfd47d7feb13407a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b8a727b7d243d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29150,24 +30030,38 @@
       <x:c r="P32" s="59" t="n"/>
       <x:c r="Q32" s="59" t="n"/>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33"/>
-      <x:c r="B33"/>
-      <x:c r="C33"/>
-      <x:c r="D33"/>
-      <x:c r="E33"/>
-      <x:c r="F33"/>
-      <x:c r="G33"/>
-      <x:c r="H33"/>
-      <x:c r="I33"/>
-      <x:c r="J33"/>
-      <x:c r="K33" s="59" t="n"/>
-      <x:c r="L33" s="59" t="n"/>
-      <x:c r="M33" s="59" t="n"/>
-      <x:c r="N33" s="59" t="n"/>
-      <x:c r="O33" s="59" t="n"/>
-      <x:c r="P33" s="59" t="n"/>
-      <x:c r="Q33" s="59" t="n"/>
+    <x:row r="33" ht="105" customHeight="1">
+      <x:c r="A33" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B33" s="170"/>
+      <x:c r="C33" s="170"/>
+      <x:c r="D33" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E33" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="F33" s="170" t="str">
+        <x:v>No chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; pre-session soreness/pain To verify</x:v>
+      </x:c>
+      <x:c r="G33" s="170"/>
+      <x:c r="H33" s="170"/>
+      <x:c r="I33" s="170" t="str">
+        <x:v>Chest + Shoulders workout - 90 min total; 17 working sets plus three preparation sets; medium pump; 20 min treadmill at 3 km/h and 12% incline</x:v>
+      </x:c>
+      <x:c r="J33" s="170" t="str">
+        <x:v>Starting energy To verify; half EAA+ (~50 mg caffeine) plus half pre-workout (~100 mg user-stated; label To verify); no coffee; no assistance/form breakdown; 3 g creatine started post-workout with whey; rail support and cardio symptoms To verify</x:v>
+      </x:c>
+      <x:c r="K33" s="222"/>
+      <x:c r="L33" s="222"/>
+      <x:c r="M33" s="222"/>
+      <x:c r="N33" s="222"/>
+      <x:c r="O33" s="222"/>
+      <x:c r="P33" s="222"/>
+      <x:c r="Q33" s="222"/>
+      <x:c r="R33" s="170"/>
+      <x:c r="S33" s="170"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34"/>
@@ -32398,7 +33292,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ede55c7f20c4c52"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2860e484e07a4b58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33819,13 +34713,83 @@
         <x:v>No compensatory cardio; require fresh readiness and no unplanned sets for Chest + Shoulders</x:v>
       </x:c>
     </x:row>
+    <x:row r="97" ht="75" customHeight="1">
+      <x:c r="A97" s="170" t="str">
+        <x:v>Friday secondary-exposure correction</x:v>
+      </x:c>
+      <x:c r="B97" s="170" t="str">
+        <x:v>Chest + Shoulders on 2026-09-04 used plate chest press, incline dumbbell press, low-to-high cable fly, cable upright row, face pull and dumbbell shrug</x:v>
+      </x:c>
+      <x:c r="C97" s="170" t="str">
+        <x:v>This avoids simply repeating Monday chest and Wednesday shoulder sessions while preserving second weekly exposure</x:v>
+      </x:c>
+      <x:c r="D97" s="170" t="str">
+        <x:v>Keep Friday as the B session; no direct shoulder press after Wednesday pressing unless the block is redesigned</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="75" customHeight="1">
+      <x:c r="A98" s="170" t="str">
+        <x:v>Chest + Shoulders performance</x:v>
+      </x:c>
+      <x:c r="B98" s="170" t="str">
+        <x:v>17 working sets plus three preparation sets completed pain-free; no RIR 1/0, assistance, breakdown or upright-row pinching</x:v>
+      </x:c>
+      <x:c r="C98" s="170" t="str">
+        <x:v>Current incline-dumbbell, cable-fly and upright-row baselines progressed; final energy was Medium-Low</x:v>
+      </x:c>
+      <x:c r="D98" s="170" t="str">
+        <x:v>Keep rep-led progression and remove one redundant cable-fly preparation set and the extra face-pull set next time</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="75" customHeight="1">
+      <x:c r="A99" s="170" t="str">
+        <x:v>Creatine monohydrate started</x:v>
+      </x:c>
+      <x:c r="B99" s="170" t="str">
+        <x:v>Vipin confirmed one stated 3 g scoop post-workout with whey on 2026-09-04</x:v>
+      </x:c>
+      <x:c r="C99" s="170" t="str">
+        <x:v>Daily consistency matters more than workout timing; a small muscle-water scale increase must not be classified as fat gain</x:v>
+      </x:c>
+      <x:c r="D99" s="170" t="str">
+        <x:v>Continue 3 g daily including rest days; product label and scoop accuracy To verify; NIH source https://ods.od.nih.gov/factsheets/ExerciseAndAthleticPerformance-HealthProfessional/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="75" customHeight="1">
+      <x:c r="A100" s="170" t="str">
+        <x:v>Caffeine routine changed</x:v>
+      </x:c>
+      <x:c r="B100" s="170" t="str">
+        <x:v>2026-09-04 used half EAA+ (~50 mg label-derived) plus half pre-workout (~100 mg user-stated), no coffee; estimated total ~150 mg</x:v>
+      </x:c>
+      <x:c r="C100" s="170" t="str">
+        <x:v>Only the EAA contribution is label-verified and late caffeine may worsen sleep despite acceptable daily totals</x:v>
+      </x:c>
+      <x:c r="D100" s="170" t="str">
+        <x:v>Obtain full pre-workout label; prefer one caffeine source and monitor bedtime, sleep onset, awakenings and morning freshness; FDA source https://www.fda.gov/consumers/consumer-updates/spilling-beans-how-much-caffeine-too-much</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="75" customHeight="1">
+      <x:c r="A101" s="170" t="str">
+        <x:v>Magnesium glycinate planned</x:v>
+      </x:c>
+      <x:c r="B101" s="170" t="str">
+        <x:v>No dose or first use confirmed; product label and elemental-magnesium amount To verify</x:v>
+      </x:c>
+      <x:c r="C101" s="170" t="str">
+        <x:v>Evidence indicates at most a modest average sleep benefit and magnesium will not offset late caffeine</x:v>
+      </x:c>
+      <x:c r="D101" s="170" t="str">
+        <x:v>Review label before use and count elemental magnesium from all supplements; NIH source https://ods.od.nih.gov/factsheets/Magnesium-HealthProfessional/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd23a4e59f3845bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f393a3d937841b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34624,6 +35588,32 @@
         <x:v>Chest + Shoulders next after fresh readiness; next Legs exactly three leg-press sets, planned RDL top load returns to 15 kg each, improve leg-curl reserve, and use three calf sets within the 18-set ceiling</x:v>
       </x:c>
     </x:row>
+    <x:row r="31" ht="125" customHeight="1">
+      <x:c r="A31" s="220" t="n">
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="B31" s="170" t="str">
+        <x:v>Chest + Shoulders</x:v>
+      </x:c>
+      <x:c r="C31" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D31" s="170" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E31" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F31" s="170" t="str">
+        <x:v>Good sleep; starting energy and pre-session soreness/pain To verify; Medium-to-Low final energy; no post-session pain or upright-row pinching; 90 min including 20 min treadmill; medium chest/shoulder pump; no assistance or form breakdown; half EAA+ plus half pre-workout, approximately 150 mg combined caffeine with pre-workout label To verify; no coffee; 3 g creatine started post-workout</x:v>
+      </x:c>
+      <x:c r="G31" s="170" t="str">
+        <x:v>Seventeen working sets plus three genuine preparation sets were completed with no RIR 1/0, pain, pinching or assistance. Friday exercise selection differed from Monday and Wednesday, and incline-dumbbell, low-to-high-fly and upright-row baselines progressed. The extra face-pull set and 20 min at 12% incline increased fatigue on the fifth consecutive training day; final energy was Medium-Low.</x:v>
+      </x:c>
+      <x:c r="H31" s="170" t="str">
+        <x:v>Back + Biceps only after Good sleep, at least Medium starting energy and no meaningful soreness/pain; cap at 16 working sets, use one chest-supported-row variation, keep RIR 2-3 and omit post-lift cardio</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -34636,7 +35626,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f72309f3f14a60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red70f3afc57f484c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34813,13 +35803,13 @@
         <x:v>Current pain or movement restrictions</x:v>
       </x:c>
       <x:c r="C10" s="170" t="str">
-        <x:v>After Legs + Calves on 2026-09-03: no hip, knee, lower-back or other pain; no assistance or reported form breakdown.</x:v>
+        <x:v>After Chest + Shoulders on 2026-09-04: no chest, shoulder, elbow, wrist or upper-biceps pain; no upright-row shoulder pinching; no assistance or reported form breakdown.</x:v>
       </x:c>
       <x:c r="D10" s="170" t="str">
-        <x:v>Known</x:v>
+        <x:v>Known with pre-session gap</x:v>
       </x:c>
       <x:c r="E10" s="170" t="str">
-        <x:v>Fresh chest, shoulder and joint readiness before Chest + Shoulders; monitor delayed leg soreness</x:v>
+        <x:v>Fresh Back + Biceps readiness; pre-session soreness/pain for 2026-09-04 remains To verify</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -34993,7 +35983,7 @@
         <x:v>Recommendations can use full commercial-gym options</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="21" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A21" s="170" t="str">
         <x:v>Training</x:v>
       </x:c>
@@ -35001,13 +35991,13 @@
         <x:v>Current sequence</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday through Thursday completed this week.</x:v>
+        <x:v>Active six-day split: Mon Chest+Triceps; Tue Back+Biceps; Wed Shoulders+Triceps; Thu Legs+Calves; Fri Chest+Shoulders; Sat Back+Biceps; Sun rest. Monday through Friday completed this week.</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
         <x:v>Known / active four-week block</x:v>
       </x:c>
       <x:c r="E21" s="170" t="str">
-        <x:v>Chest + Shoulders next; no unplanned sets and cardio only if final energy remains Medium or higher</x:v>
+        <x:v>Back + Biceps only after recovery threshold; 16 working-set cap and no cardio</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -35095,7 +36085,7 @@
         <x:v>Quantify cooked lentils next, then sabji; yogurt labels/serving weights remain To verify</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="27" ht="66" hidden="0" customHeight="1">
       <x:c r="A27" s="170" t="str">
         <x:v>Nutrition</x:v>
       </x:c>
@@ -35103,13 +36093,13 @@
         <x:v>Supplements currently used</x:v>
       </x:c>
       <x:c r="C27" s="170" t="str">
-        <x:v>MuscleTech multivitamin; fish oil; MuscleTech EAA+ Energy (user reports always taking one full 13.2 g scoop: 100 mg caffeine and 7.49 g EAAs); Ultimate Nutrition Prostar whey post-workout; Run Nutrition yeast whey at breakfast; Kapiva shilajit 500 mg after lunch</x:v>
+        <x:v>MuscleTech multivitamin; fish oil; MuscleTech EAA+ Energy now reported as half scoop; unidentified pre-workout reported as half scoop; Ultimate Nutrition Prostar whey post-workout; Run Nutrition yeast whey at breakfast; Kapiva shilajit 500 mg after lunch; creatine monohydrate started 2026-09-04 at one stated 3 g scoop post-workout. Magnesium glycinate planned but not started.</x:v>
       </x:c>
       <x:c r="D27" s="170" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E27" s="170" t="str">
-        <x:v>EAA serving habit and label verified; remaining supplement labels still needed</x:v>
+        <x:v>Obtain pre-workout, creatine and magnesium labels; verify elemental magnesium and all stimulant ingredients</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -35120,13 +36110,13 @@
         <x:v>Late caffeine exposure</x:v>
       </x:c>
       <x:c r="C28" s="170" t="str">
-        <x:v>Every workout normally includes one full EAA+ Energy scoop (100 mg caffeine). No black coffee is now the standing workout default unless Vipin reports an exception.</x:v>
+        <x:v>On 2026-09-04, half EAA+ supplied approximately 50 mg label-derived caffeine and half pre-workout supplied approximately 100 mg according to the unverified product claim; no coffee. Estimated total approximately 150 mg.</x:v>
       </x:c>
       <x:c r="D28" s="170" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="E28" s="170" t="str">
-        <x:v>Continue comparing sleep and morning freshness; EAA still provides late caffeine</x:v>
+        <x:v>Track sleep response and avoid treating two caffeine products as the standing routine until the pre-workout label is reviewed</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -35206,7 +36196,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb57474d248f4531"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce14ab8a42494eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35433,30 +36423,30 @@
         <x:v>Adjust for heat and sweat; avoid forcing excessive water</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="132" hidden="0" customHeight="1">
+    <x:row r="10" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A10" s="153" t="str">
         <x:v>Caffeine / sleep</x:v>
       </x:c>
       <x:c r="B10" s="156" t="str">
-        <x:v>100 mg caffeine from a full EAA+ Energy serving; coffee adds an unknown amount</x:v>
+        <x:v>Approximately 150 mg on 2026-09-04 from half EAA+ plus half pre-workout; no coffee</x:v>
       </x:c>
       <x:c r="C10" s="156" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="D10" s="156" t="str">
-        <x:v>Workout EAA+ label provides 100 mg caffeine. On the 2026-08-09 rest day, EAA+ was omitted; Vipin slept ~23:30-08:00 (~8.5 h) and woke fresh on 2026-08-10.</x:v>
+        <x:v>EAA label confirms 100 mg per full scoop, so half is approximately 50 mg. Pre-workout full-scoop 200 mg and half-scoop 100 mg are user-stated only.</x:v>
       </x:c>
       <x:c r="E10" s="156" t="str">
-        <x:v>Whether the improvement came from no EAA+ caffeine, the earlier chosen bedtime, rest-day recovery, or their combination; other caffeine intake that day was not reconfirmed</x:v>
+        <x:v>Pre-workout product, full ingredient panel, serving mass, other stimulants and exact dose</x:v>
       </x:c>
       <x:c r="F10" s="156" t="str">
-        <x:v>Continue avoiding extra black coffee. Compare several workout nights using EAA+ with caffeine-free rest nights; record bedtime, wake time, awakenings and morning freshness.</x:v>
+        <x:v>Prefer one caffeine source for late training; collect several sleep nights before judging tolerance</x:v>
       </x:c>
       <x:c r="G10" s="156" t="str">
-        <x:v>At least 5-7 comparable nights, including workout and rest days</x:v>
+        <x:v>Pre-workout label review plus 5-7 comparable sleep nights</x:v>
       </x:c>
       <x:c r="H10" s="158" t="str">
-        <x:v>This is the strongest caffeine-free rest-night datapoint so far, but one night is not causal proof.</x:v>
+        <x:v>Late caffeine remains the main modifiable sleep variable; FDA source https://www.fda.gov/consumers/consumer-updates/spilling-beans-how-much-caffeine-too-much</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -35485,30 +36475,30 @@
         <x:v>Dinner timing should not compromise sleep comfort</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="66" hidden="0" customHeight="1">
+    <x:row r="12" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A12" s="159" t="str">
         <x:v>Supplements</x:v>
       </x:c>
       <x:c r="B12" s="162" t="str">
-        <x:v>EAA+ Energy label verified; remaining supplement labels pending</x:v>
+        <x:v>Creatine monohydrate active at 3 g/day reported; half EAA+ active on 2026-09-04; pre-workout and magnesium labels pending</x:v>
       </x:c>
       <x:c r="C12" s="162" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="D12" s="162" t="str">
-        <x:v>1 scoop (13.2 g): 7.49 g EAAs, 100 mg caffeine, 3 kcal; label says once daily</x:v>
+        <x:v>Creatine first dose confirmed post-workout 2026-09-04. EAA label verified. Magnesium glycinate planned only.</x:v>
       </x:c>
       <x:c r="E12" s="162" t="str">
-        <x:v>Actual scoop used; labels for multivitamin, fish oil, whey products and shilajit</x:v>
+        <x:v>Creatine scoop accuracy/product label; pre-workout label; magnesium elemental dose; multivitamin magnesium</x:v>
       </x:c>
       <x:c r="F12" s="162" t="str">
-        <x:v>For late workouts, replace with caffeine-free EAA/electrolyte or water when practical</x:v>
+        <x:v>Continue creatine 3 g daily; review stimulant and magnesium labels before finalizing routine</x:v>
       </x:c>
       <x:c r="G12" s="162" t="str">
-        <x:v>Sleep trial and remaining label review</x:v>
+        <x:v>Daily creatine adherence, sleep response and label review</x:v>
       </x:c>
       <x:c r="H12" s="164" t="str">
-        <x:v>Do not exceed the package maximum of one serving daily</x:v>
+        <x:v>NIH creatine source https://ods.od.nih.gov/factsheets/ExerciseAndAthleticPerformance-HealthProfessional/; NIH magnesium source https://ods.od.nih.gov/factsheets/Magnesium-HealthProfessional/</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -35677,7 +36667,7 @@
         <x:v>Current confirmed sandwich remains quantified at 8.99 g protein. Proposed cutting substitution is 2 whole eggs + 2 whites; do not count until actual intake is confirmed.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="20" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A20" s="170" t="str">
         <x:v>Pre-workout</x:v>
       </x:c>
@@ -35685,21 +36675,23 @@
         <x:v>Before ~21:00 workout</x:v>
       </x:c>
       <x:c r="C20" s="170" t="str">
-        <x:v>Half-spoon black coffee; banana or another fruit</x:v>
+        <x:v>MuscleTech EAA+ Energy, Sour Apple; current reported workout amount changed to half scoop on 2026-09-04</x:v>
       </x:c>
       <x:c r="D20" s="371"/>
-      <x:c r="E20" s="170"/>
+      <x:c r="E20" s="170" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
       <x:c r="F20" s="170" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Exact half-scoop powder weight and whether this remains the standing routine</x:v>
       </x:c>
       <x:c r="G20" s="170" t="str">
-        <x:v>Coffee type/grams and caffeine; fruit quantity</x:v>
+        <x:v>Half of the verified full serving is approximately 3.745 g EAAs and 50 mg caffeine; do not count as dietary protein</x:v>
       </x:c>
       <x:c r="H20" s="170" t="str">
-        <x:v>Late caffeine is a sleep variable; Current no-coffee trial: omitted on 2026-08-07 and 2026-08-08</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="184.8000030517578" hidden="0" customHeight="1">
+        <x:v>Do not combine routinely with another caffeinated product until its label is reviewed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A21" s="170" t="str">
         <x:v>During workout</x:v>
       </x:c>
@@ -35707,21 +36699,22 @@
         <x:v>During ~21:00 workout</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>MuscleTech EAA+ Energy, Sour Apple
-Label serving: 1 scoop (13.2 g) in 240 mL cold water</x:v>
-      </x:c>
-      <x:c r="D21" s="371"/>
-      <x:c r="E21" s="170" t="n">
-        <x:v>3</x:v>
+        <x:v>Ultimate Nutrition Prostar whey (25 g protein) plus one stated 3 g scoop creatine monohydrate after training</x:v>
+      </x:c>
+      <x:c r="D21" s="371" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E21" s="170" t="str">
+        <x:v>Partial / To verify</x:v>
       </x:c>
       <x:c r="F21" s="170" t="str">
-        <x:v>Active</x:v>
+        <x:v>Exact whey serving/label; creatine product label and scoop accuracy</x:v>
       </x:c>
       <x:c r="G21" s="170" t="str">
-        <x:v>User confirmed on 2026-08-09 that every workout uses one full level scoop</x:v>
+        <x:v>Continue 3 g creatine daily, including rest days</x:v>
       </x:c>
       <x:c r="H21" s="170" t="str">
-        <x:v>Actual serving: 13.2 g, 7.49 g EAAs and 100 mg caffeine; no black coffee before today's workout; Equal workout energy without coffee reported after 2026-08-07 Shoulder session; overnight sleep and morning freshness pending; Follow-up 2026-08-08: ~8 h subjectively very good sleep and refreshed, energetic morning despite 100 mg EAA+ caffeine; bedtime was deliberately delayed, so continue tracking; Triceps session 2026-08-08 started ~18:30: EAA+ used, no black coffee, medium workout energy; serving amount not reconfirmed (To verify); Routine confirmed 2026-08-09: full 13.2 g scoop every workout, so the 2026-08-08 Triceps serving is resolved as 100 mg caffeine and 7.49 g EAAs</x:v>
+        <x:v>Creatine began 2026-09-04; timing is for convenience and consistency</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -36309,10 +37302,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb77180a5124e85"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ba31e2bd6944c48"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25134b61f8ec4cf9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f9dd789cb6c45fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5932c49ecb14278"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0555e607cad470d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2564ddcfaf044283"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fbb91674952403d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 5 back and biceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R25bde1780882414a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Re7908410721d4f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R3b455d177ab64146"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rb7a24c0890044062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R51bb39bd551b4431"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R7c90d73a2799405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R2e360cde33dd40b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R48bb77fa33a243ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R21954db5f6ec4f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rb4611fc9255e4ec8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R5145d3d85b474ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf118392d3ebf47f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rd831fba28df44f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Ra2a92ca9051c4a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rd8e224c000094618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rc5d3db7844d841d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R47dd1b1e28a74d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rbd8de373c58b40cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R58f8c26227884543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R530acca548c84ff1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R1df081cb3e754875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R57159138c7aa4441"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdc246d21dce34e74"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9a5905c832a24c30"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7c092a1ca724cae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86a6b5c6433a46db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0aa34563b20425b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4fd853c4ac948c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,11 +4083,11 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="str">
@@ -4421,7 +4421,7 @@
         <x:v>Saturday</x:v>
       </x:c>
       <x:c r="B18" s="59" t="str">
-        <x:v>Back + Biceps; Sunday rest</x:v>
+        <x:v>Back + Biceps - completed 2026-09-05</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="59" t="str">
@@ -4447,8 +4447,12 @@
       <x:c r="L18" s="59" t="n"/>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="92"/>
-      <x:c r="B19" s="59"/>
+      <x:c r="A19" s="92" t="str">
+        <x:v>Sunday</x:v>
+      </x:c>
+      <x:c r="B19" s="59" t="str">
+        <x:v>Complete rest / recovery</x:v>
+      </x:c>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="59" t="str">
         <x:v>Legs</x:v>
@@ -4561,16 +4565,16 @@
         <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>Low after 80 min</x:v>
+        <x:v>Medium-Low after 90 min</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Fresh readiness required</x:v>
+        <x:v>Complete rest Sunday</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
         <x:v>Monitor</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>No cardio today</x:v>
+        <x:v>Six consecutive training days completed</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4584,19 +4588,19 @@
         <x:v>Next</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Chest + Triceps</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>Five days completed</x:v>
+        <x:v>Six-day block completed</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>16 working sets; no cardio</x:v>
+        <x:v>Fresh readiness; 16-18 working sets</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>Train only after fresh readiness</x:v>
+        <x:v>No failure; cardio only if recovery supports it</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4625,7 +4629,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R505cd8568a5b4cb9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1964c19385aa47c6"/>
 </x:worksheet>
 </file>
 
@@ -27423,6 +27427,930 @@
       </x:c>
       <x:c r="N542" s="170" t="n">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="543" ht="48" customHeight="1">
+      <x:c r="A543" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B543" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C543" s="170" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D543" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E543" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F543" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G543" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H543" s="170" t="str">
+        <x:v>Controlled and unassisted; intended preparation became meaningful working volume at RIR 3</x:v>
+      </x:c>
+      <x:c r="I543" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J543" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K543" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L543" s="170" t="str">
+        <x:v>Working-volume classification based on achieved effort; remove this extra set next time</x:v>
+      </x:c>
+      <x:c r="M543" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N543" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="544" ht="48" customHeight="1">
+      <x:c r="A544" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B544" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C544" s="170" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D544" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E544" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F544" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G544" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H544" s="170" t="str">
+        <x:v>Controlled and unassisted; exact machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I544" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J544" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K544" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L544" s="170" t="str">
+        <x:v>Target exceeded with reserve</x:v>
+      </x:c>
+      <x:c r="M544" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N544" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="545" ht="48" customHeight="1">
+      <x:c r="A545" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B545" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C545" s="170" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D545" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E545" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F545" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G545" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H545" s="170" t="str">
+        <x:v>Controlled and unassisted; exact machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I545" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J545" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K545" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L545" s="170" t="str">
+        <x:v>Improved reserve</x:v>
+      </x:c>
+      <x:c r="M545" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N545" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="546" ht="48" customHeight="1">
+      <x:c r="A546" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B546" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C546" s="170" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D546" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E546" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F546" s="170" t="str">
+        <x:v>kg plates each side; machine carriage excluded</x:v>
+      </x:c>
+      <x:c r="G546" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H546" s="170" t="str">
+        <x:v>Controlled and unassisted; exact machine setup/range To verify</x:v>
+      </x:c>
+      <x:c r="I546" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J546" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K546" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L546" s="170" t="str">
+        <x:v>Strong current baseline; add no load</x:v>
+      </x:c>
+      <x:c r="M546" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N546" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="547" ht="48" customHeight="1">
+      <x:c r="A547" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B547" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C547" s="170" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D547" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E547" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F547" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G547" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H547" s="170" t="str">
+        <x:v>No reported form breakdown; elbow position and lat isolation To verify</x:v>
+      </x:c>
+      <x:c r="I547" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J547" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K547" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L547" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M547" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N547" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="548" ht="48" customHeight="1">
+      <x:c r="A548" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B548" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C548" s="170" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D548" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E548" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F548" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G548" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H548" s="170" t="str">
+        <x:v>No reported form breakdown; elbow position and lat isolation To verify</x:v>
+      </x:c>
+      <x:c r="I548" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J548" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K548" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L548" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M548" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N548" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="549" ht="48" customHeight="1">
+      <x:c r="A549" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B549" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C549" s="170" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D549" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E549" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F549" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G549" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H549" s="170" t="str">
+        <x:v>No reported form breakdown; elbow position and lat isolation To verify</x:v>
+      </x:c>
+      <x:c r="I549" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J549" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K549" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L549" s="170" t="str">
+        <x:v>Target met; add rep before load</x:v>
+      </x:c>
+      <x:c r="M549" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N549" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="550" ht="48" customHeight="1">
+      <x:c r="A550" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B550" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C550" s="170" t="str">
+        <x:v>Single-Arm Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D550" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E550" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F550" s="170" t="str">
+        <x:v>kg selected stack for each working arm; exact station/calibration To verify</x:v>
+      </x:c>
+      <x:c r="G550" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H550" s="170" t="str">
+        <x:v>No reported form breakdown; torso rotation and side-to-side match To verify</x:v>
+      </x:c>
+      <x:c r="I550" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J550" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K550" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L550" s="170" t="str">
+        <x:v>New unilateral baseline</x:v>
+      </x:c>
+      <x:c r="M550" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N550" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="551" ht="48" customHeight="1">
+      <x:c r="A551" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B551" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C551" s="170" t="str">
+        <x:v>Single-Arm Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D551" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E551" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F551" s="170" t="str">
+        <x:v>kg selected stack for each working arm; exact station/calibration To verify</x:v>
+      </x:c>
+      <x:c r="G551" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H551" s="170" t="str">
+        <x:v>No reported form breakdown; torso rotation and side-to-side match To verify</x:v>
+      </x:c>
+      <x:c r="I551" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J551" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K551" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L551" s="170" t="str">
+        <x:v>New unilateral baseline</x:v>
+      </x:c>
+      <x:c r="M551" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N551" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="552" ht="48" customHeight="1">
+      <x:c r="A552" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B552" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C552" s="170" t="str">
+        <x:v>Single-Arm Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="D552" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E552" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F552" s="170" t="str">
+        <x:v>kg selected stack for each working arm; exact station/calibration To verify</x:v>
+      </x:c>
+      <x:c r="G552" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H552" s="170" t="str">
+        <x:v>No reported form breakdown; torso rotation and side-to-side match To verify</x:v>
+      </x:c>
+      <x:c r="I552" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J552" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K552" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L552" s="170" t="str">
+        <x:v>New top-set baseline; add rep before load</x:v>
+      </x:c>
+      <x:c r="M552" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N552" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="553" ht="48" customHeight="1">
+      <x:c r="A553" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B553" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C553" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D553" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E553" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F553" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G553" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H553" s="170" t="str">
+        <x:v>No reported form breakdown; bar type and body swing To verify</x:v>
+      </x:c>
+      <x:c r="I553" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J553" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K553" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L553" s="170" t="str">
+        <x:v>Planned preparation became working volume at RIR 2</x:v>
+      </x:c>
+      <x:c r="M553" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N553" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554" ht="48" customHeight="1">
+      <x:c r="A554" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B554" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C554" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D554" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E554" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F554" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G554" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H554" s="170" t="str">
+        <x:v>No reported form breakdown; bar type and body swing To verify</x:v>
+      </x:c>
+      <x:c r="I554" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J554" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K554" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L554" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M554" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N554" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="555" ht="48" customHeight="1">
+      <x:c r="A555" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B555" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C555" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D555" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E555" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F555" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G555" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H555" s="170" t="str">
+        <x:v>No reported form breakdown; bar type and body swing To verify</x:v>
+      </x:c>
+      <x:c r="I555" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J555" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K555" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L555" s="170" t="str">
+        <x:v>Too close to failure; improve reserve</x:v>
+      </x:c>
+      <x:c r="M555" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N555" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556" ht="48" customHeight="1">
+      <x:c r="A556" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B556" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C556" s="170" t="str">
+        <x:v>Straight Bar Curl</x:v>
+      </x:c>
+      <x:c r="D556" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E556" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F556" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G556" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H556" s="170" t="str">
+        <x:v>No reported form breakdown; bar type and body swing To verify</x:v>
+      </x:c>
+      <x:c r="I556" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J556" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K556" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L556" s="170" t="str">
+        <x:v>Target met; retain load</x:v>
+      </x:c>
+      <x:c r="M556" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N556" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="557" ht="48" customHeight="1">
+      <x:c r="A557" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B557" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C557" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D557" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E557" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F557" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G557" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H557" s="170" t="str">
+        <x:v>No reported form breakdown; upper-arm contact To verify</x:v>
+      </x:c>
+      <x:c r="I557" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J557" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K557" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L557" s="170" t="str">
+        <x:v>Target met</x:v>
+      </x:c>
+      <x:c r="M557" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N557" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558" ht="48" customHeight="1">
+      <x:c r="A558" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B558" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C558" s="170" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D558" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E558" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F558" s="170" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G558" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H558" s="170" t="str">
+        <x:v>No reported form breakdown; upper-arm contact To verify</x:v>
+      </x:c>
+      <x:c r="I558" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J558" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K558" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L558" s="170" t="str">
+        <x:v>Target met; add rep before load</x:v>
+      </x:c>
+      <x:c r="M558" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N558" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559" ht="48" customHeight="1">
+      <x:c r="A559" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B559" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C559" s="170" t="str">
+        <x:v>Concentration Curl</x:v>
+      </x:c>
+      <x:c r="D559" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E559" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F559" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G559" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H559" s="170" t="str">
+        <x:v>No meaningful stimulus reported; exact tempo/range To verify</x:v>
+      </x:c>
+      <x:c r="I559" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J559" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K559" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L559" s="170" t="str">
+        <x:v>Low-fatigue preparation</x:v>
+      </x:c>
+      <x:c r="M559" s="170" t="str">
+        <x:v>Preparation</x:v>
+      </x:c>
+      <x:c r="N559" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="560" ht="48" customHeight="1">
+      <x:c r="A560" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B560" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C560" s="170" t="str">
+        <x:v>Concentration Curl</x:v>
+      </x:c>
+      <x:c r="D560" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E560" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F560" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G560" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H560" s="170" t="str">
+        <x:v>No reported form breakdown; elbow support and side-to-side match To verify</x:v>
+      </x:c>
+      <x:c r="I560" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J560" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K560" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L560" s="170" t="str">
+        <x:v>Improved reserve</x:v>
+      </x:c>
+      <x:c r="M560" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N560" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="561" ht="48" customHeight="1">
+      <x:c r="A561" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B561" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C561" s="170" t="str">
+        <x:v>Concentration Curl</x:v>
+      </x:c>
+      <x:c r="D561" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E561" s="170" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F561" s="170" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G561" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H561" s="170" t="str">
+        <x:v>No reported form breakdown; elbow support and side-to-side match To verify</x:v>
+      </x:c>
+      <x:c r="I561" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J561" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K561" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L561" s="170" t="str">
+        <x:v>Improved reserve; add rep before load</x:v>
+      </x:c>
+      <x:c r="M561" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N561" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="562" ht="48" customHeight="1">
+      <x:c r="A562" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B562" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C562" s="170" t="str">
+        <x:v>Reverse EZ Curl</x:v>
+      </x:c>
+      <x:c r="D562" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E562" s="170" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F562" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G562" s="170" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H562" s="170" t="str">
+        <x:v>No reported form breakdown; wrist position To verify</x:v>
+      </x:c>
+      <x:c r="I562" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J562" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K562" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L562" s="170" t="str">
+        <x:v>Controlled revised baseline</x:v>
+      </x:c>
+      <x:c r="M562" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N562" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="563" ht="48" customHeight="1">
+      <x:c r="A563" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B563" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C563" s="170" t="str">
+        <x:v>Reverse EZ Curl</x:v>
+      </x:c>
+      <x:c r="D563" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E563" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F563" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G563" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H563" s="170" t="str">
+        <x:v>No reported form breakdown; wrist position To verify</x:v>
+      </x:c>
+      <x:c r="I563" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="J563" s="170" t="str">
+        <x:v>Medium to High start; Medium to Low final</x:v>
+      </x:c>
+      <x:c r="K563" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L563" s="170" t="str">
+        <x:v>Reserve improved; add rep before load</x:v>
+      </x:c>
+      <x:c r="M563" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N563" s="170" t="n">
+        <x:v>3</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -27457,7 +28385,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R225780325b944d78"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raea59e7681a34c33"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27656,25 +28584,25 @@
         <x:v>Straight-Arm Pulldown</x:v>
       </x:c>
       <x:c r="C8" s="222" t="str">
-        <x:v>Not performed; replaced by second chest-supported row</x:v>
+        <x:v>50 kg x 12 @ RIR 2</x:v>
       </x:c>
       <x:c r="D8" s="222" t="str">
-        <x:v>45-50 kg</x:v>
+        <x:v>40-50 kg</x:v>
       </x:c>
       <x:c r="E8" s="222" t="str">
-        <x:v>50 kg x 12 @ RIR 2</x:v>
+        <x:v>40 kg x15 @3; 45 x15 @2; 50 x13 @2</x:v>
       </x:c>
       <x:c r="F8" s="222" t="str">
-        <x:v>Exactly 2 sets when established row machine is used</x:v>
+        <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G8" s="222" t="str">
-        <x:v>Elbows fixed</x:v>
+        <x:v>Soft elbows; pull with lats</x:v>
       </x:c>
       <x:c r="H8" s="222" t="str">
-        <x:v>Resume next Back session</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I8" s="222" t="str">
-        <x:v>Omitted to preserve 16-set ceiling after duplicate row variations</x:v>
+        <x:v>Three pain-free working sets completed</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="40" hidden="0" customHeight="1">
@@ -27886,16 +28814,16 @@
         <x:v>Plate Curl Machine</x:v>
       </x:c>
       <x:c r="C16" s="222" t="str">
-        <x:v>12.5 kg/side x 11 @ RIR 3</x:v>
+        <x:v>12.5 kg/side x 11 @ RIR 2</x:v>
       </x:c>
       <x:c r="D16" s="222" t="str">
-        <x:v>7.5-12.5 kg/side</x:v>
+        <x:v>10-12.5 kg/side</x:v>
       </x:c>
       <x:c r="E16" s="222" t="str">
-        <x:v>12.5 kg/side x 12 @ RIR 2</x:v>
+        <x:v>10 kg/side x14-15 @3; 12.5 x12 @2</x:v>
       </x:c>
       <x:c r="F16" s="222" t="str">
-        <x:v>No 15 kg until target is earned</x:v>
+        <x:v>Add rep and reserve before load</x:v>
       </x:c>
       <x:c r="G16" s="222" t="str">
         <x:v>Upper arms fixed</x:v>
@@ -27904,7 +28832,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I16" s="222" t="str">
-        <x:v>All three sets improved reserve; machine replaced incline curl in this combined session</x:v>
+        <x:v>Exactly two sets in the seven-exercise B session</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -27944,25 +28872,25 @@
         <x:v>Reverse EZ Curl</x:v>
       </x:c>
       <x:c r="C18" s="222" t="str">
-        <x:v>10 kg/side x 11 @ RIR 1</x:v>
+        <x:v>10 kg/side x 11 @ RIR 3</x:v>
       </x:c>
       <x:c r="D18" s="222" t="str">
-        <x:v>5-10 kg/side</x:v>
+        <x:v>7.5-10 kg/side</x:v>
       </x:c>
       <x:c r="E18" s="222" t="str">
-        <x:v>10 kg/side x 11 @ RIR 2</x:v>
+        <x:v>7.5 kg/side x13-15 @3; 10 kg/side x12 @2-3</x:v>
       </x:c>
       <x:c r="F18" s="222" t="str">
-        <x:v>Improve reserve</x:v>
+        <x:v>Add reps before load</x:v>
       </x:c>
       <x:c r="G18" s="222" t="str">
         <x:v>Wrists neutral</x:v>
       </x:c>
       <x:c r="H18" s="222" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I18" s="222" t="str">
-        <x:v>Bar excluded; only 2 sets used to preserve session cap</x:v>
+        <x:v>Bar excluded; exactly two sets</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -27973,25 +28901,25 @@
         <x:v>Concentration Curl</x:v>
       </x:c>
       <x:c r="C19" s="222" t="str">
-        <x:v>12.5 kg each x 10 @ RIR 1</x:v>
+        <x:v>12.5 kg each x 10 @ RIR 3</x:v>
       </x:c>
       <x:c r="D19" s="222" t="str">
-        <x:v>7.5-12.5 kg each</x:v>
+        <x:v>10-12.5 kg each</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>12.5 kg each x 10 @ RIR 2</x:v>
+        <x:v>10 kg x12-13 @3; 12.5 kg x11 @2-3</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>Improve reserve; no failure</x:v>
+        <x:v>Add reps before load; no failure</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
         <x:v>Elbow fixed; no swing</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>Clean and controlled; exactly 3 sets next time</x:v>
+        <x:v>7.5 kg x15 @4 produced little stimulus and is preparation only</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" hidden="0" customHeight="1">
@@ -28549,25 +29477,25 @@
         <x:v>Iso-Lateral High Row</x:v>
       </x:c>
       <x:c r="C39" s="170" t="str">
-        <x:v>20 kg/side x 10 @ RIR 2</x:v>
+        <x:v>20 kg/side x 12 @ RIR 3</x:v>
       </x:c>
       <x:c r="D39" s="170" t="str">
         <x:v>15-20 kg/side</x:v>
       </x:c>
       <x:c r="E39" s="170" t="str">
-        <x:v>20 kg/side x 11-12 @ RIR 2</x:v>
+        <x:v>15 kg/side x15 @3; 17.5 x13 @3; 20 x13 @2-3</x:v>
       </x:c>
       <x:c r="F39" s="170" t="str">
-        <x:v>Add reps first</x:v>
+        <x:v>Exactly three sets; add reps before load</x:v>
       </x:c>
       <x:c r="G39" s="170" t="str">
-        <x:v>Match both sides; chest stable</x:v>
+        <x:v>Chest supported; elbows follow machine path</x:v>
       </x:c>
       <x:c r="H39" s="170" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="I39" s="170" t="str">
-        <x:v>New 20 kg/side baseline</x:v>
+        <x:v>12 kg x15 @3 became extra working volume; omit it next time</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
@@ -28665,25 +29593,25 @@
         <x:v>Straight Bar Curl</x:v>
       </x:c>
       <x:c r="C43" s="170" t="str">
-        <x:v>15 kg/side x 8 @ RIR 2</x:v>
+        <x:v>15 kg/side x 9 @ RIR 2</x:v>
       </x:c>
       <x:c r="D43" s="170" t="str">
-        <x:v>10-15 kg/side</x:v>
+        <x:v>10-15 kg/side; bar excluded</x:v>
       </x:c>
       <x:c r="E43" s="170" t="str">
-        <x:v>15 kg/side x 9 @ RIR 2</x:v>
+        <x:v>10 kg/side x13 @3; 12.5 x11-12 @2; 15 x9-10 @2</x:v>
       </x:c>
       <x:c r="F43" s="170" t="str">
-        <x:v>Exactly 3 working sets; add rep before load</x:v>
+        <x:v>Exactly three sets; improve reserve before load</x:v>
       </x:c>
       <x:c r="G43" s="170" t="str">
-        <x:v>No body swing</x:v>
+        <x:v>Elbows fixed; no body swing</x:v>
       </x:c>
       <x:c r="H43" s="170" t="str">
-        <x:v>In progress</x:v>
+        <x:v>In progress / To verify</x:v>
       </x:c>
       <x:c r="I43" s="170" t="str">
-        <x:v>Bar excluded; use genuine preparation separately</x:v>
+        <x:v>Bar type and form To verify; omit 7.5 kg working set next time</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="48" customHeight="1">
@@ -28916,6 +29844,35 @@
       </x:c>
       <x:c r="I51" t="str">
         <x:v>Different machine; total plates/displayed load and starting resistance To verify; do not compare with established row machine</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="54" customHeight="1">
+      <x:c r="A52" s="170" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="B52" s="170" t="str">
+        <x:v>Single-Arm Seated Cable Row</x:v>
+      </x:c>
+      <x:c r="C52" s="170" t="str">
+        <x:v>25 kg x 10 each arm @ RIR 2</x:v>
+      </x:c>
+      <x:c r="D52" s="170" t="str">
+        <x:v>15-25 kg selected stack</x:v>
+      </x:c>
+      <x:c r="E52" s="170" t="str">
+        <x:v>15 kg x15 @3; 20 x13 @2; 25 x11 @2</x:v>
+      </x:c>
+      <x:c r="F52" s="170" t="str">
+        <x:v>Add one rep before load</x:v>
+      </x:c>
+      <x:c r="G52" s="170" t="str">
+        <x:v>Torso square; elbow toward hip</x:v>
+      </x:c>
+      <x:c r="H52" s="170" t="str">
+        <x:v>New baseline / To verify</x:v>
+      </x:c>
+      <x:c r="I52" s="170" t="str">
+        <x:v>Exact cable station/calibration and side-to-side match To verify</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28943,7 +29900,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5b8a727b7d243d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e01223b46c24002"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30063,24 +31020,38 @@
       <x:c r="R33" s="170"/>
       <x:c r="S33" s="170"/>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34"/>
-      <x:c r="B34"/>
-      <x:c r="C34"/>
-      <x:c r="D34"/>
-      <x:c r="E34"/>
-      <x:c r="F34"/>
-      <x:c r="G34"/>
-      <x:c r="H34"/>
-      <x:c r="I34"/>
-      <x:c r="J34"/>
-      <x:c r="K34" s="59" t="n"/>
-      <x:c r="L34" s="59" t="n"/>
-      <x:c r="M34" s="59" t="n"/>
-      <x:c r="N34" s="59" t="n"/>
-      <x:c r="O34" s="59" t="n"/>
-      <x:c r="P34" s="59" t="n"/>
-      <x:c r="Q34" s="59" t="n"/>
+    <x:row r="34" ht="72" customHeight="1">
+      <x:c r="A34" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B34" s="170"/>
+      <x:c r="C34" s="170"/>
+      <x:c r="D34" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E34" s="170" t="str">
+        <x:v>Medium to Low final</x:v>
+      </x:c>
+      <x:c r="F34" s="170" t="str">
+        <x:v>No pain; pre-session soreness To verify</x:v>
+      </x:c>
+      <x:c r="G34" s="170"/>
+      <x:c r="H34" s="170"/>
+      <x:c r="I34" s="170" t="str">
+        <x:v>Back + Biceps workout - 90 min total; 20 working sets plus one preparation set; medium pump; 10 min treadmill at 3 km/h and 12% incline</x:v>
+      </x:c>
+      <x:c r="J34" s="170" t="str">
+        <x:v>Started Medium-High; half EAA+ plus half pre-workout; no assistance; form breakdown/unusual sensation, coffee, creatine, rail support and cardio symptoms To verify</x:v>
+      </x:c>
+      <x:c r="K34" s="222"/>
+      <x:c r="L34" s="222"/>
+      <x:c r="M34" s="222"/>
+      <x:c r="N34" s="222"/>
+      <x:c r="O34" s="222"/>
+      <x:c r="P34" s="222"/>
+      <x:c r="Q34" s="222"/>
+      <x:c r="R34" s="170"/>
+      <x:c r="S34" s="170"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35"/>
@@ -33292,7 +34263,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2860e484e07a4b58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b02e069c2904788"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34789,7 +35760,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f393a3d937841b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539e5b87713a4669"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35614,6 +36585,32 @@
         <x:v>Back + Biceps only after Good sleep, at least Medium starting energy and no meaningful soreness/pain; cap at 16 working sets, use one chest-supported-row variation, keep RIR 2-3 and omit post-lift cardio</x:v>
       </x:c>
     </x:row>
+    <x:row r="32" ht="96" customHeight="1">
+      <x:c r="A32" s="220" t="n">
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="B32" s="170" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C32" s="170" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D32" s="170" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E32" s="170" t="str">
+        <x:v>Green/Yellow</x:v>
+      </x:c>
+      <x:c r="F32" s="170" t="str">
+        <x:v>Good sleep; Medium-High start and Medium-Low final energy; no pain; pre-session soreness To verify; 90 min including 10 min treadmill; medium back/biceps pump; no assistance; form breakdown/unusual sensation To verify; half EAA+ plus half pre-workout; coffee, creatine and exact stimulant exposure To verify</x:v>
+      </x:c>
+      <x:c r="G32" s="170" t="str">
+        <x:v>Twenty working sets plus one low-fatigue preparation set were completed without pain or assistance. New single-arm-row and revised curl baselines were established, and most working sets remained at RIR 2-3. The session exceeded the planned 18-set ceiling by two; one straight-bar set reached RIR 1, and steep cardio was added on the sixth consecutive training day despite the recovery-oriented recommendation.</x:v>
+      </x:c>
+      <x:c r="H32" s="170" t="str">
+        <x:v>Complete rest Sunday; next Back + Biceps exactly 18 working sets, remove the extra 12 kg high-row and 7.5 kg straight-bar sets, keep routine work at RIR 2-3, and use only easy cardio when recovery supports it</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -35626,7 +36623,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red70f3afc57f484c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R107e0eceef8c4443"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36196,7 +37193,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce14ab8a42494eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2371ecdb9e46c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37302,10 +38299,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5932c49ecb14278"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0555e607cad470d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2564ddcfaf044283"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fbb91674952403d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea4a624b99134b73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf3d0a4df95425c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d17b54ae5ce4663"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re258922d98374e85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 14 return workout and recovery
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf118392d3ebf47f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rd831fba28df44f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Ra2a92ca9051c4a39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="Rd8e224c000094618"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rc5d3db7844d841d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R47dd1b1e28a74d63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rbd8de373c58b40cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R58f8c26227884543"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="R530acca548c84ff1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R1df081cb3e754875"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R57159138c7aa4441"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R39175a378c984c11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4faf0b5479294d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rd805d7fbeca742d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R4df3dbe8c6e8487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rabf84ff4566b463d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R0229bbebaa474237"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R20c03e2dcee24618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R497a9c86bea145cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rac12f2b23d6447ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R4e390df4ef434bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R0147e1cae6524d74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1723,7 +1723,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9a5905c832a24c30"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5e1c366e5ca6471d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1733,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N522" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N582" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1803,7 +1803,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I58" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1820,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1838,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D96" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1850,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86a6b5c6433a46db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1989891529a413c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3955,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4fd853c4ac948c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01fdb11815e24f38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4083,7 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4091,7 +4091,7 @@
       </x:c>
       <x:c r="G5" s="53" t="n"/>
       <x:c r="H5" s="93" t="str">
-        <x:v>6-day active</x:v>
+        <x:v>Return week</x:v>
       </x:c>
       <x:c r="I5" s="53" t="n"/>
       <x:c r="J5" s="59" t="n"/>
@@ -4283,7 +4283,7 @@
         <x:v>Monday</x:v>
       </x:c>
       <x:c r="B13" s="59" t="str">
-        <x:v>Chest + Triceps - completed 2026-08-31</x:v>
+        <x:v>Chest + Triceps completed 2026-09-14</x:v>
       </x:c>
       <x:c r="C13" s="59" t="n"/>
       <x:c r="D13" s="94" t="inlineStr">
@@ -4309,7 +4309,7 @@
         <x:v>Tuesday</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
-        <x:v>Back + Biceps - completed 2026-09-01</x:v>
+        <x:v>Back + Biceps: fresh readiness first</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4327,7 +4327,7 @@
         <x:v>Wednesday</x:v>
       </x:c>
       <x:c r="B15" s="59" t="str">
-        <x:v>Shoulders + Triceps - completed 2026-09-02</x:v>
+        <x:v>Shoulders + Triceps: conditional</x:v>
       </x:c>
       <x:c r="C15" s="59" t="n"/>
       <x:c r="D15" s="90" t="inlineStr">
@@ -4349,7 +4349,7 @@
         <x:v>Thursday</x:v>
       </x:c>
       <x:c r="B16" s="59" t="str">
-        <x:v>Legs + Calves - completed 2026-09-03</x:v>
+        <x:v>Legs + Calves: conditional</x:v>
       </x:c>
       <x:c r="C16" s="59" t="n"/>
       <x:c r="D16" s="94" t="inlineStr">
@@ -4386,67 +4386,67 @@
       <x:c r="K16" s="59" t="n"/>
       <x:c r="L16" s="59" t="n"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="85" customHeight="1">
       <x:c r="A17" s="92" t="str">
         <x:v>Friday</x:v>
       </x:c>
       <x:c r="B17" s="59" t="str">
-        <x:v>Chest + Shoulders - completed 2026-09-04</x:v>
+        <x:v>Chest + Shoulders: conditional</x:v>
       </x:c>
       <x:c r="C17" s="59" t="n"/>
-      <x:c r="D17" s="59" t="str">
-        <x:v>Legs</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>Hack Squat</x:v>
-      </x:c>
-      <x:c r="F17" s="59" t="str">
-        <x:v>65 kg/side x 8 @ RIR 2</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>65 kg/side x 9 @ RIR 2</x:v>
-      </x:c>
-      <x:c r="H17" s="59" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="I17" s="59" t="str">
-        <x:v>Hold load</x:v>
+      <x:c r="D17" s="222" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="E17" s="222" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="F17" s="222" t="str">
+        <x:v>10 x 12 @3; 15 x 12 @2; 17.5 x 10 @2; 20 x 8 @2; 22.5 x 6 @2</x:v>
+      </x:c>
+      <x:c r="G17" s="222" t="str">
+        <x:v>2 sets: 15-17.5 kg/side x10-12 @3-4</x:v>
+      </x:c>
+      <x:c r="H17" s="222" t="str">
+        <x:v>Return targets</x:v>
+      </x:c>
+      <x:c r="I17" s="222" t="str">
+        <x:v>See dated target notes</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
       <x:c r="L17" s="59" t="n"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="85" customHeight="1">
       <x:c r="A18" s="92" t="str">
         <x:v>Saturday</x:v>
       </x:c>
       <x:c r="B18" s="59" t="str">
-        <x:v>Back + Biceps - completed 2026-09-05</x:v>
+        <x:v>Back + Biceps: conditional</x:v>
       </x:c>
       <x:c r="C18" s="59" t="n"/>
-      <x:c r="D18" s="59" t="str">
-        <x:v>Legs</x:v>
-      </x:c>
-      <x:c r="E18" s="59" t="str">
-        <x:v>Leg Press</x:v>
-      </x:c>
-      <x:c r="F18" s="59" t="str">
-        <x:v>160 kg x 7 unassisted @1</x:v>
-      </x:c>
-      <x:c r="G18" s="59" t="str">
-        <x:v>140 kg x 10 @ RIR 2</x:v>
-      </x:c>
-      <x:c r="H18" s="59" t="str">
-        <x:v>Modify volume/effort</x:v>
-      </x:c>
-      <x:c r="I18" s="59" t="str">
-        <x:v>Exactly 3 sets; no 160</x:v>
+      <x:c r="D18" s="222" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="E18" s="222" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="F18" s="222" t="str">
+        <x:v>15 x 12 @2; 17.5 x 10 @2; 20 x 6 @3</x:v>
+      </x:c>
+      <x:c r="G18" s="222" t="str">
+        <x:v>2 sets: 12.5-15 kg/side x10-12 @3-4</x:v>
+      </x:c>
+      <x:c r="H18" s="222" t="str">
+        <x:v>Return targets</x:v>
+      </x:c>
+      <x:c r="I18" s="222" t="str">
+        <x:v>See dated target notes</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
       <x:c r="L18" s="59" t="n"/>
     </x:row>
-    <x:row r="19" ht="30" customHeight="1">
+    <x:row r="19" ht="85" customHeight="1">
       <x:c r="A19" s="92" t="str">
         <x:v>Sunday</x:v>
       </x:c>
@@ -4454,101 +4454,101 @@
         <x:v>Complete rest / recovery</x:v>
       </x:c>
       <x:c r="C19" s="59" t="n"/>
-      <x:c r="D19" s="59" t="str">
-        <x:v>Legs</x:v>
+      <x:c r="D19" s="222" t="str">
+        <x:v>Chest + Triceps</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>DB Romanian Deadlift</x:v>
+        <x:v>Cable Fly</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>17.5 kg each x 9 @ RIR 2</x:v>
+        <x:v>20 x 15 @3; 25 x 10 @2; 25 x 10 @2</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>15 kg each x 10-11 @ RIR 2</x:v>
+        <x:v>2 sets: 15-20 kg/side x12-15 @3-4</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>Modify technique</x:v>
+        <x:v>Return targets</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>17.5 was substitution</x:v>
+        <x:v>See dated target notes</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
       <x:c r="L19" s="59" t="n"/>
     </x:row>
-    <x:row r="20" ht="30" customHeight="1">
+    <x:row r="20" ht="85" customHeight="1">
       <x:c r="A20" s="59" t="n"/>
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
-      <x:c r="D20" s="59" t="str">
-        <x:v>Legs</x:v>
+      <x:c r="D20" s="222" t="str">
+        <x:v>Chest + Triceps</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Leg Curl</x:v>
+        <x:v>Straight Bar Pushdown</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>35 kg x 9 @ RIR 1</x:v>
+        <x:v>50 x 14 @3; 55 x 11 @2; 60 x 8 @2</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>35 kg x 9-10 @ RIR 2</x:v>
+        <x:v>2 sets: 40-45 kg x12-15 @3-4</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>Modify effort</x:v>
+        <x:v>Return targets</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>No extra set</x:v>
+        <x:v>See dated target notes</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
       <x:c r="L20" s="59" t="n"/>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="85" customHeight="1">
       <x:c r="A21" s="59" t="n"/>
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
-      <x:c r="D21" s="59" t="str">
-        <x:v>Legs</x:v>
-      </x:c>
-      <x:c r="E21" s="59" t="str">
-        <x:v>Leg Extension</x:v>
-      </x:c>
-      <x:c r="F21" s="59" t="str">
-        <x:v>50 kg x 11 @ RIR 2</x:v>
-      </x:c>
-      <x:c r="G21" s="59" t="str">
-        <x:v>50 kg x 12 @ RIR 2</x:v>
-      </x:c>
-      <x:c r="H21" s="59" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="I21" s="59" t="str">
-        <x:v>Add one rep</x:v>
+      <x:c r="D21" s="222" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="E21" s="222" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="F21" s="222" t="str">
+        <x:v>35 x 14 @3; 40 x 11 @2; 45 x 9 @2</x:v>
+      </x:c>
+      <x:c r="G21" s="222" t="str">
+        <x:v>2 sets: 25-30 kg x12-15 @3-4</x:v>
+      </x:c>
+      <x:c r="H21" s="222" t="str">
+        <x:v>Return targets</x:v>
+      </x:c>
+      <x:c r="I21" s="222" t="str">
+        <x:v>See dated target notes</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
       <x:c r="L21" s="59" t="n"/>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="85" customHeight="1">
       <x:c r="A22" s="59" t="n"/>
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
-      <x:c r="D22" s="59" t="str">
-        <x:v>Calves</x:v>
-      </x:c>
-      <x:c r="E22" s="59" t="str">
-        <x:v>Standing Calf Raise</x:v>
-      </x:c>
-      <x:c r="F22" s="59" t="str">
-        <x:v>20 kg/side x 17 @ RIR 2</x:v>
-      </x:c>
-      <x:c r="G22" s="59" t="str">
-        <x:v>Repeat plus third set</x:v>
-      </x:c>
-      <x:c r="H22" s="59" t="str">
-        <x:v>In progress</x:v>
-      </x:c>
-      <x:c r="I22" s="59" t="str">
-        <x:v>Three sets next time</x:v>
+      <x:c r="D22" s="222" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="E22" s="222" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="F22" s="222" t="str">
+        <x:v>60 x 12 @2; 50 x 8 @2</x:v>
+      </x:c>
+      <x:c r="G22" s="222" t="str">
+        <x:v>2 sets: 70 kg assistance x8-12 @3-4</x:v>
+      </x:c>
+      <x:c r="H22" s="222" t="str">
+        <x:v>Return targets</x:v>
+      </x:c>
+      <x:c r="I22" s="222" t="str">
+        <x:v>See dated target notes</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4565,16 +4565,16 @@
         <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>Medium-Low after 90 min</x:v>
+        <x:v>Medium after 90 min</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Complete rest Sunday</x:v>
+        <x:v>Monitor delayed symptoms</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Monitor</x:v>
+        <x:v>No pain reported</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>Six consecutive training days completed</x:v>
+        <x:v>18 working sets exceeded lighter return plan</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4588,19 +4588,19 @@
         <x:v>Next</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
-        <x:v>Six-day block completed</x:v>
+        <x:v>Fresh readiness first</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>Fresh readiness; 16-18 working sets</x:v>
+        <x:v>10-12 work sets, RIR 3-4</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>No failure; cardio only if recovery supports it</x:v>
+        <x:v>No automatic load increases</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4629,7 +4629,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1964c19385aa47c6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae166b3f897c487b"/>
 </x:worksheet>
 </file>
 
@@ -28351,6 +28351,842 @@
       </x:c>
       <x:c r="N563" s="170" t="n">
         <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="564" ht="75" customHeight="1">
+      <x:c r="A564" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B564" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C564" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D564" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E564" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F564" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G564" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H564" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I564" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J564" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K564" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L564" s="170" t="str">
+        <x:v>User-designated warm-up retained; RIR 3 means not a very easy preparation set</x:v>
+      </x:c>
+      <x:c r="M564" s="170" t="str">
+        <x:v>Warm-up</x:v>
+      </x:c>
+      <x:c r="N564" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="565" ht="75" customHeight="1">
+      <x:c r="A565" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B565" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C565" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D565" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E565" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F565" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G565" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H565" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I565" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J565" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K565" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L565" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M565" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N565" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="566" ht="75" customHeight="1">
+      <x:c r="A566" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B566" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C566" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D566" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E566" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F566" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G566" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H566" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I566" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J566" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K566" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L566" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M566" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N566" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="567" ht="75" customHeight="1">
+      <x:c r="A567" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B567" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C567" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D567" s="170" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E567" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F567" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G567" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H567" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I567" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J567" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K567" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L567" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M567" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N567" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="568" ht="75" customHeight="1">
+      <x:c r="A568" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B568" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C568" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="D568" s="170" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E568" s="170" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F568" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G568" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H568" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I568" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J568" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K568" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L568" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M568" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N568" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="569" ht="75" customHeight="1">
+      <x:c r="A569" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B569" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C569" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D569" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E569" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F569" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G569" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H569" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I569" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J569" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K569" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L569" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M569" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N569" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="570" ht="75" customHeight="1">
+      <x:c r="A570" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B570" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C570" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D570" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E570" s="170" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F570" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G570" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H570" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I570" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J570" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K570" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L570" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M570" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N570" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="571" ht="75" customHeight="1">
+      <x:c r="A571" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B571" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C571" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="D571" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E571" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F571" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="G571" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H571" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I571" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J571" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K571" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L571" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M571" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N571" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="572" ht="75" customHeight="1">
+      <x:c r="A572" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B572" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C572" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="D572" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E572" s="170" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F572" s="170" t="str">
+        <x:v>kg each side; horizontal cable fly</x:v>
+      </x:c>
+      <x:c r="G572" s="170" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H572" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I572" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J572" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K572" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L572" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M572" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N572" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="573" ht="75" customHeight="1">
+      <x:c r="A573" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B573" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C573" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="D573" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E573" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F573" s="170" t="str">
+        <x:v>kg each side; horizontal cable fly</x:v>
+      </x:c>
+      <x:c r="G573" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H573" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I573" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J573" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K573" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L573" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M573" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N573" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="574" ht="75" customHeight="1">
+      <x:c r="A574" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B574" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C574" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="D574" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E574" s="170" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F574" s="170" t="str">
+        <x:v>kg each side; horizontal cable fly</x:v>
+      </x:c>
+      <x:c r="G574" s="170" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H574" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I574" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J574" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K574" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L574" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M574" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N574" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="575" ht="75" customHeight="1">
+      <x:c r="A575" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B575" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C575" s="170" t="str">
+        <x:v>Straight Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D575" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E575" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F575" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G575" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H575" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I575" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J575" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K575" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L575" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M575" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N575" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="576" ht="75" customHeight="1">
+      <x:c r="A576" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B576" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C576" s="170" t="str">
+        <x:v>Straight Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D576" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E576" s="170" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="F576" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G576" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H576" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I576" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J576" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K576" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L576" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M576" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N576" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="577" ht="75" customHeight="1">
+      <x:c r="A577" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B577" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C577" s="170" t="str">
+        <x:v>Straight Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="D577" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E577" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F577" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G577" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H577" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I577" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J577" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K577" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L577" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M577" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N577" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="578" ht="75" customHeight="1">
+      <x:c r="A578" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B578" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C578" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D578" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E578" s="170" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F578" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G578" s="170" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H578" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I578" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J578" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K578" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L578" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M578" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N578" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="579" ht="75" customHeight="1">
+      <x:c r="A579" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B579" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C579" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D579" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E579" s="170" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F579" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G579" s="170" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H579" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I579" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J579" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K579" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L579" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M579" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N579" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="580" ht="75" customHeight="1">
+      <x:c r="A580" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B580" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C580" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="D580" s="170" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E580" s="170" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F580" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G580" s="170" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H580" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I580" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J580" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K580" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L580" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M580" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N580" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="581" ht="75" customHeight="1">
+      <x:c r="A581" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B581" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C581" s="170" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="D581" s="170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E581" s="170" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F581" s="170" t="str">
+        <x:v>kg assistance counterweight; higher is easier</x:v>
+      </x:c>
+      <x:c r="G581" s="170" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H581" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I581" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J581" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K581" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L581" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M581" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N581" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="582" ht="75" customHeight="1">
+      <x:c r="A582" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B582" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C582" s="170" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="D582" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E582" s="170" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F582" s="170" t="str">
+        <x:v>kg assistance counterweight; higher is easier</x:v>
+      </x:c>
+      <x:c r="G582" s="170" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H582" s="170" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I582" s="170" t="str">
+        <x:v>No pain or recurrent headache</x:v>
+      </x:c>
+      <x:c r="J582" s="170" t="str">
+        <x:v>Medium start and final</x:v>
+      </x:c>
+      <x:c r="K582" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L582" s="170" t="str">
+        <x:v>Completed above lighter return prescription; hold progression pending recovery</x:v>
+      </x:c>
+      <x:c r="M582" s="170" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N582" s="170" t="n">
+        <x:v>2</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -28385,7 +29221,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raea59e7681a34c33"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffea5388e11f431a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29873,6 +30709,180 @@
       </x:c>
       <x:c r="I52" s="170" t="str">
         <x:v>Exact cable station/calibration and side-to-side match To verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="110" customHeight="1">
+      <x:c r="A53" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="B53" s="170" t="str">
+        <x:v>Flat Bench Press</x:v>
+      </x:c>
+      <x:c r="C53" s="170" t="str">
+        <x:v>10 x 12 @3; 15 x 12 @2; 17.5 x 10 @2; 20 x 8 @2; 22.5 x 6 @2</x:v>
+      </x:c>
+      <x:c r="D53" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="E53" s="170" t="str">
+        <x:v>2 sets: 15-17.5 kg/side x10-12 @3-4</x:v>
+      </x:c>
+      <x:c r="F53" s="170" t="str">
+        <x:v>Adjust downward for target reserve; no automatic increase</x:v>
+      </x:c>
+      <x:c r="G53" s="170" t="str">
+        <x:v>Controlled pain-free motion; no straining</x:v>
+      </x:c>
+      <x:c r="H53" s="170" t="str">
+        <x:v>2026-09-14 return targets</x:v>
+      </x:c>
+      <x:c r="I53" s="170" t="str">
+        <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="110" customHeight="1">
+      <x:c r="A54" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="B54" s="170" t="str">
+        <x:v>Incline Barbell Bench Press</x:v>
+      </x:c>
+      <x:c r="C54" s="170" t="str">
+        <x:v>15 x 12 @2; 17.5 x 10 @2; 20 x 6 @3</x:v>
+      </x:c>
+      <x:c r="D54" s="170" t="str">
+        <x:v>kg plates each side; bar excluded</x:v>
+      </x:c>
+      <x:c r="E54" s="170" t="str">
+        <x:v>2 sets: 12.5-15 kg/side x10-12 @3-4</x:v>
+      </x:c>
+      <x:c r="F54" s="170" t="str">
+        <x:v>Adjust downward for target reserve; no automatic increase</x:v>
+      </x:c>
+      <x:c r="G54" s="170" t="str">
+        <x:v>Controlled pain-free motion; no straining</x:v>
+      </x:c>
+      <x:c r="H54" s="170" t="str">
+        <x:v>2026-09-14 return targets</x:v>
+      </x:c>
+      <x:c r="I54" s="170" t="str">
+        <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="110" customHeight="1">
+      <x:c r="A55" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="B55" s="170" t="str">
+        <x:v>Cable Fly</x:v>
+      </x:c>
+      <x:c r="C55" s="170" t="str">
+        <x:v>20 x 15 @3; 25 x 10 @2; 25 x 10 @2</x:v>
+      </x:c>
+      <x:c r="D55" s="170" t="str">
+        <x:v>kg each side; horizontal cable fly</x:v>
+      </x:c>
+      <x:c r="E55" s="170" t="str">
+        <x:v>2 sets: 15-20 kg/side x12-15 @3-4</x:v>
+      </x:c>
+      <x:c r="F55" s="170" t="str">
+        <x:v>Adjust downward for target reserve; no automatic increase</x:v>
+      </x:c>
+      <x:c r="G55" s="170" t="str">
+        <x:v>Controlled pain-free motion; no straining</x:v>
+      </x:c>
+      <x:c r="H55" s="170" t="str">
+        <x:v>2026-09-14 return targets</x:v>
+      </x:c>
+      <x:c r="I55" s="170" t="str">
+        <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="110" customHeight="1">
+      <x:c r="A56" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="B56" s="170" t="str">
+        <x:v>Straight Bar Pushdown</x:v>
+      </x:c>
+      <x:c r="C56" s="170" t="str">
+        <x:v>50 x 14 @3; 55 x 11 @2; 60 x 8 @2</x:v>
+      </x:c>
+      <x:c r="D56" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="E56" s="170" t="str">
+        <x:v>2 sets: 40-45 kg x12-15 @3-4</x:v>
+      </x:c>
+      <x:c r="F56" s="170" t="str">
+        <x:v>Adjust downward for target reserve; no automatic increase</x:v>
+      </x:c>
+      <x:c r="G56" s="170" t="str">
+        <x:v>Controlled pain-free motion; no straining</x:v>
+      </x:c>
+      <x:c r="H56" s="170" t="str">
+        <x:v>2026-09-14 return targets</x:v>
+      </x:c>
+      <x:c r="I56" s="170" t="str">
+        <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="110" customHeight="1">
+      <x:c r="A57" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="B57" s="170" t="str">
+        <x:v>Overhead Rope Extension</x:v>
+      </x:c>
+      <x:c r="C57" s="170" t="str">
+        <x:v>35 x 14 @3; 40 x 11 @2; 45 x 9 @2</x:v>
+      </x:c>
+      <x:c r="D57" s="170" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="E57" s="170" t="str">
+        <x:v>2 sets: 25-30 kg x12-15 @3-4</x:v>
+      </x:c>
+      <x:c r="F57" s="170" t="str">
+        <x:v>Adjust downward for target reserve; no automatic increase</x:v>
+      </x:c>
+      <x:c r="G57" s="170" t="str">
+        <x:v>Controlled pain-free motion; no straining</x:v>
+      </x:c>
+      <x:c r="H57" s="170" t="str">
+        <x:v>2026-09-14 return targets</x:v>
+      </x:c>
+      <x:c r="I57" s="170" t="str">
+        <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="110" customHeight="1">
+      <x:c r="A58" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="B58" s="170" t="str">
+        <x:v>Assisted Dip Machine</x:v>
+      </x:c>
+      <x:c r="C58" s="170" t="str">
+        <x:v>60 x 12 @2; 50 x 8 @2</x:v>
+      </x:c>
+      <x:c r="D58" s="170" t="str">
+        <x:v>kg assistance counterweight; higher is easier</x:v>
+      </x:c>
+      <x:c r="E58" s="170" t="str">
+        <x:v>2 sets: 70 kg assistance x8-12 @3-4</x:v>
+      </x:c>
+      <x:c r="F58" s="170" t="str">
+        <x:v>Adjust downward for target reserve; no automatic increase</x:v>
+      </x:c>
+      <x:c r="G58" s="170" t="str">
+        <x:v>Controlled pain-free motion; no straining</x:v>
+      </x:c>
+      <x:c r="H58" s="170" t="str">
+        <x:v>2026-09-14 return targets</x:v>
+      </x:c>
+      <x:c r="I58" s="170" t="str">
+        <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -29900,7 +30910,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e01223b46c24002"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d04882cf8284675"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31053,17 +32063,29 @@
       <x:c r="R34" s="170"/>
       <x:c r="S34" s="170"/>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35"/>
-      <x:c r="B35"/>
-      <x:c r="C35"/>
-      <x:c r="D35"/>
-      <x:c r="E35"/>
-      <x:c r="F35"/>
-      <x:c r="G35"/>
-      <x:c r="H35"/>
-      <x:c r="I35"/>
-      <x:c r="J35"/>
+    <x:row r="35" ht="190" customHeight="1">
+      <x:c r="A35" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B35" s="170"/>
+      <x:c r="C35" s="170"/>
+      <x:c r="D35" s="170" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E35" s="170" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="F35" s="170" t="str">
+        <x:v>No headache/head pressure, dizziness, neck discomfort or other pain</x:v>
+      </x:c>
+      <x:c r="G35" s="170"/>
+      <x:c r="H35" s="170"/>
+      <x:c r="I35" s="170" t="str">
+        <x:v>7 min treadmill; 3 km/h; 12% incline; rail support To verify</x:v>
+      </x:c>
+      <x:c r="J35" s="170" t="str">
+        <x:v>90 minutes including 7 min treadmill at 3 km/h, 12% incline; rail support To verify. Good sleep, Medium start/final energy. No headache/head pressure, dizziness, neck discomfort, joint/other pain; no human assistance or reported form breakdown. EAA+, pre-workout, coffee, creatine and magnesium intake today To verify. User reports neurologist cleared exercise.</x:v>
+      </x:c>
       <x:c r="K35" s="59" t="n"/>
       <x:c r="L35" s="59" t="n"/>
       <x:c r="M35" s="59" t="n"/>
@@ -34263,7 +35285,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b02e069c2904788"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4429d5d4c204447"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35754,13 +36776,55 @@
         <x:v>Review label before use and count elemental magnesium from all supplements; NIH source https://ods.od.nih.gov/factsheets/Magnesium-HealthProfessional/</x:v>
       </x:c>
     </x:row>
+    <x:row r="102" ht="190" customHeight="1">
+      <x:c r="A102" s="170" t="str">
+        <x:v>2026-09-14 return context</x:v>
+      </x:c>
+      <x:c r="B102" s="170" t="str">
+        <x:v>User reports persistent back-of-head pain prompted a training break; MRI reportedly normal, neurologist cleared exercise; symptom-free for three days before return. Massage helped.</x:v>
+      </x:c>
+      <x:c r="C102" s="170" t="str">
+        <x:v>User-reported history, not independently reviewed clinical records; cause remains To verify.</x:v>
+      </x:c>
+      <x:c r="D102" s="170" t="str">
+        <x:v>Do not diagnose a nerve/vascular cause or assume massage establishes one. Follow clinician advice; stop if symptoms recur.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="190" customHeight="1">
+      <x:c r="A103" s="170" t="str">
+        <x:v>2026-09-14 return assessment</x:v>
+      </x:c>
+      <x:c r="B103" s="170" t="str">
+        <x:v>18 working sets plus one user-designated warm-up (RIR 3), six exercises. No pain, headache, dizziness, assistance or form breakdown reported; Medium final energy. Return after approximately one week off exceeded the planned 12 working sets at RIR 3-4: 14 working sets were RIR 2 and four were RIR 3. This was not a light re-entry session. Do not infer recovery or medical cause from performance alone; monitor next-day symptoms and avoid automatic load increases.</x:v>
+      </x:c>
+      <x:c r="C103" s="170" t="str">
+        <x:v>No symptoms at closeout does not establish next-day recovery. Initial plan was lighter than the completed workout.</x:v>
+      </x:c>
+      <x:c r="D103" s="170" t="str">
+        <x:v>Check delayed soreness, headache/neck symptoms, sleep and energy before next session.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="190" customHeight="1">
+      <x:c r="A104" s="170" t="str">
+        <x:v>2026-09-14 next-session targets</x:v>
+      </x:c>
+      <x:c r="B104" s="170" t="str">
+        <x:v>Next scheduled Back + Biceps only after fresh readiness and no recurrent headache, neck symptoms or limiting soreness. Start with 10-12 working sets at RIR 3-4; no failure or extra sets. Easy flat walking 5-10 min optional. Stop and seek clinician advice if headache recurs.</x:v>
+      </x:c>
+      <x:c r="C104" s="170" t="str">
+        <x:v>Avoid compensating for missed sessions with extra volume.</x:v>
+      </x:c>
+      <x:c r="D104" s="170" t="str">
+        <x:v>For each exercise show prior actual loads/reps/RIR alongside current targets and exact load basis.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539e5b87713a4669"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692c984f1ffc4b1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36611,6 +37675,32 @@
         <x:v>Complete rest Sunday; next Back + Biceps exactly 18 working sets, remove the extra 12 kg high-row and 7.5 kg straight-bar sets, keep routine work at RIR 2-3, and use only easy cardio when recovery supports it</x:v>
       </x:c>
     </x:row>
+    <x:row r="33" ht="260" customHeight="1">
+      <x:c r="A33" s="220" t="n">
+        <x:v>46279</x:v>
+      </x:c>
+      <x:c r="B33" s="170" t="str">
+        <x:v>Chest + Triceps</x:v>
+      </x:c>
+      <x:c r="C33" s="170" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D33" s="170" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E33" s="170" t="str">
+        <x:v>Return / monitor</x:v>
+      </x:c>
+      <x:c r="F33" s="170" t="str">
+        <x:v>90 minutes including 7 min treadmill at 3 km/h, 12% incline; rail support To verify. Good sleep, Medium start/final energy. No headache/head pressure, dizziness, neck discomfort, joint/other pain; no human assistance or reported form breakdown.</x:v>
+      </x:c>
+      <x:c r="G33" s="170" t="str">
+        <x:v>18 working sets plus one user-designated warm-up (RIR 3), six exercises. No pain, headache, dizziness, assistance or form breakdown reported; Medium final energy. Return after approximately one week off exceeded the planned 12 working sets at RIR 3-4: 14 working sets were RIR 2 and four were RIR 3. This was not a light re-entry session. Do not infer recovery or medical cause from performance alone; monitor next-day symptoms and avoid automatic load increases.</x:v>
+      </x:c>
+      <x:c r="H33" s="170" t="str">
+        <x:v>Next scheduled Back + Biceps only after fresh readiness and no recurrent headache, neck symptoms or limiting soreness. Start with 10-12 working sets at RIR 3-4; no failure or extra sets. Easy flat walking 5-10 min optional. Stop and seek clinician advice if headache recurs.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -36623,7 +37713,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R107e0eceef8c4443"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04206bc10cbf4219"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37193,7 +38283,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2371ecdb9e46c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bcc832898f34994"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38299,10 +39389,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea4a624b99134b73"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf3d0a4df95425c"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d17b54ae5ce4663"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re258922d98374e85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re32e5b5392264568"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ab5add18e83462b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6a1dccc521f4476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R222e1d9c243e4c53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 15 back and biceps workout
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R39175a378c984c11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4faf0b5479294d83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rd805d7fbeca742d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R4df3dbe8c6e8487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="Rabf84ff4566b463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R0229bbebaa474237"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R20c03e2dcee24618"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R497a9c86bea145cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rac12f2b23d6447ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R4e390df4ef434bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R0147e1cae6524d74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6a98311f5a0346f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra6408bd5238548e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rf3aae14e68384fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R527331f8173e457b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R1912a0bca44b4d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Re6eefc45c91140b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R9425644901ae4fa7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R0b6871c9e7bc4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rda1e234804f74e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc2d46953f32e4c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rb8590727a20c47d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -454,7 +454,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="380">
+  <x:cellXfs count="381">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -1331,6 +1331,9 @@
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1723,7 +1726,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5e1c366e5ca6471d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0d576648fb945df"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1733,7 +1736,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N582" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N599" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1803,7 +1806,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I58" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1820,7 +1823,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1838,7 +1841,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D104" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D108" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1850,7 +1853,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2552,7 +2555,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1989891529a413c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4efd725e403b419d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3955,7 +3958,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01fdb11815e24f38"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc05b3d83460641d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4083,7 +4086,8 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:v>29</x:v>
+        <x:f>COUNT('Session Summary'!A5:A34)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4309,7 +4313,7 @@
         <x:v>Tuesday</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
-        <x:v>Back + Biceps: fresh readiness first</x:v>
+        <x:v>Back + Biceps completed 2026-09-15</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4362,10 +4366,8 @@
           <x:t xml:space="preserve">Exercise</x:t>
         </x:is>
       </x:c>
-      <x:c r="F16" s="94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current Best</x:t>
-        </x:is>
+      <x:c r="F16" s="94" t="str">
+        <x:v>Latest session sets</x:v>
       </x:c>
       <x:c r="G16" s="94" t="inlineStr">
         <x:is>
@@ -4386,7 +4388,7 @@
       <x:c r="K16" s="59" t="n"/>
       <x:c r="L16" s="59" t="n"/>
     </x:row>
-    <x:row r="17" ht="85" customHeight="1">
+    <x:row r="17" ht="100" customHeight="1">
       <x:c r="A17" s="92" t="str">
         <x:v>Friday</x:v>
       </x:c>
@@ -4395,28 +4397,28 @@
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="222" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="E17" s="222" t="str">
-        <x:v>Flat Bench Press</x:v>
+        <x:v>Chest-Supported T-Bar Row</x:v>
       </x:c>
       <x:c r="F17" s="222" t="str">
-        <x:v>10 x 12 @3; 15 x 12 @2; 17.5 x 10 @2; 20 x 8 @2; 22.5 x 6 @2</x:v>
+        <x:v>20 x15 @3; 35 x15 @3; 45 x10 @3</x:v>
       </x:c>
       <x:c r="G17" s="222" t="str">
-        <x:v>2 sets: 15-17.5 kg/side x10-12 @3-4</x:v>
+        <x:v>20 x12-15 @3 preparation only if genuinely easy; 35 x15 @3; 45 x10-11 @2-3. Same machine and total plates.</x:v>
       </x:c>
       <x:c r="H17" s="222" t="str">
-        <x:v>Return targets</x:v>
+        <x:v>Recovery-led targets</x:v>
       </x:c>
       <x:c r="I17" s="222" t="str">
-        <x:v>See dated target notes</x:v>
+        <x:v>Latest dated revision</x:v>
       </x:c>
       <x:c r="J17" s="59" t="n"/>
       <x:c r="K17" s="59" t="n"/>
       <x:c r="L17" s="59" t="n"/>
     </x:row>
-    <x:row r="18" ht="85" customHeight="1">
+    <x:row r="18" ht="100" customHeight="1">
       <x:c r="A18" s="92" t="str">
         <x:v>Saturday</x:v>
       </x:c>
@@ -4425,28 +4427,28 @@
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="222" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="E18" s="222" t="str">
-        <x:v>Incline Barbell Bench Press</x:v>
+        <x:v>Straight-Arm Pulldown</x:v>
       </x:c>
       <x:c r="F18" s="222" t="str">
-        <x:v>15 x 12 @2; 17.5 x 10 @2; 20 x 6 @3</x:v>
+        <x:v>40 x15 @4; 45 x16 @3; 50 x12 @3</x:v>
       </x:c>
       <x:c r="G18" s="222" t="str">
-        <x:v>2 sets: 12.5-15 kg/side x10-12 @3-4</x:v>
+        <x:v>40 x12-15 @3-4; 45 x15-16 @3; 50 x12-13 @2-3. Agree two or three sets before starting.</x:v>
       </x:c>
       <x:c r="H18" s="222" t="str">
-        <x:v>Return targets</x:v>
+        <x:v>Recovery-led targets</x:v>
       </x:c>
       <x:c r="I18" s="222" t="str">
-        <x:v>See dated target notes</x:v>
+        <x:v>Latest dated revision</x:v>
       </x:c>
       <x:c r="J18" s="59" t="n"/>
       <x:c r="K18" s="59" t="n"/>
       <x:c r="L18" s="59" t="n"/>
     </x:row>
-    <x:row r="19" ht="85" customHeight="1">
+    <x:row r="19" ht="100" customHeight="1">
       <x:c r="A19" s="92" t="str">
         <x:v>Sunday</x:v>
       </x:c>
@@ -4455,100 +4457,100 @@
       </x:c>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="222" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Cable Fly</x:v>
+        <x:v>Iso-Lateral High Row</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>20 x 15 @3; 25 x 10 @2; 25 x 10 @2</x:v>
+        <x:v>15 x13 @2; 17.5 x11 @2; 20 x10 @2</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>2 sets: 15-20 kg/side x12-15 @3-4</x:v>
+        <x:v>15/side x13-15 @3; 17.5/side x11-12 @2-3; 20/side x10 @2-3 if three sets agreed.</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
-        <x:v>Return targets</x:v>
+        <x:v>Recovery-led targets</x:v>
       </x:c>
       <x:c r="I19" s="222" t="str">
-        <x:v>See dated target notes</x:v>
+        <x:v>Latest dated revision</x:v>
       </x:c>
       <x:c r="J19" s="59" t="n"/>
       <x:c r="K19" s="59" t="n"/>
       <x:c r="L19" s="59" t="n"/>
     </x:row>
-    <x:row r="20" ht="85" customHeight="1">
+    <x:row r="20" ht="100" customHeight="1">
       <x:c r="A20" s="59" t="n"/>
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="222" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Straight Bar Pushdown</x:v>
+        <x:v>Incline Dumbbell Curl</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>50 x 14 @3; 55 x 11 @2; 60 x 8 @2</x:v>
+        <x:v>10 x15 @1; 12.5 x10 @2; 15 x8 @1</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>2 sets: 40-45 kg x12-15 @3-4</x:v>
+        <x:v>10 each x10-12 @3; 12.5 each x8-10 @2-3. Omit 15 kg until lower loads stay controlled at target reserve.</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
-        <x:v>Return targets</x:v>
+        <x:v>Recovery-led targets</x:v>
       </x:c>
       <x:c r="I20" s="222" t="str">
-        <x:v>See dated target notes</x:v>
+        <x:v>Latest dated revision</x:v>
       </x:c>
       <x:c r="J20" s="59" t="n"/>
       <x:c r="K20" s="59" t="n"/>
       <x:c r="L20" s="59" t="n"/>
     </x:row>
-    <x:row r="21" ht="85" customHeight="1">
+    <x:row r="21" ht="100" customHeight="1">
       <x:c r="A21" s="59" t="n"/>
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="222" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="E21" s="222" t="str">
-        <x:v>Overhead Rope Extension</x:v>
+        <x:v>Hammer Curl</x:v>
       </x:c>
       <x:c r="F21" s="222" t="str">
-        <x:v>35 x 14 @3; 40 x 11 @2; 45 x 9 @2</x:v>
+        <x:v>15 x12 @2; 17.5 x11 @2</x:v>
       </x:c>
       <x:c r="G21" s="222" t="str">
-        <x:v>2 sets: 25-30 kg x12-15 @3-4</x:v>
+        <x:v>15 each x12 @2-3; 17.5 each x11-12 @2. No load increase yet.</x:v>
       </x:c>
       <x:c r="H21" s="222" t="str">
-        <x:v>Return targets</x:v>
+        <x:v>Recovery-led targets</x:v>
       </x:c>
       <x:c r="I21" s="222" t="str">
-        <x:v>See dated target notes</x:v>
+        <x:v>Latest dated revision</x:v>
       </x:c>
       <x:c r="J21" s="59" t="n"/>
       <x:c r="K21" s="59" t="n"/>
       <x:c r="L21" s="59" t="n"/>
     </x:row>
-    <x:row r="22" ht="85" customHeight="1">
+    <x:row r="22" ht="100" customHeight="1">
       <x:c r="A22" s="59" t="n"/>
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="222" t="str">
-        <x:v>Chest + Triceps</x:v>
+        <x:v>Back + Biceps</x:v>
       </x:c>
       <x:c r="E22" s="222" t="str">
-        <x:v>Assisted Dip Machine</x:v>
+        <x:v>Plate Curl Machine</x:v>
       </x:c>
       <x:c r="F22" s="222" t="str">
-        <x:v>60 x 12 @2; 50 x 8 @2</x:v>
+        <x:v>7.5 x15 @3; 10 x14 @2; 12.5 x11 @2</x:v>
       </x:c>
       <x:c r="G22" s="222" t="str">
-        <x:v>2 sets: 70 kg assistance x8-12 @3-4</x:v>
+        <x:v>10/side x14 @2-3; 12.5/side x11-12 @2. 7.5 kg preparation only if easy; avoid adding fatigue sets.</x:v>
       </x:c>
       <x:c r="H22" s="222" t="str">
-        <x:v>Return targets</x:v>
+        <x:v>Recovery-led targets</x:v>
       </x:c>
       <x:c r="I22" s="222" t="str">
-        <x:v>See dated target notes</x:v>
+        <x:v>Latest dated revision</x:v>
       </x:c>
       <x:c r="J22" s="59" t="n"/>
       <x:c r="K22" s="59" t="n"/>
@@ -4565,16 +4567,16 @@
         <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>Medium after 90 min</x:v>
+        <x:v>Medium after 75 min</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
-        <x:v>Monitor delayed symptoms</x:v>
+        <x:v>No symptoms reported</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>No pain reported</x:v>
+        <x:v>Monitor next day</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>18 working sets exceeded lighter return plan</x:v>
+        <x:v>17 sets; 15 min walk</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4588,19 +4590,19 @@
         <x:v>Next</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
         <x:v>Fresh readiness first</x:v>
       </x:c>
       <x:c r="G24" s="50" t="str">
-        <x:v>10-12 work sets, RIR 3-4</x:v>
+        <x:v>Agree workload before lifting</x:v>
       </x:c>
       <x:c r="H24" s="50" t="str">
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="I24" s="50" t="str">
-        <x:v>No automatic load increases</x:v>
+        <x:v>No automatic progression</x:v>
       </x:c>
       <x:c r="J24" s="50" t="n"/>
       <x:c r="K24" s="50" t="n"/>
@@ -4629,7 +4631,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae166b3f897c487b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfeb256f56d4c13"/>
 </x:worksheet>
 </file>
 
@@ -29186,6 +29188,754 @@
         <x:v>Working</x:v>
       </x:c>
       <x:c r="N582" s="170" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="583" ht="70" customHeight="1">
+      <x:c r="A583" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B583" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C583" s="169" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="D583" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E583" s="169" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F583" s="169" t="str">
+        <x:v>kg total added plates; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="G583" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H583" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I583" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J583" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K583" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L583" s="169" t="str">
+        <x:v>Chest support and total plates explicitly confirmed. Prior September 1 load-basis uncertainty remains historical.</x:v>
+      </x:c>
+      <x:c r="M583" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N583" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="584" ht="70" customHeight="1">
+      <x:c r="A584" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B584" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C584" s="169" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="D584" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E584" s="169" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F584" s="169" t="str">
+        <x:v>kg total added plates; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="G584" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H584" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I584" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J584" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K584" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L584" s="169" t="str">
+        <x:v>Chest support and total plates explicitly confirmed. Prior September 1 load-basis uncertainty remains historical.</x:v>
+      </x:c>
+      <x:c r="M584" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N584" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="585" ht="70" customHeight="1">
+      <x:c r="A585" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B585" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C585" s="169" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="D585" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E585" s="169" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F585" s="169" t="str">
+        <x:v>kg total added plates; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="G585" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H585" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I585" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J585" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K585" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L585" s="169" t="str">
+        <x:v>Chest support and total plates explicitly confirmed. Prior September 1 load-basis uncertainty remains historical.</x:v>
+      </x:c>
+      <x:c r="M585" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N585" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="586" ht="70" customHeight="1">
+      <x:c r="A586" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B586" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C586" s="169" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D586" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E586" s="169" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F586" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G586" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H586" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I586" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J586" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K586" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L586" s="169" t="str">
+        <x:v>First set not explicitly designated warm-up.</x:v>
+      </x:c>
+      <x:c r="M586" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N586" s="169" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="587" ht="70" customHeight="1">
+      <x:c r="A587" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B587" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C587" s="169" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D587" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E587" s="169" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F587" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G587" s="169" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H587" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I587" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J587" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K587" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L587" s="169" t="str">
+        <x:v>First set not explicitly designated warm-up.</x:v>
+      </x:c>
+      <x:c r="M587" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N587" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="588" ht="70" customHeight="1">
+      <x:c r="A588" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B588" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C588" s="169" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="D588" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E588" s="169" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="F588" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G588" s="169" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H588" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I588" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J588" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K588" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L588" s="169" t="str">
+        <x:v>First set not explicitly designated warm-up.</x:v>
+      </x:c>
+      <x:c r="M588" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N588" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="589" ht="70" customHeight="1">
+      <x:c r="A589" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B589" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C589" s="169" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D589" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E589" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F589" s="169" t="str">
+        <x:v>kg plates each side; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="G589" s="169" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H589" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I589" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J589" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K589" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L589" s="169" t="str">
+        <x:v>User identified as scheduled machine; exact model/selected grip To verify.</x:v>
+      </x:c>
+      <x:c r="M589" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N589" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="590" ht="70" customHeight="1">
+      <x:c r="A590" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B590" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C590" s="169" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D590" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E590" s="169" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F590" s="169" t="str">
+        <x:v>kg plates each side; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="G590" s="169" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H590" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I590" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J590" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K590" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L590" s="169" t="str">
+        <x:v>User identified as scheduled machine; exact model/selected grip To verify.</x:v>
+      </x:c>
+      <x:c r="M590" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N590" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="591" ht="70" customHeight="1">
+      <x:c r="A591" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B591" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C591" s="169" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="D591" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E591" s="169" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F591" s="169" t="str">
+        <x:v>kg plates each side; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="G591" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H591" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I591" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J591" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K591" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L591" s="169" t="str">
+        <x:v>User identified as scheduled machine; exact model/selected grip To verify.</x:v>
+      </x:c>
+      <x:c r="M591" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N591" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="592" ht="70" customHeight="1">
+      <x:c r="A592" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B592" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C592" s="169" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D592" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E592" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F592" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G592" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H592" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I592" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J592" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K592" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L592" s="169" t="str">
+        <x:v>Two sets near failure; next improve reserve rather than increase load.</x:v>
+      </x:c>
+      <x:c r="M592" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N592" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="593" ht="70" customHeight="1">
+      <x:c r="A593" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B593" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C593" s="169" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D593" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E593" s="169" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F593" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G593" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H593" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I593" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J593" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K593" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L593" s="169" t="str">
+        <x:v>Two sets near failure; next improve reserve rather than increase load.</x:v>
+      </x:c>
+      <x:c r="M593" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N593" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="594" ht="70" customHeight="1">
+      <x:c r="A594" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B594" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C594" s="169" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="D594" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E594" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F594" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G594" s="169" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H594" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I594" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J594" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K594" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L594" s="169" t="str">
+        <x:v>Two sets near failure; next improve reserve rather than increase load.</x:v>
+      </x:c>
+      <x:c r="M594" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N594" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="595" ht="70" customHeight="1">
+      <x:c r="A595" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B595" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C595" s="169" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D595" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E595" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F595" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G595" s="169" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H595" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I595" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J595" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K595" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L595" s="169" t="str">
+        <x:v>Matched previous repetitions and reserve.</x:v>
+      </x:c>
+      <x:c r="M595" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N595" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="596" ht="70" customHeight="1">
+      <x:c r="A596" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B596" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C596" s="169" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="D596" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E596" s="169" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F596" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G596" s="169" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H596" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I596" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J596" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K596" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L596" s="169" t="str">
+        <x:v>Matched previous repetitions and reserve.</x:v>
+      </x:c>
+      <x:c r="M596" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N596" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="597" ht="70" customHeight="1">
+      <x:c r="A597" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B597" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C597" s="169" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D597" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E597" s="169" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F597" s="169" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G597" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H597" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I597" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J597" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K597" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L597" s="169" t="str">
+        <x:v>Replaced concentration curl; top two sets matched September 5.</x:v>
+      </x:c>
+      <x:c r="M597" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N597" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="598" ht="70" customHeight="1">
+      <x:c r="A598" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B598" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C598" s="169" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D598" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E598" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F598" s="169" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G598" s="169" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H598" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I598" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J598" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K598" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L598" s="169" t="str">
+        <x:v>Replaced concentration curl; top two sets matched September 5.</x:v>
+      </x:c>
+      <x:c r="M598" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N598" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="599" ht="70" customHeight="1">
+      <x:c r="A599" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B599" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C599" s="169" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="D599" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E599" s="169" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F599" s="169" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="G599" s="169" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H599" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I599" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J599" s="169" t="str">
+        <x:v>Medium-High start; Medium final</x:v>
+      </x:c>
+      <x:c r="K599" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L599" s="169" t="str">
+        <x:v>Replaced concentration curl; top two sets matched September 5.</x:v>
+      </x:c>
+      <x:c r="M599" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N599" s="169" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -29221,7 +29971,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffea5388e11f431a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree5c384ec71f4d14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30883,6 +31633,180 @@
       </x:c>
       <x:c r="I58" s="170" t="str">
         <x:v>Dated target revision; prior targets/history retained. Conditional on symptom-free recovery; older best sets are not erased.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="120" customHeight="1">
+      <x:c r="A59" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="B59" s="169" t="str">
+        <x:v>Chest-Supported T-Bar Row</x:v>
+      </x:c>
+      <x:c r="C59" s="169" t="str">
+        <x:v>20 x15 @3; 35 x15 @3; 45 x10 @3</x:v>
+      </x:c>
+      <x:c r="D59" s="169" t="str">
+        <x:v>kg total added plates; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="E59" s="169" t="str">
+        <x:v>20 x12-15 @3 preparation only if genuinely easy; 35 x15 @3; 45 x10-11 @2-3. Same machine and total plates.</x:v>
+      </x:c>
+      <x:c r="F59" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G59" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H59" s="169" t="str">
+        <x:v>2026-09-15 targets</x:v>
+      </x:c>
+      <x:c r="I59" s="169" t="str">
+        <x:v>Dated revision; prior records retained. Chest support and total plates explicitly confirmed. Prior September 1 load-basis uncertainty remains historical.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="120" customHeight="1">
+      <x:c r="A60" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="B60" s="169" t="str">
+        <x:v>Straight-Arm Pulldown</x:v>
+      </x:c>
+      <x:c r="C60" s="169" t="str">
+        <x:v>40 x15 @4; 45 x16 @3; 50 x12 @3</x:v>
+      </x:c>
+      <x:c r="D60" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="E60" s="169" t="str">
+        <x:v>40 x12-15 @3-4; 45 x15-16 @3; 50 x12-13 @2-3. Agree two or three sets before starting.</x:v>
+      </x:c>
+      <x:c r="F60" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G60" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H60" s="169" t="str">
+        <x:v>2026-09-15 targets</x:v>
+      </x:c>
+      <x:c r="I60" s="169" t="str">
+        <x:v>Dated revision; prior records retained. First set not explicitly designated warm-up.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="120" customHeight="1">
+      <x:c r="A61" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="B61" s="169" t="str">
+        <x:v>Iso-Lateral High Row</x:v>
+      </x:c>
+      <x:c r="C61" s="169" t="str">
+        <x:v>15 x13 @2; 17.5 x11 @2; 20 x10 @2</x:v>
+      </x:c>
+      <x:c r="D61" s="169" t="str">
+        <x:v>kg plates each side; starting resistance excluded</x:v>
+      </x:c>
+      <x:c r="E61" s="169" t="str">
+        <x:v>15/side x13-15 @3; 17.5/side x11-12 @2-3; 20/side x10 @2-3 if three sets agreed.</x:v>
+      </x:c>
+      <x:c r="F61" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G61" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H61" s="169" t="str">
+        <x:v>2026-09-15 targets</x:v>
+      </x:c>
+      <x:c r="I61" s="169" t="str">
+        <x:v>Dated revision; prior records retained. User identified as scheduled machine; exact model/selected grip To verify.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="120" customHeight="1">
+      <x:c r="A62" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="B62" s="169" t="str">
+        <x:v>Incline Dumbbell Curl</x:v>
+      </x:c>
+      <x:c r="C62" s="169" t="str">
+        <x:v>10 x15 @1; 12.5 x10 @2; 15 x8 @1</x:v>
+      </x:c>
+      <x:c r="D62" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="E62" s="169" t="str">
+        <x:v>10 each x10-12 @3; 12.5 each x8-10 @2-3. Omit 15 kg until lower loads stay controlled at target reserve.</x:v>
+      </x:c>
+      <x:c r="F62" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G62" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H62" s="169" t="str">
+        <x:v>2026-09-15 targets</x:v>
+      </x:c>
+      <x:c r="I62" s="169" t="str">
+        <x:v>Dated revision; prior records retained. Two sets near failure; next improve reserve rather than increase load.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="120" customHeight="1">
+      <x:c r="A63" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="B63" s="169" t="str">
+        <x:v>Hammer Curl</x:v>
+      </x:c>
+      <x:c r="C63" s="169" t="str">
+        <x:v>15 x12 @2; 17.5 x11 @2</x:v>
+      </x:c>
+      <x:c r="D63" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="E63" s="169" t="str">
+        <x:v>15 each x12 @2-3; 17.5 each x11-12 @2. No load increase yet.</x:v>
+      </x:c>
+      <x:c r="F63" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G63" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H63" s="169" t="str">
+        <x:v>2026-09-15 targets</x:v>
+      </x:c>
+      <x:c r="I63" s="169" t="str">
+        <x:v>Dated revision; prior records retained. Matched previous repetitions and reserve.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="120" customHeight="1">
+      <x:c r="A64" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="B64" s="169" t="str">
+        <x:v>Plate Curl Machine</x:v>
+      </x:c>
+      <x:c r="C64" s="169" t="str">
+        <x:v>7.5 x15 @3; 10 x14 @2; 12.5 x11 @2</x:v>
+      </x:c>
+      <x:c r="D64" s="169" t="str">
+        <x:v>kg plates each side</x:v>
+      </x:c>
+      <x:c r="E64" s="169" t="str">
+        <x:v>10/side x14 @2-3; 12.5/side x11-12 @2. 7.5 kg preparation only if easy; avoid adding fatigue sets.</x:v>
+      </x:c>
+      <x:c r="F64" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G64" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H64" s="169" t="str">
+        <x:v>2026-09-15 targets</x:v>
+      </x:c>
+      <x:c r="I64" s="169" t="str">
+        <x:v>Dated revision; prior records retained. Replaced concentration curl; top two sets matched September 5.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -30910,7 +31834,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d04882cf8284675"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd98b03e69e0649a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32094,17 +33018,29 @@
       <x:c r="P35" s="59" t="n"/>
       <x:c r="Q35" s="59" t="n"/>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36"/>
-      <x:c r="B36"/>
-      <x:c r="C36"/>
-      <x:c r="D36"/>
-      <x:c r="E36"/>
-      <x:c r="F36"/>
-      <x:c r="G36"/>
-      <x:c r="H36"/>
-      <x:c r="I36"/>
-      <x:c r="J36"/>
+    <x:row r="36" ht="210" customHeight="1">
+      <x:c r="A36" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B36" s="169"/>
+      <x:c r="C36" s="169"/>
+      <x:c r="D36" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E36" s="169" t="str">
+        <x:v>Medium final</x:v>
+      </x:c>
+      <x:c r="F36" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="G36" s="169"/>
+      <x:c r="H36" s="169"/>
+      <x:c r="I36" s="169" t="str">
+        <x:v>15 min treadmill; 3 km/h; 12% incline; no rail support</x:v>
+      </x:c>
+      <x:c r="J36" s="169" t="str">
+        <x:v>75 minutes including 15 min treadmill at 3 km/h, 12% incline, no rail support. Good sleep; Medium-High starting energy; Medium final energy and pump. No symptoms, human-assisted reps or reported form breakdown. Full EAA+ (100 mg label-verified caffeine) plus half pre-workout (~100 mg user-stated); ~200 mg combined caffeine estimate, pre-workout label To verify. No coffee. Creatine/magnesium today To verify.</x:v>
+      </x:c>
       <x:c r="K36" s="59" t="n"/>
       <x:c r="L36" s="59" t="n"/>
       <x:c r="M36" s="59" t="n"/>
@@ -35285,7 +36221,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4429d5d4c204447"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R011ecc6536264b36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -36818,13 +37754,69 @@
         <x:v>For each exercise show prior actual loads/reps/RIR alongside current targets and exact load basis.</x:v>
       </x:c>
     </x:row>
+    <x:row r="105" ht="180" customHeight="1">
+      <x:c r="A105" s="169" t="str">
+        <x:v>2026-09-15 completion</x:v>
+      </x:c>
+      <x:c r="B105" s="169" t="str">
+        <x:v>17 working sets across six exercises: nine back and eight biceps. No separate warm-up reported; the 40 kg straight-arm set at RIR 4 is retained as performed, not silently reclassified. RIR distribution: one at 4, six at 3, eight at 2, two at 1. Machine availability changed the order and selections. Stable hammer and machine-curl top sets; higher effort on incline curls. No reported symptoms; monitor delayed recovery. Actual volume and incline exceeded the initial return prescription, but 12 sets is not a universal safety cutoff.</x:v>
+      </x:c>
+      <x:c r="C105" s="169" t="str">
+        <x:v>Self-reported symptom-free completion is encouraging; delayed recovery is not yet known.</x:v>
+      </x:c>
+      <x:c r="D105" s="169" t="str">
+        <x:v>Review next-morning symptoms, sleep, energy and soreness.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="180" customHeight="1">
+      <x:c r="A106" s="169" t="str">
+        <x:v>2026-09-15 coaching preference</x:v>
+      </x:c>
+      <x:c r="B106" s="169" t="str">
+        <x:v>Vipin objects to arbitrary limits when feeling well and wants three biceps exercises. Coach acknowledged that 12 sets is not a universal safety cutoff.</x:v>
+      </x:c>
+      <x:c r="C106" s="169" t="str">
+        <x:v>Agree a meaningful workload up front rather than repeatedly changing it mid-session. Preferences do not remove the need to assess fatigue or symptoms.</x:v>
+      </x:c>
+      <x:c r="D106" s="169" t="str">
+        <x:v>Review weekly volume and recovery; retain evidence-based advice without punitive progression language.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="180" customHeight="1">
+      <x:c r="A107" s="169" t="str">
+        <x:v>2026-09-15 supplements</x:v>
+      </x:c>
+      <x:c r="B107" s="169" t="str">
+        <x:v>Full EAA+ (100 mg label-verified caffeine) plus half pre-workout (~100 mg user-stated); ~200 mg combined caffeine estimate, pre-workout label To verify. No coffee. Creatine/magnesium today To verify.</x:v>
+      </x:c>
+      <x:c r="C107" s="169" t="str">
+        <x:v>Pre-workout caffeine amount is not independently label-verified.</x:v>
+      </x:c>
+      <x:c r="D107" s="169" t="str">
+        <x:v>Obtain product label; track sleep response without inferring caffeine caused or resolved prior headache.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="180" customHeight="1">
+      <x:c r="A108" s="169" t="str">
+        <x:v>2026-09-15 next session</x:v>
+      </x:c>
+      <x:c r="B108" s="169" t="str">
+        <x:v>Shoulders + Triceps next after fresh sleep, energy, soreness and head/neck symptom check. Agree exercise count, sets and substitutions before lifting; consider recent pressing/arm workload. Keep most sets at RIR 2-3, no forced reps; adjust to observed recovery, not energy alone. No automatic load increases.</x:v>
+      </x:c>
+      <x:c r="C108" s="169" t="str">
+        <x:v>Second consecutive return-week session completed.</x:v>
+      </x:c>
+      <x:c r="D108" s="169" t="str">
+        <x:v>Use matching historical exercise baselines and exact load basis before each exercise.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692c984f1ffc4b1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa26f63aa8b4fba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37701,6 +38693,32 @@
         <x:v>Next scheduled Back + Biceps only after fresh readiness and no recurrent headache, neck symptoms or limiting soreness. Start with 10-12 working sets at RIR 3-4; no failure or extra sets. Easy flat walking 5-10 min optional. Stop and seek clinician advice if headache recurs.</x:v>
       </x:c>
     </x:row>
+    <x:row r="34" ht="250" customHeight="1">
+      <x:c r="A34" s="380" t="n">
+        <x:v>46280</x:v>
+      </x:c>
+      <x:c r="B34" s="169" t="str">
+        <x:v>Back + Biceps</x:v>
+      </x:c>
+      <x:c r="C34" s="169" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D34" s="169" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E34" s="169" t="str">
+        <x:v>Symptom-free / monitor recovery</x:v>
+      </x:c>
+      <x:c r="F34" s="169" t="str">
+        <x:v>75 minutes including 15 min treadmill at 3 km/h, 12% incline, no rail support. Good sleep; Medium-High starting energy; Medium final energy and pump. No symptoms, human-assisted reps or reported form breakdown. Full EAA+ (100 mg label-verified caffeine) plus half pre-workout (~100 mg user-stated); ~200 mg combined caffeine estimate, pre-workout label To verify. No coffee. Creatine/magnesium today To verify.</x:v>
+      </x:c>
+      <x:c r="G34" s="169" t="str">
+        <x:v>17 working sets across six exercises: nine back and eight biceps. No separate warm-up reported; the 40 kg straight-arm set at RIR 4 is retained as performed, not silently reclassified. RIR distribution: one at 4, six at 3, eight at 2, two at 1. Machine availability changed the order and selections. Stable hammer and machine-curl top sets; higher effort on incline curls. No reported symptoms; monitor delayed recovery. Actual volume and incline exceeded the initial return prescription, but 12 sets is not a universal safety cutoff.</x:v>
+      </x:c>
+      <x:c r="H34" s="169" t="str">
+        <x:v>Shoulders + Triceps next after fresh sleep, energy, soreness and head/neck symptom check. Agree exercise count, sets and substitutions before lifting; consider recent pressing/arm workload. Keep most sets at RIR 2-3, no forced reps; adjust to observed recovery, not energy alone. No automatic load increases.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -37713,7 +38731,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04206bc10cbf4219"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc73b386cfd4c2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38283,7 +39301,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bcc832898f34994"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fca50a8a96c4eb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39389,10 +40407,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re32e5b5392264568"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ab5add18e83462b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6a1dccc521f4476"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R222e1d9c243e4c53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf817f55a144e4cf5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab66aed30cb34a13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d8165eb7366495a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34d5cecc9344e46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Log September 16 shoulders triceps and confirmed recovery
</commit_message>
<xml_diff>
--- a/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
+++ b/Vipin_Gym_Progress_Dashboard_2026-08-07_v2.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6a98311f5a0346f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Ra6408bd5238548e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="Rf3aae14e68384fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R527331f8173e457b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R1912a0bca44b4d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="Re6eefc45c91140b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="R9425644901ae4fa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="R0b6871c9e7bc4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rda1e234804f74e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="Rc2d46953f32e4c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="Rb8590727a20c47d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4d968c592d684f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R89257de04e7044c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workout Journal" sheetId="3" r:id="R06e2ab56b9d240cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercise Targets" sheetId="4" r:id="R49a9e464933a49d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Body" sheetId="5" r:id="R79903eaef603494c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Notes" sheetId="6" r:id="R2f2c6b53d9c74b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Session Summary" sheetId="7" r:id="Rea9d6af503cd4c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coaching Profile" sheetId="8" r:id="Rd74e0077d1d747ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutrition Plan" sheetId="9" r:id="Rf257d31094a84c29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos &amp; Measurements" sheetId="10" r:id="R06f81ff257004600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protein Calculator" sheetId="11" r:id="R8276107ae2104e5a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1726,7 +1726,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb0d576648fb945df"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5f7c44fcf86d4b5b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1736,7 +1736,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N599" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="28" name="WorkoutJournalTable" displayName="WorkoutJournalTable" ref="A4:N618" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -1806,7 +1806,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="31" name="ExerciseTargetsTable" displayName="ExerciseTargetsTable" ref="A4:I70" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="Muscle"/>
     <x:tableColumn id="2" name="Exercise"/>
@@ -1823,7 +1823,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="33" name="RecoveryTable" displayName="RecoveryTable" ref="A4:J37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Weight (kg)"/>
@@ -1841,7 +1841,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D108" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="ProgramNotesTable" displayName="ProgramNotesTable" ref="A4:D112" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Category"/>
     <x:tableColumn id="2" name="Rule / Observation"/>
@@ -1853,7 +1853,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="SessionSummaryTable" displayName="SessionSummaryTable" ref="A4:H35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Workout"/>
@@ -2555,7 +2555,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4efd725e403b419d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff27b6bc6867478f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3958,7 +3958,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc05b3d83460641d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c57a7d0cc764df5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4086,8 +4086,8 @@
       </x:c>
       <x:c r="C5" s="59" t="n"/>
       <x:c r="D5" s="93" t="n">
-        <x:f>COUNT('Session Summary'!A5:A34)</x:f>
-        <x:v>30</x:v>
+        <x:f>COUNT('Session Summary'!A5:A35)</x:f>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E5" s="53" t="n"/>
       <x:c r="F5" s="93" t="n">
@@ -4313,7 +4313,7 @@
         <x:v>Tuesday</x:v>
       </x:c>
       <x:c r="B14" s="59" t="str">
-        <x:v>Back + Biceps completed 2026-09-15</x:v>
+        <x:v>Shoulders + Triceps completed 2026-09-16</x:v>
       </x:c>
       <x:c r="C14" s="59" t="n"/>
       <x:c r="D14" s="59" t="n"/>
@@ -4397,16 +4397,16 @@
       </x:c>
       <x:c r="C17" s="59" t="n"/>
       <x:c r="D17" s="222" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="E17" s="222" t="str">
-        <x:v>Chest-Supported T-Bar Row</x:v>
+        <x:v>Dumbbell Shoulder Press</x:v>
       </x:c>
       <x:c r="F17" s="222" t="str">
-        <x:v>20 x15 @3; 35 x15 @3; 45 x10 @3</x:v>
+        <x:v>17.5 x12 @3; 20 x12 @3; 22.5 x10 @2; 25 x7 @2</x:v>
       </x:c>
       <x:c r="G17" s="222" t="str">
-        <x:v>20 x12-15 @3 preparation only if genuinely easy; 35 x15 @3; 45 x10-11 @2-3. Same machine and total plates.</x:v>
+        <x:v>17.5 each x12-15 @3; 20 x12-13 @2-3; 22.5 x10-11 @2. Optional 25 x7-8 @2 replaces a set if agreed, not automatically added.</x:v>
       </x:c>
       <x:c r="H17" s="222" t="str">
         <x:v>Recovery-led targets</x:v>
@@ -4427,16 +4427,16 @@
       </x:c>
       <x:c r="C18" s="59" t="n"/>
       <x:c r="D18" s="222" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="E18" s="222" t="str">
-        <x:v>Straight-Arm Pulldown</x:v>
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
       </x:c>
       <x:c r="F18" s="222" t="str">
-        <x:v>40 x15 @4; 45 x16 @3; 50 x12 @3</x:v>
+        <x:v>2.5 x20 @3; 5 x14 @3; 7.5 x10 @2</x:v>
       </x:c>
       <x:c r="G18" s="222" t="str">
-        <x:v>40 x12-15 @3-4; 45 x15-16 @3; 50 x12-13 @2-3. Agree two or three sets before starting.</x:v>
+        <x:v>2.5/side x15-20 @3; 5 x14-15 @2-3; 7.5 x10-11 @2. Hold load.</x:v>
       </x:c>
       <x:c r="H18" s="222" t="str">
         <x:v>Recovery-led targets</x:v>
@@ -4457,16 +4457,16 @@
       </x:c>
       <x:c r="C19" s="59" t="n"/>
       <x:c r="D19" s="222" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="E19" s="222" t="str">
-        <x:v>Iso-Lateral High Row</x:v>
+        <x:v>Reverse Pec Deck</x:v>
       </x:c>
       <x:c r="F19" s="222" t="str">
-        <x:v>15 x13 @2; 17.5 x11 @2; 20 x10 @2</x:v>
+        <x:v>30 x15 @3; 35 x12 @2; 40 x8 @2</x:v>
       </x:c>
       <x:c r="G19" s="222" t="str">
-        <x:v>15/side x13-15 @3; 17.5/side x11-12 @2-3; 20/side x10 @2-3 if three sets agreed.</x:v>
+        <x:v>30 x15 @3; 35 x12-13 @2; 40 x8-9 @2 if three sets agreed.</x:v>
       </x:c>
       <x:c r="H19" s="222" t="str">
         <x:v>Recovery-led targets</x:v>
@@ -4483,16 +4483,16 @@
       <x:c r="B20" s="59" t="n"/>
       <x:c r="C20" s="59" t="n"/>
       <x:c r="D20" s="222" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="E20" s="222" t="str">
-        <x:v>Incline Dumbbell Curl</x:v>
+        <x:v>Rope Pushdown</x:v>
       </x:c>
       <x:c r="F20" s="222" t="str">
-        <x:v>10 x15 @1; 12.5 x10 @2; 15 x8 @1</x:v>
+        <x:v>30 x17 @2; 35 x11 @2; 40 x9 @3</x:v>
       </x:c>
       <x:c r="G20" s="222" t="str">
-        <x:v>10 each x10-12 @3; 12.5 each x8-10 @2-3. Omit 15 kg until lower loads stay controlled at target reserve.</x:v>
+        <x:v>30 x15-17 @3; 35 x11-13 @2; 40 x9-10 @2-3 if third set agreed.</x:v>
       </x:c>
       <x:c r="H20" s="222" t="str">
         <x:v>Recovery-led targets</x:v>
@@ -4509,16 +4509,16 @@
       <x:c r="B21" s="59" t="n"/>
       <x:c r="C21" s="59" t="n"/>
       <x:c r="D21" s="222" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="E21" s="222" t="str">
-        <x:v>Hammer Curl</x:v>
+        <x:v>Single-Arm Cable Pushdown</x:v>
       </x:c>
       <x:c r="F21" s="222" t="str">
-        <x:v>15 x12 @2; 17.5 x11 @2</x:v>
+        <x:v>5 x20 @3; 10 x15 @3; 15 x11 @3</x:v>
       </x:c>
       <x:c r="G21" s="222" t="str">
-        <x:v>15 each x12 @2-3; 17.5 each x11-12 @2. No load increase yet.</x:v>
+        <x:v>10 each arm x15 @3; 15 x11-12 @2-3. 5 kg preparation only if genuinely easy.</x:v>
       </x:c>
       <x:c r="H21" s="222" t="str">
         <x:v>Recovery-led targets</x:v>
@@ -4535,16 +4535,16 @@
       <x:c r="B22" s="59" t="n"/>
       <x:c r="C22" s="59" t="n"/>
       <x:c r="D22" s="222" t="str">
-        <x:v>Back + Biceps</x:v>
+        <x:v>Shoulders + Triceps</x:v>
       </x:c>
       <x:c r="E22" s="222" t="str">
-        <x:v>Plate Curl Machine</x:v>
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
       </x:c>
       <x:c r="F22" s="222" t="str">
-        <x:v>7.5 x15 @3; 10 x14 @2; 12.5 x11 @2</x:v>
+        <x:v>20 x15 @3; 25 x12 @2; 30 x8 @2</x:v>
       </x:c>
       <x:c r="G22" s="222" t="str">
-        <x:v>10/side x14 @2-3; 12.5/side x11-12 @2. 7.5 kg preparation only if easy; avoid adding fatigue sets.</x:v>
+        <x:v>20 total x15 @3; 25 x12-13 @2; 30 x8-9 @2 if third set agreed. Hold load.</x:v>
       </x:c>
       <x:c r="H22" s="222" t="str">
         <x:v>Recovery-led targets</x:v>
@@ -4567,16 +4567,16 @@
         <x:v>Final energy</x:v>
       </x:c>
       <x:c r="F23" s="50" t="str">
-        <x:v>Medium after 75 min</x:v>
+        <x:v>Medium to High after 90 min</x:v>
       </x:c>
       <x:c r="G23" s="50" t="str">
         <x:v>No symptoms reported</x:v>
       </x:c>
       <x:c r="H23" s="50" t="str">
-        <x:v>Monitor next day</x:v>
+        <x:v>Very good pump</x:v>
       </x:c>
       <x:c r="I23" s="50" t="str">
-        <x:v>17 sets; 15 min walk</x:v>
+        <x:v>19 sets; 15 min walk</x:v>
       </x:c>
       <x:c r="J23" s="50" t="n"/>
       <x:c r="K23" s="50" t="n"/>
@@ -4590,7 +4590,7 @@
         <x:v>Next</x:v>
       </x:c>
       <x:c r="E24" s="50" t="str">
-        <x:v>Shoulders + Triceps</x:v>
+        <x:v>Legs + Calves</x:v>
       </x:c>
       <x:c r="F24" s="50" t="str">
         <x:v>Fresh readiness first</x:v>
@@ -4631,7 +4631,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfeb256f56d4c13"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62d5ec4c06e141d5"/>
 </x:worksheet>
 </file>
 
@@ -29936,6 +29936,842 @@
         <x:v>Working</x:v>
       </x:c>
       <x:c r="N599" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="600" ht="70" customHeight="1">
+      <x:c r="A600" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B600" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C600" s="169" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D600" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E600" s="169" t="n">
+        <x:v>17.5</x:v>
+      </x:c>
+      <x:c r="F600" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G600" s="169" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H600" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I600" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J600" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K600" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L600" s="169" t="str">
+        <x:v>Four working sets; no warm-up reported. Hold load and rebuild reps.</x:v>
+      </x:c>
+      <x:c r="M600" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N600" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="601" ht="70" customHeight="1">
+      <x:c r="A601" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B601" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C601" s="169" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D601" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E601" s="169" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F601" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G601" s="169" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H601" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I601" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J601" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K601" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L601" s="169" t="str">
+        <x:v>Four working sets; no warm-up reported. Hold load and rebuild reps.</x:v>
+      </x:c>
+      <x:c r="M601" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N601" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="602" ht="70" customHeight="1">
+      <x:c r="A602" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B602" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C602" s="169" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D602" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E602" s="169" t="n">
+        <x:v>22.5</x:v>
+      </x:c>
+      <x:c r="F602" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G602" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H602" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I602" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J602" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K602" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L602" s="169" t="str">
+        <x:v>Four working sets; no warm-up reported. Hold load and rebuild reps.</x:v>
+      </x:c>
+      <x:c r="M602" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N602" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="603" ht="70" customHeight="1">
+      <x:c r="A603" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B603" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C603" s="169" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="D603" s="169" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E603" s="169" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F603" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="G603" s="169" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H603" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I603" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J603" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K603" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L603" s="169" t="str">
+        <x:v>Four working sets; no warm-up reported. Hold load and rebuild reps.</x:v>
+      </x:c>
+      <x:c r="M603" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N603" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="604" ht="70" customHeight="1">
+      <x:c r="A604" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B604" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C604" s="169" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D604" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E604" s="169" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="F604" s="169" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="G604" s="169" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H604" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I604" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J604" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K604" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L604" s="169" t="str">
+        <x:v>Same established per-side convention; starting resistance excluded.</x:v>
+      </x:c>
+      <x:c r="M604" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N604" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="605" ht="70" customHeight="1">
+      <x:c r="A605" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B605" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C605" s="169" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D605" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E605" s="169" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F605" s="169" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="G605" s="169" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="H605" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I605" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J605" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K605" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L605" s="169" t="str">
+        <x:v>Same established per-side convention; starting resistance excluded.</x:v>
+      </x:c>
+      <x:c r="M605" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N605" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="606" ht="70" customHeight="1">
+      <x:c r="A606" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B606" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C606" s="169" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="D606" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E606" s="169" t="n">
+        <x:v>7.5</x:v>
+      </x:c>
+      <x:c r="F606" s="169" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="G606" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H606" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I606" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J606" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K606" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L606" s="169" t="str">
+        <x:v>Same established per-side convention; starting resistance excluded.</x:v>
+      </x:c>
+      <x:c r="M606" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N606" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="607" ht="70" customHeight="1">
+      <x:c r="A607" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B607" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C607" s="169" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D607" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E607" s="169" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F607" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G607" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H607" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I607" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J607" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K607" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L607" s="169" t="str">
+        <x:v>Controlled work with reserve; no pain reported.</x:v>
+      </x:c>
+      <x:c r="M607" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N607" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="608" ht="70" customHeight="1">
+      <x:c r="A608" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B608" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C608" s="169" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D608" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E608" s="169" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F608" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G608" s="169" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H608" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I608" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J608" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K608" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L608" s="169" t="str">
+        <x:v>Controlled work with reserve; no pain reported.</x:v>
+      </x:c>
+      <x:c r="M608" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N608" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="609" ht="70" customHeight="1">
+      <x:c r="A609" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B609" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C609" s="169" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="D609" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E609" s="169" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F609" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G609" s="169" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H609" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I609" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J609" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K609" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L609" s="169" t="str">
+        <x:v>Controlled work with reserve; no pain reported.</x:v>
+      </x:c>
+      <x:c r="M609" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N609" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="610" ht="70" customHeight="1">
+      <x:c r="A610" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B610" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C610" s="169" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D610" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E610" s="169" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F610" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G610" s="169" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H610" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I610" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J610" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K610" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L610" s="169" t="str">
+        <x:v>Retain actual reported RIR even though top set had more reserve.</x:v>
+      </x:c>
+      <x:c r="M610" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N610" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="611" ht="70" customHeight="1">
+      <x:c r="A611" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B611" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C611" s="169" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D611" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E611" s="169" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="F611" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G611" s="169" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H611" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I611" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J611" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K611" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L611" s="169" t="str">
+        <x:v>Retain actual reported RIR even though top set had more reserve.</x:v>
+      </x:c>
+      <x:c r="M611" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N611" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="612" ht="70" customHeight="1">
+      <x:c r="A612" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B612" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C612" s="169" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="D612" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E612" s="169" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F612" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="G612" s="169" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H612" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I612" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J612" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K612" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L612" s="169" t="str">
+        <x:v>Retain actual reported RIR even though top set had more reserve.</x:v>
+      </x:c>
+      <x:c r="M612" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N612" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="613" ht="70" customHeight="1">
+      <x:c r="A613" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B613" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C613" s="169" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D613" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E613" s="169" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F613" s="169" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="G613" s="169" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H613" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I613" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J613" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K613" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L613" s="169" t="str">
+        <x:v>Both arms same reps confirmed. Paired sets counted once, not doubled.</x:v>
+      </x:c>
+      <x:c r="M613" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N613" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="614" ht="70" customHeight="1">
+      <x:c r="A614" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B614" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C614" s="169" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D614" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E614" s="169" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F614" s="169" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="G614" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H614" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I614" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J614" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K614" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L614" s="169" t="str">
+        <x:v>Both arms same reps confirmed. Paired sets counted once, not doubled.</x:v>
+      </x:c>
+      <x:c r="M614" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N614" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="615" ht="70" customHeight="1">
+      <x:c r="A615" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B615" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C615" s="169" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="D615" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E615" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F615" s="169" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="G615" s="169" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H615" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I615" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J615" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K615" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L615" s="169" t="str">
+        <x:v>Both arms same reps confirmed. Paired sets counted once, not doubled.</x:v>
+      </x:c>
+      <x:c r="M615" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N615" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="616" ht="70" customHeight="1">
+      <x:c r="A616" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B616" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C616" s="169" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D616" s="169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E616" s="169" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F616" s="169" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="G616" s="169" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="H616" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I616" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J616" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K616" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L616" s="169" t="str">
+        <x:v>One total dumbbell, not per side.</x:v>
+      </x:c>
+      <x:c r="M616" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N616" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="617" ht="70" customHeight="1">
+      <x:c r="A617" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B617" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C617" s="169" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D617" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E617" s="169" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F617" s="169" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="G617" s="169" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H617" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I617" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J617" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K617" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L617" s="169" t="str">
+        <x:v>One total dumbbell, not per side.</x:v>
+      </x:c>
+      <x:c r="M617" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N617" s="169" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="618" ht="70" customHeight="1">
+      <x:c r="A618" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B618" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C618" s="169" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="D618" s="169" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E618" s="169" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F618" s="169" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="G618" s="169" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H618" s="169" t="str">
+        <x:v>No human-assisted reps or reported form breakdown</x:v>
+      </x:c>
+      <x:c r="I618" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="J618" s="169" t="str">
+        <x:v>Medium-High start and final</x:v>
+      </x:c>
+      <x:c r="K618" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="L618" s="169" t="str">
+        <x:v>One total dumbbell, not per side.</x:v>
+      </x:c>
+      <x:c r="M618" s="169" t="str">
+        <x:v>Working</x:v>
+      </x:c>
+      <x:c r="N618" s="169" t="n">
         <x:v>2</x:v>
       </x:c>
     </x:row>
@@ -29971,7 +30807,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree5c384ec71f4d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c65015f719a4a68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31807,6 +32643,180 @@
       </x:c>
       <x:c r="I64" s="169" t="str">
         <x:v>Dated revision; prior records retained. Replaced concentration curl; top two sets matched September 5.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="120" customHeight="1">
+      <x:c r="A65" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="B65" s="169" t="str">
+        <x:v>Dumbbell Shoulder Press</x:v>
+      </x:c>
+      <x:c r="C65" s="169" t="str">
+        <x:v>17.5 x12 @3; 20 x12 @3; 22.5 x10 @2; 25 x7 @2</x:v>
+      </x:c>
+      <x:c r="D65" s="169" t="str">
+        <x:v>kg each dumbbell</x:v>
+      </x:c>
+      <x:c r="E65" s="169" t="str">
+        <x:v>17.5 each x12-15 @3; 20 x12-13 @2-3; 22.5 x10-11 @2. Optional 25 x7-8 @2 replaces a set if agreed, not automatically added.</x:v>
+      </x:c>
+      <x:c r="F65" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G65" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H65" s="169" t="str">
+        <x:v>2026-09-16 targets</x:v>
+      </x:c>
+      <x:c r="I65" s="169" t="str">
+        <x:v>Dated session results, not lifetime bests; prior records retained. Four working sets; no warm-up reported. Hold load and rebuild reps.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="120" customHeight="1">
+      <x:c r="A66" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="B66" s="169" t="str">
+        <x:v>Plate-Loaded Lateral Raise Machine</x:v>
+      </x:c>
+      <x:c r="C66" s="169" t="str">
+        <x:v>2.5 x20 @3; 5 x14 @3; 7.5 x10 @2</x:v>
+      </x:c>
+      <x:c r="D66" s="169" t="str">
+        <x:v>kg plate each side; unloaded resistance To verify</x:v>
+      </x:c>
+      <x:c r="E66" s="169" t="str">
+        <x:v>2.5/side x15-20 @3; 5 x14-15 @2-3; 7.5 x10-11 @2. Hold load.</x:v>
+      </x:c>
+      <x:c r="F66" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G66" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H66" s="169" t="str">
+        <x:v>2026-09-16 targets</x:v>
+      </x:c>
+      <x:c r="I66" s="169" t="str">
+        <x:v>Dated session results, not lifetime bests; prior records retained. Same established per-side convention; starting resistance excluded.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="120" customHeight="1">
+      <x:c r="A67" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="B67" s="169" t="str">
+        <x:v>Reverse Pec Deck</x:v>
+      </x:c>
+      <x:c r="C67" s="169" t="str">
+        <x:v>30 x15 @3; 35 x12 @2; 40 x8 @2</x:v>
+      </x:c>
+      <x:c r="D67" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="E67" s="169" t="str">
+        <x:v>30 x15 @3; 35 x12-13 @2; 40 x8-9 @2 if three sets agreed.</x:v>
+      </x:c>
+      <x:c r="F67" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G67" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H67" s="169" t="str">
+        <x:v>2026-09-16 targets</x:v>
+      </x:c>
+      <x:c r="I67" s="169" t="str">
+        <x:v>Dated session results, not lifetime bests; prior records retained. Controlled work with reserve; no pain reported.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="120" customHeight="1">
+      <x:c r="A68" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="B68" s="169" t="str">
+        <x:v>Rope Pushdown</x:v>
+      </x:c>
+      <x:c r="C68" s="169" t="str">
+        <x:v>30 x17 @2; 35 x11 @2; 40 x9 @3</x:v>
+      </x:c>
+      <x:c r="D68" s="169" t="str">
+        <x:v>kg total stack</x:v>
+      </x:c>
+      <x:c r="E68" s="169" t="str">
+        <x:v>30 x15-17 @3; 35 x11-13 @2; 40 x9-10 @2-3 if third set agreed.</x:v>
+      </x:c>
+      <x:c r="F68" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G68" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H68" s="169" t="str">
+        <x:v>2026-09-16 targets</x:v>
+      </x:c>
+      <x:c r="I68" s="169" t="str">
+        <x:v>Dated session results, not lifetime bests; prior records retained. Retain actual reported RIR even though top set had more reserve.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="120" customHeight="1">
+      <x:c r="A69" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="B69" s="169" t="str">
+        <x:v>Single-Arm Cable Pushdown</x:v>
+      </x:c>
+      <x:c r="C69" s="169" t="str">
+        <x:v>5 x20 @3; 10 x15 @3; 15 x11 @3</x:v>
+      </x:c>
+      <x:c r="D69" s="169" t="str">
+        <x:v>kg stack setting each arm</x:v>
+      </x:c>
+      <x:c r="E69" s="169" t="str">
+        <x:v>10 each arm x15 @3; 15 x11-12 @2-3. 5 kg preparation only if genuinely easy.</x:v>
+      </x:c>
+      <x:c r="F69" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G69" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H69" s="169" t="str">
+        <x:v>2026-09-16 targets</x:v>
+      </x:c>
+      <x:c r="I69" s="169" t="str">
+        <x:v>Dated session results, not lifetime bests; prior records retained. Both arms same reps confirmed. Paired sets counted once, not doubled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="120" customHeight="1">
+      <x:c r="A70" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="B70" s="169" t="str">
+        <x:v>Seated Two-Hand Overhead Dumbbell Extension</x:v>
+      </x:c>
+      <x:c r="C70" s="169" t="str">
+        <x:v>20 x15 @3; 25 x12 @2; 30 x8 @2</x:v>
+      </x:c>
+      <x:c r="D70" s="169" t="str">
+        <x:v>kg one dumbbell held with both hands</x:v>
+      </x:c>
+      <x:c r="E70" s="169" t="str">
+        <x:v>20 total x15 @3; 25 x12-13 @2; 30 x8-9 @2 if third set agreed. Hold load.</x:v>
+      </x:c>
+      <x:c r="F70" s="169" t="str">
+        <x:v>Progress reps/reserve before load; agree set count first</x:v>
+      </x:c>
+      <x:c r="G70" s="169" t="str">
+        <x:v>Controlled pain-free motion</x:v>
+      </x:c>
+      <x:c r="H70" s="169" t="str">
+        <x:v>2026-09-16 targets</x:v>
+      </x:c>
+      <x:c r="I70" s="169" t="str">
+        <x:v>Dated session results, not lifetime bests; prior records retained. One total dumbbell, not per side.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -31834,7 +32844,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd98b03e69e0649a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d6c5a96906c470c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33049,17 +34059,29 @@
       <x:c r="P36" s="59" t="n"/>
       <x:c r="Q36" s="59" t="n"/>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37"/>
-      <x:c r="B37"/>
-      <x:c r="C37"/>
-      <x:c r="D37"/>
-      <x:c r="E37"/>
-      <x:c r="F37"/>
-      <x:c r="G37"/>
-      <x:c r="H37"/>
-      <x:c r="I37"/>
-      <x:c r="J37"/>
+    <x:row r="37" ht="260" customHeight="1">
+      <x:c r="A37" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B37" s="169"/>
+      <x:c r="C37" s="169"/>
+      <x:c r="D37" s="169" t="str">
+        <x:v>Good</x:v>
+      </x:c>
+      <x:c r="E37" s="169" t="str">
+        <x:v>Medium to High final (initially Medium)</x:v>
+      </x:c>
+      <x:c r="F37" s="169" t="str">
+        <x:v>No headache, head pressure, dizziness, neck discomfort or joint/other pain</x:v>
+      </x:c>
+      <x:c r="G37" s="169"/>
+      <x:c r="H37" s="169"/>
+      <x:c r="I37" s="169" t="str">
+        <x:v>15 min treadmill; average 3.3 km/h; 12% incline; no rail support</x:v>
+      </x:c>
+      <x:c r="J37" s="169" t="str">
+        <x:v>90 minutes including 15 min treadmill at average 3.3 km/h, 12% incline, no rail support. Good sleep; Medium-High starting energy; final energy Medium to High (initially described Medium); Very good pump. No headache, head pressure, dizziness, neck or joint pain, human-assisted reps or form breakdown. No core reported. Full EAA+ (100 mg label-verified caffeine) plus half pre-workout (~100 mg user-stated); ~200 mg combined caffeine estimate, pre-workout label To verify. No coffee. Creatine/magnesium today To verify.</x:v>
+      </x:c>
       <x:c r="K37" s="59" t="n"/>
       <x:c r="L37" s="59" t="n"/>
       <x:c r="M37" s="59" t="n"/>
@@ -36221,7 +37243,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R011ecc6536264b36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4145049525714b93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -37810,13 +38832,69 @@
         <x:v>Use matching historical exercise baselines and exact load basis before each exercise.</x:v>
       </x:c>
     </x:row>
+    <x:row r="109" ht="180" customHeight="1">
+      <x:c r="A109" s="169" t="str">
+        <x:v>2026-09-16 completion</x:v>
+      </x:c>
+      <x:c r="B109" s="169" t="str">
+        <x:v>19 working sets across six exercises: ten shoulders and nine direct triceps. No warm-up sets reported. Ten sets at RIR 3 and nine at RIR 2. Lateral raise 7.5/side x10 @2 is two reps above September 2; overhead dumbbell 30 x8 @2 is one rep above. Shoulder press 25 x7 @2 remains below prior x9 @2. Symptom-free completion and good remaining energy are encouraging; delayed recovery is pending. Actual 19 sets exceeded the initial 15-set plan; agree volume upfront using weekly workload and recovery, not an arbitrary safety cutoff.</x:v>
+      </x:c>
+      <x:c r="C109" s="169" t="str">
+        <x:v>Self-reported symptom-free completion is encouraging; delayed recovery is not yet known.</x:v>
+      </x:c>
+      <x:c r="D109" s="169" t="str">
+        <x:v>Review next-morning symptoms, sleep, energy and soreness.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="180" customHeight="1">
+      <x:c r="A110" s="169" t="str">
+        <x:v>2026-09-16 treadmill habit</x:v>
+      </x:c>
+      <x:c r="B110" s="169" t="str">
+        <x:v>User explicitly confirms no rail support today and says he never uses it.</x:v>
+      </x:c>
+      <x:c r="C110" s="169" t="str">
+        <x:v>Standing self-reported habit, not retrospective verification of every older session.</x:v>
+      </x:c>
+      <x:c r="D110" s="169" t="str">
+        <x:v>Preserve older uncertain entries unchanged; record rail status for future sessions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="180" customHeight="1">
+      <x:c r="A111" s="169" t="str">
+        <x:v>2026-09-16 supplements</x:v>
+      </x:c>
+      <x:c r="B111" s="169" t="str">
+        <x:v>Full EAA+ (100 mg label-verified caffeine) plus half pre-workout (~100 mg user-stated); ~200 mg combined caffeine estimate, pre-workout label To verify. No coffee. Creatine/magnesium today To verify.</x:v>
+      </x:c>
+      <x:c r="C111" s="169" t="str">
+        <x:v>Pre-workout caffeine amount is not independently label-verified.</x:v>
+      </x:c>
+      <x:c r="D111" s="169" t="str">
+        <x:v>Obtain product label; track sleep response without inferring causation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="180" customHeight="1">
+      <x:c r="A112" s="169" t="str">
+        <x:v>2026-09-16 next session</x:v>
+      </x:c>
+      <x:c r="B112" s="169" t="str">
+        <x:v>Thursday Legs + Calves next after fresh sleep, energy, soreness and head/neck symptom check. Preserve goal of stronger legs and fuller thighs. Agree sets and cardio before lifting; use most working sets at RIR 2-3 without forced reps. Hold shoulder/triceps loads and build controlled reps. No automatic increases.</x:v>
+      </x:c>
+      <x:c r="C112" s="169" t="str">
+        <x:v>Third consecutive return-week session completed.</x:v>
+      </x:c>
+      <x:c r="D112" s="169" t="str">
+        <x:v>Use matching historical exercise baselines and exact load basis before each exercise.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa26f63aa8b4fba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc09a2c7442d4c06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38719,6 +39797,32 @@
         <x:v>Shoulders + Triceps next after fresh sleep, energy, soreness and head/neck symptom check. Agree exercise count, sets and substitutions before lifting; consider recent pressing/arm workload. Keep most sets at RIR 2-3, no forced reps; adjust to observed recovery, not energy alone. No automatic load increases.</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="250" customHeight="1">
+      <x:c r="A35" s="380" t="n">
+        <x:v>46281</x:v>
+      </x:c>
+      <x:c r="B35" s="169" t="str">
+        <x:v>Shoulders + Triceps</x:v>
+      </x:c>
+      <x:c r="C35" s="169" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D35" s="169" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E35" s="169" t="str">
+        <x:v>Symptom-free / monitor recovery</x:v>
+      </x:c>
+      <x:c r="F35" s="169" t="str">
+        <x:v>90 minutes including 15 min treadmill at average 3.3 km/h, 12% incline, no rail support. Good sleep; Medium-High starting energy; final energy Medium to High (initially described Medium); Very good pump. No headache, head pressure, dizziness, neck or joint pain, human-assisted reps or form breakdown. No core reported. Full EAA+ (100 mg label-verified caffeine) plus half pre-workout (~100 mg user-stated); ~200 mg combined caffeine estimate, pre-workout label To verify. No coffee. Creatine/magnesium today To verify.</x:v>
+      </x:c>
+      <x:c r="G35" s="169" t="str">
+        <x:v>19 working sets across six exercises: ten shoulders and nine direct triceps. No warm-up sets reported. Ten sets at RIR 3 and nine at RIR 2. Lateral raise 7.5/side x10 @2 is two reps above September 2; overhead dumbbell 30 x8 @2 is one rep above. Shoulder press 25 x7 @2 remains below prior x9 @2. Symptom-free completion and good remaining energy are encouraging; delayed recovery is pending. Actual 19 sets exceeded the initial 15-set plan; agree volume upfront using weekly workload and recovery, not an arbitrary safety cutoff.</x:v>
+      </x:c>
+      <x:c r="H35" s="169" t="str">
+        <x:v>Thursday Legs + Calves next after fresh sleep, energy, soreness and head/neck symptom check. Preserve goal of stronger legs and fuller thighs. Agree sets and cardio before lifting; use most working sets at RIR 2-3 without forced reps. Hold shoulder/triceps loads and build controlled reps. No automatic increases.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
@@ -38731,7 +39835,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc73b386cfd4c2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55d8064a39694e69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39301,7 +40405,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fca50a8a96c4eb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc6d1ed100c54046"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40407,10 +41511,10 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf817f55a144e4cf5"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab66aed30cb34a13"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d8165eb7366495a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc34d5cecc9344e46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba5179200eb64411"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9cf8dcc019d4918"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra774d94ae31441a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c6c9bc8ac343a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>